<commit_message>
added evaluation loading to all examples and updated results sheet
</commit_message>
<xml_diff>
--- a/results/compiled results.xlsx
+++ b/results/compiled results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\elish\Desktop\Aims Project\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2650DEAD-700D-4576-9CE9-D084CBF64DA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF659FA7-A9AD-48FF-A05A-A03CC0C9EDC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{DA4D96B0-492C-4945-A9C4-EFCA6D6BC722}"/>
+    <workbookView xWindow="4752" yWindow="3240" windowWidth="17280" windowHeight="8880" xr2:uid="{DA4D96B0-492C-4945-A9C4-EFCA6D6BC722}"/>
   </bookViews>
   <sheets>
     <sheet name="dynamic v2 " sheetId="1" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="49">
   <si>
     <t xml:space="preserve">Model </t>
   </si>
@@ -185,6 +185,18 @@
   </si>
   <si>
     <t>CIA ee</t>
+  </si>
+  <si>
+    <t>EE Min (x,y,z)</t>
+  </si>
+  <si>
+    <t>EE Max (x,y,z)</t>
+  </si>
+  <si>
+    <t>WB Min (x,y,z)</t>
+  </si>
+  <si>
+    <t>WB Max (x,y,z)</t>
   </si>
 </sst>
 </file>
@@ -217,9 +229,58 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="6">
     <border>
       <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
       <right/>
       <top/>
       <bottom/>
@@ -229,21 +290,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -258,6 +312,42 @@
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -599,779 +689,779 @@
     <col min="1" max="1" width="15.5546875" customWidth="1"/>
     <col min="2" max="2" width="8.77734375" style="1" customWidth="1"/>
     <col min="3" max="13" width="8.88671875" style="1"/>
-    <col min="14" max="14" width="14.88671875" style="5" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.33203125" style="6" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="10.21875" style="6" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="17.21875" style="6" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="15" style="6" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.33203125" style="7" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="15.44140625" style="7" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="14.33203125" style="6" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="10.109375" style="7" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="12.33203125" style="6" customWidth="1"/>
-    <col min="24" max="24" width="5.109375" style="6" customWidth="1"/>
-    <col min="25" max="25" width="10.109375" style="6" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="10.88671875" style="6" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="7.109375" style="6" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="14" style="6" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="8.5546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="14.88671875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.33203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="10.21875" style="3" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="17.21875" style="3" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="15" style="3" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="15.44140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="14.33203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="10.109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="12.33203125" style="3" customWidth="1"/>
+    <col min="24" max="24" width="5.109375" style="3" customWidth="1"/>
+    <col min="25" max="25" width="10.109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="10.88671875" style="3" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="7.109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="14" style="3" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="8.5546875" style="2" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:29" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
-      <c r="K1" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="L1" s="4"/>
-      <c r="M1" s="4"/>
+      <c r="A1" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="16" t="s">
+        <v>45</v>
+      </c>
+      <c r="C1" s="17"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="F1" s="17"/>
+      <c r="G1" s="18"/>
+      <c r="H1" s="17" t="s">
+        <v>47</v>
+      </c>
+      <c r="I1" s="17"/>
+      <c r="J1" s="18"/>
+      <c r="K1" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="L1" s="17"/>
+      <c r="M1" s="18"/>
     </row>
     <row r="2" spans="1:29" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2" s="10">
         <v>0.270000010728836</v>
       </c>
-      <c r="C2" s="3">
+      <c r="C2" s="2">
         <v>0.34999999403953502</v>
       </c>
-      <c r="D2" s="3">
+      <c r="D2" s="9">
         <v>0.34999999403953502</v>
       </c>
-      <c r="E2" s="3">
+      <c r="E2" s="2">
         <v>0.46999999880790699</v>
       </c>
-      <c r="F2" s="3">
+      <c r="F2" s="2">
         <v>0.62999999523162797</v>
       </c>
-      <c r="G2" s="3">
+      <c r="G2" s="9">
         <v>0.55000001192092896</v>
       </c>
-      <c r="H2" s="3">
+      <c r="H2" s="2">
         <v>-0.855000019073486</v>
       </c>
-      <c r="I2" s="3">
+      <c r="I2" s="2">
         <v>-0.855000019073486</v>
       </c>
-      <c r="J2" s="3">
+      <c r="J2" s="9">
         <v>-0.10000000149011599</v>
       </c>
-      <c r="K2" s="3">
+      <c r="K2" s="11">
         <v>0.855000019073486</v>
       </c>
-      <c r="L2" s="3">
+      <c r="L2" s="2">
         <v>0.855000019073486</v>
       </c>
-      <c r="M2" s="3">
+      <c r="M2" s="9">
         <v>1.1900000572204501</v>
       </c>
     </row>
     <row r="3" spans="1:29" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="A3" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B3" s="11">
         <v>0.270000010728836</v>
       </c>
-      <c r="C3" s="3">
+      <c r="C3" s="2">
         <v>0.34999999403953502</v>
       </c>
-      <c r="D3" s="3">
+      <c r="D3" s="9">
         <v>0.34999999403953502</v>
       </c>
-      <c r="E3" s="3">
+      <c r="E3" s="2">
         <v>0.46999999880790699</v>
       </c>
-      <c r="F3" s="3">
+      <c r="F3" s="2">
         <v>0.62999999523162797</v>
       </c>
-      <c r="G3" s="3">
+      <c r="G3" s="9">
         <v>0.55000001192092896</v>
       </c>
-      <c r="H3" s="3">
+      <c r="H3" s="2">
         <v>-0.855000019073486</v>
       </c>
-      <c r="I3" s="3">
+      <c r="I3" s="2">
         <v>-0.855000019073486</v>
       </c>
-      <c r="J3" s="3">
+      <c r="J3" s="9">
         <v>-0.10000000149011599</v>
       </c>
-      <c r="K3" s="3">
+      <c r="K3" s="11">
         <v>0.855000019073486</v>
       </c>
-      <c r="L3" s="3">
+      <c r="L3" s="2">
         <v>0.855000019073486</v>
       </c>
-      <c r="M3" s="3">
+      <c r="M3" s="9">
         <v>1.1900000572204501</v>
       </c>
     </row>
     <row r="4" spans="1:29" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+      <c r="A4" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B4" s="11">
         <v>0.270000010728836</v>
       </c>
-      <c r="C4" s="3">
+      <c r="C4" s="2">
         <v>0.20000000298023199</v>
       </c>
-      <c r="D4" s="3">
+      <c r="D4" s="9">
         <v>0.34999999403953502</v>
       </c>
-      <c r="E4" s="3">
+      <c r="E4" s="2">
         <v>0.46999999880790699</v>
       </c>
-      <c r="F4" s="3">
+      <c r="F4" s="2">
         <v>0.77999997138976995</v>
       </c>
-      <c r="G4" s="3">
+      <c r="G4" s="9">
         <v>0.55000001192092896</v>
       </c>
-      <c r="H4" s="3">
+      <c r="H4" s="2">
         <v>-0.855000019073486</v>
       </c>
-      <c r="I4" s="3">
+      <c r="I4" s="2">
         <v>-0.855000019073486</v>
       </c>
-      <c r="J4" s="3">
+      <c r="J4" s="9">
         <v>-0.10000000149011599</v>
       </c>
-      <c r="K4" s="3">
+      <c r="K4" s="11">
         <v>0.855000019073486</v>
       </c>
-      <c r="L4" s="3">
+      <c r="L4" s="2">
         <v>0.855000019073486</v>
       </c>
-      <c r="M4" s="3">
+      <c r="M4" s="9">
         <v>1.1900000572204501</v>
       </c>
     </row>
     <row r="5" spans="1:29" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+      <c r="A5" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="3">
+      <c r="B5" s="11">
         <v>5.9999998658895402E-2</v>
       </c>
-      <c r="C5" s="3">
+      <c r="C5" s="2">
         <v>0.15000000596046401</v>
       </c>
-      <c r="D5" s="3">
+      <c r="D5" s="9">
         <v>0.25</v>
       </c>
-      <c r="E5" s="3">
+      <c r="E5" s="2">
         <v>0.46000000834464999</v>
       </c>
-      <c r="F5" s="3">
+      <c r="F5" s="2">
         <v>0.82999998331069902</v>
       </c>
-      <c r="G5" s="3">
+      <c r="G5" s="9">
         <v>0.64999997615814198</v>
       </c>
-      <c r="H5" s="3">
-        <v>0</v>
-      </c>
-      <c r="I5" s="3">
-        <v>0</v>
-      </c>
-      <c r="J5" s="3">
+      <c r="H5" s="2">
+        <v>0</v>
+      </c>
+      <c r="I5" s="2">
+        <v>0</v>
+      </c>
+      <c r="J5" s="9">
         <v>0.15000000596046401</v>
       </c>
-      <c r="K5" s="3">
+      <c r="K5" s="11">
         <v>0.30000001192092801</v>
       </c>
-      <c r="L5" s="3">
+      <c r="L5" s="2">
         <v>0.30000001192092801</v>
       </c>
-      <c r="M5" s="3">
+      <c r="M5" s="9">
         <v>0.44999998807907099</v>
       </c>
     </row>
     <row r="6" spans="1:29" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
+      <c r="A6" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="3">
+      <c r="B6" s="11">
         <v>0.17000000178813901</v>
       </c>
-      <c r="C6" s="3">
+      <c r="C6" s="2">
         <v>0.15000000596046401</v>
       </c>
-      <c r="D6" s="3">
+      <c r="D6" s="9">
         <v>0.25</v>
       </c>
-      <c r="E6" s="3">
+      <c r="E6" s="2">
         <v>0.56999999284744196</v>
       </c>
-      <c r="F6" s="3">
+      <c r="F6" s="2">
         <v>0.82999998331069902</v>
       </c>
-      <c r="G6" s="3">
+      <c r="G6" s="9">
         <v>0.64999997615814198</v>
       </c>
-      <c r="H6" s="3">
+      <c r="H6" s="2">
         <v>-0.855000019073486</v>
       </c>
-      <c r="I6" s="3">
+      <c r="I6" s="2">
         <v>-0.855000019073486</v>
       </c>
-      <c r="J6" s="3">
+      <c r="J6" s="9">
         <v>-0.10000000149011599</v>
       </c>
-      <c r="K6" s="3">
+      <c r="K6" s="11">
         <v>0.855000019073486</v>
       </c>
-      <c r="L6" s="3">
+      <c r="L6" s="2">
         <v>0.855000019073486</v>
       </c>
-      <c r="M6" s="3">
+      <c r="M6" s="9">
         <v>1.1900000572204501</v>
       </c>
     </row>
     <row r="7" spans="1:29" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+      <c r="A7" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="3">
+      <c r="B7" s="11">
         <v>0.17000000178813901</v>
       </c>
-      <c r="C7" s="3">
+      <c r="C7" s="2">
         <v>0.15000000596046401</v>
       </c>
-      <c r="D7" s="3">
+      <c r="D7" s="9">
         <v>0.25</v>
       </c>
-      <c r="E7" s="3">
+      <c r="E7" s="2">
         <v>0.56999999284744196</v>
       </c>
-      <c r="F7" s="3">
+      <c r="F7" s="2">
         <v>0.82999998331069902</v>
       </c>
-      <c r="G7" s="3">
+      <c r="G7" s="9">
         <v>0.64999997615814198</v>
       </c>
-      <c r="H7" s="3">
+      <c r="H7" s="2">
         <v>-0.855000019073486</v>
       </c>
-      <c r="I7" s="3">
+      <c r="I7" s="2">
         <v>-0.855000019073486</v>
       </c>
-      <c r="J7" s="3">
+      <c r="J7" s="9">
         <v>-0.10000000149011599</v>
       </c>
-      <c r="K7" s="3">
+      <c r="K7" s="11">
         <v>0.855000019073486</v>
       </c>
-      <c r="L7" s="3">
+      <c r="L7" s="2">
         <v>0.855000019073486</v>
       </c>
-      <c r="M7" s="3">
+      <c r="M7" s="9">
         <v>1.1900000572204501</v>
       </c>
     </row>
     <row r="8" spans="1:29" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
+      <c r="A8" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="B8" s="3">
+      <c r="B8" s="11">
         <v>0.17000000178813901</v>
       </c>
-      <c r="C8" s="3">
+      <c r="C8" s="2">
         <v>0.15000000596046401</v>
       </c>
-      <c r="D8" s="3">
+      <c r="D8" s="9">
         <v>0.25</v>
       </c>
-      <c r="E8" s="3">
+      <c r="E8" s="2">
         <v>0.56999999284744196</v>
       </c>
-      <c r="F8" s="3">
+      <c r="F8" s="2">
         <v>0.82999998331069902</v>
       </c>
-      <c r="G8" s="3">
+      <c r="G8" s="9">
         <v>0.64999997615814198</v>
       </c>
-      <c r="H8" s="3">
-        <v>0</v>
-      </c>
-      <c r="I8" s="3">
-        <v>0</v>
-      </c>
-      <c r="J8" s="3">
-        <v>0</v>
-      </c>
-      <c r="K8" s="3">
+      <c r="H8" s="2">
+        <v>0</v>
+      </c>
+      <c r="I8" s="2">
+        <v>0</v>
+      </c>
+      <c r="J8" s="9">
+        <v>0</v>
+      </c>
+      <c r="K8" s="11">
         <v>0.60000002384185702</v>
       </c>
-      <c r="L8" s="3">
+      <c r="L8" s="2">
         <v>0.89999997615814198</v>
       </c>
-      <c r="M8" s="3">
+      <c r="M8" s="9">
         <v>0.69999998807907104</v>
       </c>
     </row>
     <row r="9" spans="1:29" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
+      <c r="A9" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="3">
+      <c r="B9" s="12">
         <v>0.17000000178813901</v>
       </c>
-      <c r="C9" s="3">
+      <c r="C9" s="13">
         <v>0.15000000596046401</v>
       </c>
-      <c r="D9" s="3">
+      <c r="D9" s="14">
         <v>0.25</v>
       </c>
-      <c r="E9" s="3">
+      <c r="E9" s="13">
         <v>0.56999999284744196</v>
       </c>
-      <c r="F9" s="3">
+      <c r="F9" s="13">
         <v>0.82999998331069902</v>
       </c>
-      <c r="G9" s="3">
+      <c r="G9" s="14">
         <v>0.64999997615814198</v>
       </c>
-      <c r="H9" s="3">
+      <c r="H9" s="13">
         <v>-0.855000019073486</v>
       </c>
-      <c r="I9" s="3">
+      <c r="I9" s="13">
         <v>-0.855000019073486</v>
       </c>
-      <c r="J9" s="3">
+      <c r="J9" s="14">
         <v>-0.10000000149011599</v>
       </c>
-      <c r="K9" s="3">
+      <c r="K9" s="12">
         <v>0.855000019073486</v>
       </c>
-      <c r="L9" s="3">
+      <c r="L9" s="13">
         <v>0.855000019073486</v>
       </c>
-      <c r="M9" s="3">
+      <c r="M9" s="14">
         <v>1.1900000572204501</v>
       </c>
     </row>
     <row r="13" spans="1:29" x14ac:dyDescent="0.3">
-      <c r="O13" s="8" t="s">
+      <c r="O13" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="P13" s="8" t="s">
+      <c r="P13" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="Q13" s="8" t="s">
+      <c r="Q13" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="R13" s="8" t="s">
+      <c r="R13" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="S13" s="9" t="s">
+      <c r="S13" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="T13" s="9" t="s">
+      <c r="T13" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="U13" s="8" t="s">
+      <c r="U13" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="V13" s="9" t="s">
+      <c r="V13" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="W13" s="8" t="s">
+      <c r="W13" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="X13" s="8" t="s">
+      <c r="X13" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="Y13" s="8" t="s">
+      <c r="Y13" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="Z13" s="8" t="s">
+      <c r="Z13" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="AA13" s="8" t="s">
+      <c r="AA13" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="AB13" s="8" t="s">
+      <c r="AB13" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="AC13" s="10" t="s">
+      <c r="AC13" s="7" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="14" spans="1:29" x14ac:dyDescent="0.3">
-      <c r="N14" s="5" t="s">
+      <c r="N14" t="s">
         <v>21</v>
       </c>
-      <c r="O14" s="6" t="s">
+      <c r="O14" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="P14" s="6" t="s">
+      <c r="P14" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="Q14" s="6" t="s">
+      <c r="Q14" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="R14" s="6" t="s">
+      <c r="R14" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="S14" s="7" t="s">
+      <c r="S14" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="T14" s="7" t="s">
+      <c r="T14" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="U14" s="6" t="s">
+      <c r="U14" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="V14" s="7" t="s">
+      <c r="V14" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="W14" s="6" t="s">
+      <c r="W14" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="X14" s="6" t="s">
+      <c r="X14" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="Y14" s="6" t="s">
+      <c r="Y14" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="Z14" s="6" t="s">
+      <c r="Z14" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="AA14" s="6" t="s">
+      <c r="AA14" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="AB14" s="6" t="s">
+      <c r="AB14" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="AC14" s="3" t="s">
+      <c r="AC14" s="2" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="15" spans="1:29" x14ac:dyDescent="0.3">
-      <c r="N15" s="5" t="s">
+      <c r="N15" t="s">
         <v>39</v>
       </c>
-      <c r="O15" s="6">
+      <c r="O15" s="3">
         <v>2.0934814092646199E-2</v>
       </c>
-      <c r="P15" s="6">
+      <c r="P15" s="3">
         <v>6.9102947542359794E-2</v>
       </c>
-      <c r="Q15" s="6">
+      <c r="Q15" s="3">
         <v>3.4711742221484802E-3</v>
       </c>
-      <c r="R15" s="6">
+      <c r="R15" s="3">
         <v>5.1547613905872898E-3</v>
       </c>
-      <c r="S15" s="7">
-        <v>0</v>
-      </c>
-      <c r="T15" s="7">
-        <v>0</v>
-      </c>
-      <c r="U15" s="6">
-        <v>0</v>
-      </c>
-      <c r="V15" s="7">
-        <v>0</v>
-      </c>
-      <c r="Y15" s="6">
+      <c r="S15" s="4">
+        <v>0</v>
+      </c>
+      <c r="T15" s="4">
+        <v>0</v>
+      </c>
+      <c r="U15" s="3">
+        <v>0</v>
+      </c>
+      <c r="V15" s="4">
+        <v>0</v>
+      </c>
+      <c r="Y15" s="3">
         <v>1.2800000000000001E-2</v>
       </c>
-      <c r="Z15" s="6">
+      <c r="Z15" s="3">
         <v>3.7720889999999998</v>
       </c>
-      <c r="AA15" s="6">
+      <c r="AA15" s="3">
         <v>10.6272727272727</v>
       </c>
-      <c r="AB15" s="6">
+      <c r="AB15" s="3">
         <v>1.169</v>
       </c>
-      <c r="AC15" s="3">
+      <c r="AC15" s="2">
         <v>13031.0716310962</v>
       </c>
     </row>
     <row r="16" spans="1:29" x14ac:dyDescent="0.3">
-      <c r="N16" s="5" t="s">
+      <c r="N16" t="s">
         <v>38</v>
       </c>
-      <c r="O16" s="6">
+      <c r="O16" s="3">
         <v>2.15380052361E-2</v>
       </c>
-      <c r="P16" s="6">
+      <c r="P16" s="3">
         <v>7.1027378762642202E-2</v>
       </c>
-      <c r="Q16" s="6">
+      <c r="Q16" s="3">
         <v>3.5160645750315399E-3</v>
       </c>
-      <c r="R16" s="6">
+      <c r="R16" s="3">
         <v>5.3275300875990804E-3</v>
       </c>
-      <c r="S16" s="7">
-        <v>0</v>
-      </c>
-      <c r="T16" s="7">
-        <v>0</v>
-      </c>
-      <c r="U16" s="6">
-        <v>0</v>
-      </c>
-      <c r="V16" s="7">
-        <v>0</v>
-      </c>
-      <c r="Y16" s="6">
+      <c r="S16" s="4">
+        <v>0</v>
+      </c>
+      <c r="T16" s="4">
+        <v>0</v>
+      </c>
+      <c r="U16" s="3">
+        <v>0</v>
+      </c>
+      <c r="V16" s="4">
+        <v>0</v>
+      </c>
+      <c r="Y16" s="3">
         <v>2.3199999999999998E-2</v>
       </c>
-      <c r="Z16" s="6">
+      <c r="Z16" s="3">
         <v>3.81633599999999</v>
       </c>
-      <c r="AA16" s="6">
+      <c r="AA16" s="3">
         <v>9.4181818181818109</v>
       </c>
-      <c r="AB16" s="6">
+      <c r="AB16" s="3">
         <v>1.036</v>
       </c>
-      <c r="AC16" s="3">
+      <c r="AC16" s="2">
         <v>12973.6600451822</v>
       </c>
     </row>
     <row r="17" spans="14:29" x14ac:dyDescent="0.3">
-      <c r="N17" s="5" t="s">
+      <c r="N17" t="s">
         <v>37</v>
       </c>
-      <c r="O17" s="6">
+      <c r="O17" s="3">
         <v>2.15380070530449E-2</v>
       </c>
-      <c r="P17" s="6">
+      <c r="P17" s="3">
         <v>7.1027379034489802E-2</v>
       </c>
-      <c r="Q17" s="6">
+      <c r="Q17" s="3">
         <v>3.5160658977784098E-3</v>
       </c>
-      <c r="R17" s="6">
+      <c r="R17" s="3">
         <v>5.3275314460857499E-3</v>
       </c>
-      <c r="S17" s="7">
-        <v>0</v>
-      </c>
-      <c r="T17" s="7">
-        <v>0</v>
-      </c>
-      <c r="U17" s="6">
-        <v>0</v>
-      </c>
-      <c r="V17" s="7">
+      <c r="S17" s="4">
+        <v>0</v>
+      </c>
+      <c r="T17" s="4">
+        <v>0</v>
+      </c>
+      <c r="U17" s="3">
+        <v>0</v>
+      </c>
+      <c r="V17" s="4">
         <v>100</v>
       </c>
-      <c r="Y17" s="6">
+      <c r="Y17" s="3">
         <v>2.7199999999999998E-2</v>
       </c>
-      <c r="Z17" s="6">
+      <c r="Z17" s="3">
         <v>0.79200000000000004</v>
       </c>
-      <c r="AA17" s="6">
+      <c r="AA17" s="3">
         <v>9.4363636363636303</v>
       </c>
-      <c r="AB17" s="6">
+      <c r="AB17" s="3">
         <v>1.038</v>
       </c>
-      <c r="AC17" s="3">
+      <c r="AC17" s="2">
         <v>12973.6597628543</v>
       </c>
     </row>
     <row r="18" spans="14:29" x14ac:dyDescent="0.3">
-      <c r="N18" s="5" t="s">
+      <c r="N18" t="s">
         <v>40</v>
       </c>
-      <c r="O18" s="6">
+      <c r="O18" s="3">
         <v>2.1538025413604299E-2</v>
       </c>
-      <c r="P18" s="6">
+      <c r="P18" s="3">
         <v>7.1027374073324795E-2</v>
       </c>
-      <c r="Q18" s="6">
+      <c r="Q18" s="3">
         <v>3.51608576948721E-3</v>
       </c>
-      <c r="R18" s="6">
+      <c r="R18" s="3">
         <v>5.3275228677729302E-3</v>
       </c>
-      <c r="S18" s="7">
-        <v>0</v>
-      </c>
-      <c r="T18" s="7">
-        <v>0</v>
-      </c>
-      <c r="U18" s="6">
-        <v>0</v>
-      </c>
-      <c r="V18" s="7">
-        <v>0</v>
-      </c>
-      <c r="Y18" s="6">
+      <c r="S18" s="4">
+        <v>0</v>
+      </c>
+      <c r="T18" s="4">
+        <v>0</v>
+      </c>
+      <c r="U18" s="3">
+        <v>0</v>
+      </c>
+      <c r="V18" s="4">
+        <v>0</v>
+      </c>
+      <c r="Y18" s="3">
         <v>0.10879999999999899</v>
       </c>
-      <c r="Z18" s="6">
+      <c r="Z18" s="3">
         <v>3.81633599999999</v>
       </c>
-      <c r="AA18" s="6">
+      <c r="AA18" s="3">
         <v>9.1999999999999993</v>
       </c>
-      <c r="AB18" s="6">
+      <c r="AB18" s="3">
         <v>1.012</v>
       </c>
-      <c r="AC18" s="3">
+      <c r="AC18" s="2">
         <v>12973.665448292701</v>
       </c>
     </row>
     <row r="19" spans="14:29" x14ac:dyDescent="0.3">
-      <c r="N19" s="5" t="s">
+      <c r="N19" t="s">
         <v>41</v>
       </c>
-      <c r="O19" s="6">
+      <c r="O19" s="3">
         <v>2.1538025413604299E-2</v>
       </c>
-      <c r="P19" s="6">
+      <c r="P19" s="3">
         <v>7.1027374073324795E-2</v>
       </c>
-      <c r="Q19" s="6">
+      <c r="Q19" s="3">
         <v>3.51608576948721E-3</v>
       </c>
-      <c r="R19" s="6">
+      <c r="R19" s="3">
         <v>5.3275228677729302E-3</v>
       </c>
-      <c r="S19" s="7">
-        <v>0</v>
-      </c>
-      <c r="T19" s="7">
-        <v>0</v>
-      </c>
-      <c r="U19" s="6">
-        <v>0</v>
-      </c>
-      <c r="V19" s="7">
-        <v>0</v>
-      </c>
-      <c r="Y19" s="6">
+      <c r="S19" s="4">
+        <v>0</v>
+      </c>
+      <c r="T19" s="4">
+        <v>0</v>
+      </c>
+      <c r="U19" s="3">
+        <v>0</v>
+      </c>
+      <c r="V19" s="4">
+        <v>0</v>
+      </c>
+      <c r="Y19" s="3">
         <v>0.10879999999999899</v>
       </c>
-      <c r="Z19" s="6">
+      <c r="Z19" s="3">
         <v>3.81633599999999</v>
       </c>
-      <c r="AA19" s="6">
+      <c r="AA19" s="3">
         <v>9.1999999999999993</v>
       </c>
-      <c r="AB19" s="6">
+      <c r="AB19" s="3">
         <v>1.012</v>
       </c>
-      <c r="AC19" s="3">
+      <c r="AC19" s="2">
         <v>12973.665448292701</v>
       </c>
     </row>
     <row r="20" spans="14:29" x14ac:dyDescent="0.3">
-      <c r="N20" s="5" t="s">
+      <c r="N20" t="s">
         <v>42</v>
       </c>
-      <c r="O20" s="6">
+      <c r="O20" s="3">
         <v>2.1538025413604299E-2</v>
       </c>
-      <c r="P20" s="6">
+      <c r="P20" s="3">
         <v>7.1027374073324795E-2</v>
       </c>
-      <c r="Q20" s="6">
+      <c r="Q20" s="3">
         <v>3.51608576948721E-3</v>
       </c>
-      <c r="R20" s="6">
+      <c r="R20" s="3">
         <v>5.3275228677729302E-3</v>
       </c>
-      <c r="S20" s="7">
-        <v>0</v>
-      </c>
-      <c r="T20" s="7">
-        <v>0</v>
-      </c>
-      <c r="U20" s="6">
-        <v>0</v>
-      </c>
-      <c r="V20" s="7">
+      <c r="S20" s="4">
+        <v>0</v>
+      </c>
+      <c r="T20" s="4">
+        <v>0</v>
+      </c>
+      <c r="U20" s="3">
+        <v>0</v>
+      </c>
+      <c r="V20" s="4">
         <v>100</v>
       </c>
-      <c r="Y20" s="6">
+      <c r="Y20" s="3">
         <v>0.10879999999999899</v>
       </c>
-      <c r="Z20" s="6">
+      <c r="Z20" s="3">
         <v>0.378</v>
       </c>
-      <c r="AA20" s="6">
+      <c r="AA20" s="3">
         <v>9.1999999999999993</v>
       </c>
-      <c r="AB20" s="6">
+      <c r="AB20" s="3">
         <v>1.012</v>
       </c>
-      <c r="AC20" s="3">
+      <c r="AC20" s="2">
         <v>12973.665448292701</v>
       </c>
     </row>
     <row r="21" spans="14:29" x14ac:dyDescent="0.3">
-      <c r="N21" s="5" t="s">
+      <c r="N21" t="s">
         <v>43</v>
       </c>
-      <c r="O21" s="6">
+      <c r="O21" s="3">
         <v>2.1538025413604299E-2</v>
       </c>
-      <c r="P21" s="6">
+      <c r="P21" s="3">
         <v>7.1027374073324795E-2</v>
       </c>
-      <c r="Q21" s="6">
+      <c r="Q21" s="3">
         <v>3.51608576948721E-3</v>
       </c>
-      <c r="R21" s="6">
+      <c r="R21" s="3">
         <v>5.3275228677729302E-3</v>
       </c>
-      <c r="S21" s="7">
-        <v>0</v>
-      </c>
-      <c r="T21" s="7">
-        <v>0</v>
-      </c>
-      <c r="U21" s="6">
-        <v>0</v>
-      </c>
-      <c r="V21" s="7">
-        <v>0</v>
-      </c>
-      <c r="Y21" s="6">
+      <c r="S21" s="4">
+        <v>0</v>
+      </c>
+      <c r="T21" s="4">
+        <v>0</v>
+      </c>
+      <c r="U21" s="3">
+        <v>0</v>
+      </c>
+      <c r="V21" s="4">
+        <v>0</v>
+      </c>
+      <c r="Y21" s="3">
         <v>0.10879999999999899</v>
       </c>
-      <c r="Z21" s="6">
+      <c r="Z21" s="3">
         <v>3.81633599999999</v>
       </c>
-      <c r="AA21" s="6">
+      <c r="AA21" s="3">
         <v>9.1999999999999993</v>
       </c>
-      <c r="AB21" s="6">
+      <c r="AB21" s="3">
         <v>1.012</v>
       </c>
-      <c r="AC21" s="3">
+      <c r="AC21" s="2">
         <v>12973.665448292701</v>
       </c>
     </row>
@@ -1395,26 +1485,26 @@
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4" t="s">
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4" t="s">
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
-      <c r="K1" s="4" t="s">
+      <c r="I1" s="19"/>
+      <c r="J1" s="19"/>
+      <c r="K1" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="L1" s="4"/>
-      <c r="M1" s="4"/>
+      <c r="L1" s="19"/>
+      <c r="M1" s="19"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
@@ -1471,26 +1561,26 @@
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4" t="s">
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4" t="s">
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
-      <c r="K1" s="4" t="s">
+      <c r="I1" s="19"/>
+      <c r="J1" s="19"/>
+      <c r="K1" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="L1" s="4"/>
-      <c r="M1" s="4"/>
+      <c r="L1" s="19"/>
+      <c r="M1" s="19"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
@@ -1547,26 +1637,26 @@
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4" t="s">
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4" t="s">
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
-      <c r="K1" s="4" t="s">
+      <c r="I1" s="19"/>
+      <c r="J1" s="19"/>
+      <c r="K1" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="L1" s="4"/>
-      <c r="M1" s="4"/>
+      <c r="L1" s="19"/>
+      <c r="M1" s="19"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
@@ -1626,26 +1716,26 @@
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4" t="s">
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4" t="s">
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
-      <c r="K1" s="4" t="s">
+      <c r="I1" s="19"/>
+      <c r="J1" s="19"/>
+      <c r="K1" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="L1" s="4"/>
-      <c r="M1" s="4"/>
+      <c r="L1" s="19"/>
+      <c r="M1" s="19"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
@@ -1705,26 +1795,26 @@
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4" t="s">
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4" t="s">
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
-      <c r="K1" s="4" t="s">
+      <c r="I1" s="19"/>
+      <c r="J1" s="19"/>
+      <c r="K1" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="L1" s="4"/>
-      <c r="M1" s="4"/>
+      <c r="L1" s="19"/>
+      <c r="M1" s="19"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
@@ -1784,26 +1874,26 @@
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4" t="s">
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4" t="s">
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
-      <c r="K1" s="4" t="s">
+      <c r="I1" s="19"/>
+      <c r="J1" s="19"/>
+      <c r="K1" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="L1" s="4"/>
-      <c r="M1" s="4"/>
+      <c r="L1" s="19"/>
+      <c r="M1" s="19"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
@@ -1860,26 +1950,26 @@
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4" t="s">
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4" t="s">
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
-      <c r="K1" s="4" t="s">
+      <c r="I1" s="19"/>
+      <c r="J1" s="19"/>
+      <c r="K1" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="L1" s="4"/>
-      <c r="M1" s="4"/>
+      <c r="L1" s="19"/>
+      <c r="M1" s="19"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
@@ -1936,26 +2026,26 @@
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4" t="s">
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4" t="s">
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
-      <c r="K1" s="4" t="s">
+      <c r="I1" s="19"/>
+      <c r="J1" s="19"/>
+      <c r="K1" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="L1" s="4"/>
-      <c r="M1" s="4"/>
+      <c r="L1" s="19"/>
+      <c r="M1" s="19"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
@@ -2012,26 +2102,26 @@
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4" t="s">
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4" t="s">
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
-      <c r="K1" s="4" t="s">
+      <c r="I1" s="19"/>
+      <c r="J1" s="19"/>
+      <c r="K1" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="L1" s="4"/>
-      <c r="M1" s="4"/>
+      <c r="L1" s="19"/>
+      <c r="M1" s="19"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
@@ -2088,26 +2178,26 @@
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4" t="s">
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4" t="s">
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
-      <c r="K1" s="4" t="s">
+      <c r="I1" s="19"/>
+      <c r="J1" s="19"/>
+      <c r="K1" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="L1" s="4"/>
-      <c r="M1" s="4"/>
+      <c r="L1" s="19"/>
+      <c r="M1" s="19"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
@@ -2164,26 +2254,26 @@
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4" t="s">
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4" t="s">
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
-      <c r="K1" s="4" t="s">
+      <c r="I1" s="19"/>
+      <c r="J1" s="19"/>
+      <c r="K1" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="L1" s="4"/>
-      <c r="M1" s="4"/>
+      <c r="L1" s="19"/>
+      <c r="M1" s="19"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" t="s">

</xml_diff>

<commit_message>
completed dynamic motion results and v1 result multiple safety
</commit_message>
<xml_diff>
--- a/results/compiled results.xlsx
+++ b/results/compiled results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\elish\Desktop\Aims Project\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0CA14D8-B090-480F-86FC-EEDC7115E07C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C95190C6-65E3-4C35-BB00-80E40F8F7AFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{DA4D96B0-492C-4945-A9C4-EFCA6D6BC722}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{DA4D96B0-492C-4945-A9C4-EFCA6D6BC722}"/>
   </bookViews>
   <sheets>
     <sheet name="Dynamic results" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="390" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="435" uniqueCount="52">
   <si>
     <t xml:space="preserve">Model </t>
   </si>
@@ -414,15 +414,6 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -451,10 +442,25 @@
     <xf numFmtId="2" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -464,12 +470,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -839,26 +839,26 @@
       <c r="A2" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="31" t="s">
         <v>40</v>
       </c>
-      <c r="C2" s="20"/>
-      <c r="D2" s="21"/>
-      <c r="E2" s="20" t="s">
+      <c r="C2" s="32"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="32" t="s">
         <v>41</v>
       </c>
-      <c r="F2" s="20"/>
-      <c r="G2" s="21"/>
-      <c r="H2" s="20" t="s">
+      <c r="F2" s="32"/>
+      <c r="G2" s="33"/>
+      <c r="H2" s="32" t="s">
         <v>42</v>
       </c>
-      <c r="I2" s="20"/>
-      <c r="J2" s="20"/>
-      <c r="K2" s="19" t="s">
+      <c r="I2" s="32"/>
+      <c r="J2" s="32"/>
+      <c r="K2" s="31" t="s">
         <v>43</v>
       </c>
-      <c r="L2" s="20"/>
-      <c r="M2" s="20"/>
+      <c r="L2" s="32"/>
+      <c r="M2" s="32"/>
     </row>
     <row r="3" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
@@ -1607,26 +1607,26 @@
       <c r="A27" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B27" s="19" t="s">
+      <c r="B27" s="31" t="s">
         <v>40</v>
       </c>
-      <c r="C27" s="20"/>
-      <c r="D27" s="21"/>
-      <c r="E27" s="20" t="s">
+      <c r="C27" s="32"/>
+      <c r="D27" s="33"/>
+      <c r="E27" s="32" t="s">
         <v>41</v>
       </c>
-      <c r="F27" s="20"/>
-      <c r="G27" s="21"/>
-      <c r="H27" s="20" t="s">
+      <c r="F27" s="32"/>
+      <c r="G27" s="33"/>
+      <c r="H27" s="32" t="s">
         <v>42</v>
       </c>
-      <c r="I27" s="20"/>
-      <c r="J27" s="20"/>
-      <c r="K27" s="19" t="s">
+      <c r="I27" s="32"/>
+      <c r="J27" s="32"/>
+      <c r="K27" s="31" t="s">
         <v>43</v>
       </c>
-      <c r="L27" s="20"/>
-      <c r="M27" s="20"/>
+      <c r="L27" s="32"/>
+      <c r="M27" s="32"/>
     </row>
     <row r="28" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A28" s="14" t="s">
@@ -2324,26 +2324,26 @@
       <c r="A47" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B47" s="19" t="s">
+      <c r="B47" s="31" t="s">
         <v>40</v>
       </c>
-      <c r="C47" s="20"/>
-      <c r="D47" s="21"/>
-      <c r="E47" s="20" t="s">
+      <c r="C47" s="32"/>
+      <c r="D47" s="33"/>
+      <c r="E47" s="32" t="s">
         <v>41</v>
       </c>
-      <c r="F47" s="20"/>
-      <c r="G47" s="21"/>
-      <c r="H47" s="20" t="s">
+      <c r="F47" s="32"/>
+      <c r="G47" s="33"/>
+      <c r="H47" s="32" t="s">
         <v>42</v>
       </c>
-      <c r="I47" s="20"/>
-      <c r="J47" s="20"/>
-      <c r="K47" s="19" t="s">
+      <c r="I47" s="32"/>
+      <c r="J47" s="32"/>
+      <c r="K47" s="31" t="s">
         <v>43</v>
       </c>
-      <c r="L47" s="20"/>
-      <c r="M47" s="20"/>
+      <c r="L47" s="32"/>
+      <c r="M47" s="32"/>
     </row>
     <row r="48" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A48" s="12" t="s">
@@ -3039,26 +3039,26 @@
       <c r="A70" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B70" s="19" t="s">
+      <c r="B70" s="31" t="s">
         <v>40</v>
       </c>
-      <c r="C70" s="20"/>
-      <c r="D70" s="21"/>
-      <c r="E70" s="20" t="s">
+      <c r="C70" s="32"/>
+      <c r="D70" s="33"/>
+      <c r="E70" s="32" t="s">
         <v>41</v>
       </c>
-      <c r="F70" s="20"/>
-      <c r="G70" s="21"/>
-      <c r="H70" s="20" t="s">
+      <c r="F70" s="32"/>
+      <c r="G70" s="33"/>
+      <c r="H70" s="32" t="s">
         <v>42</v>
       </c>
-      <c r="I70" s="20"/>
-      <c r="J70" s="20"/>
-      <c r="K70" s="19" t="s">
+      <c r="I70" s="32"/>
+      <c r="J70" s="32"/>
+      <c r="K70" s="31" t="s">
         <v>43</v>
       </c>
-      <c r="L70" s="20"/>
-      <c r="M70" s="20"/>
+      <c r="L70" s="32"/>
+      <c r="M70" s="32"/>
     </row>
     <row r="71" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A71" s="14" t="s">
@@ -3395,7 +3395,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="81" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="81" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B81"/>
       <c r="C81"/>
       <c r="D81"/>
@@ -3411,8 +3411,47 @@
       <c r="N81" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="82" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="O81" s="3">
+        <v>2.4033445388934701E-2</v>
+      </c>
+      <c r="P81" s="3">
+        <v>7.6803144918766594E-2</v>
+      </c>
+      <c r="Q81" s="3">
+        <v>4.8029022631287596E-3</v>
+      </c>
+      <c r="R81" s="3">
+        <v>5.3988458797210896E-3</v>
+      </c>
+      <c r="S81" s="2">
+        <v>0</v>
+      </c>
+      <c r="T81" s="4">
+        <v>0</v>
+      </c>
+      <c r="U81" s="3">
+        <v>0</v>
+      </c>
+      <c r="V81" s="2">
+        <v>100</v>
+      </c>
+      <c r="Y81" s="3">
+        <v>0.10373</v>
+      </c>
+      <c r="Z81" s="3">
+        <v>0.37646399999999902</v>
+      </c>
+      <c r="AA81" s="2">
+        <v>23.072727272727199</v>
+      </c>
+      <c r="AB81" s="3">
+        <v>2.5379999999999998</v>
+      </c>
+      <c r="AC81" s="2">
+        <v>15983.961540287601</v>
+      </c>
+    </row>
+    <row r="82" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B82"/>
       <c r="C82"/>
       <c r="D82"/>
@@ -3428,8 +3467,47 @@
       <c r="N82" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="83" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="O82" s="3">
+        <v>2.4583666008142602E-2</v>
+      </c>
+      <c r="P82" s="3">
+        <v>7.6668707340654396E-2</v>
+      </c>
+      <c r="Q82" s="3">
+        <v>5.4081451391882404E-3</v>
+      </c>
+      <c r="R82" s="3">
+        <v>5.44948977927794E-3</v>
+      </c>
+      <c r="S82" s="2">
+        <v>0</v>
+      </c>
+      <c r="T82" s="4">
+        <v>0</v>
+      </c>
+      <c r="U82" s="3">
+        <v>0</v>
+      </c>
+      <c r="V82" s="2">
+        <v>44.045454545454497</v>
+      </c>
+      <c r="Y82" s="3">
+        <v>0.17599999999999999</v>
+      </c>
+      <c r="Z82" s="3">
+        <v>1.1199999999999899</v>
+      </c>
+      <c r="AA82" s="2">
+        <v>2.28181818181818</v>
+      </c>
+      <c r="AB82" s="3">
+        <v>0.251</v>
+      </c>
+      <c r="AC82" s="2">
+        <v>16008.168786464999</v>
+      </c>
+    </row>
+    <row r="83" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B83"/>
       <c r="C83"/>
       <c r="D83"/>
@@ -3445,8 +3523,47 @@
       <c r="N83" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="84" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="O83" s="3">
+        <v>2.45856273437772E-2</v>
+      </c>
+      <c r="P83" s="3">
+        <v>7.6668376666935906E-2</v>
+      </c>
+      <c r="Q83" s="3">
+        <v>5.4103026680408801E-3</v>
+      </c>
+      <c r="R83" s="3">
+        <v>5.45196247760113E-3</v>
+      </c>
+      <c r="S83" s="2">
+        <v>0</v>
+      </c>
+      <c r="T83" s="4">
+        <v>0</v>
+      </c>
+      <c r="U83" s="3">
+        <v>0</v>
+      </c>
+      <c r="V83" s="2">
+        <v>0</v>
+      </c>
+      <c r="Y83" s="3">
+        <v>1.4543999999999999</v>
+      </c>
+      <c r="Z83" s="3">
+        <v>4.3177019999999997</v>
+      </c>
+      <c r="AA83" s="2">
+        <v>2.1818181818181799</v>
+      </c>
+      <c r="AB83" s="3">
+        <v>0.24</v>
+      </c>
+      <c r="AC83" s="2">
+        <v>16008.4204858513</v>
+      </c>
+    </row>
+    <row r="84" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B84"/>
       <c r="C84"/>
       <c r="D84"/>
@@ -3462,8 +3579,47 @@
       <c r="N84" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="85" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="O84" s="3">
+        <v>2.4585621925057501E-2</v>
+      </c>
+      <c r="P84" s="3">
+        <v>7.6668378186270897E-2</v>
+      </c>
+      <c r="Q84" s="3">
+        <v>5.4102968139911698E-3</v>
+      </c>
+      <c r="R84" s="3">
+        <v>5.4519646896899702E-3</v>
+      </c>
+      <c r="S84" s="2">
+        <v>0</v>
+      </c>
+      <c r="T84" s="4">
+        <v>0</v>
+      </c>
+      <c r="U84" s="3">
+        <v>0</v>
+      </c>
+      <c r="V84" s="2">
+        <v>100</v>
+      </c>
+      <c r="Y84" s="3">
+        <v>0.29519999999999902</v>
+      </c>
+      <c r="Z84" s="3">
+        <v>0.68320000000000003</v>
+      </c>
+      <c r="AA84" s="2">
+        <v>2.19999999999999</v>
+      </c>
+      <c r="AB84" s="3">
+        <v>0.24199999999999999</v>
+      </c>
+      <c r="AC84" s="2">
+        <v>16008.4219888916</v>
+      </c>
+    </row>
+    <row r="85" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B85"/>
       <c r="C85"/>
       <c r="D85"/>
@@ -3479,8 +3635,47 @@
       <c r="N85" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="86" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="O85" s="3">
+        <v>2.4585621925057501E-2</v>
+      </c>
+      <c r="P85" s="3">
+        <v>7.6668378186270897E-2</v>
+      </c>
+      <c r="Q85" s="3">
+        <v>5.4102968139911698E-3</v>
+      </c>
+      <c r="R85" s="3">
+        <v>5.4519646896899702E-3</v>
+      </c>
+      <c r="S85" s="2">
+        <v>0</v>
+      </c>
+      <c r="T85" s="4">
+        <v>0</v>
+      </c>
+      <c r="U85" s="3">
+        <v>0</v>
+      </c>
+      <c r="V85" s="2">
+        <v>19.063636363636299</v>
+      </c>
+      <c r="Y85" s="3">
+        <v>0.29519999999999902</v>
+      </c>
+      <c r="Z85" s="3">
+        <v>1.5960000000000001</v>
+      </c>
+      <c r="AA85" s="2">
+        <v>2.19999999999999</v>
+      </c>
+      <c r="AB85" s="3">
+        <v>0.24199999999999999</v>
+      </c>
+      <c r="AC85" s="2">
+        <v>16008.4219888916</v>
+      </c>
+    </row>
+    <row r="86" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B86"/>
       <c r="C86"/>
       <c r="D86"/>
@@ -3497,7 +3692,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="87" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="87" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B87"/>
       <c r="C87"/>
       <c r="D87"/>
@@ -3513,14 +3708,100 @@
       <c r="N87" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="88" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="O87" s="3">
+        <v>2.4585621925057501E-2</v>
+      </c>
+      <c r="P87" s="3">
+        <v>7.6668378186270897E-2</v>
+      </c>
+      <c r="Q87" s="3">
+        <v>5.4102968139911698E-3</v>
+      </c>
+      <c r="R87" s="3">
+        <v>5.4519646896899702E-3</v>
+      </c>
+      <c r="S87" s="2">
+        <v>0</v>
+      </c>
+      <c r="T87" s="4">
+        <v>0</v>
+      </c>
+      <c r="U87" s="3">
+        <v>0</v>
+      </c>
+      <c r="V87" s="2">
+        <v>19.063636363636299</v>
+      </c>
+      <c r="Y87" s="3">
+        <v>0.29519999999999902</v>
+      </c>
+      <c r="Z87" s="3">
+        <v>1.5960000000000001</v>
+      </c>
+      <c r="AA87" s="2">
+        <v>2.19999999999999</v>
+      </c>
+      <c r="AB87" s="3">
+        <v>0.24199999999999999</v>
+      </c>
+      <c r="AC87" s="2">
+        <v>16008.4219888916</v>
+      </c>
+    </row>
+    <row r="88" spans="2:29" x14ac:dyDescent="0.3">
       <c r="N88" t="s">
         <v>38</v>
       </c>
+      <c r="O88" s="3">
+        <v>2.4585621925057501E-2</v>
+      </c>
+      <c r="P88" s="3">
+        <v>7.6668378186270897E-2</v>
+      </c>
+      <c r="Q88" s="3">
+        <v>5.4102968139911698E-3</v>
+      </c>
+      <c r="R88" s="3">
+        <v>5.4519646896899702E-3</v>
+      </c>
+      <c r="S88" s="2">
+        <v>0</v>
+      </c>
+      <c r="T88" s="4">
+        <v>0</v>
+      </c>
+      <c r="U88" s="3">
+        <v>0</v>
+      </c>
+      <c r="V88" s="2">
+        <v>19.063636363636299</v>
+      </c>
+      <c r="Y88" s="3">
+        <v>0.29519999999999902</v>
+      </c>
+      <c r="Z88" s="3">
+        <v>1.5960000000000001</v>
+      </c>
+      <c r="AA88" s="2">
+        <v>2.19999999999999</v>
+      </c>
+      <c r="AB88" s="3">
+        <v>0.24199999999999999</v>
+      </c>
+      <c r="AC88" s="2">
+        <v>16008.4219888916</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="E2:G2"/>
+    <mergeCell ref="H2:J2"/>
+    <mergeCell ref="K2:M2"/>
+    <mergeCell ref="B27:D27"/>
+    <mergeCell ref="E27:G27"/>
+    <mergeCell ref="H27:J27"/>
+    <mergeCell ref="K27:M27"/>
     <mergeCell ref="B70:D70"/>
     <mergeCell ref="E70:G70"/>
     <mergeCell ref="H70:J70"/>
@@ -3529,14 +3810,6 @@
     <mergeCell ref="E47:G47"/>
     <mergeCell ref="H47:J47"/>
     <mergeCell ref="K47:M47"/>
-    <mergeCell ref="B2:D2"/>
-    <mergeCell ref="E2:G2"/>
-    <mergeCell ref="H2:J2"/>
-    <mergeCell ref="K2:M2"/>
-    <mergeCell ref="B27:D27"/>
-    <mergeCell ref="E27:G27"/>
-    <mergeCell ref="H27:J27"/>
-    <mergeCell ref="K27:M27"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3544,43 +3817,52 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7131F0C-F05D-45F0-8B49-786E37E66573}">
-  <dimension ref="A1:O83"/>
+  <dimension ref="A1:AD83"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.6640625" customWidth="1"/>
+    <col min="16" max="19" width="12.44140625" style="3" customWidth="1"/>
+    <col min="20" max="21" width="8.88671875" style="2"/>
+    <col min="22" max="22" width="12.44140625" style="3" customWidth="1"/>
+    <col min="23" max="23" width="10.77734375" style="2" customWidth="1"/>
+    <col min="24" max="24" width="15.77734375" style="3" customWidth="1"/>
+    <col min="25" max="27" width="12.44140625" style="3" customWidth="1"/>
+    <col min="28" max="28" width="8.88671875" style="2"/>
+    <col min="29" max="29" width="12.44140625" style="3" customWidth="1"/>
+    <col min="30" max="30" width="14.109375" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="31" t="s">
         <v>40</v>
       </c>
-      <c r="C2" s="20"/>
-      <c r="D2" s="21"/>
-      <c r="E2" s="20" t="s">
+      <c r="C2" s="32"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="32" t="s">
         <v>41</v>
       </c>
-      <c r="F2" s="20"/>
-      <c r="G2" s="21"/>
-      <c r="H2" s="20" t="s">
+      <c r="F2" s="32"/>
+      <c r="G2" s="33"/>
+      <c r="H2" s="32" t="s">
         <v>42</v>
       </c>
-      <c r="I2" s="20"/>
-      <c r="J2" s="20"/>
-      <c r="K2" s="19" t="s">
+      <c r="I2" s="32"/>
+      <c r="J2" s="32"/>
+      <c r="K2" s="31" t="s">
         <v>43</v>
       </c>
-      <c r="L2" s="20"/>
-      <c r="M2" s="20"/>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="L2" s="32"/>
+      <c r="M2" s="32"/>
+    </row>
+    <row r="3" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
         <v>1</v>
       </c>
@@ -3621,7 +3903,7 @@
         <v>1.1900000572204501</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A4" s="12" t="s">
         <v>2</v>
       </c>
@@ -3662,7 +3944,7 @@
         <v>1.1900000572204501</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>3</v>
       </c>
@@ -3703,7 +3985,7 @@
         <v>1.1399999856948799</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A6" s="14" t="s">
         <v>4</v>
       </c>
@@ -3744,7 +4026,7 @@
         <v>1.25</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>7</v>
       </c>
@@ -3785,7 +4067,7 @@
         <v>0.730000019073486</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A8" s="12" t="s">
         <v>5</v>
       </c>
@@ -3826,7 +4108,7 @@
         <v>0.81999999284744196</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A9" s="12" t="s">
         <v>17</v>
       </c>
@@ -3867,7 +4149,7 @@
         <v>0.81999999284744196</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A10" s="13" t="s">
         <v>6</v>
       </c>
@@ -3884,22 +4166,114 @@
       <c r="L10" s="10"/>
       <c r="M10" s="10"/>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="P12" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q12" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="R12" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="S12" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="T12" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="U12" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="V12" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="W12" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="X12" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="Y12" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z12" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA12" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="AB12" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="AC12" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="AD12" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O13" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O14" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P14" s="3">
+        <v>0.208803427881982</v>
+      </c>
+      <c r="Q14" s="3">
+        <v>3.2646891997723602E-2</v>
+      </c>
+      <c r="R14" s="3">
+        <v>0.20774180079319299</v>
+      </c>
+      <c r="S14" s="3">
+        <v>3.1069445262637101E-2</v>
+      </c>
+      <c r="T14" s="2">
+        <v>100</v>
+      </c>
+      <c r="U14" s="2">
+        <v>1.81694009620145E-3</v>
+      </c>
+      <c r="V14" s="3">
+        <v>1.81694009620145E-3</v>
+      </c>
+      <c r="W14" s="2">
+        <v>0</v>
+      </c>
+      <c r="X14" s="3">
+        <v>5.6548667764616201E-2</v>
+      </c>
+      <c r="Y14" s="3">
+        <v>5.6548667764616201E-2</v>
+      </c>
+      <c r="Z14" s="3">
+        <v>0.02</v>
+      </c>
+      <c r="AA14" s="3">
+        <v>3.81633599999999</v>
+      </c>
+      <c r="AB14" s="2">
+        <v>100</v>
+      </c>
+      <c r="AC14" s="3">
+        <v>11</v>
+      </c>
+      <c r="AD14" s="2">
+        <v>5331.3170567901097</v>
+      </c>
+    </row>
+    <row r="15" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O15" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O16" t="s">
         <v>33</v>
       </c>
@@ -3938,26 +4312,26 @@
       <c r="A24" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B24" s="19" t="s">
+      <c r="B24" s="31" t="s">
         <v>40</v>
       </c>
-      <c r="C24" s="20"/>
-      <c r="D24" s="21"/>
-      <c r="E24" s="20" t="s">
+      <c r="C24" s="32"/>
+      <c r="D24" s="33"/>
+      <c r="E24" s="32" t="s">
         <v>41</v>
       </c>
-      <c r="F24" s="20"/>
-      <c r="G24" s="21"/>
-      <c r="H24" s="20" t="s">
+      <c r="F24" s="32"/>
+      <c r="G24" s="33"/>
+      <c r="H24" s="32" t="s">
         <v>42</v>
       </c>
-      <c r="I24" s="20"/>
-      <c r="J24" s="20"/>
-      <c r="K24" s="19" t="s">
+      <c r="I24" s="32"/>
+      <c r="J24" s="32"/>
+      <c r="K24" s="31" t="s">
         <v>43</v>
       </c>
-      <c r="L24" s="20"/>
-      <c r="M24" s="20"/>
+      <c r="L24" s="32"/>
+      <c r="M24" s="32"/>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A25" s="14" t="s">
@@ -4287,82 +4661,127 @@
         <v>0.62999999523162797</v>
       </c>
     </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O34" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O35" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P35" s="3">
+        <v>0.292965027710332</v>
+      </c>
+      <c r="Q35" s="3">
+        <v>5.9460140223132098E-2</v>
+      </c>
+      <c r="R35" s="3">
+        <v>0.29305596943231199</v>
+      </c>
+      <c r="S35" s="3">
+        <v>5.9339420540317801E-2</v>
+      </c>
+      <c r="T35" s="2">
+        <v>100</v>
+      </c>
+      <c r="U35" s="2">
+        <v>8.0292745229176999E-3</v>
+      </c>
+      <c r="V35" s="3">
+        <v>8.0292745229176999E-3</v>
+      </c>
+      <c r="W35" s="2">
+        <v>12.2272727272727</v>
+      </c>
+      <c r="X35" s="3">
+        <v>5.6548667764616201E-2</v>
+      </c>
+      <c r="Y35" s="3">
+        <v>5.6548667764616201E-2</v>
+      </c>
+      <c r="Z35" s="3">
+        <v>1.2799999999999899E-3</v>
+      </c>
+      <c r="AA35" s="3">
+        <v>3.1303999999999998</v>
+      </c>
+      <c r="AB35" s="2">
+        <v>100</v>
+      </c>
+      <c r="AC35" s="3">
+        <v>11</v>
+      </c>
+      <c r="AD35" s="2">
+        <v>4943.45004945858</v>
+      </c>
+    </row>
+    <row r="36" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O36" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O37" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O38" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O39" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O40" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O41" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O42" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A44" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B44" s="19" t="s">
+      <c r="B44" s="31" t="s">
         <v>40</v>
       </c>
-      <c r="C44" s="20"/>
-      <c r="D44" s="21"/>
-      <c r="E44" s="20" t="s">
+      <c r="C44" s="32"/>
+      <c r="D44" s="33"/>
+      <c r="E44" s="32" t="s">
         <v>41</v>
       </c>
-      <c r="F44" s="20"/>
-      <c r="G44" s="21"/>
-      <c r="H44" s="20" t="s">
+      <c r="F44" s="32"/>
+      <c r="G44" s="33"/>
+      <c r="H44" s="32" t="s">
         <v>42</v>
       </c>
-      <c r="I44" s="20"/>
-      <c r="J44" s="20"/>
-      <c r="K44" s="19" t="s">
+      <c r="I44" s="32"/>
+      <c r="J44" s="32"/>
+      <c r="K44" s="31" t="s">
         <v>43</v>
       </c>
-      <c r="L44" s="20"/>
-      <c r="M44" s="20"/>
-    </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="L44" s="32"/>
+      <c r="M44" s="32"/>
+    </row>
+    <row r="45" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A45" s="14" t="s">
         <v>1</v>
       </c>
@@ -4403,7 +4822,7 @@
         <v>0.75</v>
       </c>
     </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A46" s="12" t="s">
         <v>2</v>
       </c>
@@ -4444,7 +4863,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="47" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A47" s="5" t="s">
         <v>3</v>
       </c>
@@ -4485,7 +4904,7 @@
         <v>0.65299999713897705</v>
       </c>
     </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A48" s="14" t="s">
         <v>4</v>
       </c>
@@ -4741,34 +5160,34 @@
       </c>
     </row>
     <row r="65" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A65" s="22" t="s">
-        <v>0</v>
-      </c>
-      <c r="B65" s="33" t="s">
+      <c r="A65" s="19" t="s">
+        <v>0</v>
+      </c>
+      <c r="B65" s="34" t="s">
         <v>40</v>
       </c>
-      <c r="C65" s="32"/>
-      <c r="D65" s="34"/>
-      <c r="E65" s="35" t="s">
+      <c r="C65" s="35"/>
+      <c r="D65" s="36"/>
+      <c r="E65" s="37" t="s">
         <v>41</v>
       </c>
-      <c r="F65" s="32"/>
-      <c r="G65" s="34"/>
-      <c r="H65" s="35" t="s">
+      <c r="F65" s="35"/>
+      <c r="G65" s="36"/>
+      <c r="H65" s="37" t="s">
         <v>42</v>
       </c>
-      <c r="I65" s="32"/>
-      <c r="J65" s="36"/>
-      <c r="K65" s="33" t="s">
+      <c r="I65" s="35"/>
+      <c r="J65" s="38"/>
+      <c r="K65" s="34" t="s">
         <v>43</v>
       </c>
-      <c r="L65" s="32"/>
-      <c r="M65" s="32"/>
-      <c r="N65" s="24"/>
-      <c r="O65" s="24"/>
+      <c r="L65" s="35"/>
+      <c r="M65" s="35"/>
+      <c r="N65" s="21"/>
+      <c r="O65" s="21"/>
     </row>
     <row r="66" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A66" s="25" t="s">
+      <c r="A66" s="22" t="s">
         <v>1</v>
       </c>
       <c r="B66" s="15">
@@ -4807,451 +5226,451 @@
       <c r="M66" s="16">
         <v>0.72000002861022905</v>
       </c>
-      <c r="N66" s="24"/>
-      <c r="O66" s="24"/>
+      <c r="N66" s="21"/>
+      <c r="O66" s="21"/>
     </row>
     <row r="67" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A67" s="25" t="s">
+      <c r="A67" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="B67" s="26">
+      <c r="B67" s="23">
         <v>0.140000000596046</v>
       </c>
-      <c r="C67" s="26">
+      <c r="C67" s="23">
         <v>-0.5</v>
       </c>
-      <c r="D67" s="27">
+      <c r="D67" s="24">
         <v>5.0000000745057997E-2</v>
       </c>
-      <c r="E67" s="26">
+      <c r="E67" s="23">
         <v>0.56000000238418501</v>
       </c>
-      <c r="F67" s="26">
+      <c r="F67" s="23">
         <v>0.5</v>
       </c>
-      <c r="G67" s="27">
+      <c r="G67" s="24">
         <v>0.64999997615814198</v>
       </c>
-      <c r="H67" s="26">
+      <c r="H67" s="23">
         <v>-0.72000002861022905</v>
       </c>
-      <c r="I67" s="26">
+      <c r="I67" s="23">
         <v>-1.3200000524520801</v>
       </c>
-      <c r="J67" s="26">
+      <c r="J67" s="23">
         <v>-0.11999999731779</v>
       </c>
-      <c r="K67" s="28">
+      <c r="K67" s="25">
         <v>0.11999999731779</v>
       </c>
-      <c r="L67" s="26">
+      <c r="L67" s="23">
         <v>0.11999999731779</v>
       </c>
-      <c r="M67" s="26">
+      <c r="M67" s="23">
         <v>0.72000002861022905</v>
       </c>
-      <c r="N67" s="24"/>
-      <c r="O67" s="24"/>
+      <c r="N67" s="21"/>
+      <c r="O67" s="21"/>
     </row>
     <row r="68" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A68" s="22" t="s">
+      <c r="A68" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="B68" s="29">
+      <c r="B68" s="26">
         <v>-0.50999999046325595</v>
       </c>
-      <c r="C68" s="29">
+      <c r="C68" s="26">
         <v>-0.75499999523162797</v>
       </c>
-      <c r="D68" s="30">
+      <c r="D68" s="27">
         <v>-3.2999999821186003E-2</v>
       </c>
-      <c r="E68" s="29">
+      <c r="E68" s="26">
         <v>0.5</v>
       </c>
-      <c r="F68" s="29">
+      <c r="F68" s="26">
         <v>1.25499999523162</v>
       </c>
-      <c r="G68" s="30">
+      <c r="G68" s="27">
         <v>0.77700001001357999</v>
       </c>
-      <c r="H68" s="29">
+      <c r="H68" s="26">
         <v>-0.81000000238418501</v>
       </c>
-      <c r="I68" s="29">
+      <c r="I68" s="26">
         <v>-1.3049999475479099</v>
       </c>
-      <c r="J68" s="29">
+      <c r="J68" s="26">
         <v>-0.38299998641014099</v>
       </c>
-      <c r="K68" s="31">
+      <c r="K68" s="28">
         <v>0.60000002384185702</v>
       </c>
-      <c r="L68" s="29">
+      <c r="L68" s="26">
         <v>1.20500004291534</v>
       </c>
-      <c r="M68" s="29">
+      <c r="M68" s="26">
         <v>0.92699998617172197</v>
       </c>
-      <c r="N68" s="24"/>
-      <c r="O68" s="24"/>
+      <c r="N68" s="21"/>
+      <c r="O68" s="21"/>
     </row>
     <row r="69" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A69" s="25" t="s">
+      <c r="A69" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="B69" s="26">
+      <c r="B69" s="23">
         <v>0.140000000596046</v>
       </c>
-      <c r="C69" s="26">
+      <c r="C69" s="23">
         <v>-0.60000002384185702</v>
       </c>
-      <c r="D69" s="27">
+      <c r="D69" s="24">
         <v>0.10000000149011599</v>
       </c>
-      <c r="E69" s="26">
+      <c r="E69" s="23">
         <v>0.55000001192092896</v>
       </c>
-      <c r="F69" s="26">
+      <c r="F69" s="23">
         <v>0.60000002384185702</v>
       </c>
-      <c r="G69" s="27">
+      <c r="G69" s="24">
         <v>0.60000002384185702</v>
       </c>
-      <c r="H69" s="26">
+      <c r="H69" s="23">
         <v>-0.80000001192092896</v>
       </c>
-      <c r="I69" s="26">
+      <c r="I69" s="23">
         <v>-0.80000001192092896</v>
       </c>
-      <c r="J69" s="26">
+      <c r="J69" s="23">
         <v>-0.20000000298023199</v>
       </c>
-      <c r="K69" s="28">
+      <c r="K69" s="25">
         <v>0.25</v>
       </c>
-      <c r="L69" s="26">
+      <c r="L69" s="23">
         <v>0.80000001192092896</v>
       </c>
-      <c r="M69" s="26">
+      <c r="M69" s="23">
         <v>0.85000002384185702</v>
       </c>
-      <c r="N69" s="24"/>
-      <c r="O69" s="24"/>
+      <c r="N69" s="21"/>
+      <c r="O69" s="21"/>
     </row>
     <row r="70" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A70" s="22" t="s">
+      <c r="A70" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="B70" s="29">
+      <c r="B70" s="26">
         <v>0.140000000596046</v>
       </c>
-      <c r="C70" s="29">
+      <c r="C70" s="26">
         <v>-0.60000002384185702</v>
       </c>
-      <c r="D70" s="30">
+      <c r="D70" s="27">
         <v>5.0000000745057997E-2</v>
       </c>
-      <c r="E70" s="29">
+      <c r="E70" s="26">
         <v>0.55000001192092896</v>
       </c>
-      <c r="F70" s="29">
+      <c r="F70" s="26">
         <v>0.60000002384185702</v>
       </c>
-      <c r="G70" s="30">
+      <c r="G70" s="27">
         <v>0.64999997615814198</v>
       </c>
-      <c r="H70" s="29">
+      <c r="H70" s="26">
         <v>-0.20000000298023199</v>
       </c>
-      <c r="I70" s="29">
+      <c r="I70" s="26">
         <v>-0.80000001192092896</v>
       </c>
-      <c r="J70" s="29">
+      <c r="J70" s="26">
         <v>-0.20000000298023199</v>
       </c>
-      <c r="K70" s="31">
+      <c r="K70" s="28">
         <v>0.75</v>
       </c>
-      <c r="L70" s="29">
+      <c r="L70" s="26">
         <v>0.80000001192092896</v>
       </c>
-      <c r="M70" s="29">
+      <c r="M70" s="26">
         <v>0.85000002384185702</v>
       </c>
-      <c r="N70" s="24"/>
-      <c r="O70" s="24"/>
+      <c r="N70" s="21"/>
+      <c r="O70" s="21"/>
     </row>
     <row r="71" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A71" s="25" t="s">
+      <c r="A71" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="B71" s="26"/>
-      <c r="C71" s="26"/>
-      <c r="D71" s="27"/>
-      <c r="E71" s="26"/>
-      <c r="F71" s="26"/>
-      <c r="G71" s="27"/>
-      <c r="H71" s="26"/>
-      <c r="I71" s="26"/>
-      <c r="J71" s="26"/>
-      <c r="K71" s="28"/>
-      <c r="L71" s="26"/>
-      <c r="M71" s="26"/>
-      <c r="N71" s="24"/>
-      <c r="O71" s="24"/>
+      <c r="B71" s="23"/>
+      <c r="C71" s="23"/>
+      <c r="D71" s="24"/>
+      <c r="E71" s="23"/>
+      <c r="F71" s="23"/>
+      <c r="G71" s="24"/>
+      <c r="H71" s="23"/>
+      <c r="I71" s="23"/>
+      <c r="J71" s="23"/>
+      <c r="K71" s="25"/>
+      <c r="L71" s="23"/>
+      <c r="M71" s="23"/>
+      <c r="N71" s="21"/>
+      <c r="O71" s="21"/>
     </row>
     <row r="72" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A72" s="25" t="s">
+      <c r="A72" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="B72" s="26">
+      <c r="B72" s="23">
         <v>0.140000000596046</v>
       </c>
-      <c r="C72" s="26">
+      <c r="C72" s="23">
         <v>-0.60000002384185702</v>
       </c>
-      <c r="D72" s="27">
+      <c r="D72" s="24">
         <v>5.0000000745057997E-2</v>
       </c>
-      <c r="E72" s="26">
+      <c r="E72" s="23">
         <v>0.55000001192092896</v>
       </c>
-      <c r="F72" s="26">
+      <c r="F72" s="23">
         <v>0.60000002384185702</v>
       </c>
-      <c r="G72" s="27">
+      <c r="G72" s="24">
         <v>0.64999997615814198</v>
       </c>
-      <c r="H72" s="26">
+      <c r="H72" s="23">
         <v>-0.20000000298023199</v>
       </c>
-      <c r="I72" s="26">
+      <c r="I72" s="23">
         <v>-0.80000001192092896</v>
       </c>
-      <c r="J72" s="26">
+      <c r="J72" s="23">
         <v>-0.20000000298023199</v>
       </c>
-      <c r="K72" s="28">
+      <c r="K72" s="25">
         <v>0.75</v>
       </c>
-      <c r="L72" s="26">
+      <c r="L72" s="23">
         <v>0.80000001192092896</v>
       </c>
-      <c r="M72" s="26">
+      <c r="M72" s="23">
         <v>0.85000002384185702</v>
       </c>
-      <c r="N72" s="24"/>
-      <c r="O72" s="24"/>
+      <c r="N72" s="21"/>
+      <c r="O72" s="21"/>
     </row>
     <row r="73" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A73" s="23" t="s">
+      <c r="A73" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="B73" s="31">
+      <c r="B73" s="28">
         <v>0.140000000596046</v>
       </c>
-      <c r="C73" s="29">
+      <c r="C73" s="26">
         <v>-0.60000002384185702</v>
       </c>
-      <c r="D73" s="29">
+      <c r="D73" s="26">
         <v>5.0000000745057997E-2</v>
       </c>
-      <c r="E73" s="31">
+      <c r="E73" s="28">
         <v>0.55000001192092896</v>
       </c>
-      <c r="F73" s="29">
+      <c r="F73" s="26">
         <v>0.60000002384185702</v>
       </c>
-      <c r="G73" s="29">
+      <c r="G73" s="26">
         <v>0.64999997615814198</v>
       </c>
-      <c r="H73" s="31">
+      <c r="H73" s="28">
         <v>-0.20000000298023199</v>
       </c>
-      <c r="I73" s="29">
+      <c r="I73" s="26">
         <v>-0.80000001192092896</v>
       </c>
-      <c r="J73" s="29">
+      <c r="J73" s="26">
         <v>-0.20000000298023199</v>
       </c>
-      <c r="K73" s="31">
+      <c r="K73" s="28">
         <v>0.75</v>
       </c>
-      <c r="L73" s="29">
+      <c r="L73" s="26">
         <v>0.80000001192092896</v>
       </c>
-      <c r="M73" s="29">
+      <c r="M73" s="26">
         <v>0.85000002384185702</v>
       </c>
-      <c r="N73" s="24"/>
-      <c r="O73" s="24"/>
+      <c r="N73" s="21"/>
+      <c r="O73" s="21"/>
     </row>
     <row r="74" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A74" s="24"/>
-      <c r="B74" s="24"/>
-      <c r="C74" s="24"/>
-      <c r="D74" s="24"/>
-      <c r="E74" s="24"/>
-      <c r="F74" s="24"/>
-      <c r="G74" s="24"/>
-      <c r="H74" s="24"/>
-      <c r="I74" s="24"/>
-      <c r="J74" s="24"/>
-      <c r="K74" s="24"/>
-      <c r="L74" s="24"/>
-      <c r="M74" s="24"/>
-      <c r="N74" s="24"/>
-      <c r="O74" s="24"/>
+      <c r="A74" s="21"/>
+      <c r="B74" s="21"/>
+      <c r="C74" s="21"/>
+      <c r="D74" s="21"/>
+      <c r="E74" s="21"/>
+      <c r="F74" s="21"/>
+      <c r="G74" s="21"/>
+      <c r="H74" s="21"/>
+      <c r="I74" s="21"/>
+      <c r="J74" s="21"/>
+      <c r="K74" s="21"/>
+      <c r="L74" s="21"/>
+      <c r="M74" s="21"/>
+      <c r="N74" s="21"/>
+      <c r="O74" s="21"/>
     </row>
     <row r="75" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A75" s="24"/>
-      <c r="B75" s="24"/>
-      <c r="C75" s="24"/>
-      <c r="D75" s="24"/>
-      <c r="E75" s="24"/>
-      <c r="F75" s="24"/>
-      <c r="G75" s="24"/>
-      <c r="H75" s="24"/>
-      <c r="I75" s="24"/>
-      <c r="J75" s="24"/>
-      <c r="K75" s="24"/>
-      <c r="L75" s="24"/>
-      <c r="M75" s="24"/>
-      <c r="N75" s="24"/>
+      <c r="A75" s="21"/>
+      <c r="B75" s="21"/>
+      <c r="C75" s="21"/>
+      <c r="D75" s="21"/>
+      <c r="E75" s="21"/>
+      <c r="F75" s="21"/>
+      <c r="G75" s="21"/>
+      <c r="H75" s="21"/>
+      <c r="I75" s="21"/>
+      <c r="J75" s="21"/>
+      <c r="K75" s="21"/>
+      <c r="L75" s="21"/>
+      <c r="M75" s="21"/>
+      <c r="N75" s="21"/>
       <c r="O75" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="76" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A76" s="24"/>
-      <c r="B76" s="24"/>
-      <c r="C76" s="24"/>
-      <c r="D76" s="24"/>
-      <c r="E76" s="24"/>
-      <c r="F76" s="24"/>
-      <c r="G76" s="24"/>
-      <c r="H76" s="24"/>
-      <c r="I76" s="24"/>
-      <c r="J76" s="24"/>
-      <c r="K76" s="24"/>
-      <c r="L76" s="24"/>
-      <c r="M76" s="24"/>
-      <c r="N76" s="24"/>
+      <c r="A76" s="21"/>
+      <c r="B76" s="21"/>
+      <c r="C76" s="21"/>
+      <c r="D76" s="21"/>
+      <c r="E76" s="21"/>
+      <c r="F76" s="21"/>
+      <c r="G76" s="21"/>
+      <c r="H76" s="21"/>
+      <c r="I76" s="21"/>
+      <c r="J76" s="21"/>
+      <c r="K76" s="21"/>
+      <c r="L76" s="21"/>
+      <c r="M76" s="21"/>
+      <c r="N76" s="21"/>
       <c r="O76" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="77" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A77" s="24"/>
-      <c r="B77" s="24"/>
-      <c r="C77" s="24"/>
-      <c r="D77" s="24"/>
-      <c r="E77" s="24"/>
-      <c r="F77" s="24"/>
-      <c r="G77" s="24"/>
-      <c r="H77" s="24"/>
-      <c r="I77" s="24"/>
-      <c r="J77" s="24"/>
-      <c r="K77" s="24"/>
-      <c r="L77" s="24"/>
-      <c r="M77" s="24"/>
-      <c r="N77" s="24"/>
+      <c r="A77" s="21"/>
+      <c r="B77" s="21"/>
+      <c r="C77" s="21"/>
+      <c r="D77" s="21"/>
+      <c r="E77" s="21"/>
+      <c r="F77" s="21"/>
+      <c r="G77" s="21"/>
+      <c r="H77" s="21"/>
+      <c r="I77" s="21"/>
+      <c r="J77" s="21"/>
+      <c r="K77" s="21"/>
+      <c r="L77" s="21"/>
+      <c r="M77" s="21"/>
+      <c r="N77" s="21"/>
       <c r="O77" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="78" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A78" s="24"/>
-      <c r="B78" s="24"/>
-      <c r="C78" s="24"/>
-      <c r="D78" s="24"/>
-      <c r="E78" s="24"/>
-      <c r="F78" s="24"/>
-      <c r="G78" s="24"/>
-      <c r="H78" s="24"/>
-      <c r="I78" s="24"/>
-      <c r="J78" s="24"/>
-      <c r="K78" s="24"/>
-      <c r="L78" s="24"/>
-      <c r="M78" s="24"/>
-      <c r="N78" s="24"/>
+      <c r="A78" s="21"/>
+      <c r="B78" s="21"/>
+      <c r="C78" s="21"/>
+      <c r="D78" s="21"/>
+      <c r="E78" s="21"/>
+      <c r="F78" s="21"/>
+      <c r="G78" s="21"/>
+      <c r="H78" s="21"/>
+      <c r="I78" s="21"/>
+      <c r="J78" s="21"/>
+      <c r="K78" s="21"/>
+      <c r="L78" s="21"/>
+      <c r="M78" s="21"/>
+      <c r="N78" s="21"/>
       <c r="O78" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="79" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A79" s="24"/>
-      <c r="B79" s="24"/>
-      <c r="C79" s="24"/>
-      <c r="D79" s="24"/>
-      <c r="E79" s="24"/>
-      <c r="F79" s="24"/>
-      <c r="G79" s="24"/>
-      <c r="H79" s="24"/>
-      <c r="I79" s="24"/>
-      <c r="J79" s="24"/>
-      <c r="K79" s="24"/>
-      <c r="L79" s="24"/>
-      <c r="M79" s="24"/>
-      <c r="N79" s="24"/>
+      <c r="A79" s="21"/>
+      <c r="B79" s="21"/>
+      <c r="C79" s="21"/>
+      <c r="D79" s="21"/>
+      <c r="E79" s="21"/>
+      <c r="F79" s="21"/>
+      <c r="G79" s="21"/>
+      <c r="H79" s="21"/>
+      <c r="I79" s="21"/>
+      <c r="J79" s="21"/>
+      <c r="K79" s="21"/>
+      <c r="L79" s="21"/>
+      <c r="M79" s="21"/>
+      <c r="N79" s="21"/>
       <c r="O79" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="80" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A80" s="24"/>
-      <c r="B80" s="24"/>
-      <c r="C80" s="24"/>
-      <c r="D80" s="24"/>
-      <c r="E80" s="24"/>
-      <c r="F80" s="24"/>
-      <c r="G80" s="24"/>
-      <c r="H80" s="24"/>
-      <c r="I80" s="24"/>
-      <c r="J80" s="24"/>
-      <c r="K80" s="24"/>
-      <c r="L80" s="24"/>
-      <c r="M80" s="24"/>
-      <c r="N80" s="24"/>
+      <c r="A80" s="21"/>
+      <c r="B80" s="21"/>
+      <c r="C80" s="21"/>
+      <c r="D80" s="21"/>
+      <c r="E80" s="21"/>
+      <c r="F80" s="21"/>
+      <c r="G80" s="21"/>
+      <c r="H80" s="21"/>
+      <c r="I80" s="21"/>
+      <c r="J80" s="21"/>
+      <c r="K80" s="21"/>
+      <c r="L80" s="21"/>
+      <c r="M80" s="21"/>
+      <c r="N80" s="21"/>
       <c r="O80" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="81" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A81" s="24"/>
-      <c r="B81" s="24"/>
-      <c r="C81" s="24"/>
-      <c r="D81" s="24"/>
-      <c r="E81" s="24"/>
-      <c r="F81" s="24"/>
-      <c r="G81" s="24"/>
-      <c r="H81" s="24"/>
-      <c r="I81" s="24"/>
-      <c r="J81" s="24"/>
-      <c r="K81" s="24"/>
-      <c r="L81" s="24"/>
-      <c r="M81" s="24"/>
-      <c r="N81" s="24"/>
+      <c r="A81" s="21"/>
+      <c r="B81" s="21"/>
+      <c r="C81" s="21"/>
+      <c r="D81" s="21"/>
+      <c r="E81" s="21"/>
+      <c r="F81" s="21"/>
+      <c r="G81" s="21"/>
+      <c r="H81" s="21"/>
+      <c r="I81" s="21"/>
+      <c r="J81" s="21"/>
+      <c r="K81" s="21"/>
+      <c r="L81" s="21"/>
+      <c r="M81" s="21"/>
+      <c r="N81" s="21"/>
       <c r="O81" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="82" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A82" s="24"/>
-      <c r="B82" s="24"/>
-      <c r="C82" s="24"/>
-      <c r="D82" s="24"/>
-      <c r="E82" s="24"/>
-      <c r="F82" s="24"/>
-      <c r="G82" s="24"/>
-      <c r="H82" s="24"/>
-      <c r="I82" s="24"/>
-      <c r="J82" s="24"/>
-      <c r="K82" s="24"/>
-      <c r="L82" s="24"/>
-      <c r="M82" s="24"/>
-      <c r="N82" s="24"/>
+      <c r="A82" s="21"/>
+      <c r="B82" s="21"/>
+      <c r="C82" s="21"/>
+      <c r="D82" s="21"/>
+      <c r="E82" s="21"/>
+      <c r="F82" s="21"/>
+      <c r="G82" s="21"/>
+      <c r="H82" s="21"/>
+      <c r="I82" s="21"/>
+      <c r="J82" s="21"/>
+      <c r="K82" s="21"/>
+      <c r="L82" s="21"/>
+      <c r="M82" s="21"/>
+      <c r="N82" s="21"/>
       <c r="O82" t="s">
         <v>37</v>
       </c>
@@ -5263,6 +5682,14 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="E2:G2"/>
+    <mergeCell ref="H2:J2"/>
+    <mergeCell ref="K2:M2"/>
+    <mergeCell ref="B24:D24"/>
+    <mergeCell ref="E24:G24"/>
+    <mergeCell ref="H24:J24"/>
+    <mergeCell ref="K24:M24"/>
     <mergeCell ref="B65:D65"/>
     <mergeCell ref="E65:G65"/>
     <mergeCell ref="H65:J65"/>
@@ -5271,14 +5698,6 @@
     <mergeCell ref="E44:G44"/>
     <mergeCell ref="H44:J44"/>
     <mergeCell ref="K44:M44"/>
-    <mergeCell ref="B2:D2"/>
-    <mergeCell ref="E2:G2"/>
-    <mergeCell ref="H2:J2"/>
-    <mergeCell ref="K2:M2"/>
-    <mergeCell ref="B24:D24"/>
-    <mergeCell ref="E24:G24"/>
-    <mergeCell ref="H24:J24"/>
-    <mergeCell ref="K24:M24"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -5286,43 +5705,43 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA087EBE-083C-402B-95D7-A249E10AE281}">
-  <dimension ref="A1:O81"/>
+  <dimension ref="A1:AD81"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="31" t="s">
         <v>40</v>
       </c>
-      <c r="C2" s="20"/>
-      <c r="D2" s="21"/>
-      <c r="E2" s="20" t="s">
+      <c r="C2" s="32"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="32" t="s">
         <v>41</v>
       </c>
-      <c r="F2" s="20"/>
-      <c r="G2" s="21"/>
-      <c r="H2" s="20" t="s">
+      <c r="F2" s="32"/>
+      <c r="G2" s="33"/>
+      <c r="H2" s="32" t="s">
         <v>42</v>
       </c>
-      <c r="I2" s="20"/>
-      <c r="J2" s="20"/>
-      <c r="K2" s="19" t="s">
+      <c r="I2" s="32"/>
+      <c r="J2" s="32"/>
+      <c r="K2" s="31" t="s">
         <v>43</v>
       </c>
-      <c r="L2" s="20"/>
-      <c r="M2" s="20"/>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="L2" s="32"/>
+      <c r="M2" s="32"/>
+    </row>
+    <row r="3" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
         <v>1</v>
       </c>
@@ -5363,7 +5782,7 @@
         <v>1.1900000572204501</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A4" s="12" t="s">
         <v>2</v>
       </c>
@@ -5404,7 +5823,7 @@
         <v>1.1900000572204501</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>3</v>
       </c>
@@ -5445,7 +5864,7 @@
         <v>1.1900000572204501</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A6" s="14" t="s">
         <v>4</v>
       </c>
@@ -5486,7 +5905,7 @@
         <v>0.80000001192092896</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>7</v>
       </c>
@@ -5527,7 +5946,7 @@
         <v>0.69999998807907104</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A8" s="12" t="s">
         <v>5</v>
       </c>
@@ -5544,7 +5963,7 @@
       <c r="L8" s="2"/>
       <c r="M8" s="2"/>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A9" s="12" t="s">
         <v>17</v>
       </c>
@@ -5585,68 +6004,115 @@
         <v>0.69999998807907104</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A10" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="37">
+      <c r="B10" s="29">
         <v>0.20000000298023199</v>
       </c>
-      <c r="C10" s="38">
+      <c r="C10" s="30">
         <v>-0.44999998807907099</v>
       </c>
-      <c r="D10" s="38">
-        <v>0</v>
-      </c>
-      <c r="E10" s="37">
+      <c r="D10" s="30">
+        <v>0</v>
+      </c>
+      <c r="E10" s="29">
         <v>0.60000002384185702</v>
       </c>
-      <c r="F10" s="38">
+      <c r="F10" s="30">
         <v>0.44999998807907099</v>
       </c>
-      <c r="G10" s="38">
+      <c r="G10" s="30">
         <v>0.69999998807907104</v>
       </c>
-      <c r="H10" s="37">
-        <v>0</v>
-      </c>
-      <c r="I10" s="38">
+      <c r="H10" s="29">
+        <v>0</v>
+      </c>
+      <c r="I10" s="30">
         <v>-0.46000000834464999</v>
       </c>
-      <c r="J10" s="38">
+      <c r="J10" s="30">
         <v>-0.10000000149011599</v>
       </c>
-      <c r="K10" s="37">
+      <c r="K10" s="29">
         <v>0.60000002384185702</v>
       </c>
-      <c r="L10" s="38">
+      <c r="L10" s="30">
         <v>0.46000000834464999</v>
       </c>
-      <c r="M10" s="38">
+      <c r="M10" s="30">
         <v>0.69999998807907104</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="P11" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q11" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="R11" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="S11" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="T11" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="U11" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="V11" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="W11" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="X11" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="Y11" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z11" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA11" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="AB11" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="AC11" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="AD11" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O12" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O13" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O14" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O15" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O16" t="s">
         <v>35</v>
       </c>
@@ -5675,26 +6141,26 @@
       <c r="A23" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B23" s="19" t="s">
+      <c r="B23" s="31" t="s">
         <v>40</v>
       </c>
-      <c r="C23" s="20"/>
-      <c r="D23" s="21"/>
-      <c r="E23" s="20" t="s">
+      <c r="C23" s="32"/>
+      <c r="D23" s="33"/>
+      <c r="E23" s="32" t="s">
         <v>41</v>
       </c>
-      <c r="F23" s="20"/>
-      <c r="G23" s="21"/>
-      <c r="H23" s="20" t="s">
+      <c r="F23" s="32"/>
+      <c r="G23" s="33"/>
+      <c r="H23" s="32" t="s">
         <v>42</v>
       </c>
-      <c r="I23" s="20"/>
-      <c r="J23" s="20"/>
-      <c r="K23" s="19" t="s">
+      <c r="I23" s="32"/>
+      <c r="J23" s="32"/>
+      <c r="K23" s="31" t="s">
         <v>43</v>
       </c>
-      <c r="L23" s="20"/>
-      <c r="M23" s="20"/>
+      <c r="L23" s="32"/>
+      <c r="M23" s="32"/>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A24" s="14" t="s">
@@ -5963,40 +6429,40 @@
       <c r="A31" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="B31" s="37">
+      <c r="B31" s="29">
         <v>0.230000004172325</v>
       </c>
-      <c r="C31" s="38">
+      <c r="C31" s="30">
         <v>-0.259999990463256</v>
       </c>
-      <c r="D31" s="38">
+      <c r="D31" s="30">
         <v>0.18999999761581399</v>
       </c>
-      <c r="E31" s="37">
+      <c r="E31" s="29">
         <v>0.40999999642372098</v>
       </c>
-      <c r="F31" s="38">
+      <c r="F31" s="30">
         <v>0.259999990463256</v>
       </c>
-      <c r="G31" s="38">
+      <c r="G31" s="30">
         <v>0.50999999046325595</v>
       </c>
-      <c r="H31" s="37">
+      <c r="H31" s="29">
         <v>-0.855000019073486</v>
       </c>
-      <c r="I31" s="38">
+      <c r="I31" s="30">
         <v>-0.855000019073486</v>
       </c>
-      <c r="J31" s="38">
+      <c r="J31" s="30">
         <v>-0.10000000149011599</v>
       </c>
-      <c r="K31" s="37">
+      <c r="K31" s="29">
         <v>0.855000019073486</v>
       </c>
-      <c r="L31" s="38">
+      <c r="L31" s="30">
         <v>0.855000019073486</v>
       </c>
-      <c r="M31" s="38">
+      <c r="M31" s="30">
         <v>1.1900000572204501</v>
       </c>
     </row>
@@ -6049,26 +6515,26 @@
       <c r="A44" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B44" s="19" t="s">
+      <c r="B44" s="31" t="s">
         <v>40</v>
       </c>
-      <c r="C44" s="20"/>
-      <c r="D44" s="21"/>
-      <c r="E44" s="20" t="s">
+      <c r="C44" s="32"/>
+      <c r="D44" s="33"/>
+      <c r="E44" s="32" t="s">
         <v>41</v>
       </c>
-      <c r="F44" s="20"/>
-      <c r="G44" s="21"/>
-      <c r="H44" s="20" t="s">
+      <c r="F44" s="32"/>
+      <c r="G44" s="33"/>
+      <c r="H44" s="32" t="s">
         <v>42</v>
       </c>
-      <c r="I44" s="20"/>
-      <c r="J44" s="20"/>
-      <c r="K44" s="19" t="s">
+      <c r="I44" s="32"/>
+      <c r="J44" s="32"/>
+      <c r="K44" s="31" t="s">
         <v>43</v>
       </c>
-      <c r="L44" s="20"/>
-      <c r="M44" s="20"/>
+      <c r="L44" s="32"/>
+      <c r="M44" s="32"/>
     </row>
     <row r="45" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A45" s="14" t="s">
@@ -6337,40 +6803,40 @@
       <c r="A52" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="B52" s="37">
+      <c r="B52" s="29">
         <v>0.230000004172325</v>
       </c>
-      <c r="C52" s="38">
+      <c r="C52" s="30">
         <v>-0.259999990463256</v>
       </c>
-      <c r="D52" s="38">
+      <c r="D52" s="30">
         <v>0.18999999761581399</v>
       </c>
-      <c r="E52" s="37">
+      <c r="E52" s="29">
         <v>0.40999999642372098</v>
       </c>
-      <c r="F52" s="38">
+      <c r="F52" s="30">
         <v>0.259999990463256</v>
       </c>
-      <c r="G52" s="38">
+      <c r="G52" s="30">
         <v>0.50999999046325595</v>
       </c>
-      <c r="H52" s="37">
+      <c r="H52" s="29">
         <v>-1.9999999552965102E-2</v>
       </c>
-      <c r="I52" s="38">
+      <c r="I52" s="30">
         <v>-0.28000000119209201</v>
       </c>
-      <c r="J52" s="38">
+      <c r="J52" s="30">
         <v>-1.9999999552965102E-2</v>
       </c>
-      <c r="K52" s="37">
+      <c r="K52" s="29">
         <v>0.43000000715255698</v>
       </c>
-      <c r="L52" s="38">
+      <c r="L52" s="30">
         <v>0.28000000119209201</v>
       </c>
-      <c r="M52" s="38">
+      <c r="M52" s="30">
         <v>0.52999997138976995</v>
       </c>
     </row>
@@ -6420,523 +6886,531 @@
       </c>
     </row>
     <row r="64" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A64" s="22" t="s">
-        <v>0</v>
-      </c>
-      <c r="B64" s="33" t="s">
+      <c r="A64" s="19" t="s">
+        <v>0</v>
+      </c>
+      <c r="B64" s="34" t="s">
         <v>40</v>
       </c>
-      <c r="C64" s="32"/>
-      <c r="D64" s="34"/>
-      <c r="E64" s="35" t="s">
+      <c r="C64" s="35"/>
+      <c r="D64" s="36"/>
+      <c r="E64" s="37" t="s">
         <v>41</v>
       </c>
-      <c r="F64" s="32"/>
-      <c r="G64" s="34"/>
-      <c r="H64" s="35" t="s">
+      <c r="F64" s="35"/>
+      <c r="G64" s="36"/>
+      <c r="H64" s="37" t="s">
         <v>42</v>
       </c>
-      <c r="I64" s="32"/>
-      <c r="J64" s="36"/>
-      <c r="K64" s="33" t="s">
+      <c r="I64" s="35"/>
+      <c r="J64" s="38"/>
+      <c r="K64" s="34" t="s">
         <v>43</v>
       </c>
-      <c r="L64" s="32"/>
-      <c r="M64" s="32"/>
-      <c r="N64" s="24"/>
-      <c r="O64" s="24"/>
+      <c r="L64" s="35"/>
+      <c r="M64" s="35"/>
+      <c r="N64" s="21"/>
+      <c r="O64" s="21"/>
     </row>
     <row r="65" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A65" s="25" t="s">
+      <c r="A65" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="B65" s="26">
+      <c r="B65" s="23">
         <v>0.18999999761581399</v>
       </c>
-      <c r="C65" s="26">
+      <c r="C65" s="23">
         <v>-0.55000001192092896</v>
       </c>
-      <c r="D65" s="27">
+      <c r="D65" s="24">
         <v>5.0000000745057997E-2</v>
       </c>
-      <c r="E65" s="26">
+      <c r="E65" s="23">
         <v>0.50999999046325595</v>
       </c>
-      <c r="F65" s="26">
+      <c r="F65" s="23">
         <v>0.55000001192092896</v>
       </c>
-      <c r="G65" s="27">
+      <c r="G65" s="24">
         <v>0.64999997615814198</v>
       </c>
-      <c r="H65" s="26">
+      <c r="H65" s="23">
         <v>-0.40500000119209201</v>
       </c>
-      <c r="I65" s="26">
+      <c r="I65" s="23">
         <v>-0.62999999523162797</v>
       </c>
-      <c r="J65" s="26">
+      <c r="J65" s="23">
         <v>1.49999996647238E-2</v>
       </c>
-      <c r="K65" s="28">
+      <c r="K65" s="25">
         <v>0.33500000834464999</v>
       </c>
-      <c r="L65" s="26">
+      <c r="L65" s="23">
         <v>0.61000001430511397</v>
       </c>
-      <c r="M65" s="26">
+      <c r="M65" s="23">
         <v>0.65499997138976995</v>
       </c>
-      <c r="N65" s="24"/>
-      <c r="O65" s="24"/>
+      <c r="N65" s="21"/>
+      <c r="O65" s="21"/>
     </row>
     <row r="66" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A66" s="25" t="s">
+      <c r="A66" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="B66" s="26">
+      <c r="B66" s="23">
         <v>0.18999999761581399</v>
       </c>
-      <c r="C66" s="26">
+      <c r="C66" s="23">
         <v>-0.55000001192092896</v>
       </c>
-      <c r="D66" s="27">
+      <c r="D66" s="24">
         <v>5.0000000745057997E-2</v>
       </c>
-      <c r="E66" s="26">
+      <c r="E66" s="23">
         <v>0.50999999046325595</v>
       </c>
-      <c r="F66" s="26">
+      <c r="F66" s="23">
         <v>0.55000001192092896</v>
       </c>
-      <c r="G66" s="27">
+      <c r="G66" s="24">
         <v>0.64999997615814198</v>
       </c>
-      <c r="H66" s="26">
+      <c r="H66" s="23">
         <v>-0.41999998688697798</v>
       </c>
-      <c r="I66" s="26">
+      <c r="I66" s="23">
         <v>-0.92000001668929998</v>
       </c>
-      <c r="J66" s="26">
+      <c r="J66" s="23">
         <v>2.9999999329447701E-2</v>
       </c>
-      <c r="K66" s="28">
+      <c r="K66" s="25">
         <v>0.31999999284744202</v>
       </c>
-      <c r="L66" s="26">
+      <c r="L66" s="23">
         <v>0.31999999284744202</v>
       </c>
-      <c r="M66" s="26">
+      <c r="M66" s="23">
         <v>0.67000001668929998</v>
       </c>
-      <c r="N66" s="24"/>
-      <c r="O66" s="24"/>
+      <c r="N66" s="21"/>
+      <c r="O66" s="21"/>
     </row>
     <row r="67" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A67" s="22" t="s">
+      <c r="A67" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="B67" s="29">
+      <c r="B67" s="26">
         <v>-0.55000001192092896</v>
       </c>
-      <c r="C67" s="29">
+      <c r="C67" s="26">
         <v>-0.75</v>
       </c>
-      <c r="D67" s="30">
+      <c r="D67" s="27">
         <v>-2.9999999329447701E-2</v>
       </c>
-      <c r="E67" s="29">
+      <c r="E67" s="26">
         <v>0.44999998807907099</v>
       </c>
-      <c r="F67" s="29">
+      <c r="F67" s="26">
         <v>1.25</v>
       </c>
-      <c r="G67" s="30">
+      <c r="G67" s="27">
         <v>0.76999998092651301</v>
       </c>
-      <c r="H67" s="29">
+      <c r="H67" s="26">
         <v>-1.04999995231628</v>
       </c>
-      <c r="I67" s="29">
+      <c r="I67" s="26">
         <v>-1.3500000238418499</v>
       </c>
-      <c r="J67" s="29">
+      <c r="J67" s="26">
         <v>-0.57999998331069902</v>
       </c>
-      <c r="K67" s="31">
+      <c r="K67" s="28">
         <v>0.34999999403953502</v>
       </c>
-      <c r="L67" s="29">
+      <c r="L67" s="26">
         <v>1.25</v>
       </c>
-      <c r="M67" s="29">
+      <c r="M67" s="26">
         <v>0.72000002861022905</v>
       </c>
-      <c r="N67" s="24"/>
-      <c r="O67" s="24"/>
+      <c r="N67" s="21"/>
+      <c r="O67" s="21"/>
     </row>
     <row r="68" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A68" s="25" t="s">
+      <c r="A68" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="B68" s="26">
+      <c r="B68" s="23">
         <v>0.140000000596046</v>
       </c>
-      <c r="C68" s="26">
+      <c r="C68" s="23">
         <v>-0.60000002384185702</v>
       </c>
-      <c r="D68" s="27">
+      <c r="D68" s="24">
         <v>5.0000000745057997E-2</v>
       </c>
-      <c r="E68" s="26">
+      <c r="E68" s="23">
         <v>0.55000001192092896</v>
       </c>
-      <c r="F68" s="26">
+      <c r="F68" s="23">
         <v>0.60000002384185702</v>
       </c>
-      <c r="G68" s="27">
+      <c r="G68" s="24">
         <v>0.64999997615814198</v>
       </c>
-      <c r="H68" s="26">
+      <c r="H68" s="23">
         <v>-0.20000000298023199</v>
       </c>
-      <c r="I68" s="26">
+      <c r="I68" s="23">
         <v>-0.80000001192092896</v>
       </c>
-      <c r="J68" s="26">
+      <c r="J68" s="23">
         <v>-0.20000000298023199</v>
       </c>
-      <c r="K68" s="28">
+      <c r="K68" s="25">
         <v>0.75</v>
       </c>
-      <c r="L68" s="26">
+      <c r="L68" s="23">
         <v>0.80000001192092896</v>
       </c>
-      <c r="M68" s="26">
+      <c r="M68" s="23">
         <v>0.85000002384185702</v>
       </c>
-      <c r="N68" s="24"/>
-      <c r="O68" s="24"/>
+      <c r="N68" s="21"/>
+      <c r="O68" s="21"/>
     </row>
     <row r="69" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A69" s="22" t="s">
+      <c r="A69" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="B69" s="29">
+      <c r="B69" s="26">
         <v>0.140000000596046</v>
       </c>
-      <c r="C69" s="29">
+      <c r="C69" s="26">
         <v>-0.60000002384185702</v>
       </c>
-      <c r="D69" s="30">
+      <c r="D69" s="27">
         <v>5.0000000745057997E-2</v>
       </c>
-      <c r="E69" s="29">
+      <c r="E69" s="26">
         <v>0.55000001192092896</v>
       </c>
-      <c r="F69" s="29">
+      <c r="F69" s="26">
         <v>0.60000002384185702</v>
       </c>
-      <c r="G69" s="30">
+      <c r="G69" s="27">
         <v>0.64999997615814198</v>
       </c>
-      <c r="H69" s="29">
+      <c r="H69" s="26">
         <v>-0.20000000298023199</v>
       </c>
-      <c r="I69" s="29">
+      <c r="I69" s="26">
         <v>-0.80000001192092896</v>
       </c>
-      <c r="J69" s="29">
+      <c r="J69" s="26">
         <v>-0.20000000298023199</v>
       </c>
-      <c r="K69" s="31">
+      <c r="K69" s="28">
         <v>0.75</v>
       </c>
-      <c r="L69" s="29">
+      <c r="L69" s="26">
         <v>0.80000001192092896</v>
       </c>
-      <c r="M69" s="29">
+      <c r="M69" s="26">
         <v>0.85000002384185702</v>
       </c>
-      <c r="N69" s="24"/>
-      <c r="O69" s="24"/>
+      <c r="N69" s="21"/>
+      <c r="O69" s="21"/>
     </row>
     <row r="70" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A70" s="25" t="s">
+      <c r="A70" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="B70" s="26"/>
-      <c r="C70" s="26"/>
-      <c r="D70" s="27"/>
-      <c r="E70" s="26"/>
-      <c r="F70" s="26"/>
-      <c r="G70" s="27"/>
-      <c r="H70" s="26"/>
-      <c r="I70" s="26"/>
-      <c r="J70" s="26"/>
-      <c r="K70" s="28"/>
-      <c r="L70" s="26"/>
-      <c r="M70" s="26"/>
-      <c r="N70" s="24"/>
-      <c r="O70" s="24"/>
+      <c r="B70" s="23"/>
+      <c r="C70" s="23"/>
+      <c r="D70" s="24"/>
+      <c r="E70" s="23"/>
+      <c r="F70" s="23"/>
+      <c r="G70" s="24"/>
+      <c r="H70" s="23"/>
+      <c r="I70" s="23"/>
+      <c r="J70" s="23"/>
+      <c r="K70" s="25"/>
+      <c r="L70" s="23"/>
+      <c r="M70" s="23"/>
+      <c r="N70" s="21"/>
+      <c r="O70" s="21"/>
     </row>
     <row r="71" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A71" s="25" t="s">
+      <c r="A71" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="B71" s="26">
+      <c r="B71" s="23">
         <v>0.140000000596046</v>
       </c>
-      <c r="C71" s="26">
+      <c r="C71" s="23">
         <v>-0.60000002384185702</v>
       </c>
-      <c r="D71" s="27">
+      <c r="D71" s="24">
         <v>5.0000000745057997E-2</v>
       </c>
-      <c r="E71" s="26">
+      <c r="E71" s="23">
         <v>0.55000001192092896</v>
       </c>
-      <c r="F71" s="26">
+      <c r="F71" s="23">
         <v>0.60000002384185702</v>
       </c>
-      <c r="G71" s="27">
+      <c r="G71" s="24">
         <v>0.64999997615814198</v>
       </c>
-      <c r="H71" s="26">
+      <c r="H71" s="23">
         <v>-0.20000000298023199</v>
       </c>
-      <c r="I71" s="26">
+      <c r="I71" s="23">
         <v>-0.80000001192092896</v>
       </c>
-      <c r="J71" s="26">
+      <c r="J71" s="23">
         <v>-0.20000000298023199</v>
       </c>
-      <c r="K71" s="28">
+      <c r="K71" s="25">
         <v>0.75</v>
       </c>
-      <c r="L71" s="26">
+      <c r="L71" s="23">
         <v>0.80000001192092896</v>
       </c>
-      <c r="M71" s="26">
+      <c r="M71" s="23">
         <v>0.85000002384185702</v>
       </c>
-      <c r="N71" s="24"/>
-      <c r="O71" s="24"/>
+      <c r="N71" s="21"/>
+      <c r="O71" s="21"/>
     </row>
     <row r="72" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A72" s="23" t="s">
+      <c r="A72" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="B72" s="31">
+      <c r="B72" s="28">
         <v>0.140000000596046</v>
       </c>
-      <c r="C72" s="29">
+      <c r="C72" s="26">
         <v>-0.60000002384185702</v>
       </c>
-      <c r="D72" s="29">
+      <c r="D72" s="26">
         <v>5.0000000745057997E-2</v>
       </c>
-      <c r="E72" s="31">
+      <c r="E72" s="28">
         <v>0.55000001192092896</v>
       </c>
-      <c r="F72" s="29">
+      <c r="F72" s="26">
         <v>0.60000002384185702</v>
       </c>
-      <c r="G72" s="29">
+      <c r="G72" s="26">
         <v>0.64999997615814198</v>
       </c>
-      <c r="H72" s="31">
+      <c r="H72" s="28">
         <v>-0.20000000298023199</v>
       </c>
-      <c r="I72" s="29">
+      <c r="I72" s="26">
         <v>-0.80000001192092896</v>
       </c>
-      <c r="J72" s="29">
+      <c r="J72" s="26">
         <v>-0.20000000298023199</v>
       </c>
-      <c r="K72" s="31">
+      <c r="K72" s="28">
         <v>0.75</v>
       </c>
-      <c r="L72" s="29">
+      <c r="L72" s="26">
         <v>0.80000001192092896</v>
       </c>
-      <c r="M72" s="29">
+      <c r="M72" s="26">
         <v>0.85000002384185702</v>
       </c>
-      <c r="N72" s="24"/>
-      <c r="O72" s="24"/>
+      <c r="N72" s="21"/>
+      <c r="O72" s="21"/>
     </row>
     <row r="73" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A73" s="24"/>
-      <c r="B73" s="24"/>
-      <c r="C73" s="24"/>
-      <c r="D73" s="24"/>
-      <c r="E73" s="24"/>
-      <c r="F73" s="24"/>
-      <c r="G73" s="24"/>
-      <c r="H73" s="24"/>
-      <c r="I73" s="24"/>
-      <c r="J73" s="24"/>
-      <c r="K73" s="24"/>
-      <c r="L73" s="24"/>
-      <c r="M73" s="24"/>
-      <c r="N73" s="24"/>
-      <c r="O73" s="24"/>
+      <c r="A73" s="21"/>
+      <c r="B73" s="21"/>
+      <c r="C73" s="21"/>
+      <c r="D73" s="21"/>
+      <c r="E73" s="21"/>
+      <c r="F73" s="21"/>
+      <c r="G73" s="21"/>
+      <c r="H73" s="21"/>
+      <c r="I73" s="21"/>
+      <c r="J73" s="21"/>
+      <c r="K73" s="21"/>
+      <c r="L73" s="21"/>
+      <c r="M73" s="21"/>
+      <c r="N73" s="21"/>
+      <c r="O73" s="21"/>
     </row>
     <row r="74" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A74" s="24"/>
-      <c r="B74" s="24"/>
-      <c r="C74" s="24"/>
-      <c r="D74" s="24"/>
-      <c r="E74" s="24"/>
-      <c r="F74" s="24"/>
-      <c r="G74" s="24"/>
-      <c r="H74" s="24"/>
-      <c r="I74" s="24"/>
-      <c r="J74" s="24"/>
-      <c r="K74" s="24"/>
-      <c r="L74" s="24"/>
-      <c r="M74" s="24"/>
-      <c r="N74" s="24"/>
-      <c r="O74" s="24" t="s">
+      <c r="A74" s="21"/>
+      <c r="B74" s="21"/>
+      <c r="C74" s="21"/>
+      <c r="D74" s="21"/>
+      <c r="E74" s="21"/>
+      <c r="F74" s="21"/>
+      <c r="G74" s="21"/>
+      <c r="H74" s="21"/>
+      <c r="I74" s="21"/>
+      <c r="J74" s="21"/>
+      <c r="K74" s="21"/>
+      <c r="L74" s="21"/>
+      <c r="M74" s="21"/>
+      <c r="N74" s="21"/>
+      <c r="O74" s="21" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="75" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A75" s="24"/>
-      <c r="B75" s="24"/>
-      <c r="C75" s="24"/>
-      <c r="D75" s="24"/>
-      <c r="E75" s="24"/>
-      <c r="F75" s="24"/>
-      <c r="G75" s="24"/>
-      <c r="H75" s="24"/>
-      <c r="I75" s="24"/>
-      <c r="J75" s="24"/>
-      <c r="K75" s="24"/>
-      <c r="L75" s="24"/>
-      <c r="M75" s="24"/>
-      <c r="N75" s="24"/>
-      <c r="O75" s="24" t="s">
+      <c r="A75" s="21"/>
+      <c r="B75" s="21"/>
+      <c r="C75" s="21"/>
+      <c r="D75" s="21"/>
+      <c r="E75" s="21"/>
+      <c r="F75" s="21"/>
+      <c r="G75" s="21"/>
+      <c r="H75" s="21"/>
+      <c r="I75" s="21"/>
+      <c r="J75" s="21"/>
+      <c r="K75" s="21"/>
+      <c r="L75" s="21"/>
+      <c r="M75" s="21"/>
+      <c r="N75" s="21"/>
+      <c r="O75" s="21" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="76" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A76" s="24"/>
-      <c r="B76" s="24"/>
-      <c r="C76" s="24"/>
-      <c r="D76" s="24"/>
-      <c r="E76" s="24"/>
-      <c r="F76" s="24"/>
-      <c r="G76" s="24"/>
-      <c r="H76" s="24"/>
-      <c r="I76" s="24"/>
-      <c r="J76" s="24"/>
-      <c r="K76" s="24"/>
-      <c r="L76" s="24"/>
-      <c r="M76" s="24"/>
-      <c r="N76" s="24"/>
-      <c r="O76" s="24" t="s">
+      <c r="A76" s="21"/>
+      <c r="B76" s="21"/>
+      <c r="C76" s="21"/>
+      <c r="D76" s="21"/>
+      <c r="E76" s="21"/>
+      <c r="F76" s="21"/>
+      <c r="G76" s="21"/>
+      <c r="H76" s="21"/>
+      <c r="I76" s="21"/>
+      <c r="J76" s="21"/>
+      <c r="K76" s="21"/>
+      <c r="L76" s="21"/>
+      <c r="M76" s="21"/>
+      <c r="N76" s="21"/>
+      <c r="O76" s="21" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="77" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A77" s="24"/>
-      <c r="B77" s="24"/>
-      <c r="C77" s="24"/>
-      <c r="D77" s="24"/>
-      <c r="E77" s="24"/>
-      <c r="F77" s="24"/>
-      <c r="G77" s="24"/>
-      <c r="H77" s="24"/>
-      <c r="I77" s="24"/>
-      <c r="J77" s="24"/>
-      <c r="K77" s="24"/>
-      <c r="L77" s="24"/>
-      <c r="M77" s="24"/>
-      <c r="N77" s="24"/>
-      <c r="O77" s="24" t="s">
+      <c r="A77" s="21"/>
+      <c r="B77" s="21"/>
+      <c r="C77" s="21"/>
+      <c r="D77" s="21"/>
+      <c r="E77" s="21"/>
+      <c r="F77" s="21"/>
+      <c r="G77" s="21"/>
+      <c r="H77" s="21"/>
+      <c r="I77" s="21"/>
+      <c r="J77" s="21"/>
+      <c r="K77" s="21"/>
+      <c r="L77" s="21"/>
+      <c r="M77" s="21"/>
+      <c r="N77" s="21"/>
+      <c r="O77" s="21" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="78" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A78" s="24"/>
-      <c r="B78" s="24"/>
-      <c r="C78" s="24"/>
-      <c r="D78" s="24"/>
-      <c r="E78" s="24"/>
-      <c r="F78" s="24"/>
-      <c r="G78" s="24"/>
-      <c r="H78" s="24"/>
-      <c r="I78" s="24"/>
-      <c r="J78" s="24"/>
-      <c r="K78" s="24"/>
-      <c r="L78" s="24"/>
-      <c r="M78" s="24"/>
-      <c r="N78" s="24"/>
-      <c r="O78" s="24" t="s">
+      <c r="A78" s="21"/>
+      <c r="B78" s="21"/>
+      <c r="C78" s="21"/>
+      <c r="D78" s="21"/>
+      <c r="E78" s="21"/>
+      <c r="F78" s="21"/>
+      <c r="G78" s="21"/>
+      <c r="H78" s="21"/>
+      <c r="I78" s="21"/>
+      <c r="J78" s="21"/>
+      <c r="K78" s="21"/>
+      <c r="L78" s="21"/>
+      <c r="M78" s="21"/>
+      <c r="N78" s="21"/>
+      <c r="O78" s="21" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="79" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A79" s="24"/>
-      <c r="B79" s="24"/>
-      <c r="C79" s="24"/>
-      <c r="D79" s="24"/>
-      <c r="E79" s="24"/>
-      <c r="F79" s="24"/>
-      <c r="G79" s="24"/>
-      <c r="H79" s="24"/>
-      <c r="I79" s="24"/>
-      <c r="J79" s="24"/>
-      <c r="K79" s="24"/>
-      <c r="L79" s="24"/>
-      <c r="M79" s="24"/>
-      <c r="N79" s="24"/>
-      <c r="O79" s="24" t="s">
+      <c r="A79" s="21"/>
+      <c r="B79" s="21"/>
+      <c r="C79" s="21"/>
+      <c r="D79" s="21"/>
+      <c r="E79" s="21"/>
+      <c r="F79" s="21"/>
+      <c r="G79" s="21"/>
+      <c r="H79" s="21"/>
+      <c r="I79" s="21"/>
+      <c r="J79" s="21"/>
+      <c r="K79" s="21"/>
+      <c r="L79" s="21"/>
+      <c r="M79" s="21"/>
+      <c r="N79" s="21"/>
+      <c r="O79" s="21" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="80" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A80" s="24"/>
-      <c r="B80" s="24"/>
-      <c r="C80" s="24"/>
-      <c r="D80" s="24"/>
-      <c r="E80" s="24"/>
-      <c r="F80" s="24"/>
-      <c r="G80" s="24"/>
-      <c r="H80" s="24"/>
-      <c r="I80" s="24"/>
-      <c r="J80" s="24"/>
-      <c r="K80" s="24"/>
-      <c r="L80" s="24"/>
-      <c r="M80" s="24"/>
-      <c r="N80" s="24"/>
-      <c r="O80" s="24" t="s">
+      <c r="A80" s="21"/>
+      <c r="B80" s="21"/>
+      <c r="C80" s="21"/>
+      <c r="D80" s="21"/>
+      <c r="E80" s="21"/>
+      <c r="F80" s="21"/>
+      <c r="G80" s="21"/>
+      <c r="H80" s="21"/>
+      <c r="I80" s="21"/>
+      <c r="J80" s="21"/>
+      <c r="K80" s="21"/>
+      <c r="L80" s="21"/>
+      <c r="M80" s="21"/>
+      <c r="N80" s="21"/>
+      <c r="O80" s="21" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="81" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A81" s="24"/>
-      <c r="B81" s="24"/>
-      <c r="C81" s="24"/>
-      <c r="D81" s="24"/>
-      <c r="E81" s="24"/>
-      <c r="F81" s="24"/>
-      <c r="G81" s="24"/>
-      <c r="H81" s="24"/>
-      <c r="I81" s="24"/>
-      <c r="J81" s="24"/>
-      <c r="K81" s="24"/>
-      <c r="L81" s="24"/>
-      <c r="M81" s="24"/>
-      <c r="N81" s="24"/>
-      <c r="O81" s="24" t="s">
+      <c r="A81" s="21"/>
+      <c r="B81" s="21"/>
+      <c r="C81" s="21"/>
+      <c r="D81" s="21"/>
+      <c r="E81" s="21"/>
+      <c r="F81" s="21"/>
+      <c r="G81" s="21"/>
+      <c r="H81" s="21"/>
+      <c r="I81" s="21"/>
+      <c r="J81" s="21"/>
+      <c r="K81" s="21"/>
+      <c r="L81" s="21"/>
+      <c r="M81" s="21"/>
+      <c r="N81" s="21"/>
+      <c r="O81" s="21" t="s">
         <v>38</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="E2:G2"/>
+    <mergeCell ref="H2:J2"/>
+    <mergeCell ref="K2:M2"/>
+    <mergeCell ref="B23:D23"/>
+    <mergeCell ref="E23:G23"/>
+    <mergeCell ref="H23:J23"/>
+    <mergeCell ref="K23:M23"/>
     <mergeCell ref="B44:D44"/>
     <mergeCell ref="E44:G44"/>
     <mergeCell ref="H44:J44"/>
@@ -6945,14 +7419,6 @@
     <mergeCell ref="E64:G64"/>
     <mergeCell ref="H64:J64"/>
     <mergeCell ref="K64:M64"/>
-    <mergeCell ref="B2:D2"/>
-    <mergeCell ref="E2:G2"/>
-    <mergeCell ref="H2:J2"/>
-    <mergeCell ref="K2:M2"/>
-    <mergeCell ref="B23:D23"/>
-    <mergeCell ref="E23:G23"/>
-    <mergeCell ref="H23:J23"/>
-    <mergeCell ref="K23:M23"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -6960,43 +7426,43 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB1CCC97-D0A7-4837-9497-07689BD5D6D2}">
-  <dimension ref="A1:O82"/>
+  <dimension ref="A1:AD82"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="31" t="s">
         <v>40</v>
       </c>
-      <c r="C2" s="20"/>
-      <c r="D2" s="21"/>
-      <c r="E2" s="20" t="s">
+      <c r="C2" s="32"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="32" t="s">
         <v>41</v>
       </c>
-      <c r="F2" s="20"/>
-      <c r="G2" s="21"/>
-      <c r="H2" s="20" t="s">
+      <c r="F2" s="32"/>
+      <c r="G2" s="33"/>
+      <c r="H2" s="32" t="s">
         <v>42</v>
       </c>
-      <c r="I2" s="20"/>
-      <c r="J2" s="20"/>
-      <c r="K2" s="19" t="s">
+      <c r="I2" s="32"/>
+      <c r="J2" s="32"/>
+      <c r="K2" s="31" t="s">
         <v>43</v>
       </c>
-      <c r="L2" s="20"/>
-      <c r="M2" s="20"/>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="L2" s="32"/>
+      <c r="M2" s="32"/>
+    </row>
+    <row r="3" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
         <v>1</v>
       </c>
@@ -7037,7 +7503,7 @@
         <v>1.1900000572204501</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A4" s="12" t="s">
         <v>2</v>
       </c>
@@ -7078,7 +7544,7 @@
         <v>1.1900000572204501</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>3</v>
       </c>
@@ -7119,7 +7585,7 @@
         <v>1.1900000572204501</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A6" s="14" t="s">
         <v>4</v>
       </c>
@@ -7160,7 +7626,7 @@
         <v>0.55000001192092896</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>7</v>
       </c>
@@ -7201,7 +7667,7 @@
         <v>0.60000002384185702</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A8" s="12" t="s">
         <v>5</v>
       </c>
@@ -7218,7 +7684,7 @@
       <c r="L8" s="2"/>
       <c r="M8" s="2"/>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A9" s="12" t="s">
         <v>17</v>
       </c>
@@ -7259,7 +7725,7 @@
         <v>0.60000002384185702</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A10" s="13" t="s">
         <v>6</v>
       </c>
@@ -7276,27 +7742,74 @@
       <c r="L10" s="10"/>
       <c r="M10" s="10"/>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="P11" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q11" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="R11" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="S11" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="T11" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="U11" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="V11" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="W11" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="X11" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="Y11" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z11" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA11" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="AB11" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="AC11" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="AD11" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O12" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O13" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O14" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O15" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O16" t="s">
         <v>35</v>
       </c>
@@ -7325,26 +7838,26 @@
       <c r="A23" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B23" s="19" t="s">
+      <c r="B23" s="31" t="s">
         <v>40</v>
       </c>
-      <c r="C23" s="20"/>
-      <c r="D23" s="21"/>
-      <c r="E23" s="20" t="s">
+      <c r="C23" s="32"/>
+      <c r="D23" s="33"/>
+      <c r="E23" s="32" t="s">
         <v>41</v>
       </c>
-      <c r="F23" s="20"/>
-      <c r="G23" s="21"/>
-      <c r="H23" s="20" t="s">
+      <c r="F23" s="32"/>
+      <c r="G23" s="33"/>
+      <c r="H23" s="32" t="s">
         <v>42</v>
       </c>
-      <c r="I23" s="20"/>
-      <c r="J23" s="20"/>
-      <c r="K23" s="19" t="s">
+      <c r="I23" s="32"/>
+      <c r="J23" s="32"/>
+      <c r="K23" s="31" t="s">
         <v>43</v>
       </c>
-      <c r="L23" s="20"/>
-      <c r="M23" s="20"/>
+      <c r="L23" s="32"/>
+      <c r="M23" s="32"/>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A24" s="14" t="s">
@@ -7675,26 +8188,26 @@
       <c r="A44" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B44" s="19" t="s">
+      <c r="B44" s="31" t="s">
         <v>40</v>
       </c>
-      <c r="C44" s="20"/>
-      <c r="D44" s="21"/>
-      <c r="E44" s="20" t="s">
+      <c r="C44" s="32"/>
+      <c r="D44" s="33"/>
+      <c r="E44" s="32" t="s">
         <v>41</v>
       </c>
-      <c r="F44" s="20"/>
-      <c r="G44" s="21"/>
-      <c r="H44" s="20" t="s">
+      <c r="F44" s="32"/>
+      <c r="G44" s="33"/>
+      <c r="H44" s="32" t="s">
         <v>42</v>
       </c>
-      <c r="I44" s="20"/>
-      <c r="J44" s="20"/>
-      <c r="K44" s="19" t="s">
+      <c r="I44" s="32"/>
+      <c r="J44" s="32"/>
+      <c r="K44" s="31" t="s">
         <v>43</v>
       </c>
-      <c r="L44" s="20"/>
-      <c r="M44" s="20"/>
+      <c r="L44" s="32"/>
+      <c r="M44" s="32"/>
     </row>
     <row r="45" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A45" s="14" t="s">
@@ -7998,523 +8511,531 @@
       </c>
     </row>
     <row r="65" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A65" s="22" t="s">
-        <v>0</v>
-      </c>
-      <c r="B65" s="33" t="s">
+      <c r="A65" s="19" t="s">
+        <v>0</v>
+      </c>
+      <c r="B65" s="34" t="s">
         <v>40</v>
       </c>
-      <c r="C65" s="32"/>
-      <c r="D65" s="34"/>
-      <c r="E65" s="35" t="s">
+      <c r="C65" s="35"/>
+      <c r="D65" s="36"/>
+      <c r="E65" s="37" t="s">
         <v>41</v>
       </c>
-      <c r="F65" s="32"/>
-      <c r="G65" s="34"/>
-      <c r="H65" s="35" t="s">
+      <c r="F65" s="35"/>
+      <c r="G65" s="36"/>
+      <c r="H65" s="37" t="s">
         <v>42</v>
       </c>
-      <c r="I65" s="32"/>
-      <c r="J65" s="36"/>
-      <c r="K65" s="33" t="s">
+      <c r="I65" s="35"/>
+      <c r="J65" s="38"/>
+      <c r="K65" s="34" t="s">
         <v>43</v>
       </c>
-      <c r="L65" s="32"/>
-      <c r="M65" s="32"/>
-      <c r="N65" s="24"/>
-      <c r="O65" s="24"/>
+      <c r="L65" s="35"/>
+      <c r="M65" s="35"/>
+      <c r="N65" s="21"/>
+      <c r="O65" s="21"/>
     </row>
     <row r="66" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A66" s="25" t="s">
+      <c r="A66" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="B66" s="26">
+      <c r="B66" s="23">
         <v>0.34499999880790699</v>
       </c>
-      <c r="C66" s="26">
+      <c r="C66" s="23">
         <v>-1</v>
       </c>
-      <c r="D66" s="27">
+      <c r="D66" s="24">
         <v>0.125</v>
       </c>
-      <c r="E66" s="26">
+      <c r="E66" s="23">
         <v>0.55500000715255704</v>
       </c>
-      <c r="F66" s="26">
-        <v>0</v>
-      </c>
-      <c r="G66" s="27">
+      <c r="F66" s="23">
+        <v>0</v>
+      </c>
+      <c r="G66" s="24">
         <v>0.52499997615814198</v>
       </c>
-      <c r="H66" s="26">
+      <c r="H66" s="23">
         <v>0.245000004768371</v>
       </c>
-      <c r="I66" s="26">
+      <c r="I66" s="23">
         <v>-1.1000000238418499</v>
       </c>
-      <c r="J66" s="26">
+      <c r="J66" s="23">
         <v>2.5000000372528999E-2</v>
       </c>
-      <c r="K66" s="28">
+      <c r="K66" s="25">
         <v>0.65499997138976995</v>
       </c>
-      <c r="L66" s="26">
+      <c r="L66" s="23">
         <v>0.10000000149011599</v>
       </c>
-      <c r="M66" s="26">
+      <c r="M66" s="23">
         <v>0.625</v>
       </c>
-      <c r="N66" s="24"/>
-      <c r="O66" s="24"/>
+      <c r="N66" s="21"/>
+      <c r="O66" s="21"/>
     </row>
     <row r="67" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A67" s="25" t="s">
+      <c r="A67" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="B67" s="26">
+      <c r="B67" s="23">
         <v>0.34700000286102201</v>
       </c>
-      <c r="C67" s="26">
+      <c r="C67" s="23">
         <v>-1</v>
       </c>
-      <c r="D67" s="27">
+      <c r="D67" s="24">
         <v>0.125</v>
       </c>
-      <c r="E67" s="26">
+      <c r="E67" s="23">
         <v>0.55299997329711903</v>
       </c>
-      <c r="F67" s="26">
-        <v>0</v>
-      </c>
-      <c r="G67" s="27">
+      <c r="F67" s="23">
+        <v>0</v>
+      </c>
+      <c r="G67" s="24">
         <v>0.52499997615814198</v>
       </c>
-      <c r="H67" s="26">
+      <c r="H67" s="23">
         <v>0.22200000286102201</v>
       </c>
-      <c r="I67" s="26">
+      <c r="I67" s="23">
         <v>-1.1000000238418499</v>
       </c>
-      <c r="J67" s="26">
+      <c r="J67" s="23">
         <v>5.0000000745057997E-2</v>
       </c>
-      <c r="K67" s="28">
+      <c r="K67" s="25">
         <v>0.67799997329711903</v>
       </c>
-      <c r="L67" s="26">
+      <c r="L67" s="23">
         <v>0.10000000149011599</v>
       </c>
-      <c r="M67" s="26">
+      <c r="M67" s="23">
         <v>0.60000002384185702</v>
       </c>
-      <c r="N67" s="24"/>
-      <c r="O67" s="24"/>
+      <c r="N67" s="21"/>
+      <c r="O67" s="21"/>
     </row>
     <row r="68" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A68" s="22" t="s">
+      <c r="A68" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="B68" s="29">
+      <c r="B68" s="26">
         <v>0.140000000596046</v>
       </c>
-      <c r="C68" s="29">
+      <c r="C68" s="26">
         <v>-0.60000002384185702</v>
       </c>
-      <c r="D68" s="30">
+      <c r="D68" s="27">
         <v>5.0000000745057997E-2</v>
       </c>
-      <c r="E68" s="29">
+      <c r="E68" s="26">
         <v>0.55000001192092896</v>
       </c>
-      <c r="F68" s="29">
+      <c r="F68" s="26">
         <v>0.60000002384185702</v>
       </c>
-      <c r="G68" s="30">
+      <c r="G68" s="27">
         <v>0.64999997615814198</v>
       </c>
-      <c r="H68" s="29">
+      <c r="H68" s="26">
         <v>-0.10000000149011599</v>
       </c>
-      <c r="I68" s="29">
+      <c r="I68" s="26">
         <v>-0.69999998807907104</v>
       </c>
-      <c r="J68" s="29">
+      <c r="J68" s="26">
         <v>-5.0000000745057997E-2</v>
       </c>
-      <c r="K68" s="31">
+      <c r="K68" s="28">
         <v>0.64999997615814198</v>
       </c>
-      <c r="L68" s="29">
+      <c r="L68" s="26">
         <v>0.69999998807907104</v>
       </c>
-      <c r="M68" s="29">
+      <c r="M68" s="26">
         <v>0.75</v>
       </c>
-      <c r="N68" s="24"/>
-      <c r="O68" s="24"/>
+      <c r="N68" s="21"/>
+      <c r="O68" s="21"/>
     </row>
     <row r="69" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A69" s="25" t="s">
+      <c r="A69" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="B69" s="26">
+      <c r="B69" s="23">
         <v>0.140000000596046</v>
       </c>
-      <c r="C69" s="26">
+      <c r="C69" s="23">
         <v>-0.60000002384185702</v>
       </c>
-      <c r="D69" s="27">
+      <c r="D69" s="24">
         <v>5.0000000745057997E-2</v>
       </c>
-      <c r="E69" s="26">
+      <c r="E69" s="23">
         <v>0.55000001192092896</v>
       </c>
-      <c r="F69" s="26">
+      <c r="F69" s="23">
         <v>0.60000002384185702</v>
       </c>
-      <c r="G69" s="27">
+      <c r="G69" s="24">
         <v>0.64999997615814198</v>
       </c>
-      <c r="H69" s="26">
+      <c r="H69" s="23">
         <v>-0.20000000298023199</v>
       </c>
-      <c r="I69" s="26">
+      <c r="I69" s="23">
         <v>-0.69999998807907104</v>
       </c>
-      <c r="J69" s="26">
+      <c r="J69" s="23">
         <v>-0.20000000298023199</v>
       </c>
-      <c r="K69" s="28">
+      <c r="K69" s="25">
         <v>0.64999997615814198</v>
       </c>
-      <c r="L69" s="26">
+      <c r="L69" s="23">
         <v>0.69999998807907104</v>
       </c>
-      <c r="M69" s="26">
+      <c r="M69" s="23">
         <v>0.75</v>
       </c>
-      <c r="N69" s="24"/>
-      <c r="O69" s="24"/>
+      <c r="N69" s="21"/>
+      <c r="O69" s="21"/>
     </row>
     <row r="70" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A70" s="22" t="s">
+      <c r="A70" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="B70" s="29">
+      <c r="B70" s="26">
         <v>0.140000000596046</v>
       </c>
-      <c r="C70" s="29">
+      <c r="C70" s="26">
         <v>-0.60000002384185702</v>
       </c>
-      <c r="D70" s="30">
+      <c r="D70" s="27">
         <v>5.0000000745057997E-2</v>
       </c>
-      <c r="E70" s="29">
+      <c r="E70" s="26">
         <v>0.55000001192092896</v>
       </c>
-      <c r="F70" s="29">
+      <c r="F70" s="26">
         <v>0.60000002384185702</v>
       </c>
-      <c r="G70" s="30">
+      <c r="G70" s="27">
         <v>0.64999997615814198</v>
       </c>
-      <c r="H70" s="29">
+      <c r="H70" s="26">
         <v>-0.20000000298023199</v>
       </c>
-      <c r="I70" s="29">
+      <c r="I70" s="26">
         <v>-0.80000001192092896</v>
       </c>
-      <c r="J70" s="29">
+      <c r="J70" s="26">
         <v>-0.20000000298023199</v>
       </c>
-      <c r="K70" s="31">
+      <c r="K70" s="28">
         <v>0.75</v>
       </c>
-      <c r="L70" s="29">
+      <c r="L70" s="26">
         <v>0.80000001192092896</v>
       </c>
-      <c r="M70" s="29">
+      <c r="M70" s="26">
         <v>0.85000002384185702</v>
       </c>
-      <c r="N70" s="24"/>
-      <c r="O70" s="24"/>
+      <c r="N70" s="21"/>
+      <c r="O70" s="21"/>
     </row>
     <row r="71" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A71" s="25" t="s">
+      <c r="A71" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="B71" s="26"/>
-      <c r="C71" s="26"/>
-      <c r="D71" s="27"/>
-      <c r="E71" s="26"/>
-      <c r="F71" s="26"/>
-      <c r="G71" s="27"/>
-      <c r="H71" s="26"/>
-      <c r="I71" s="26"/>
-      <c r="J71" s="26"/>
-      <c r="K71" s="28"/>
-      <c r="L71" s="26"/>
-      <c r="M71" s="26"/>
-      <c r="N71" s="24"/>
-      <c r="O71" s="24"/>
+      <c r="B71" s="23"/>
+      <c r="C71" s="23"/>
+      <c r="D71" s="24"/>
+      <c r="E71" s="23"/>
+      <c r="F71" s="23"/>
+      <c r="G71" s="24"/>
+      <c r="H71" s="23"/>
+      <c r="I71" s="23"/>
+      <c r="J71" s="23"/>
+      <c r="K71" s="25"/>
+      <c r="L71" s="23"/>
+      <c r="M71" s="23"/>
+      <c r="N71" s="21"/>
+      <c r="O71" s="21"/>
     </row>
     <row r="72" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A72" s="25" t="s">
+      <c r="A72" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="B72" s="26">
+      <c r="B72" s="23">
         <v>0.140000000596046</v>
       </c>
-      <c r="C72" s="26">
+      <c r="C72" s="23">
         <v>-0.60000002384185702</v>
       </c>
-      <c r="D72" s="27">
+      <c r="D72" s="24">
         <v>5.0000000745057997E-2</v>
       </c>
-      <c r="E72" s="26">
+      <c r="E72" s="23">
         <v>0.55000001192092896</v>
       </c>
-      <c r="F72" s="26">
+      <c r="F72" s="23">
         <v>0.60000002384185702</v>
       </c>
-      <c r="G72" s="27">
+      <c r="G72" s="24">
         <v>0.64999997615814198</v>
       </c>
-      <c r="H72" s="26">
+      <c r="H72" s="23">
         <v>-0.20000000298023199</v>
       </c>
-      <c r="I72" s="26">
+      <c r="I72" s="23">
         <v>-0.80000001192092896</v>
       </c>
-      <c r="J72" s="26">
+      <c r="J72" s="23">
         <v>-0.20000000298023199</v>
       </c>
-      <c r="K72" s="28">
+      <c r="K72" s="25">
         <v>0.75</v>
       </c>
-      <c r="L72" s="26">
+      <c r="L72" s="23">
         <v>0.80000001192092896</v>
       </c>
-      <c r="M72" s="26">
+      <c r="M72" s="23">
         <v>0.85000002384185702</v>
       </c>
-      <c r="N72" s="24"/>
-      <c r="O72" s="24"/>
+      <c r="N72" s="21"/>
+      <c r="O72" s="21"/>
     </row>
     <row r="73" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A73" s="23" t="s">
+      <c r="A73" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="B73" s="31">
+      <c r="B73" s="28">
         <v>0.140000000596046</v>
       </c>
-      <c r="C73" s="29">
+      <c r="C73" s="26">
         <v>-0.60000002384185702</v>
       </c>
-      <c r="D73" s="29">
+      <c r="D73" s="26">
         <v>5.0000000745057997E-2</v>
       </c>
-      <c r="E73" s="31">
+      <c r="E73" s="28">
         <v>0.55000001192092896</v>
       </c>
-      <c r="F73" s="29">
+      <c r="F73" s="26">
         <v>0.60000002384185702</v>
       </c>
-      <c r="G73" s="29">
+      <c r="G73" s="26">
         <v>0.64999997615814198</v>
       </c>
-      <c r="H73" s="31">
+      <c r="H73" s="28">
         <v>-0.20000000298023199</v>
       </c>
-      <c r="I73" s="29">
+      <c r="I73" s="26">
         <v>-0.80000001192092896</v>
       </c>
-      <c r="J73" s="29">
+      <c r="J73" s="26">
         <v>-0.10000000149011599</v>
       </c>
-      <c r="K73" s="31">
+      <c r="K73" s="28">
         <v>0.75</v>
       </c>
-      <c r="L73" s="29">
+      <c r="L73" s="26">
         <v>0.80000001192092896</v>
       </c>
-      <c r="M73" s="29">
+      <c r="M73" s="26">
         <v>0.85000002384185702</v>
       </c>
-      <c r="N73" s="24"/>
-      <c r="O73" s="24"/>
+      <c r="N73" s="21"/>
+      <c r="O73" s="21"/>
     </row>
     <row r="74" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A74" s="24"/>
-      <c r="B74" s="24"/>
-      <c r="C74" s="24"/>
-      <c r="D74" s="24"/>
-      <c r="E74" s="24"/>
-      <c r="F74" s="24"/>
-      <c r="G74" s="24"/>
-      <c r="H74" s="24"/>
-      <c r="I74" s="24"/>
-      <c r="J74" s="24"/>
-      <c r="K74" s="24"/>
-      <c r="L74" s="24"/>
-      <c r="M74" s="24"/>
-      <c r="N74" s="24"/>
-      <c r="O74" s="24"/>
+      <c r="A74" s="21"/>
+      <c r="B74" s="21"/>
+      <c r="C74" s="21"/>
+      <c r="D74" s="21"/>
+      <c r="E74" s="21"/>
+      <c r="F74" s="21"/>
+      <c r="G74" s="21"/>
+      <c r="H74" s="21"/>
+      <c r="I74" s="21"/>
+      <c r="J74" s="21"/>
+      <c r="K74" s="21"/>
+      <c r="L74" s="21"/>
+      <c r="M74" s="21"/>
+      <c r="N74" s="21"/>
+      <c r="O74" s="21"/>
     </row>
     <row r="75" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A75" s="24"/>
-      <c r="B75" s="24"/>
-      <c r="C75" s="24"/>
-      <c r="D75" s="24"/>
-      <c r="E75" s="24"/>
-      <c r="F75" s="24"/>
-      <c r="G75" s="24"/>
-      <c r="H75" s="24"/>
-      <c r="I75" s="24"/>
-      <c r="J75" s="24"/>
-      <c r="K75" s="24"/>
-      <c r="L75" s="24"/>
-      <c r="M75" s="24"/>
-      <c r="N75" s="24"/>
-      <c r="O75" s="24" t="s">
+      <c r="A75" s="21"/>
+      <c r="B75" s="21"/>
+      <c r="C75" s="21"/>
+      <c r="D75" s="21"/>
+      <c r="E75" s="21"/>
+      <c r="F75" s="21"/>
+      <c r="G75" s="21"/>
+      <c r="H75" s="21"/>
+      <c r="I75" s="21"/>
+      <c r="J75" s="21"/>
+      <c r="K75" s="21"/>
+      <c r="L75" s="21"/>
+      <c r="M75" s="21"/>
+      <c r="N75" s="21"/>
+      <c r="O75" s="21" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="76" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A76" s="24"/>
-      <c r="B76" s="24"/>
-      <c r="C76" s="24"/>
-      <c r="D76" s="24"/>
-      <c r="E76" s="24"/>
-      <c r="F76" s="24"/>
-      <c r="G76" s="24"/>
-      <c r="H76" s="24"/>
-      <c r="I76" s="24"/>
-      <c r="J76" s="24"/>
-      <c r="K76" s="24"/>
-      <c r="L76" s="24"/>
-      <c r="M76" s="24"/>
-      <c r="N76" s="24"/>
-      <c r="O76" s="24" t="s">
+      <c r="A76" s="21"/>
+      <c r="B76" s="21"/>
+      <c r="C76" s="21"/>
+      <c r="D76" s="21"/>
+      <c r="E76" s="21"/>
+      <c r="F76" s="21"/>
+      <c r="G76" s="21"/>
+      <c r="H76" s="21"/>
+      <c r="I76" s="21"/>
+      <c r="J76" s="21"/>
+      <c r="K76" s="21"/>
+      <c r="L76" s="21"/>
+      <c r="M76" s="21"/>
+      <c r="N76" s="21"/>
+      <c r="O76" s="21" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="77" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A77" s="24"/>
-      <c r="B77" s="24"/>
-      <c r="C77" s="24"/>
-      <c r="D77" s="24"/>
-      <c r="E77" s="24"/>
-      <c r="F77" s="24"/>
-      <c r="G77" s="24"/>
-      <c r="H77" s="24"/>
-      <c r="I77" s="24"/>
-      <c r="J77" s="24"/>
-      <c r="K77" s="24"/>
-      <c r="L77" s="24"/>
-      <c r="M77" s="24"/>
-      <c r="N77" s="24"/>
-      <c r="O77" s="24" t="s">
+      <c r="A77" s="21"/>
+      <c r="B77" s="21"/>
+      <c r="C77" s="21"/>
+      <c r="D77" s="21"/>
+      <c r="E77" s="21"/>
+      <c r="F77" s="21"/>
+      <c r="G77" s="21"/>
+      <c r="H77" s="21"/>
+      <c r="I77" s="21"/>
+      <c r="J77" s="21"/>
+      <c r="K77" s="21"/>
+      <c r="L77" s="21"/>
+      <c r="M77" s="21"/>
+      <c r="N77" s="21"/>
+      <c r="O77" s="21" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="78" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A78" s="24"/>
-      <c r="B78" s="24"/>
-      <c r="C78" s="24"/>
-      <c r="D78" s="24"/>
-      <c r="E78" s="24"/>
-      <c r="F78" s="24"/>
-      <c r="G78" s="24"/>
-      <c r="H78" s="24"/>
-      <c r="I78" s="24"/>
-      <c r="J78" s="24"/>
-      <c r="K78" s="24"/>
-      <c r="L78" s="24"/>
-      <c r="M78" s="24"/>
-      <c r="N78" s="24"/>
-      <c r="O78" s="24" t="s">
+      <c r="A78" s="21"/>
+      <c r="B78" s="21"/>
+      <c r="C78" s="21"/>
+      <c r="D78" s="21"/>
+      <c r="E78" s="21"/>
+      <c r="F78" s="21"/>
+      <c r="G78" s="21"/>
+      <c r="H78" s="21"/>
+      <c r="I78" s="21"/>
+      <c r="J78" s="21"/>
+      <c r="K78" s="21"/>
+      <c r="L78" s="21"/>
+      <c r="M78" s="21"/>
+      <c r="N78" s="21"/>
+      <c r="O78" s="21" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="79" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A79" s="24"/>
-      <c r="B79" s="24"/>
-      <c r="C79" s="24"/>
-      <c r="D79" s="24"/>
-      <c r="E79" s="24"/>
-      <c r="F79" s="24"/>
-      <c r="G79" s="24"/>
-      <c r="H79" s="24"/>
-      <c r="I79" s="24"/>
-      <c r="J79" s="24"/>
-      <c r="K79" s="24"/>
-      <c r="L79" s="24"/>
-      <c r="M79" s="24"/>
-      <c r="N79" s="24"/>
-      <c r="O79" s="24" t="s">
+      <c r="A79" s="21"/>
+      <c r="B79" s="21"/>
+      <c r="C79" s="21"/>
+      <c r="D79" s="21"/>
+      <c r="E79" s="21"/>
+      <c r="F79" s="21"/>
+      <c r="G79" s="21"/>
+      <c r="H79" s="21"/>
+      <c r="I79" s="21"/>
+      <c r="J79" s="21"/>
+      <c r="K79" s="21"/>
+      <c r="L79" s="21"/>
+      <c r="M79" s="21"/>
+      <c r="N79" s="21"/>
+      <c r="O79" s="21" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="80" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A80" s="24"/>
-      <c r="B80" s="24"/>
-      <c r="C80" s="24"/>
-      <c r="D80" s="24"/>
-      <c r="E80" s="24"/>
-      <c r="F80" s="24"/>
-      <c r="G80" s="24"/>
-      <c r="H80" s="24"/>
-      <c r="I80" s="24"/>
-      <c r="J80" s="24"/>
-      <c r="K80" s="24"/>
-      <c r="L80" s="24"/>
-      <c r="M80" s="24"/>
-      <c r="N80" s="24"/>
-      <c r="O80" s="24" t="s">
+      <c r="A80" s="21"/>
+      <c r="B80" s="21"/>
+      <c r="C80" s="21"/>
+      <c r="D80" s="21"/>
+      <c r="E80" s="21"/>
+      <c r="F80" s="21"/>
+      <c r="G80" s="21"/>
+      <c r="H80" s="21"/>
+      <c r="I80" s="21"/>
+      <c r="J80" s="21"/>
+      <c r="K80" s="21"/>
+      <c r="L80" s="21"/>
+      <c r="M80" s="21"/>
+      <c r="N80" s="21"/>
+      <c r="O80" s="21" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="81" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A81" s="24"/>
-      <c r="B81" s="24"/>
-      <c r="C81" s="24"/>
-      <c r="D81" s="24"/>
-      <c r="E81" s="24"/>
-      <c r="F81" s="24"/>
-      <c r="G81" s="24"/>
-      <c r="H81" s="24"/>
-      <c r="I81" s="24"/>
-      <c r="J81" s="24"/>
-      <c r="K81" s="24"/>
-      <c r="L81" s="24"/>
-      <c r="M81" s="24"/>
-      <c r="N81" s="24"/>
-      <c r="O81" s="24" t="s">
+      <c r="A81" s="21"/>
+      <c r="B81" s="21"/>
+      <c r="C81" s="21"/>
+      <c r="D81" s="21"/>
+      <c r="E81" s="21"/>
+      <c r="F81" s="21"/>
+      <c r="G81" s="21"/>
+      <c r="H81" s="21"/>
+      <c r="I81" s="21"/>
+      <c r="J81" s="21"/>
+      <c r="K81" s="21"/>
+      <c r="L81" s="21"/>
+      <c r="M81" s="21"/>
+      <c r="N81" s="21"/>
+      <c r="O81" s="21" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="82" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A82" s="24"/>
-      <c r="B82" s="24"/>
-      <c r="C82" s="24"/>
-      <c r="D82" s="24"/>
-      <c r="E82" s="24"/>
-      <c r="F82" s="24"/>
-      <c r="G82" s="24"/>
-      <c r="H82" s="24"/>
-      <c r="I82" s="24"/>
-      <c r="J82" s="24"/>
-      <c r="K82" s="24"/>
-      <c r="L82" s="24"/>
-      <c r="M82" s="24"/>
-      <c r="N82" s="24"/>
-      <c r="O82" s="24" t="s">
+      <c r="A82" s="21"/>
+      <c r="B82" s="21"/>
+      <c r="C82" s="21"/>
+      <c r="D82" s="21"/>
+      <c r="E82" s="21"/>
+      <c r="F82" s="21"/>
+      <c r="G82" s="21"/>
+      <c r="H82" s="21"/>
+      <c r="I82" s="21"/>
+      <c r="J82" s="21"/>
+      <c r="K82" s="21"/>
+      <c r="L82" s="21"/>
+      <c r="M82" s="21"/>
+      <c r="N82" s="21"/>
+      <c r="O82" s="21" t="s">
         <v>38</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="E2:G2"/>
+    <mergeCell ref="H2:J2"/>
+    <mergeCell ref="K2:M2"/>
+    <mergeCell ref="B23:D23"/>
+    <mergeCell ref="E23:G23"/>
+    <mergeCell ref="H23:J23"/>
+    <mergeCell ref="K23:M23"/>
     <mergeCell ref="B44:D44"/>
     <mergeCell ref="E44:G44"/>
     <mergeCell ref="H44:J44"/>
@@ -8523,14 +9044,6 @@
     <mergeCell ref="E65:G65"/>
     <mergeCell ref="H65:J65"/>
     <mergeCell ref="K65:M65"/>
-    <mergeCell ref="B2:D2"/>
-    <mergeCell ref="E2:G2"/>
-    <mergeCell ref="H2:J2"/>
-    <mergeCell ref="K2:M2"/>
-    <mergeCell ref="B23:D23"/>
-    <mergeCell ref="E23:G23"/>
-    <mergeCell ref="H23:J23"/>
-    <mergeCell ref="K23:M23"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>

<commit_message>
multiple safety conditions results all models plus pnp results
</commit_message>
<xml_diff>
--- a/results/compiled results.xlsx
+++ b/results/compiled results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\elish\Desktop\Aims Project\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C95190C6-65E3-4C35-BB00-80E40F8F7AFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F74E363-4632-4736-8BF7-AA89281F44D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{DA4D96B0-492C-4945-A9C4-EFCA6D6BC722}"/>
   </bookViews>
@@ -4272,43 +4272,313 @@
       <c r="O15" t="s">
         <v>51</v>
       </c>
+      <c r="P15" s="3">
+        <v>0.205705302011014</v>
+      </c>
+      <c r="Q15" s="3">
+        <v>0.10480522342236601</v>
+      </c>
+      <c r="R15" s="3">
+        <v>0.20691336023293999</v>
+      </c>
+      <c r="S15" s="3">
+        <v>0.10594480432336199</v>
+      </c>
+      <c r="T15" s="2">
+        <v>0</v>
+      </c>
+      <c r="U15" s="2">
+        <v>4.7640653619619E-2</v>
+      </c>
+      <c r="V15" s="3">
+        <v>4.7640653619619E-2</v>
+      </c>
+      <c r="W15" s="2">
+        <v>0</v>
+      </c>
+      <c r="X15" s="3">
+        <v>5.6548667764616201E-2</v>
+      </c>
+      <c r="Y15" s="3">
+        <v>5.6548667764616201E-2</v>
+      </c>
+      <c r="Z15" s="3">
+        <v>6.3199999999999895E-2</v>
+      </c>
+      <c r="AA15" s="3">
+        <v>3.81633599999999</v>
+      </c>
+      <c r="AB15" s="2">
+        <v>93.6</v>
+      </c>
+      <c r="AC15" s="3">
+        <v>10.295999999999999</v>
+      </c>
+      <c r="AD15" s="2">
+        <v>8331.0174627980305</v>
+      </c>
     </row>
     <row r="16" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O16" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P16" s="3">
+        <v>0.20094616602850901</v>
+      </c>
+      <c r="Q16" s="3">
+        <v>0.107460022996064</v>
+      </c>
+      <c r="R16" s="3">
+        <v>0.20170607435510901</v>
+      </c>
+      <c r="S16" s="3">
+        <v>0.108864617481995</v>
+      </c>
+      <c r="T16" s="2">
+        <v>0</v>
+      </c>
+      <c r="U16" s="2">
+        <v>4.7640653619619E-2</v>
+      </c>
+      <c r="V16" s="3">
+        <v>4.7640653619619E-2</v>
+      </c>
+      <c r="W16" s="2">
+        <v>0</v>
+      </c>
+      <c r="X16" s="3">
+        <v>5.6548667764616201E-2</v>
+      </c>
+      <c r="Y16" s="3">
+        <v>5.6548667764616201E-2</v>
+      </c>
+      <c r="Z16" s="3">
+        <v>2.3199999999999901E-2</v>
+      </c>
+      <c r="AA16" s="3">
+        <v>2.619904</v>
+      </c>
+      <c r="AB16" s="2">
+        <v>98.918181818181793</v>
+      </c>
+      <c r="AC16" s="3">
+        <v>10.881</v>
+      </c>
+      <c r="AD16" s="2">
+        <v>7108.14468373205</v>
+      </c>
+    </row>
+    <row r="17" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O17" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P17" s="3">
+        <v>0.36366496008710802</v>
+      </c>
+      <c r="Q17" s="3">
+        <v>8.5103341494056503E-2</v>
+      </c>
+      <c r="R17" s="3">
+        <v>0.36356107891046802</v>
+      </c>
+      <c r="S17" s="3">
+        <v>8.5107195582413003E-2</v>
+      </c>
+      <c r="T17" s="2">
+        <v>0</v>
+      </c>
+      <c r="U17" s="2">
+        <v>5.6548667764616201E-2</v>
+      </c>
+      <c r="V17" s="3">
+        <v>5.6548667764616201E-2</v>
+      </c>
+      <c r="W17" s="2">
+        <v>87.1</v>
+      </c>
+      <c r="X17" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y17" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z17" s="3">
+        <v>0.156799999999999</v>
+      </c>
+      <c r="AA17" s="3">
+        <v>0.37631999999999999</v>
+      </c>
+      <c r="AB17" s="2">
+        <v>100</v>
+      </c>
+      <c r="AC17" s="3">
+        <v>11</v>
+      </c>
+      <c r="AD17" s="2">
+        <v>4079.1357275988898</v>
+      </c>
+    </row>
+    <row r="18" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O18" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P18" s="3">
+        <v>0.261901664151098</v>
+      </c>
+      <c r="Q18" s="3">
+        <v>0.124405443576612</v>
+      </c>
+      <c r="R18" s="3">
+        <v>0.261743363290594</v>
+      </c>
+      <c r="S18" s="3">
+        <v>0.124877538651196</v>
+      </c>
+      <c r="T18" s="2">
+        <v>0</v>
+      </c>
+      <c r="U18" s="2">
+        <v>5.6548667764616201E-2</v>
+      </c>
+      <c r="V18" s="3">
+        <v>5.6548667764616201E-2</v>
+      </c>
+      <c r="W18" s="2">
+        <v>100</v>
+      </c>
+      <c r="X18" s="3">
+        <v>5.6548667764616201E-2</v>
+      </c>
+      <c r="Y18" s="3">
+        <v>5.6548667764616201E-2</v>
+      </c>
+      <c r="Z18" s="3">
+        <v>0.13119999999999901</v>
+      </c>
+      <c r="AA18" s="3">
+        <v>0.38370899999999902</v>
+      </c>
+      <c r="AB18" s="2">
+        <v>100</v>
+      </c>
+      <c r="AC18" s="3">
+        <v>11</v>
+      </c>
+      <c r="AD18" s="2">
+        <v>9698.3661137017607</v>
+      </c>
+    </row>
+    <row r="19" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O19" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P19" s="3">
+        <v>0.33054050800014101</v>
+      </c>
+      <c r="Q19" s="3">
+        <v>0.116855717031366</v>
+      </c>
+      <c r="R19" s="3">
+        <v>0.33034728905099198</v>
+      </c>
+      <c r="S19" s="3">
+        <v>0.117266130962788</v>
+      </c>
+      <c r="T19" s="2">
+        <v>0</v>
+      </c>
+      <c r="U19" s="2">
+        <v>5.6548667764616201E-2</v>
+      </c>
+      <c r="V19" s="3">
+        <v>5.6548667764616201E-2</v>
+      </c>
+      <c r="W19" s="2">
+        <v>100</v>
+      </c>
+      <c r="X19" s="3">
+        <v>5.6548667764616201E-2</v>
+      </c>
+      <c r="Y19" s="3">
+        <v>5.6548667764616201E-2</v>
+      </c>
+      <c r="Z19" s="3">
+        <v>0.156799999999999</v>
+      </c>
+      <c r="AA19" s="3">
+        <v>0.37440000000000001</v>
+      </c>
+      <c r="AB19" s="2">
+        <v>100</v>
+      </c>
+      <c r="AC19" s="3">
+        <v>11</v>
+      </c>
+      <c r="AD19" s="2">
+        <v>13665.8515410358</v>
+      </c>
+    </row>
+    <row r="20" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O20" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P20" s="3">
+        <v>0.33834814301107202</v>
+      </c>
+      <c r="Q20" s="3">
+        <v>0.11752130295997699</v>
+      </c>
+      <c r="R20" s="3">
+        <v>0.33837069477188497</v>
+      </c>
+      <c r="S20" s="3">
+        <v>0.117818134227457</v>
+      </c>
+      <c r="T20" s="2">
+        <v>0</v>
+      </c>
+      <c r="U20" s="2">
+        <v>5.6548667764616201E-2</v>
+      </c>
+      <c r="V20" s="3">
+        <v>5.6548667764616201E-2</v>
+      </c>
+      <c r="W20" s="2">
+        <v>100</v>
+      </c>
+      <c r="X20" s="3">
+        <v>5.6548667764616201E-2</v>
+      </c>
+      <c r="Y20" s="3">
+        <v>5.6548667764616201E-2</v>
+      </c>
+      <c r="Z20" s="3">
+        <v>0.156799999999999</v>
+      </c>
+      <c r="AA20" s="3">
+        <v>0.33629999999999899</v>
+      </c>
+      <c r="AB20" s="2">
+        <v>100</v>
+      </c>
+      <c r="AC20" s="3">
+        <v>11</v>
+      </c>
+      <c r="AD20" s="2">
+        <v>13585.1360406514</v>
+      </c>
+    </row>
+    <row r="21" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O21" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A24" s="5" t="s">
         <v>0</v>
       </c>
@@ -4333,7 +4603,7 @@
       <c r="L24" s="32"/>
       <c r="M24" s="32"/>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A25" s="14" t="s">
         <v>1</v>
       </c>
@@ -4374,7 +4644,7 @@
         <v>0.64999997615814198</v>
       </c>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A26" s="12" t="s">
         <v>2</v>
       </c>
@@ -4415,7 +4685,7 @@
         <v>0.224999994039535</v>
       </c>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A27" s="5" t="s">
         <v>3</v>
       </c>
@@ -4456,7 +4726,7 @@
         <v>0.72399997711181596</v>
       </c>
     </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A28" s="14" t="s">
         <v>4</v>
       </c>
@@ -4497,7 +4767,7 @@
         <v>0.59500002861022905</v>
       </c>
     </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A29" s="5" t="s">
         <v>7</v>
       </c>
@@ -4538,7 +4808,7 @@
         <v>0.63999998569488503</v>
       </c>
     </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A30" s="12" t="s">
         <v>5</v>
       </c>
@@ -4579,7 +4849,7 @@
         <v>0.63999998569488503</v>
       </c>
     </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A31" s="12" t="s">
         <v>17</v>
       </c>
@@ -4620,7 +4890,7 @@
         <v>0.63999998569488503</v>
       </c>
     </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A32" s="13" t="s">
         <v>6</v>
       </c>
@@ -4720,35 +4990,350 @@
       <c r="O36" t="s">
         <v>51</v>
       </c>
+      <c r="P36" s="3">
+        <v>0.20570530200000001</v>
+      </c>
+      <c r="Q36" s="3">
+        <v>0.104805223</v>
+      </c>
+      <c r="R36" s="3">
+        <v>0.20691335999999999</v>
+      </c>
+      <c r="S36" s="3">
+        <v>0.105944804</v>
+      </c>
+      <c r="T36" s="2">
+        <v>0</v>
+      </c>
+      <c r="U36" s="2">
+        <v>4.7640653999999998E-2</v>
+      </c>
+      <c r="V36" s="3">
+        <v>4.7640653999999998E-2</v>
+      </c>
+      <c r="W36" s="2">
+        <v>0</v>
+      </c>
+      <c r="X36" s="3">
+        <v>5.6548668000000003E-2</v>
+      </c>
+      <c r="Y36" s="3">
+        <v>5.6548668000000003E-2</v>
+      </c>
+      <c r="Z36" s="3">
+        <v>6.3200000000000006E-2</v>
+      </c>
+      <c r="AA36" s="3">
+        <v>3.8163360000000002</v>
+      </c>
+      <c r="AB36" s="2">
+        <v>93.6</v>
+      </c>
+      <c r="AC36" s="3">
+        <v>10.295999999999999</v>
+      </c>
+      <c r="AD36" s="2">
+        <v>8331.0174630000001</v>
+      </c>
     </row>
     <row r="37" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O37" t="s">
         <v>33</v>
       </c>
+      <c r="P37" s="3">
+        <v>0.39636884812880002</v>
+      </c>
+      <c r="Q37" s="3">
+        <v>7.6429860888034801E-2</v>
+      </c>
+      <c r="R37" s="3">
+        <v>0.39609779115274402</v>
+      </c>
+      <c r="S37" s="3">
+        <v>7.6770326473487097E-2</v>
+      </c>
+      <c r="T37" s="2">
+        <v>25.363636363636299</v>
+      </c>
+      <c r="U37" s="2">
+        <v>1.6374037031865098E-2</v>
+      </c>
+      <c r="V37" s="3">
+        <v>1.6374037031865098E-2</v>
+      </c>
+      <c r="W37" s="2">
+        <v>100</v>
+      </c>
+      <c r="X37" s="3">
+        <v>1.5038879272304601E-2</v>
+      </c>
+      <c r="Y37" s="3">
+        <v>1.5038879272304601E-2</v>
+      </c>
+      <c r="Z37" s="3">
+        <v>3.8114000000000002E-2</v>
+      </c>
+      <c r="AA37" s="3">
+        <v>8.7437999999999905E-2</v>
+      </c>
+      <c r="AB37" s="2">
+        <v>100</v>
+      </c>
+      <c r="AC37" s="3">
+        <v>11</v>
+      </c>
+      <c r="AD37" s="2">
+        <v>9736.55635166092</v>
+      </c>
     </row>
     <row r="38" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O38" t="s">
         <v>32</v>
       </c>
+      <c r="P38" s="3">
+        <v>0.45759959561025798</v>
+      </c>
+      <c r="Q38" s="3">
+        <v>3.3647610214357297E-2</v>
+      </c>
+      <c r="R38" s="3">
+        <v>0.45767954838810199</v>
+      </c>
+      <c r="S38" s="3">
+        <v>3.3615140563021402E-2</v>
+      </c>
+      <c r="T38" s="2">
+        <v>100</v>
+      </c>
+      <c r="U38" s="2">
+        <v>0</v>
+      </c>
+      <c r="V38" s="3">
+        <v>0</v>
+      </c>
+      <c r="W38" s="2">
+        <v>54.754545454545401</v>
+      </c>
+      <c r="X38" s="3">
+        <v>2.9574444486077399E-2</v>
+      </c>
+      <c r="Y38" s="3">
+        <v>2.9574444486077399E-2</v>
+      </c>
+      <c r="Z38" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA38" s="3">
+        <v>0.88751999999999898</v>
+      </c>
+      <c r="AB38" s="2">
+        <v>100</v>
+      </c>
+      <c r="AC38" s="3">
+        <v>11</v>
+      </c>
+      <c r="AD38" s="2">
+        <v>5202.9112099563299</v>
+      </c>
     </row>
     <row r="39" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O39" t="s">
         <v>35</v>
       </c>
+      <c r="P39" s="3">
+        <v>0.40507656031128503</v>
+      </c>
+      <c r="Q39" s="3">
+        <v>0.14868149934542199</v>
+      </c>
+      <c r="R39" s="3">
+        <v>0.40439103966173201</v>
+      </c>
+      <c r="S39" s="3">
+        <v>0.14916030078762699</v>
+      </c>
+      <c r="T39" s="2">
+        <v>0</v>
+      </c>
+      <c r="U39" s="2">
+        <v>1.6374037031865098E-2</v>
+      </c>
+      <c r="V39" s="3">
+        <v>1.6374037031865098E-2</v>
+      </c>
+      <c r="W39" s="2">
+        <v>100</v>
+      </c>
+      <c r="X39" s="3">
+        <v>1.9369750605491599E-2</v>
+      </c>
+      <c r="Y39" s="3">
+        <v>1.9369750605491599E-2</v>
+      </c>
+      <c r="Z39" s="3">
+        <v>3.9780000000000003E-2</v>
+      </c>
+      <c r="AA39" s="3">
+        <v>0.11193</v>
+      </c>
+      <c r="AB39" s="2">
+        <v>100</v>
+      </c>
+      <c r="AC39" s="3">
+        <v>11</v>
+      </c>
+      <c r="AD39" s="2">
+        <v>9052.5473879033907</v>
+      </c>
     </row>
     <row r="40" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O40" t="s">
         <v>36</v>
       </c>
+      <c r="P40" s="3">
+        <v>0.527889263524429</v>
+      </c>
+      <c r="Q40" s="3">
+        <v>0.116368844458883</v>
+      </c>
+      <c r="R40" s="3">
+        <v>0.532471639682636</v>
+      </c>
+      <c r="S40" s="3">
+        <v>0.11462148137252599</v>
+      </c>
+      <c r="T40" s="2">
+        <v>0</v>
+      </c>
+      <c r="U40" s="2">
+        <v>1.6374037031865098E-2</v>
+      </c>
+      <c r="V40" s="3">
+        <v>1.6374037031865098E-2</v>
+      </c>
+      <c r="W40" s="2">
+        <v>100</v>
+      </c>
+      <c r="X40" s="3">
+        <v>1.9369750605491599E-2</v>
+      </c>
+      <c r="Y40" s="3">
+        <v>1.9369750605491599E-2</v>
+      </c>
+      <c r="Z40" s="3">
+        <v>3.9780000000000003E-2</v>
+      </c>
+      <c r="AA40" s="3">
+        <v>0.107584</v>
+      </c>
+      <c r="AB40" s="2">
+        <v>100</v>
+      </c>
+      <c r="AC40" s="3">
+        <v>11</v>
+      </c>
+      <c r="AD40" s="2">
+        <v>9105.1182521936098</v>
+      </c>
     </row>
     <row r="41" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O41" t="s">
         <v>37</v>
       </c>
+      <c r="P41" s="3">
+        <v>0.52887767906368</v>
+      </c>
+      <c r="Q41" s="3">
+        <v>0.116791657860364</v>
+      </c>
+      <c r="R41" s="3">
+        <v>0.53410663516087997</v>
+      </c>
+      <c r="S41" s="3">
+        <v>0.114291997076247</v>
+      </c>
+      <c r="T41" s="2">
+        <v>0</v>
+      </c>
+      <c r="U41" s="2">
+        <v>1.6374037031865098E-2</v>
+      </c>
+      <c r="V41" s="3">
+        <v>1.6374037031865098E-2</v>
+      </c>
+      <c r="W41" s="2">
+        <v>100</v>
+      </c>
+      <c r="X41" s="3">
+        <v>1.7956312720886099E-2</v>
+      </c>
+      <c r="Y41" s="3">
+        <v>1.7956312720886099E-2</v>
+      </c>
+      <c r="Z41" s="3">
+        <v>3.9780000000000003E-2</v>
+      </c>
+      <c r="AA41" s="3">
+        <v>0.10496</v>
+      </c>
+      <c r="AB41" s="2">
+        <v>100</v>
+      </c>
+      <c r="AC41" s="3">
+        <v>11</v>
+      </c>
+      <c r="AD41" s="2">
+        <v>8998.4913450118693</v>
+      </c>
     </row>
     <row r="42" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O42" t="s">
         <v>38</v>
+      </c>
+      <c r="P42" s="3">
+        <v>0.52881868088098205</v>
+      </c>
+      <c r="Q42" s="3">
+        <v>0.116735197855005</v>
+      </c>
+      <c r="R42" s="3">
+        <v>0.53410105514998096</v>
+      </c>
+      <c r="S42" s="3">
+        <v>0.11429433206974</v>
+      </c>
+      <c r="T42" s="2">
+        <v>0</v>
+      </c>
+      <c r="U42" s="2">
+        <v>1.6374037031865098E-2</v>
+      </c>
+      <c r="V42" s="3">
+        <v>1.6374037031865098E-2</v>
+      </c>
+      <c r="W42" s="2">
+        <v>100</v>
+      </c>
+      <c r="X42" s="3">
+        <v>1.7956312720886099E-2</v>
+      </c>
+      <c r="Y42" s="3">
+        <v>1.7956312720886099E-2</v>
+      </c>
+      <c r="Z42" s="3">
+        <v>3.9780000000000003E-2</v>
+      </c>
+      <c r="AA42" s="3">
+        <v>0.10332</v>
+      </c>
+      <c r="AB42" s="2">
+        <v>100</v>
+      </c>
+      <c r="AC42" s="3">
+        <v>11</v>
+      </c>
+      <c r="AD42" s="2">
+        <v>8998.2516377375905</v>
       </c>
     </row>
     <row r="43" spans="1:30" x14ac:dyDescent="0.3">
@@ -4945,7 +5530,7 @@
         <v>0.55000001192092896</v>
       </c>
     </row>
-    <row r="49" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A49" s="5" t="s">
         <v>7</v>
       </c>
@@ -4986,7 +5571,7 @@
         <v>0.64999997615814198</v>
       </c>
     </row>
-    <row r="50" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A50" s="12" t="s">
         <v>5</v>
       </c>
@@ -5027,7 +5612,7 @@
         <v>1.2350000143051101</v>
       </c>
     </row>
-    <row r="51" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A51" s="12" t="s">
         <v>17</v>
       </c>
@@ -5068,7 +5653,7 @@
         <v>1.1900000572204501</v>
       </c>
     </row>
-    <row r="52" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A52" s="13" t="s">
         <v>6</v>
       </c>
@@ -5109,57 +5694,417 @@
         <v>1.1900000572204501</v>
       </c>
     </row>
-    <row r="54" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O54" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="55" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O55" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="56" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P55" s="3">
+        <v>0.24152868270713199</v>
+      </c>
+      <c r="Q55" s="3">
+        <v>5.6402546228257702E-2</v>
+      </c>
+      <c r="R55" s="3">
+        <v>0.24067999376510699</v>
+      </c>
+      <c r="S55" s="3">
+        <v>5.6033894231103998E-2</v>
+      </c>
+      <c r="T55" s="2">
+        <v>89.745454545454507</v>
+      </c>
+      <c r="U55" s="2">
+        <v>1.4495889241012999E-2</v>
+      </c>
+      <c r="V55" s="3">
+        <v>1.4495889241012999E-2</v>
+      </c>
+      <c r="W55" s="2">
+        <v>0</v>
+      </c>
+      <c r="X55" s="3">
+        <v>5.3722281573936603E-2</v>
+      </c>
+      <c r="Y55" s="3">
+        <v>5.3722281573936603E-2</v>
+      </c>
+      <c r="Z55" s="3">
+        <v>6.1559999999999896E-3</v>
+      </c>
+      <c r="AA55" s="3">
+        <v>1</v>
+      </c>
+      <c r="AB55" s="2">
+        <v>100</v>
+      </c>
+      <c r="AC55" s="3">
+        <v>11</v>
+      </c>
+      <c r="AD55" s="2">
+        <v>4988.0428367251698</v>
+      </c>
+    </row>
+    <row r="56" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O56" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="57" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P56" s="3">
+        <v>0.24153136628727301</v>
+      </c>
+      <c r="Q56" s="3">
+        <v>5.6402456665812797E-2</v>
+      </c>
+      <c r="R56" s="3">
+        <v>0.24068003797366799</v>
+      </c>
+      <c r="S56" s="3">
+        <v>5.6033890013490198E-2</v>
+      </c>
+      <c r="T56" s="2">
+        <v>89.745454545454507</v>
+      </c>
+      <c r="U56" s="2">
+        <v>1.4495889241012999E-2</v>
+      </c>
+      <c r="V56" s="3">
+        <v>1.4495889241012999E-2</v>
+      </c>
+      <c r="W56" s="2">
+        <v>0</v>
+      </c>
+      <c r="X56" s="3">
+        <v>5.6548667764616201E-2</v>
+      </c>
+      <c r="Y56" s="3">
+        <v>5.6548667764616201E-2</v>
+      </c>
+      <c r="Z56" s="3">
+        <v>6.1559999999999896E-3</v>
+      </c>
+      <c r="AA56" s="3">
+        <v>2.52</v>
+      </c>
+      <c r="AB56" s="2">
+        <v>100</v>
+      </c>
+      <c r="AC56" s="3">
+        <v>11</v>
+      </c>
+      <c r="AD56" s="2">
+        <v>4988.5894963933697</v>
+      </c>
+    </row>
+    <row r="57" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O57" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="58" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P57" s="3">
+        <v>0.49126895243375501</v>
+      </c>
+      <c r="Q57" s="3">
+        <v>4.1231954899859001E-2</v>
+      </c>
+      <c r="R57" s="3">
+        <v>0.491560159835985</v>
+      </c>
+      <c r="S57" s="3">
+        <v>4.0996484534822603E-2</v>
+      </c>
+      <c r="T57" s="2">
+        <v>100</v>
+      </c>
+      <c r="U57" s="2">
+        <v>2.72150547943637E-4</v>
+      </c>
+      <c r="V57" s="3">
+        <v>2.72150547943637E-4</v>
+      </c>
+      <c r="W57" s="2">
+        <v>100</v>
+      </c>
+      <c r="X57" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y57" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z57" s="3">
+        <v>1.1904E-2</v>
+      </c>
+      <c r="AA57" s="3">
+        <v>0.115374</v>
+      </c>
+      <c r="AB57" s="2">
+        <v>100</v>
+      </c>
+      <c r="AC57" s="3">
+        <v>11</v>
+      </c>
+      <c r="AD57" s="2">
+        <v>4547.7666107106497</v>
+      </c>
+    </row>
+    <row r="58" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O58" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="59" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P58" s="3">
+        <v>0.36203522476231298</v>
+      </c>
+      <c r="Q58" s="3">
+        <v>5.3083689656963098E-2</v>
+      </c>
+      <c r="R58" s="3">
+        <v>0.361717770882652</v>
+      </c>
+      <c r="S58" s="3">
+        <v>5.3024782722781001E-2</v>
+      </c>
+      <c r="T58" s="2">
+        <v>77.609090909090895</v>
+      </c>
+      <c r="U58" s="2">
+        <v>1.8172761741243E-2</v>
+      </c>
+      <c r="V58" s="3">
+        <v>1.8172761741243E-2</v>
+      </c>
+      <c r="W58" s="2">
+        <v>100</v>
+      </c>
+      <c r="X58" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y58" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z58" s="3">
+        <v>2.1839999999999998E-2</v>
+      </c>
+      <c r="AA58" s="3">
+        <v>0.12676399999999999</v>
+      </c>
+      <c r="AB58" s="2">
+        <v>100</v>
+      </c>
+      <c r="AC58" s="3">
+        <v>11</v>
+      </c>
+      <c r="AD58" s="2">
+        <v>7096.2458818271198</v>
+      </c>
+    </row>
+    <row r="59" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O59" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="60" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P59" s="3">
+        <v>0.39959914338580699</v>
+      </c>
+      <c r="Q59" s="3">
+        <v>0.171224398304928</v>
+      </c>
+      <c r="R59" s="3">
+        <v>0.39956351079470498</v>
+      </c>
+      <c r="S59" s="3">
+        <v>0.17206327397843399</v>
+      </c>
+      <c r="T59" s="2">
+        <v>0</v>
+      </c>
+      <c r="U59" s="2">
+        <v>1.6374037031865098E-2</v>
+      </c>
+      <c r="V59" s="3">
+        <v>1.6374037031865098E-2</v>
+      </c>
+      <c r="W59" s="2">
+        <v>100</v>
+      </c>
+      <c r="X59" s="3">
+        <v>2.25392034638357E-2</v>
+      </c>
+      <c r="Y59" s="3">
+        <v>2.25392034638357E-2</v>
+      </c>
+      <c r="Z59" s="3">
+        <v>4.2431999999999997E-2</v>
+      </c>
+      <c r="AA59" s="3">
+        <v>0.1386</v>
+      </c>
+      <c r="AB59" s="2">
+        <v>100</v>
+      </c>
+      <c r="AC59" s="3">
+        <v>11</v>
+      </c>
+      <c r="AD59" s="2">
+        <v>10455.3265531918</v>
+      </c>
+    </row>
+    <row r="60" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O60" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="61" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P60" s="3">
+        <v>0.64763181116499502</v>
+      </c>
+      <c r="Q60" s="3">
+        <v>0.10714481663194</v>
+      </c>
+      <c r="R60" s="3">
+        <v>0.64971300819234501</v>
+      </c>
+      <c r="S60" s="3">
+        <v>0.106991123965878</v>
+      </c>
+      <c r="T60" s="2">
+        <v>100</v>
+      </c>
+      <c r="U60" s="2">
+        <v>0</v>
+      </c>
+      <c r="V60" s="3">
+        <v>0</v>
+      </c>
+      <c r="W60" s="2">
+        <v>0</v>
+      </c>
+      <c r="X60" s="3">
+        <v>5.6548667764616201E-2</v>
+      </c>
+      <c r="Y60" s="3">
+        <v>5.6548667764616201E-2</v>
+      </c>
+      <c r="Z60" s="3">
+        <v>7.9999999999999996E-6</v>
+      </c>
+      <c r="AA60" s="3">
+        <v>3.81633599999999</v>
+      </c>
+      <c r="AB60" s="2">
+        <v>100</v>
+      </c>
+      <c r="AC60" s="3">
+        <v>11</v>
+      </c>
+      <c r="AD60" s="2">
+        <v>2868.1308666606101</v>
+      </c>
+    </row>
+    <row r="61" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O61" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="62" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P61" s="3">
+        <v>0.32782759329432998</v>
+      </c>
+      <c r="Q61" s="3">
+        <v>0.185228338581368</v>
+      </c>
+      <c r="R61" s="3">
+        <v>0.325449546302851</v>
+      </c>
+      <c r="S61" s="3">
+        <v>0.18633972352994799</v>
+      </c>
+      <c r="T61" s="2">
+        <v>0</v>
+      </c>
+      <c r="U61" s="2">
+        <v>1.6374037031865098E-2</v>
+      </c>
+      <c r="V61" s="3">
+        <v>1.6374037031865098E-2</v>
+      </c>
+      <c r="W61" s="2">
+        <v>100</v>
+      </c>
+      <c r="X61" s="3">
+        <v>2.25392034638357E-2</v>
+      </c>
+      <c r="Y61" s="3">
+        <v>2.25392034638357E-2</v>
+      </c>
+      <c r="Z61" s="3">
+        <v>3.9780000000000003E-2</v>
+      </c>
+      <c r="AA61" s="3">
+        <v>0.12676399999999999</v>
+      </c>
+      <c r="AB61" s="2">
+        <v>100</v>
+      </c>
+      <c r="AC61" s="3">
+        <v>11</v>
+      </c>
+      <c r="AD61" s="2">
+        <v>9726.6027333685197</v>
+      </c>
+    </row>
+    <row r="62" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O62" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="64" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P62" s="3">
+        <v>0.54419239100000005</v>
+      </c>
+      <c r="Q62" s="3">
+        <v>0.1364098</v>
+      </c>
+      <c r="R62" s="3">
+        <v>0.54768143000000002</v>
+      </c>
+      <c r="S62" s="3">
+        <v>0.137002452</v>
+      </c>
+      <c r="T62" s="2">
+        <v>100</v>
+      </c>
+      <c r="U62" s="2">
+        <v>0</v>
+      </c>
+      <c r="V62" s="3">
+        <v>0</v>
+      </c>
+      <c r="W62" s="2">
+        <v>100</v>
+      </c>
+      <c r="X62" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y62" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z62" s="3">
+        <v>2.7999999999999998E-4</v>
+      </c>
+      <c r="AA62" s="3">
+        <v>1.584E-2</v>
+      </c>
+      <c r="AB62" s="2">
+        <v>100</v>
+      </c>
+      <c r="AC62" s="3">
+        <v>11</v>
+      </c>
+      <c r="AD62" s="2">
+        <v>10448.12103</v>
+      </c>
+    </row>
+    <row r="64" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="65" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A65" s="19" t="s">
         <v>0</v>
       </c>
@@ -5186,7 +6131,7 @@
       <c r="N65" s="21"/>
       <c r="O65" s="21"/>
     </row>
-    <row r="66" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A66" s="22" t="s">
         <v>1</v>
       </c>
@@ -5229,7 +6174,7 @@
       <c r="N66" s="21"/>
       <c r="O66" s="21"/>
     </row>
-    <row r="67" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A67" s="22" t="s">
         <v>2</v>
       </c>
@@ -5272,7 +6217,7 @@
       <c r="N67" s="21"/>
       <c r="O67" s="21"/>
     </row>
-    <row r="68" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A68" s="19" t="s">
         <v>3</v>
       </c>
@@ -5315,7 +6260,7 @@
       <c r="N68" s="21"/>
       <c r="O68" s="21"/>
     </row>
-    <row r="69" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A69" s="22" t="s">
         <v>4</v>
       </c>
@@ -5358,7 +6303,7 @@
       <c r="N69" s="21"/>
       <c r="O69" s="21"/>
     </row>
-    <row r="70" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A70" s="19" t="s">
         <v>7</v>
       </c>
@@ -5401,7 +6346,7 @@
       <c r="N70" s="21"/>
       <c r="O70" s="21"/>
     </row>
-    <row r="71" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A71" s="22" t="s">
         <v>5</v>
       </c>
@@ -5420,7 +6365,7 @@
       <c r="N71" s="21"/>
       <c r="O71" s="21"/>
     </row>
-    <row r="72" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A72" s="22" t="s">
         <v>17</v>
       </c>
@@ -5463,7 +6408,7 @@
       <c r="N72" s="21"/>
       <c r="O72" s="21"/>
     </row>
-    <row r="73" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A73" s="20" t="s">
         <v>6</v>
       </c>
@@ -5506,7 +6451,7 @@
       <c r="N73" s="21"/>
       <c r="O73" s="21"/>
     </row>
-    <row r="74" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A74" s="21"/>
       <c r="B74" s="21"/>
       <c r="C74" s="21"/>
@@ -5523,7 +6468,7 @@
       <c r="N74" s="21"/>
       <c r="O74" s="21"/>
     </row>
-    <row r="75" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A75" s="21"/>
       <c r="B75" s="21"/>
       <c r="C75" s="21"/>
@@ -5542,7 +6487,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="76" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A76" s="21"/>
       <c r="B76" s="21"/>
       <c r="C76" s="21"/>
@@ -5560,8 +6505,53 @@
       <c r="O76" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="77" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P76" s="3">
+        <v>0.70879072300000001</v>
+      </c>
+      <c r="Q76" s="3">
+        <v>0.12970775700000001</v>
+      </c>
+      <c r="R76" s="3">
+        <v>0.74383465000000004</v>
+      </c>
+      <c r="S76" s="3">
+        <v>6.9465451999999997E-2</v>
+      </c>
+      <c r="T76" s="2">
+        <v>0</v>
+      </c>
+      <c r="U76" s="2">
+        <v>5.6548668000000003E-2</v>
+      </c>
+      <c r="V76" s="3">
+        <v>5.6548668000000003E-2</v>
+      </c>
+      <c r="W76" s="2">
+        <v>99.754545449999995</v>
+      </c>
+      <c r="X76" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y76" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z76" s="3">
+        <v>0.3024</v>
+      </c>
+      <c r="AA76" s="3">
+        <v>1.0160640000000001</v>
+      </c>
+      <c r="AB76" s="2">
+        <v>100</v>
+      </c>
+      <c r="AC76" s="3">
+        <v>11</v>
+      </c>
+      <c r="AD76" s="2">
+        <v>1510.5934870000001</v>
+      </c>
+    </row>
+    <row r="77" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A77" s="21"/>
       <c r="B77" s="21"/>
       <c r="C77" s="21"/>
@@ -5579,8 +6569,53 @@
       <c r="O77" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="78" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P77" s="3">
+        <v>0.70879071959919404</v>
+      </c>
+      <c r="Q77" s="3">
+        <v>0.12970776262285599</v>
+      </c>
+      <c r="R77" s="3">
+        <v>0.74383464783216802</v>
+      </c>
+      <c r="S77" s="3">
+        <v>6.9465459047769698E-2</v>
+      </c>
+      <c r="T77" s="2">
+        <v>0</v>
+      </c>
+      <c r="U77" s="2">
+        <v>5.6548667764616201E-2</v>
+      </c>
+      <c r="V77" s="3">
+        <v>5.6548667764616201E-2</v>
+      </c>
+      <c r="W77" s="2">
+        <v>99.754545454545394</v>
+      </c>
+      <c r="X77" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y77" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z77" s="3">
+        <v>0.252</v>
+      </c>
+      <c r="AA77" s="3">
+        <v>1.0160640000000001</v>
+      </c>
+      <c r="AB77" s="2">
+        <v>100</v>
+      </c>
+      <c r="AC77" s="3">
+        <v>11</v>
+      </c>
+      <c r="AD77" s="2">
+        <v>1510.59370258337</v>
+      </c>
+    </row>
+    <row r="78" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A78" s="21"/>
       <c r="B78" s="21"/>
       <c r="C78" s="21"/>
@@ -5598,8 +6633,53 @@
       <c r="O78" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="79" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P78" s="3">
+        <v>0.19671244991665399</v>
+      </c>
+      <c r="Q78" s="3">
+        <v>7.3385994064906299E-2</v>
+      </c>
+      <c r="R78" s="3">
+        <v>0.21064040329979999</v>
+      </c>
+      <c r="S78" s="3">
+        <v>4.9692216629041497E-2</v>
+      </c>
+      <c r="T78" s="2">
+        <v>0</v>
+      </c>
+      <c r="U78" s="2">
+        <v>5.6548667764616201E-2</v>
+      </c>
+      <c r="V78" s="3">
+        <v>5.6548667764616201E-2</v>
+      </c>
+      <c r="W78" s="2">
+        <v>0</v>
+      </c>
+      <c r="X78" s="3">
+        <v>5.6548667764616201E-2</v>
+      </c>
+      <c r="Y78" s="3">
+        <v>5.6548667764616201E-2</v>
+      </c>
+      <c r="Z78" s="3">
+        <v>1.6362000000000001</v>
+      </c>
+      <c r="AA78" s="3">
+        <v>4.6362209999999999</v>
+      </c>
+      <c r="AB78" s="2">
+        <v>87.718181818181804</v>
+      </c>
+      <c r="AC78" s="3">
+        <v>9.6489999999999991</v>
+      </c>
+      <c r="AD78" s="2">
+        <v>14623.2034990794</v>
+      </c>
+    </row>
+    <row r="79" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A79" s="21"/>
       <c r="B79" s="21"/>
       <c r="C79" s="21"/>
@@ -5617,8 +6697,53 @@
       <c r="O79" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="80" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P79" s="3">
+        <v>0.28138346033538097</v>
+      </c>
+      <c r="Q79" s="3">
+        <v>1.6642141468699301E-2</v>
+      </c>
+      <c r="R79" s="3">
+        <v>0.27976099772787699</v>
+      </c>
+      <c r="S79" s="3">
+        <v>4.2988078863015599E-3</v>
+      </c>
+      <c r="T79" s="2">
+        <v>0</v>
+      </c>
+      <c r="U79" s="2">
+        <v>5.6548667764616201E-2</v>
+      </c>
+      <c r="V79" s="3">
+        <v>5.6548667764616201E-2</v>
+      </c>
+      <c r="W79" s="2">
+        <v>48.754545454545401</v>
+      </c>
+      <c r="X79" s="3">
+        <v>2.2252947962927601E-3</v>
+      </c>
+      <c r="Y79" s="3">
+        <v>2.2252947962927601E-3</v>
+      </c>
+      <c r="Z79" s="3">
+        <v>0.246</v>
+      </c>
+      <c r="AA79" s="3">
+        <v>1.764</v>
+      </c>
+      <c r="AB79" s="2">
+        <v>100</v>
+      </c>
+      <c r="AC79" s="3">
+        <v>11</v>
+      </c>
+      <c r="AD79" s="2">
+        <v>7664.0583359410903</v>
+      </c>
+    </row>
+    <row r="80" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A80" s="21"/>
       <c r="B80" s="21"/>
       <c r="C80" s="21"/>
@@ -5636,8 +6761,53 @@
       <c r="O80" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="81" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P80" s="3">
+        <v>0.206062935883218</v>
+      </c>
+      <c r="Q80" s="3">
+        <v>7.7527046881941897E-2</v>
+      </c>
+      <c r="R80" s="3">
+        <v>0.22095070765303701</v>
+      </c>
+      <c r="S80" s="3">
+        <v>5.3603689337032398E-2</v>
+      </c>
+      <c r="T80" s="2">
+        <v>0</v>
+      </c>
+      <c r="U80" s="2">
+        <v>5.6548667764616201E-2</v>
+      </c>
+      <c r="V80" s="3">
+        <v>5.6548667764616201E-2</v>
+      </c>
+      <c r="W80" s="2">
+        <v>4.1545454545454499</v>
+      </c>
+      <c r="X80" s="3">
+        <v>5.6548667764616201E-2</v>
+      </c>
+      <c r="Y80" s="3">
+        <v>5.6548667764616201E-2</v>
+      </c>
+      <c r="Z80" s="3">
+        <v>0.29519999999999902</v>
+      </c>
+      <c r="AA80" s="3">
+        <v>1.5960000000000001</v>
+      </c>
+      <c r="AB80" s="2">
+        <v>90.172727272727201</v>
+      </c>
+      <c r="AC80" s="3">
+        <v>9.9190000000000005</v>
+      </c>
+      <c r="AD80" s="2">
+        <v>9853.7325300468692</v>
+      </c>
+    </row>
+    <row r="81" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A81" s="21"/>
       <c r="B81" s="21"/>
       <c r="C81" s="21"/>
@@ -5656,7 +6826,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="82" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A82" s="21"/>
       <c r="B82" s="21"/>
       <c r="C82" s="21"/>
@@ -5674,10 +6844,100 @@
       <c r="O82" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="83" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P82" s="3">
+        <v>0.206062935883218</v>
+      </c>
+      <c r="Q82" s="3">
+        <v>7.7527046881941897E-2</v>
+      </c>
+      <c r="R82" s="3">
+        <v>0.22095070765303701</v>
+      </c>
+      <c r="S82" s="3">
+        <v>5.3603689337032398E-2</v>
+      </c>
+      <c r="T82" s="2">
+        <v>0</v>
+      </c>
+      <c r="U82" s="2">
+        <v>5.6548667764616201E-2</v>
+      </c>
+      <c r="V82" s="3">
+        <v>5.6548667764616201E-2</v>
+      </c>
+      <c r="W82" s="2">
+        <v>4.1545454545454499</v>
+      </c>
+      <c r="X82" s="3">
+        <v>5.6548667764616201E-2</v>
+      </c>
+      <c r="Y82" s="3">
+        <v>5.6548667764616201E-2</v>
+      </c>
+      <c r="Z82" s="3">
+        <v>0.29519999999999902</v>
+      </c>
+      <c r="AA82" s="3">
+        <v>1.5960000000000001</v>
+      </c>
+      <c r="AB82" s="2">
+        <v>90.172727272727201</v>
+      </c>
+      <c r="AC82" s="3">
+        <v>9.9190000000000005</v>
+      </c>
+      <c r="AD82" s="2">
+        <v>9853.7325300468692</v>
+      </c>
+    </row>
+    <row r="83" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O83" t="s">
         <v>38</v>
+      </c>
+      <c r="P83" s="3">
+        <v>0.206062935883218</v>
+      </c>
+      <c r="Q83" s="3">
+        <v>7.7527046881941897E-2</v>
+      </c>
+      <c r="R83" s="3">
+        <v>0.22095070765303701</v>
+      </c>
+      <c r="S83" s="3">
+        <v>5.3603689337032398E-2</v>
+      </c>
+      <c r="T83" s="2">
+        <v>0</v>
+      </c>
+      <c r="U83" s="2">
+        <v>5.6548667764616201E-2</v>
+      </c>
+      <c r="V83" s="3">
+        <v>5.6548667764616201E-2</v>
+      </c>
+      <c r="W83" s="2">
+        <v>4.1545454545454499</v>
+      </c>
+      <c r="X83" s="3">
+        <v>5.6548667764616201E-2</v>
+      </c>
+      <c r="Y83" s="3">
+        <v>5.6548667764616201E-2</v>
+      </c>
+      <c r="Z83" s="3">
+        <v>0.29519999999999902</v>
+      </c>
+      <c r="AA83" s="3">
+        <v>1.5960000000000001</v>
+      </c>
+      <c r="AB83" s="2">
+        <v>90.172727272727201</v>
+      </c>
+      <c r="AC83" s="3">
+        <v>9.9190000000000005</v>
+      </c>
+      <c r="AD83" s="2">
+        <v>9853.7325300468692</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
full results from all examples
</commit_message>
<xml_diff>
--- a/results/compiled results.xlsx
+++ b/results/compiled results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\elish\Desktop\Aims Project\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F74E363-4632-4736-8BF7-AA89281F44D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1909A0AB-C71F-4994-83C5-EDF42BF29570}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{DA4D96B0-492C-4945-A9C4-EFCA6D6BC722}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{DA4D96B0-492C-4945-A9C4-EFCA6D6BC722}"/>
   </bookViews>
   <sheets>
     <sheet name="Dynamic results" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="435" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="443" uniqueCount="51">
   <si>
     <t xml:space="preserve">Model </t>
   </si>
@@ -146,9 +146,6 @@
     <t>l 70b</t>
   </si>
   <si>
-    <t>l 8b</t>
-  </si>
-  <si>
     <t>g 31b</t>
   </si>
   <si>
@@ -204,8 +201,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.000"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -358,7 +356,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -472,6 +470,12 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -832,7 +836,7 @@
   <sheetData>
     <row r="1" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:29" x14ac:dyDescent="0.3">
@@ -840,22 +844,22 @@
         <v>0</v>
       </c>
       <c r="B2" s="31" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C2" s="32"/>
       <c r="D2" s="33"/>
       <c r="E2" s="32" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F2" s="32"/>
       <c r="G2" s="33"/>
       <c r="H2" s="32" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I2" s="32"/>
       <c r="J2" s="32"/>
       <c r="K2" s="31" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L2" s="32"/>
       <c r="M2" s="32"/>
@@ -1255,7 +1259,7 @@
         <v>9</v>
       </c>
       <c r="T15" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="U15" s="3" t="s">
         <v>9</v>
@@ -1287,7 +1291,7 @@
     </row>
     <row r="16" spans="1:29" x14ac:dyDescent="0.3">
       <c r="N16" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="O16" s="3">
         <v>2.0934814092646199E-2</v>
@@ -1331,7 +1335,7 @@
     </row>
     <row r="17" spans="1:29" x14ac:dyDescent="0.3">
       <c r="N17" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="18" spans="1:29" x14ac:dyDescent="0.3">
@@ -1424,7 +1428,7 @@
     </row>
     <row r="20" spans="1:29" x14ac:dyDescent="0.3">
       <c r="N20" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="O20" s="3">
         <v>2.1538025413604299E-2</v>
@@ -1468,7 +1472,7 @@
     </row>
     <row r="21" spans="1:29" x14ac:dyDescent="0.3">
       <c r="N21" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="O21" s="3">
         <v>2.1538025413604299E-2</v>
@@ -1512,7 +1516,7 @@
     </row>
     <row r="22" spans="1:29" x14ac:dyDescent="0.3">
       <c r="N22" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="O22" s="3">
         <v>2.1538025413604299E-2</v>
@@ -1556,7 +1560,7 @@
     </row>
     <row r="23" spans="1:29" x14ac:dyDescent="0.3">
       <c r="N23" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="O23" s="3">
         <v>2.1538025413604299E-2</v>
@@ -1600,7 +1604,7 @@
     </row>
     <row r="26" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="27" spans="1:29" x14ac:dyDescent="0.3">
@@ -1608,22 +1612,22 @@
         <v>0</v>
       </c>
       <c r="B27" s="31" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C27" s="32"/>
       <c r="D27" s="33"/>
       <c r="E27" s="32" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F27" s="32"/>
       <c r="G27" s="33"/>
       <c r="H27" s="32" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I27" s="32"/>
       <c r="J27" s="32"/>
       <c r="K27" s="31" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L27" s="32"/>
       <c r="M27" s="32"/>
@@ -1963,7 +1967,7 @@
     </row>
     <row r="38" spans="1:29" x14ac:dyDescent="0.3">
       <c r="N38" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="O38" s="3">
         <v>9.0957692494960204E-2</v>
@@ -2009,7 +2013,7 @@
     </row>
     <row r="39" spans="1:29" x14ac:dyDescent="0.3">
       <c r="N39" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="O39" s="3">
         <v>2.0584563579292298E-2</v>
@@ -2141,7 +2145,7 @@
     </row>
     <row r="42" spans="1:29" x14ac:dyDescent="0.3">
       <c r="N42" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="O42" s="3">
         <v>2.1628472999999999E-2</v>
@@ -2185,7 +2189,7 @@
     </row>
     <row r="43" spans="1:29" x14ac:dyDescent="0.3">
       <c r="N43" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="O43" s="3">
         <v>2.1628472999999999E-2</v>
@@ -2229,7 +2233,7 @@
     </row>
     <row r="44" spans="1:29" x14ac:dyDescent="0.3">
       <c r="N44" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="O44" s="3">
         <v>2.1628472652915998E-2</v>
@@ -2273,7 +2277,7 @@
     </row>
     <row r="45" spans="1:29" x14ac:dyDescent="0.3">
       <c r="N45" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="O45" s="3">
         <v>2.1628472652915998E-2</v>
@@ -2317,7 +2321,7 @@
     </row>
     <row r="46" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="47" spans="1:29" x14ac:dyDescent="0.3">
@@ -2325,29 +2329,29 @@
         <v>0</v>
       </c>
       <c r="B47" s="31" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C47" s="32"/>
       <c r="D47" s="33"/>
       <c r="E47" s="32" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F47" s="32"/>
       <c r="G47" s="33"/>
       <c r="H47" s="32" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I47" s="32"/>
       <c r="J47" s="32"/>
       <c r="K47" s="31" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L47" s="32"/>
       <c r="M47" s="32"/>
     </row>
     <row r="48" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A48" s="12" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B48" s="7">
         <v>0.259999990463256</v>
@@ -2388,7 +2392,7 @@
     </row>
     <row r="49" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A49" s="12" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B49" s="7">
         <v>0.234999999403953</v>
@@ -2680,7 +2684,7 @@
     </row>
     <row r="59" spans="1:29" x14ac:dyDescent="0.3">
       <c r="N59" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="O59" s="3">
         <v>2.0811572863993801E-2</v>
@@ -2724,7 +2728,7 @@
     </row>
     <row r="60" spans="1:29" x14ac:dyDescent="0.3">
       <c r="N60" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="O60" s="3">
         <v>6.0352238096435099E-2</v>
@@ -2856,7 +2860,7 @@
     </row>
     <row r="63" spans="1:29" x14ac:dyDescent="0.3">
       <c r="N63" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="O63" s="3">
         <v>2.1628472999999999E-2</v>
@@ -2900,7 +2904,7 @@
     </row>
     <row r="64" spans="1:29" x14ac:dyDescent="0.3">
       <c r="N64" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="O64" s="3">
         <v>2.1628472652915998E-2</v>
@@ -2944,7 +2948,7 @@
     </row>
     <row r="65" spans="1:29" x14ac:dyDescent="0.3">
       <c r="N65" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="O65" s="3">
         <v>2.1628472999999999E-2</v>
@@ -2988,7 +2992,7 @@
     </row>
     <row r="66" spans="1:29" x14ac:dyDescent="0.3">
       <c r="N66" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="O66" s="3">
         <v>2.1628472652915998E-2</v>
@@ -3032,7 +3036,7 @@
     </row>
     <row r="69" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="70" spans="1:29" x14ac:dyDescent="0.3">
@@ -3040,22 +3044,22 @@
         <v>0</v>
       </c>
       <c r="B70" s="31" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C70" s="32"/>
       <c r="D70" s="33"/>
       <c r="E70" s="32" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F70" s="32"/>
       <c r="G70" s="33"/>
       <c r="H70" s="32" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I70" s="32"/>
       <c r="J70" s="32"/>
       <c r="K70" s="31" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L70" s="32"/>
       <c r="M70" s="32"/>
@@ -3409,7 +3413,7 @@
       <c r="L81"/>
       <c r="M81"/>
       <c r="N81" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="O81" s="3">
         <v>2.4033445388934701E-2</v>
@@ -3465,7 +3469,7 @@
       <c r="L82"/>
       <c r="M82"/>
       <c r="N82" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="O82" s="3">
         <v>2.4583666008142602E-2</v>
@@ -3633,7 +3637,7 @@
       <c r="L85"/>
       <c r="M85"/>
       <c r="N85" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="O85" s="3">
         <v>2.4585621925057501E-2</v>
@@ -3689,7 +3693,7 @@
       <c r="L86"/>
       <c r="M86"/>
       <c r="N86" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="87" spans="2:29" x14ac:dyDescent="0.3">
@@ -3706,7 +3710,7 @@
       <c r="L87"/>
       <c r="M87"/>
       <c r="N87" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="O87" s="3">
         <v>2.4585621925057501E-2</v>
@@ -3750,7 +3754,7 @@
     </row>
     <row r="88" spans="2:29" x14ac:dyDescent="0.3">
       <c r="N88" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="O88" s="3">
         <v>2.4585621925057501E-2</v>
@@ -3834,7 +3838,7 @@
   <sheetData>
     <row r="1" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:30" x14ac:dyDescent="0.3">
@@ -3842,22 +3846,22 @@
         <v>0</v>
       </c>
       <c r="B2" s="31" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C2" s="32"/>
       <c r="D2" s="33"/>
       <c r="E2" s="32" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F2" s="32"/>
       <c r="G2" s="33"/>
       <c r="H2" s="32" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I2" s="32"/>
       <c r="J2" s="32"/>
       <c r="K2" s="31" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L2" s="32"/>
       <c r="M2" s="32"/>
@@ -4220,43 +4224,43 @@
     </row>
     <row r="14" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O14" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="P14" s="3">
-        <v>0.208803427881982</v>
+        <v>0.20880342800000001</v>
       </c>
       <c r="Q14" s="3">
-        <v>3.2646891997723602E-2</v>
+        <v>3.2646891999999997E-2</v>
       </c>
       <c r="R14" s="3">
-        <v>0.20774180079319299</v>
+        <v>0.207741801</v>
       </c>
       <c r="S14" s="3">
-        <v>3.1069445262637101E-2</v>
+        <v>3.1069445000000001E-2</v>
       </c>
       <c r="T14" s="2">
         <v>100</v>
       </c>
       <c r="U14" s="2">
-        <v>1.81694009620145E-3</v>
+        <v>1.81694E-3</v>
       </c>
       <c r="V14" s="3">
-        <v>1.81694009620145E-3</v>
+        <v>1.81694E-3</v>
       </c>
       <c r="W14" s="2">
         <v>0</v>
       </c>
       <c r="X14" s="3">
-        <v>5.6548667764616201E-2</v>
+        <v>5.6548668000000003E-2</v>
       </c>
       <c r="Y14" s="3">
-        <v>5.6548667764616201E-2</v>
+        <v>5.6548668000000003E-2</v>
       </c>
       <c r="Z14" s="3">
         <v>0.02</v>
       </c>
       <c r="AA14" s="3">
-        <v>3.81633599999999</v>
+        <v>3.8163360000000002</v>
       </c>
       <c r="AB14" s="2">
         <v>100</v>
@@ -4265,33 +4269,33 @@
         <v>11</v>
       </c>
       <c r="AD14" s="2">
-        <v>5331.3170567901097</v>
+        <v>5331.3170570000002</v>
       </c>
     </row>
     <row r="15" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O15" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="P15" s="3">
-        <v>0.205705302011014</v>
+        <v>0.208803427881982</v>
       </c>
       <c r="Q15" s="3">
-        <v>0.10480522342236601</v>
+        <v>3.2646891997723602E-2</v>
       </c>
       <c r="R15" s="3">
-        <v>0.20691336023293999</v>
+        <v>0.20774180079319299</v>
       </c>
       <c r="S15" s="3">
-        <v>0.10594480432336199</v>
+        <v>3.1069445262637101E-2</v>
       </c>
       <c r="T15" s="2">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="U15" s="2">
-        <v>4.7640653619619E-2</v>
+        <v>1.81694009620145E-3</v>
       </c>
       <c r="V15" s="3">
-        <v>4.7640653619619E-2</v>
+        <v>1.81694009620145E-3</v>
       </c>
       <c r="W15" s="2">
         <v>0</v>
@@ -4303,19 +4307,19 @@
         <v>5.6548667764616201E-2</v>
       </c>
       <c r="Z15" s="3">
-        <v>6.3199999999999895E-2</v>
+        <v>0.02</v>
       </c>
       <c r="AA15" s="3">
         <v>3.81633599999999</v>
       </c>
       <c r="AB15" s="2">
-        <v>93.6</v>
+        <v>100</v>
       </c>
       <c r="AC15" s="3">
-        <v>10.295999999999999</v>
+        <v>11</v>
       </c>
       <c r="AD15" s="2">
-        <v>8331.0174627980305</v>
+        <v>5331.3170567901097</v>
       </c>
     </row>
     <row r="16" spans="1:30" x14ac:dyDescent="0.3">
@@ -4323,16 +4327,16 @@
         <v>33</v>
       </c>
       <c r="P16" s="3">
-        <v>0.20094616602850901</v>
+        <v>0.205705302011014</v>
       </c>
       <c r="Q16" s="3">
-        <v>0.107460022996064</v>
+        <v>0.10480522342236601</v>
       </c>
       <c r="R16" s="3">
-        <v>0.20170607435510901</v>
+        <v>0.20691336023293999</v>
       </c>
       <c r="S16" s="3">
-        <v>0.108864617481995</v>
+        <v>0.10594480432336199</v>
       </c>
       <c r="T16" s="2">
         <v>0</v>
@@ -4353,19 +4357,19 @@
         <v>5.6548667764616201E-2</v>
       </c>
       <c r="Z16" s="3">
-        <v>2.3199999999999901E-2</v>
+        <v>6.3199999999999895E-2</v>
       </c>
       <c r="AA16" s="3">
-        <v>2.619904</v>
+        <v>3.81633599999999</v>
       </c>
       <c r="AB16" s="2">
-        <v>98.918181818181793</v>
+        <v>93.6</v>
       </c>
       <c r="AC16" s="3">
-        <v>10.881</v>
+        <v>10.295999999999999</v>
       </c>
       <c r="AD16" s="2">
-        <v>7108.14468373205</v>
+        <v>8331.0174627980305</v>
       </c>
     </row>
     <row r="17" spans="1:30" x14ac:dyDescent="0.3">
@@ -4373,66 +4377,66 @@
         <v>32</v>
       </c>
       <c r="P17" s="3">
-        <v>0.36366496008710802</v>
+        <v>0.20094616602850901</v>
       </c>
       <c r="Q17" s="3">
-        <v>8.5103341494056503E-2</v>
+        <v>0.107460022996064</v>
       </c>
       <c r="R17" s="3">
-        <v>0.36356107891046802</v>
+        <v>0.20170607435510901</v>
       </c>
       <c r="S17" s="3">
-        <v>8.5107195582413003E-2</v>
+        <v>0.108864617481995</v>
       </c>
       <c r="T17" s="2">
         <v>0</v>
       </c>
       <c r="U17" s="2">
+        <v>4.7640653619619E-2</v>
+      </c>
+      <c r="V17" s="3">
+        <v>4.7640653619619E-2</v>
+      </c>
+      <c r="W17" s="2">
+        <v>0</v>
+      </c>
+      <c r="X17" s="3">
         <v>5.6548667764616201E-2</v>
       </c>
-      <c r="V17" s="3">
+      <c r="Y17" s="3">
         <v>5.6548667764616201E-2</v>
       </c>
-      <c r="W17" s="2">
-        <v>87.1</v>
-      </c>
-      <c r="X17" s="3">
-        <v>0</v>
-      </c>
-      <c r="Y17" s="3">
-        <v>0</v>
-      </c>
       <c r="Z17" s="3">
-        <v>0.156799999999999</v>
+        <v>2.3199999999999901E-2</v>
       </c>
       <c r="AA17" s="3">
-        <v>0.37631999999999999</v>
+        <v>2.619904</v>
       </c>
       <c r="AB17" s="2">
-        <v>100</v>
+        <v>98.918181818181793</v>
       </c>
       <c r="AC17" s="3">
-        <v>11</v>
+        <v>10.881</v>
       </c>
       <c r="AD17" s="2">
-        <v>4079.1357275988898</v>
+        <v>7108.14468373205</v>
       </c>
     </row>
     <row r="18" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O18" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="P18" s="3">
-        <v>0.261901664151098</v>
+        <v>0.36366496008710802</v>
       </c>
       <c r="Q18" s="3">
-        <v>0.124405443576612</v>
+        <v>8.5103341494056503E-2</v>
       </c>
       <c r="R18" s="3">
-        <v>0.261743363290594</v>
+        <v>0.36356107891046802</v>
       </c>
       <c r="S18" s="3">
-        <v>0.124877538651196</v>
+        <v>8.5107195582413003E-2</v>
       </c>
       <c r="T18" s="2">
         <v>0</v>
@@ -4444,19 +4448,19 @@
         <v>5.6548667764616201E-2</v>
       </c>
       <c r="W18" s="2">
-        <v>100</v>
+        <v>87.1</v>
       </c>
       <c r="X18" s="3">
-        <v>5.6548667764616201E-2</v>
+        <v>0</v>
       </c>
       <c r="Y18" s="3">
-        <v>5.6548667764616201E-2</v>
+        <v>0</v>
       </c>
       <c r="Z18" s="3">
-        <v>0.13119999999999901</v>
+        <v>0.156799999999999</v>
       </c>
       <c r="AA18" s="3">
-        <v>0.38370899999999902</v>
+        <v>0.37631999999999999</v>
       </c>
       <c r="AB18" s="2">
         <v>100</v>
@@ -4465,24 +4469,24 @@
         <v>11</v>
       </c>
       <c r="AD18" s="2">
-        <v>9698.3661137017607</v>
+        <v>4079.1357275988898</v>
       </c>
     </row>
     <row r="19" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O19" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="P19" s="3">
-        <v>0.33054050800014101</v>
+        <v>0.261901664151098</v>
       </c>
       <c r="Q19" s="3">
-        <v>0.116855717031366</v>
+        <v>0.124405443576612</v>
       </c>
       <c r="R19" s="3">
-        <v>0.33034728905099198</v>
+        <v>0.261743363290594</v>
       </c>
       <c r="S19" s="3">
-        <v>0.117266130962788</v>
+        <v>0.124877538651196</v>
       </c>
       <c r="T19" s="2">
         <v>0</v>
@@ -4503,10 +4507,10 @@
         <v>5.6548667764616201E-2</v>
       </c>
       <c r="Z19" s="3">
-        <v>0.156799999999999</v>
+        <v>0.13119999999999901</v>
       </c>
       <c r="AA19" s="3">
-        <v>0.37440000000000001</v>
+        <v>0.38370899999999902</v>
       </c>
       <c r="AB19" s="2">
         <v>100</v>
@@ -4515,24 +4519,24 @@
         <v>11</v>
       </c>
       <c r="AD19" s="2">
-        <v>13665.8515410358</v>
+        <v>9698.3661137017607</v>
       </c>
     </row>
     <row r="20" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O20" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="P20" s="3">
-        <v>0.33834814301107202</v>
+        <v>0.33054050800014101</v>
       </c>
       <c r="Q20" s="3">
-        <v>0.11752130295997699</v>
+        <v>0.116855717031366</v>
       </c>
       <c r="R20" s="3">
-        <v>0.33837069477188497</v>
+        <v>0.33034728905099198</v>
       </c>
       <c r="S20" s="3">
-        <v>0.117818134227457</v>
+        <v>0.117266130962788</v>
       </c>
       <c r="T20" s="2">
         <v>0</v>
@@ -4556,7 +4560,7 @@
         <v>0.156799999999999</v>
       </c>
       <c r="AA20" s="3">
-        <v>0.33629999999999899</v>
+        <v>0.37440000000000001</v>
       </c>
       <c r="AB20" s="2">
         <v>100</v>
@@ -4565,17 +4569,62 @@
         <v>11</v>
       </c>
       <c r="AD20" s="2">
-        <v>13585.1360406514</v>
+        <v>13665.8515410358</v>
       </c>
     </row>
     <row r="21" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O21" t="s">
-        <v>38</v>
+        <v>37</v>
+      </c>
+      <c r="P21" s="3">
+        <v>0.33834814301107202</v>
+      </c>
+      <c r="Q21" s="3">
+        <v>0.11752130295997699</v>
+      </c>
+      <c r="R21" s="3">
+        <v>0.33837069477188497</v>
+      </c>
+      <c r="S21" s="3">
+        <v>0.117818134227457</v>
+      </c>
+      <c r="T21" s="2">
+        <v>0</v>
+      </c>
+      <c r="U21" s="2">
+        <v>5.6548667764616201E-2</v>
+      </c>
+      <c r="V21" s="3">
+        <v>5.6548667764616201E-2</v>
+      </c>
+      <c r="W21" s="2">
+        <v>100</v>
+      </c>
+      <c r="X21" s="3">
+        <v>5.6548667764616201E-2</v>
+      </c>
+      <c r="Y21" s="3">
+        <v>5.6548667764616201E-2</v>
+      </c>
+      <c r="Z21" s="3">
+        <v>0.156799999999999</v>
+      </c>
+      <c r="AA21" s="3">
+        <v>0.33629999999999899</v>
+      </c>
+      <c r="AB21" s="2">
+        <v>100</v>
+      </c>
+      <c r="AC21" s="3">
+        <v>11</v>
+      </c>
+      <c r="AD21" s="2">
+        <v>13585.1360406514</v>
       </c>
     </row>
     <row r="23" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="24" spans="1:30" x14ac:dyDescent="0.3">
@@ -4583,22 +4632,22 @@
         <v>0</v>
       </c>
       <c r="B24" s="31" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C24" s="32"/>
       <c r="D24" s="33"/>
       <c r="E24" s="32" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F24" s="32"/>
       <c r="G24" s="33"/>
       <c r="H24" s="32" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I24" s="32"/>
       <c r="J24" s="32"/>
       <c r="K24" s="31" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L24" s="32"/>
       <c r="M24" s="32"/>
@@ -4938,7 +4987,7 @@
     </row>
     <row r="35" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O35" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="P35" s="3">
         <v>0.292965027710332</v>
@@ -4988,7 +5037,7 @@
     </row>
     <row r="36" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O36" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="P36" s="3">
         <v>0.20570530200000001</v>
@@ -5138,7 +5187,7 @@
     </row>
     <row r="39" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O39" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="P39" s="3">
         <v>0.40507656031128503</v>
@@ -5188,7 +5237,7 @@
     </row>
     <row r="40" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O40" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="P40" s="3">
         <v>0.527889263524429</v>
@@ -5238,7 +5287,7 @@
     </row>
     <row r="41" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O41" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="P41" s="3">
         <v>0.52887767906368</v>
@@ -5288,7 +5337,7 @@
     </row>
     <row r="42" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O42" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="P42" s="3">
         <v>0.52881868088098205</v>
@@ -5338,7 +5387,7 @@
     </row>
     <row r="43" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="44" spans="1:30" x14ac:dyDescent="0.3">
@@ -5346,22 +5395,22 @@
         <v>0</v>
       </c>
       <c r="B44" s="31" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C44" s="32"/>
       <c r="D44" s="33"/>
       <c r="E44" s="32" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F44" s="32"/>
       <c r="G44" s="33"/>
       <c r="H44" s="32" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I44" s="32"/>
       <c r="J44" s="32"/>
       <c r="K44" s="31" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L44" s="32"/>
       <c r="M44" s="32"/>
@@ -5701,7 +5750,7 @@
     </row>
     <row r="55" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O55" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="P55" s="3">
         <v>0.24152868270713199</v>
@@ -5751,7 +5800,7 @@
     </row>
     <row r="56" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O56" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="P56" s="3">
         <v>0.24153136628727301</v>
@@ -5901,7 +5950,7 @@
     </row>
     <row r="59" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O59" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="P59" s="3">
         <v>0.39959914338580699</v>
@@ -5951,7 +6000,7 @@
     </row>
     <row r="60" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O60" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="P60" s="3">
         <v>0.64763181116499502</v>
@@ -6001,7 +6050,7 @@
     </row>
     <row r="61" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O61" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="P61" s="3">
         <v>0.32782759329432998</v>
@@ -6051,7 +6100,7 @@
     </row>
     <row r="62" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O62" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="P62" s="3">
         <v>0.54419239100000005</v>
@@ -6101,7 +6150,7 @@
     </row>
     <row r="64" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="65" spans="1:30" x14ac:dyDescent="0.3">
@@ -6109,22 +6158,22 @@
         <v>0</v>
       </c>
       <c r="B65" s="34" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C65" s="35"/>
       <c r="D65" s="36"/>
       <c r="E65" s="37" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F65" s="35"/>
       <c r="G65" s="36"/>
       <c r="H65" s="37" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I65" s="35"/>
       <c r="J65" s="38"/>
       <c r="K65" s="34" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L65" s="35"/>
       <c r="M65" s="35"/>
@@ -6503,7 +6552,7 @@
       <c r="M76" s="21"/>
       <c r="N76" s="21"/>
       <c r="O76" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="P76" s="3">
         <v>0.70879072300000001</v>
@@ -6567,7 +6616,7 @@
       <c r="M77" s="21"/>
       <c r="N77" s="21"/>
       <c r="O77" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="P77" s="3">
         <v>0.70879071959919404</v>
@@ -6759,7 +6808,7 @@
       <c r="M80" s="21"/>
       <c r="N80" s="21"/>
       <c r="O80" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="P80" s="3">
         <v>0.206062935883218</v>
@@ -6823,7 +6872,7 @@
       <c r="M81" s="21"/>
       <c r="N81" s="21"/>
       <c r="O81" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="82" spans="1:30" x14ac:dyDescent="0.3">
@@ -6842,7 +6891,7 @@
       <c r="M82" s="21"/>
       <c r="N82" s="21"/>
       <c r="O82" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="P82" s="3">
         <v>0.206062935883218</v>
@@ -6892,7 +6941,7 @@
     </row>
     <row r="83" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O83" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="P83" s="3">
         <v>0.206062935883218</v>
@@ -6965,15 +7014,27 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA087EBE-083C-402B-95D7-A249E10AE281}">
-  <dimension ref="A1:AD81"/>
+  <dimension ref="A1:AD82"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.77734375" customWidth="1"/>
+    <col min="16" max="19" width="9" style="3" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="16" style="2" customWidth="1"/>
+    <col min="21" max="21" width="10.33203125" style="3" customWidth="1"/>
+    <col min="22" max="22" width="9" style="3" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="9" style="2" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="9" style="3" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="12.33203125" style="3" customWidth="1"/>
+    <col min="26" max="26" width="12" style="3" customWidth="1"/>
+    <col min="27" max="27" width="16" style="3" customWidth="1"/>
+    <col min="28" max="28" width="9" style="2" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="9" style="3" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="9.88671875" style="2" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:30" x14ac:dyDescent="0.3">
@@ -6981,22 +7042,22 @@
         <v>0</v>
       </c>
       <c r="B2" s="31" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C2" s="32"/>
       <c r="D2" s="33"/>
       <c r="E2" s="32" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F2" s="32"/>
       <c r="G2" s="33"/>
       <c r="H2" s="32" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I2" s="32"/>
       <c r="J2" s="32"/>
       <c r="K2" s="31" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L2" s="32"/>
       <c r="M2" s="32"/>
@@ -7321,7 +7382,7 @@
       <c r="T11" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="U11" s="4" t="s">
+      <c r="U11" s="3" t="s">
         <v>23</v>
       </c>
       <c r="V11" s="3" t="s">
@@ -7359,70 +7420,345 @@
     </row>
     <row r="13" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O13" t="s">
-        <v>34</v>
+        <v>49</v>
+      </c>
+      <c r="P13" s="3">
+        <v>4.2014315000000003E-2</v>
+      </c>
+      <c r="Q13" s="3">
+        <v>4.5367003000000003E-2</v>
+      </c>
+      <c r="R13" s="3">
+        <v>3.3585647000000003E-2</v>
+      </c>
+      <c r="S13" s="3">
+        <v>2.2475227E-2</v>
+      </c>
+      <c r="T13" s="2">
+        <v>0</v>
+      </c>
+      <c r="U13" s="3">
+        <v>1.7944689999999999E-3</v>
+      </c>
+      <c r="V13" s="3">
+        <v>1.7944689999999999E-3</v>
+      </c>
+      <c r="W13" s="2">
+        <v>0</v>
+      </c>
+      <c r="X13" s="3">
+        <v>3.3335779999999998E-3</v>
+      </c>
+      <c r="Y13" s="3">
+        <v>3.3335779999999998E-3</v>
+      </c>
+      <c r="Z13" s="3">
+        <v>2.7040000000000002E-2</v>
+      </c>
+      <c r="AA13" s="3">
+        <v>3.8163360000000002</v>
+      </c>
+      <c r="AB13" s="2">
+        <v>45.56818182</v>
+      </c>
+      <c r="AC13" s="3">
+        <v>5.0125000000000002</v>
+      </c>
+      <c r="AD13" s="2">
+        <v>5218.4328599999999</v>
       </c>
     </row>
     <row r="14" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O14" t="s">
-        <v>33</v>
+        <v>50</v>
+      </c>
+      <c r="P14" s="3">
+        <v>4.2014338702453899E-2</v>
+      </c>
+      <c r="Q14" s="3">
+        <v>4.5367001376787397E-2</v>
+      </c>
+      <c r="R14" s="3">
+        <v>3.3585671741942401E-2</v>
+      </c>
+      <c r="S14" s="3">
+        <v>2.2475229587933299E-2</v>
+      </c>
+      <c r="T14" s="2">
+        <v>0</v>
+      </c>
+      <c r="U14" s="3">
+        <v>1.7221527280616E-3</v>
+      </c>
+      <c r="V14" s="3">
+        <v>1.7221527280616E-3</v>
+      </c>
+      <c r="W14" s="2">
+        <v>0</v>
+      </c>
+      <c r="X14" s="3">
+        <v>3.3335776281149501E-3</v>
+      </c>
+      <c r="Y14" s="3">
+        <v>3.3335776281149501E-3</v>
+      </c>
+      <c r="Z14" s="3">
+        <v>2.496E-2</v>
+      </c>
+      <c r="AA14" s="3">
+        <v>3.81633599999999</v>
+      </c>
+      <c r="AB14" s="2">
+        <v>45.454545454545404</v>
+      </c>
+      <c r="AC14" s="3">
+        <v>5</v>
+      </c>
+      <c r="AD14" s="2">
+        <v>5218.4318246387002</v>
       </c>
     </row>
     <row r="15" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O15" t="s">
-        <v>32</v>
+        <v>33</v>
+      </c>
+      <c r="P15" s="3">
+        <v>4.2014348E-2</v>
+      </c>
+      <c r="Q15" s="3">
+        <v>4.5366978000000002E-2</v>
+      </c>
+      <c r="R15" s="3">
+        <v>3.3585688000000002E-2</v>
+      </c>
+      <c r="S15" s="3">
+        <v>2.2475209999999999E-2</v>
+      </c>
+      <c r="T15" s="2">
+        <v>0</v>
+      </c>
+      <c r="U15" s="3">
+        <v>1.799536E-3</v>
+      </c>
+      <c r="V15" s="3">
+        <v>1.799536E-3</v>
+      </c>
+      <c r="W15" s="2">
+        <v>0</v>
+      </c>
+      <c r="X15" s="3">
+        <v>3.3335779999999998E-3</v>
+      </c>
+      <c r="Y15" s="3">
+        <v>3.3335779999999998E-3</v>
+      </c>
+      <c r="Z15" s="3">
+        <v>5.1200000000000002E-2</v>
+      </c>
+      <c r="AA15" s="3">
+        <v>3.3281999999999998</v>
+      </c>
+      <c r="AB15" s="2">
+        <v>45.60606061</v>
+      </c>
+      <c r="AC15" s="3">
+        <v>5.016666667</v>
+      </c>
+      <c r="AD15" s="2">
+        <v>5218.4308760000004</v>
       </c>
     </row>
     <row r="16" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O16" t="s">
+        <v>32</v>
+      </c>
+      <c r="P16" s="3">
+        <v>5.7919755000000003E-2</v>
+      </c>
+      <c r="Q16" s="3">
+        <v>4.5499654E-2</v>
+      </c>
+      <c r="R16" s="3">
+        <v>4.9692238999999999E-2</v>
+      </c>
+      <c r="S16" s="3">
+        <v>2.4941772000000001E-2</v>
+      </c>
+      <c r="T16" s="2">
+        <v>0</v>
+      </c>
+      <c r="U16" s="3">
+        <v>2.5963639999999999E-3</v>
+      </c>
+      <c r="V16" s="3">
+        <v>2.5963639999999999E-3</v>
+      </c>
+      <c r="W16" s="2">
+        <v>100</v>
+      </c>
+      <c r="X16" s="3">
+        <v>3.3335779999999998E-3</v>
+      </c>
+      <c r="Y16" s="3">
+        <v>3.3335779999999998E-3</v>
+      </c>
+      <c r="Z16" s="3">
+        <v>0.11423999999999999</v>
+      </c>
+      <c r="AA16" s="3">
+        <v>0.441</v>
+      </c>
+      <c r="AB16" s="2">
+        <v>100</v>
+      </c>
+      <c r="AC16" s="3">
+        <v>11</v>
+      </c>
+      <c r="AD16" s="2">
+        <v>8629.9956860000002</v>
+      </c>
+    </row>
+    <row r="17" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="O17" t="s">
+        <v>34</v>
+      </c>
+      <c r="P17" s="3">
+        <v>0.32352501569431402</v>
+      </c>
+      <c r="Q17" s="3">
+        <v>8.0327988032312295E-2</v>
+      </c>
+      <c r="R17" s="3">
+        <v>0.318604672838811</v>
+      </c>
+      <c r="S17" s="3">
+        <v>8.0458833222313703E-2</v>
+      </c>
+      <c r="T17" s="2">
+        <v>0</v>
+      </c>
+      <c r="U17" s="3">
+        <v>2.5963635446017101E-3</v>
+      </c>
+      <c r="V17" s="3">
+        <v>2.5963635446017101E-3</v>
+      </c>
+      <c r="W17" s="2">
+        <v>100</v>
+      </c>
+      <c r="X17" s="3">
+        <v>2.1407571476495602E-3</v>
+      </c>
+      <c r="Y17" s="3">
+        <v>2.1407571476495602E-3</v>
+      </c>
+      <c r="Z17" s="3">
+        <v>0.11592</v>
+      </c>
+      <c r="AA17" s="3">
+        <v>0.16799999999999901</v>
+      </c>
+      <c r="AB17" s="2">
+        <v>100</v>
+      </c>
+      <c r="AC17" s="3">
+        <v>11</v>
+      </c>
+      <c r="AD17" s="2">
+        <v>6370.8851921161804</v>
+      </c>
+    </row>
+    <row r="18" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="O18" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="O17" t="s">
+    <row r="19" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="O19" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="O18" t="s">
+      <c r="P19" s="3">
+        <v>0.16022386699999999</v>
+      </c>
+      <c r="Q19" s="3">
+        <v>2.9896869E-2</v>
+      </c>
+      <c r="R19" s="3">
+        <v>0.15472997599999999</v>
+      </c>
+      <c r="S19" s="3">
+        <v>1.9367807000000001E-2</v>
+      </c>
+      <c r="T19" s="2">
+        <v>0</v>
+      </c>
+      <c r="U19" s="3">
+        <v>2.5963639999999999E-3</v>
+      </c>
+      <c r="V19" s="3">
+        <v>2.5963639999999999E-3</v>
+      </c>
+      <c r="W19" s="2">
+        <v>35.265151520000003</v>
+      </c>
+      <c r="X19" s="3">
+        <v>3.3335779999999998E-3</v>
+      </c>
+      <c r="Y19" s="3">
+        <v>3.3335779999999998E-3</v>
+      </c>
+      <c r="Z19" s="3">
+        <v>0.12096</v>
+      </c>
+      <c r="AA19" s="3">
+        <v>0.71399999999999997</v>
+      </c>
+      <c r="AB19" s="2">
+        <v>100</v>
+      </c>
+      <c r="AC19" s="3">
+        <v>11</v>
+      </c>
+      <c r="AD19" s="2">
+        <v>4566.317556</v>
+      </c>
+    </row>
+    <row r="20" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="O20" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="O19" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.3">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="23" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A23" s="5" t="s">
         <v>0</v>
       </c>
       <c r="B23" s="31" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C23" s="32"/>
       <c r="D23" s="33"/>
       <c r="E23" s="32" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F23" s="32"/>
       <c r="G23" s="33"/>
       <c r="H23" s="32" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I23" s="32"/>
       <c r="J23" s="32"/>
       <c r="K23" s="31" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L23" s="32"/>
       <c r="M23" s="32"/>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A24" s="14" t="s">
         <v>1</v>
       </c>
@@ -7463,7 +7799,7 @@
         <v>0.30500000715255698</v>
       </c>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A25" s="12" t="s">
         <v>2</v>
       </c>
@@ -7504,7 +7840,7 @@
         <v>0.75499999523162797</v>
       </c>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A26" s="5" t="s">
         <v>3</v>
       </c>
@@ -7545,7 +7881,7 @@
         <v>1.0740000009536701</v>
       </c>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A27" s="14" t="s">
         <v>4</v>
       </c>
@@ -7586,7 +7922,7 @@
         <v>0.64499998092651301</v>
       </c>
     </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A28" s="5" t="s">
         <v>7</v>
       </c>
@@ -7627,7 +7963,7 @@
         <v>0.51999998092651301</v>
       </c>
     </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A29" s="12" t="s">
         <v>5</v>
       </c>
@@ -7644,7 +7980,7 @@
       <c r="L29" s="2"/>
       <c r="M29" s="2"/>
     </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A30" s="12" t="s">
         <v>17</v>
       </c>
@@ -7685,7 +8021,7 @@
         <v>0.56000000238418501</v>
       </c>
     </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A31" s="13" t="s">
         <v>6</v>
       </c>
@@ -7726,77 +8062,352 @@
         <v>1.1900000572204501</v>
       </c>
     </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O33" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O34" t="s">
+        <v>49</v>
+      </c>
+      <c r="P34" s="3">
+        <v>0.60818880816893195</v>
+      </c>
+      <c r="Q34" s="3">
+        <v>5.6804182423719297E-2</v>
+      </c>
+      <c r="R34" s="3">
+        <v>0.61669829615651806</v>
+      </c>
+      <c r="S34" s="3">
+        <v>4.0396311880573403E-2</v>
+      </c>
+      <c r="T34" s="2">
+        <v>100</v>
+      </c>
+      <c r="U34" s="3">
+        <v>0</v>
+      </c>
+      <c r="V34" s="3">
+        <v>0</v>
+      </c>
+      <c r="W34" s="2">
+        <v>100</v>
+      </c>
+      <c r="X34" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y34" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z34" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA34" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB34" s="2">
+        <v>100</v>
+      </c>
+      <c r="AC34" s="3">
+        <v>11</v>
+      </c>
+      <c r="AD34" s="2">
+        <v>6451.6821721451197</v>
+      </c>
+    </row>
+    <row r="35" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="O35" t="s">
+        <v>50</v>
+      </c>
+      <c r="P35" s="3">
+        <v>0.35510066930148498</v>
+      </c>
+      <c r="Q35" s="3">
+        <v>4.0702674721002197E-2</v>
+      </c>
+      <c r="R35" s="3">
+        <v>0.35632095236091998</v>
+      </c>
+      <c r="S35" s="3">
+        <v>4.2391921745013598E-2</v>
+      </c>
+      <c r="T35" s="2">
+        <v>100</v>
+      </c>
+      <c r="U35" s="3">
+        <v>0</v>
+      </c>
+      <c r="V35" s="3">
+        <v>0</v>
+      </c>
+      <c r="W35" s="2">
+        <v>100</v>
+      </c>
+      <c r="X35" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y35" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z35" s="3">
+        <v>2.72E-4</v>
+      </c>
+      <c r="AA35" s="3">
+        <v>2.7599999999999899E-3</v>
+      </c>
+      <c r="AB35" s="2">
+        <v>100</v>
+      </c>
+      <c r="AC35" s="3">
+        <v>11</v>
+      </c>
+      <c r="AD35" s="2">
+        <v>4822.5589480135704</v>
+      </c>
+    </row>
+    <row r="36" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="O36" t="s">
+        <v>33</v>
+      </c>
+      <c r="P36" s="3">
+        <v>4.2911879E-2</v>
+      </c>
+      <c r="Q36" s="3">
+        <v>4.7610356E-2</v>
+      </c>
+      <c r="R36" s="3">
+        <v>3.3634046000000001E-2</v>
+      </c>
+      <c r="S36" s="3">
+        <v>2.2448250999999999E-2</v>
+      </c>
+      <c r="T36" s="2">
+        <v>0</v>
+      </c>
+      <c r="U36" s="3">
+        <v>4.4100000000000001E-5</v>
+      </c>
+      <c r="V36" s="3">
+        <v>4.4100000000000001E-5</v>
+      </c>
+      <c r="W36" s="2">
+        <v>0</v>
+      </c>
+      <c r="X36" s="3">
+        <v>3.3335779999999998E-3</v>
+      </c>
+      <c r="Y36" s="3">
+        <v>3.3335779999999998E-3</v>
+      </c>
+      <c r="Z36" s="3">
+        <v>3.5496E-2</v>
+      </c>
+      <c r="AA36" s="3">
+        <v>1.504656</v>
+      </c>
+      <c r="AB36" s="2">
+        <v>47.196969699999997</v>
+      </c>
+      <c r="AC36" s="3">
+        <v>5.1916666669999998</v>
+      </c>
+      <c r="AD36" s="2">
+        <v>5175.2255839999998</v>
+      </c>
+    </row>
+    <row r="37" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="O37" t="s">
+        <v>32</v>
+      </c>
+      <c r="P37" s="3">
+        <v>0.22597246600000001</v>
+      </c>
+      <c r="Q37" s="3">
+        <v>2.0079974E-2</v>
+      </c>
+      <c r="R37" s="3">
+        <v>0.22275471699999999</v>
+      </c>
+      <c r="S37" s="3">
+        <v>1.4879814E-2</v>
+      </c>
+      <c r="T37" s="2">
+        <v>0</v>
+      </c>
+      <c r="U37" s="3">
+        <v>0</v>
+      </c>
+      <c r="V37" s="3">
+        <v>0</v>
+      </c>
+      <c r="W37" s="2">
+        <v>37.462121209999999</v>
+      </c>
+      <c r="X37" s="3">
+        <v>3.3335779999999998E-3</v>
+      </c>
+      <c r="Y37" s="3">
+        <v>3.3335779999999998E-3</v>
+      </c>
+      <c r="Z37" s="3">
+        <v>2.0331999999999999E-2</v>
+      </c>
+      <c r="AA37" s="3">
+        <v>3.7867519999999999</v>
+      </c>
+      <c r="AB37" s="2">
+        <v>100</v>
+      </c>
+      <c r="AC37" s="3">
+        <v>11</v>
+      </c>
+      <c r="AD37" s="2">
+        <v>4593.5556189999998</v>
+      </c>
+    </row>
+    <row r="38" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="O38" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="O35" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="O36" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="O37" t="s">
+      <c r="P38" s="3">
+        <v>0.216140047</v>
+      </c>
+      <c r="Q38" s="3">
+        <v>8.5321912999999999E-2</v>
+      </c>
+      <c r="R38" s="3">
+        <v>0.197299206</v>
+      </c>
+      <c r="S38" s="3">
+        <v>6.1894022E-2</v>
+      </c>
+      <c r="T38" s="2">
+        <v>0</v>
+      </c>
+      <c r="U38" s="3">
+        <v>0</v>
+      </c>
+      <c r="V38" s="3">
+        <v>0</v>
+      </c>
+      <c r="W38" s="2">
+        <v>100</v>
+      </c>
+      <c r="X38" s="3">
+        <v>1.7400000000000001E-6</v>
+      </c>
+      <c r="Y38" s="3">
+        <v>1.7400000000000001E-6</v>
+      </c>
+      <c r="Z38" s="3">
+        <v>1.5911999999999999E-2</v>
+      </c>
+      <c r="AA38" s="3">
+        <v>7.3111999999999996E-2</v>
+      </c>
+      <c r="AB38" s="2">
+        <v>100</v>
+      </c>
+      <c r="AC38" s="3">
+        <v>11</v>
+      </c>
+      <c r="AD38" s="2">
+        <v>7088.2309420000001</v>
+      </c>
+    </row>
+    <row r="39" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="O39" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="O38" t="s">
+    <row r="40" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="O40" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="O39" t="s">
+      <c r="P40" s="3">
+        <v>0.420673144</v>
+      </c>
+      <c r="Q40" s="3">
+        <v>5.9976452E-2</v>
+      </c>
+      <c r="R40" s="3">
+        <v>0.42202424999999999</v>
+      </c>
+      <c r="S40" s="3">
+        <v>5.5791974000000001E-2</v>
+      </c>
+      <c r="T40" s="2">
+        <v>0</v>
+      </c>
+      <c r="U40" s="3">
+        <v>0</v>
+      </c>
+      <c r="V40" s="3">
+        <v>0</v>
+      </c>
+      <c r="W40" s="2">
+        <v>100</v>
+      </c>
+      <c r="X40" s="3">
+        <v>4.5711699999999999E-4</v>
+      </c>
+      <c r="Y40" s="3">
+        <v>4.5711699999999999E-4</v>
+      </c>
+      <c r="Z40" s="3">
+        <v>1.5911999999999999E-2</v>
+      </c>
+      <c r="AA40" s="3">
+        <v>0.129076</v>
+      </c>
+      <c r="AB40" s="2">
+        <v>100</v>
+      </c>
+      <c r="AC40" s="3">
+        <v>11</v>
+      </c>
+      <c r="AD40" s="2">
+        <v>4997.4142389999997</v>
+      </c>
+    </row>
+    <row r="41" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="O41" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="O40" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.3">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="44" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A44" s="5" t="s">
         <v>0</v>
       </c>
       <c r="B44" s="31" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C44" s="32"/>
       <c r="D44" s="33"/>
       <c r="E44" s="32" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F44" s="32"/>
       <c r="G44" s="33"/>
       <c r="H44" s="32" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I44" s="32"/>
       <c r="J44" s="32"/>
       <c r="K44" s="31" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L44" s="32"/>
       <c r="M44" s="32"/>
     </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A45" s="14" t="s">
         <v>1</v>
       </c>
@@ -7837,7 +8448,7 @@
         <v>0.61400002241134599</v>
       </c>
     </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A46" s="12" t="s">
         <v>2</v>
       </c>
@@ -7878,7 +8489,7 @@
         <v>0.69999998807907104</v>
       </c>
     </row>
-    <row r="47" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A47" s="5" t="s">
         <v>3</v>
       </c>
@@ -7919,7 +8530,7 @@
         <v>0.605000019073486</v>
       </c>
     </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A48" s="14" t="s">
         <v>4</v>
       </c>
@@ -7960,7 +8571,7 @@
         <v>0.52999997138976995</v>
       </c>
     </row>
-    <row r="49" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A49" s="5" t="s">
         <v>7</v>
       </c>
@@ -8001,7 +8612,7 @@
         <v>1.1900000572204501</v>
       </c>
     </row>
-    <row r="50" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A50" s="12" t="s">
         <v>5</v>
       </c>
@@ -8018,7 +8629,7 @@
       <c r="L50" s="2"/>
       <c r="M50" s="2"/>
     </row>
-    <row r="51" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A51" s="12" t="s">
         <v>17</v>
       </c>
@@ -8059,7 +8670,7 @@
         <v>1.1900000572204501</v>
       </c>
     </row>
-    <row r="52" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A52" s="13" t="s">
         <v>6</v>
       </c>
@@ -8100,79 +8711,354 @@
         <v>0.52999997138976995</v>
       </c>
     </row>
-    <row r="54" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O54" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="55" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O55" t="s">
+        <v>49</v>
+      </c>
+      <c r="P55" s="3">
+        <v>0.17555779906965399</v>
+      </c>
+      <c r="Q55" s="3">
+        <v>5.7706774050752203E-2</v>
+      </c>
+      <c r="R55" s="3">
+        <v>0.17131422624349399</v>
+      </c>
+      <c r="S55" s="3">
+        <v>5.7216426093038501E-2</v>
+      </c>
+      <c r="T55" s="2">
+        <v>78.901515151515099</v>
+      </c>
+      <c r="U55" s="3">
+        <v>0</v>
+      </c>
+      <c r="V55" s="3">
+        <v>0</v>
+      </c>
+      <c r="W55" s="2">
+        <v>100</v>
+      </c>
+      <c r="X55" s="3">
+        <v>3.0723742111518101E-3</v>
+      </c>
+      <c r="Y55" s="3">
+        <v>3.0723742111518101E-3</v>
+      </c>
+      <c r="Z55" s="3">
+        <v>3.5639999999999899E-3</v>
+      </c>
+      <c r="AA55" s="3">
+        <v>0.15509999999999999</v>
+      </c>
+      <c r="AB55" s="2">
+        <v>100</v>
+      </c>
+      <c r="AC55" s="3">
+        <v>11</v>
+      </c>
+      <c r="AD55" s="2">
+        <v>14794.7714566631</v>
+      </c>
+    </row>
+    <row r="56" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="O56" t="s">
+        <v>50</v>
+      </c>
+      <c r="P56" s="3">
+        <v>0.122592693107468</v>
+      </c>
+      <c r="Q56" s="3">
+        <v>4.71632749613572E-2</v>
+      </c>
+      <c r="R56" s="3">
+        <v>0.11577056490922299</v>
+      </c>
+      <c r="S56" s="3">
+        <v>4.05254965779848E-2</v>
+      </c>
+      <c r="T56" s="2">
+        <v>76.931818181818102</v>
+      </c>
+      <c r="U56" s="3">
+        <v>0</v>
+      </c>
+      <c r="V56" s="3">
+        <v>0</v>
+      </c>
+      <c r="W56" s="2">
+        <v>100</v>
+      </c>
+      <c r="X56" s="3">
+        <v>3.0723742111518101E-3</v>
+      </c>
+      <c r="Y56" s="3">
+        <v>3.0723742111518101E-3</v>
+      </c>
+      <c r="Z56" s="3">
+        <v>4.0699999999999903E-3</v>
+      </c>
+      <c r="AA56" s="3">
+        <v>0.23485</v>
+      </c>
+      <c r="AB56" s="2">
+        <v>100</v>
+      </c>
+      <c r="AC56" s="3">
+        <v>11</v>
+      </c>
+      <c r="AD56" s="2">
+        <v>12290.5093045413</v>
+      </c>
+    </row>
+    <row r="57" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="O57" t="s">
+        <v>33</v>
+      </c>
+      <c r="P57" s="3">
+        <v>0.33531475500000002</v>
+      </c>
+      <c r="Q57" s="3">
+        <v>3.8711674000000001E-2</v>
+      </c>
+      <c r="R57" s="3">
+        <v>0.33155639399999998</v>
+      </c>
+      <c r="S57" s="3">
+        <v>3.8257272000000002E-2</v>
+      </c>
+      <c r="T57" s="2">
+        <v>0</v>
+      </c>
+      <c r="U57" s="3">
+        <v>1.167345E-3</v>
+      </c>
+      <c r="V57" s="3">
+        <v>1.167345E-3</v>
+      </c>
+      <c r="W57" s="2">
+        <v>100</v>
+      </c>
+      <c r="X57" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y57" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z57" s="3">
+        <v>5.3039999999999997E-2</v>
+      </c>
+      <c r="AA57" s="3">
+        <v>0.33465600000000001</v>
+      </c>
+      <c r="AB57" s="2">
+        <v>100</v>
+      </c>
+      <c r="AC57" s="3">
+        <v>11</v>
+      </c>
+      <c r="AD57" s="2">
+        <v>4325.1634789999998</v>
+      </c>
+    </row>
+    <row r="58" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="O58" t="s">
+        <v>32</v>
+      </c>
+      <c r="P58" s="3">
+        <v>0.25543057400000002</v>
+      </c>
+      <c r="Q58" s="3">
+        <v>8.7359440999999996E-2</v>
+      </c>
+      <c r="R58" s="3">
+        <v>0.238834243</v>
+      </c>
+      <c r="S58" s="3">
+        <v>7.0005949999999997E-2</v>
+      </c>
+      <c r="T58" s="2">
+        <v>0</v>
+      </c>
+      <c r="U58" s="3">
+        <v>0</v>
+      </c>
+      <c r="V58" s="3">
+        <v>0</v>
+      </c>
+      <c r="W58" s="2">
+        <v>100</v>
+      </c>
+      <c r="X58" s="3">
+        <v>4.4100000000000001E-5</v>
+      </c>
+      <c r="Y58" s="3">
+        <v>4.4100000000000001E-5</v>
+      </c>
+      <c r="Z58" s="3">
+        <v>1.5911999999999999E-2</v>
+      </c>
+      <c r="AA58" s="3">
+        <v>8.7999999999999995E-2</v>
+      </c>
+      <c r="AB58" s="2">
+        <v>100</v>
+      </c>
+      <c r="AC58" s="3">
+        <v>11</v>
+      </c>
+      <c r="AD58" s="2">
+        <v>6936.4021849999999</v>
+      </c>
+    </row>
+    <row r="59" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="O59" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="56" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="O56" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="57" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="O57" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="58" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="O58" t="s">
+      <c r="P59" s="3">
+        <v>7.0549890000000004E-2</v>
+      </c>
+      <c r="Q59" s="3">
+        <v>3.7363296999999997E-2</v>
+      </c>
+      <c r="R59" s="3">
+        <v>6.2647734999999996E-2</v>
+      </c>
+      <c r="S59" s="3">
+        <v>1.7313859999999999E-3</v>
+      </c>
+      <c r="T59" s="2">
+        <v>0</v>
+      </c>
+      <c r="U59" s="3">
+        <v>0</v>
+      </c>
+      <c r="V59" s="3">
+        <v>0</v>
+      </c>
+      <c r="W59" s="2">
+        <v>74.659090910000003</v>
+      </c>
+      <c r="X59" s="3">
+        <v>1.7400000000000001E-6</v>
+      </c>
+      <c r="Y59" s="3">
+        <v>1.7400000000000001E-6</v>
+      </c>
+      <c r="Z59" s="3">
+        <v>1.5911999999999999E-2</v>
+      </c>
+      <c r="AA59" s="3">
+        <v>2.7291240000000001</v>
+      </c>
+      <c r="AB59" s="2">
+        <v>100</v>
+      </c>
+      <c r="AC59" s="3">
+        <v>11</v>
+      </c>
+      <c r="AD59" s="2">
+        <v>4758.0608389999998</v>
+      </c>
+    </row>
+    <row r="60" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="O60" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="59" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="O59" t="s">
+    <row r="61" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="O61" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="60" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="O60" t="s">
+      <c r="P61" s="3">
+        <v>4.2555557000000001E-2</v>
+      </c>
+      <c r="Q61" s="3">
+        <v>4.7794402E-2</v>
+      </c>
+      <c r="R61" s="3">
+        <v>3.3294799999999999E-2</v>
+      </c>
+      <c r="S61" s="3">
+        <v>2.2750368999999999E-2</v>
+      </c>
+      <c r="T61" s="2">
+        <v>0</v>
+      </c>
+      <c r="U61" s="3">
+        <v>0</v>
+      </c>
+      <c r="V61" s="3">
+        <v>0</v>
+      </c>
+      <c r="W61" s="2">
+        <v>0</v>
+      </c>
+      <c r="X61" s="3">
+        <v>3.3335779999999998E-3</v>
+      </c>
+      <c r="Y61" s="3">
+        <v>3.3335779999999998E-3</v>
+      </c>
+      <c r="Z61" s="3">
+        <v>1.5911999999999999E-2</v>
+      </c>
+      <c r="AA61" s="3">
+        <v>3.8163360000000002</v>
+      </c>
+      <c r="AB61" s="2">
+        <v>54.204545449999998</v>
+      </c>
+      <c r="AC61" s="3">
+        <v>5.9625000000000004</v>
+      </c>
+      <c r="AD61" s="2">
+        <v>5178.2805109999999</v>
+      </c>
+    </row>
+    <row r="62" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="O62" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="61" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="O61" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="63" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="64" spans="1:15" x14ac:dyDescent="0.3">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="64" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A64" s="19" t="s">
         <v>0</v>
       </c>
       <c r="B64" s="34" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C64" s="35"/>
       <c r="D64" s="36"/>
       <c r="E64" s="37" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F64" s="35"/>
       <c r="G64" s="36"/>
       <c r="H64" s="37" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I64" s="35"/>
       <c r="J64" s="38"/>
       <c r="K64" s="34" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L64" s="35"/>
       <c r="M64" s="35"/>
       <c r="N64" s="21"/>
       <c r="O64" s="21"/>
     </row>
-    <row r="65" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A65" s="22" t="s">
         <v>1</v>
       </c>
@@ -8215,7 +9101,7 @@
       <c r="N65" s="21"/>
       <c r="O65" s="21"/>
     </row>
-    <row r="66" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A66" s="22" t="s">
         <v>2</v>
       </c>
@@ -8258,7 +9144,7 @@
       <c r="N66" s="21"/>
       <c r="O66" s="21"/>
     </row>
-    <row r="67" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A67" s="19" t="s">
         <v>3</v>
       </c>
@@ -8301,7 +9187,7 @@
       <c r="N67" s="21"/>
       <c r="O67" s="21"/>
     </row>
-    <row r="68" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A68" s="22" t="s">
         <v>4</v>
       </c>
@@ -8344,7 +9230,7 @@
       <c r="N68" s="21"/>
       <c r="O68" s="21"/>
     </row>
-    <row r="69" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A69" s="19" t="s">
         <v>7</v>
       </c>
@@ -8387,7 +9273,7 @@
       <c r="N69" s="21"/>
       <c r="O69" s="21"/>
     </row>
-    <row r="70" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A70" s="22" t="s">
         <v>5</v>
       </c>
@@ -8406,7 +9292,7 @@
       <c r="N70" s="21"/>
       <c r="O70" s="21"/>
     </row>
-    <row r="71" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A71" s="22" t="s">
         <v>17</v>
       </c>
@@ -8449,7 +9335,7 @@
       <c r="N71" s="21"/>
       <c r="O71" s="21"/>
     </row>
-    <row r="72" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A72" s="20" t="s">
         <v>6</v>
       </c>
@@ -8492,7 +9378,7 @@
       <c r="N72" s="21"/>
       <c r="O72" s="21"/>
     </row>
-    <row r="73" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A73" s="21"/>
       <c r="B73" s="21"/>
       <c r="C73" s="21"/>
@@ -8509,7 +9395,7 @@
       <c r="N73" s="21"/>
       <c r="O73" s="21"/>
     </row>
-    <row r="74" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A74" s="21"/>
       <c r="B74" s="21"/>
       <c r="C74" s="21"/>
@@ -8524,11 +9410,11 @@
       <c r="L74" s="21"/>
       <c r="M74" s="21"/>
       <c r="N74" s="21"/>
-      <c r="O74" s="21" t="s">
+      <c r="O74" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="75" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A75" s="21"/>
       <c r="B75" s="21"/>
       <c r="C75" s="21"/>
@@ -8543,11 +9429,56 @@
       <c r="L75" s="21"/>
       <c r="M75" s="21"/>
       <c r="N75" s="21"/>
-      <c r="O75" s="21" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="76" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="O75" t="s">
+        <v>49</v>
+      </c>
+      <c r="P75" s="3">
+        <v>0.36265725399999998</v>
+      </c>
+      <c r="Q75" s="3">
+        <v>3.7780846E-2</v>
+      </c>
+      <c r="R75" s="3">
+        <v>0.35737406100000002</v>
+      </c>
+      <c r="S75" s="3">
+        <v>3.1152862E-2</v>
+      </c>
+      <c r="T75" s="2">
+        <v>0</v>
+      </c>
+      <c r="U75" s="3">
+        <v>2.7615159999999999E-3</v>
+      </c>
+      <c r="V75" s="3">
+        <v>2.7615159999999999E-3</v>
+      </c>
+      <c r="W75" s="2">
+        <v>28.06818182</v>
+      </c>
+      <c r="X75" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y75" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z75" s="3">
+        <v>0.2112</v>
+      </c>
+      <c r="AA75" s="3">
+        <v>0.59519999999999995</v>
+      </c>
+      <c r="AB75" s="2">
+        <v>100</v>
+      </c>
+      <c r="AC75" s="3">
+        <v>11</v>
+      </c>
+      <c r="AD75" s="2">
+        <v>4485.8906280000001</v>
+      </c>
+    </row>
+    <row r="76" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A76" s="21"/>
       <c r="B76" s="21"/>
       <c r="C76" s="21"/>
@@ -8562,11 +9493,56 @@
       <c r="L76" s="21"/>
       <c r="M76" s="21"/>
       <c r="N76" s="21"/>
-      <c r="O76" s="21" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="77" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="O76" t="s">
+        <v>50</v>
+      </c>
+      <c r="P76" s="3">
+        <v>0.348315708</v>
+      </c>
+      <c r="Q76" s="3">
+        <v>3.9609232000000001E-2</v>
+      </c>
+      <c r="R76" s="3">
+        <v>0.34317238700000002</v>
+      </c>
+      <c r="S76" s="3">
+        <v>3.2814257999999999E-2</v>
+      </c>
+      <c r="T76" s="2">
+        <v>0</v>
+      </c>
+      <c r="U76" s="3">
+        <v>2.7615159999999999E-3</v>
+      </c>
+      <c r="V76" s="3">
+        <v>2.7615159999999999E-3</v>
+      </c>
+      <c r="W76" s="2">
+        <v>54.166666669999998</v>
+      </c>
+      <c r="X76" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y76" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z76" s="3">
+        <v>0.2112</v>
+      </c>
+      <c r="AA76" s="3">
+        <v>0.58726400000000001</v>
+      </c>
+      <c r="AB76" s="2">
+        <v>100</v>
+      </c>
+      <c r="AC76" s="3">
+        <v>11</v>
+      </c>
+      <c r="AD76" s="2">
+        <v>4443.0176229999997</v>
+      </c>
+    </row>
+    <row r="77" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A77" s="21"/>
       <c r="B77" s="21"/>
       <c r="C77" s="21"/>
@@ -8581,11 +9557,56 @@
       <c r="L77" s="21"/>
       <c r="M77" s="21"/>
       <c r="N77" s="21"/>
-      <c r="O77" s="21" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="78" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="O77" t="s">
+        <v>33</v>
+      </c>
+      <c r="P77" s="3">
+        <v>0.218810434</v>
+      </c>
+      <c r="Q77" s="3">
+        <v>5.5642596000000002E-2</v>
+      </c>
+      <c r="R77" s="3">
+        <v>0.20642369299999999</v>
+      </c>
+      <c r="S77" s="3">
+        <v>3.0677823E-2</v>
+      </c>
+      <c r="T77" s="2">
+        <v>0</v>
+      </c>
+      <c r="U77" s="3">
+        <v>1.4408050000000001E-3</v>
+      </c>
+      <c r="V77" s="3">
+        <v>1.4408050000000001E-3</v>
+      </c>
+      <c r="W77" s="2">
+        <v>40.151515150000002</v>
+      </c>
+      <c r="X77" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y77" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z77" s="3">
+        <v>1.6</v>
+      </c>
+      <c r="AA77" s="3">
+        <v>4.7320000000000002</v>
+      </c>
+      <c r="AB77" s="2">
+        <v>100</v>
+      </c>
+      <c r="AC77" s="3">
+        <v>11</v>
+      </c>
+      <c r="AD77" s="2">
+        <v>7135.7513470000004</v>
+      </c>
+    </row>
+    <row r="78" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A78" s="21"/>
       <c r="B78" s="21"/>
       <c r="C78" s="21"/>
@@ -8600,11 +9621,56 @@
       <c r="L78" s="21"/>
       <c r="M78" s="21"/>
       <c r="N78" s="21"/>
-      <c r="O78" s="21" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="79" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="O78" t="s">
+        <v>32</v>
+      </c>
+      <c r="P78" s="3">
+        <v>2.5382371000000001E-2</v>
+      </c>
+      <c r="Q78" s="3">
+        <v>7.4474062999999993E-2</v>
+      </c>
+      <c r="R78" s="3">
+        <v>7.1542890000000003E-3</v>
+      </c>
+      <c r="S78" s="3">
+        <v>4.9539229999999998E-3</v>
+      </c>
+      <c r="T78" s="2">
+        <v>0</v>
+      </c>
+      <c r="U78" s="3">
+        <v>3.3335779999999998E-3</v>
+      </c>
+      <c r="V78" s="3">
+        <v>3.3335779999999998E-3</v>
+      </c>
+      <c r="W78" s="2">
+        <v>8.5227272729999992</v>
+      </c>
+      <c r="X78" s="3">
+        <v>3.3335779999999998E-3</v>
+      </c>
+      <c r="Y78" s="3">
+        <v>3.3335779999999998E-3</v>
+      </c>
+      <c r="Z78" s="3">
+        <v>0.29520000000000002</v>
+      </c>
+      <c r="AA78" s="3">
+        <v>1.5960000000000001</v>
+      </c>
+      <c r="AB78" s="2">
+        <v>41.477272730000003</v>
+      </c>
+      <c r="AC78" s="3">
+        <v>4.5625</v>
+      </c>
+      <c r="AD78" s="2">
+        <v>16165.30091</v>
+      </c>
+    </row>
+    <row r="79" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A79" s="21"/>
       <c r="B79" s="21"/>
       <c r="C79" s="21"/>
@@ -8619,11 +9685,56 @@
       <c r="L79" s="21"/>
       <c r="M79" s="21"/>
       <c r="N79" s="21"/>
-      <c r="O79" s="21" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="80" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="O79" t="s">
+        <v>34</v>
+      </c>
+      <c r="P79" s="3">
+        <v>2.5382371000000001E-2</v>
+      </c>
+      <c r="Q79" s="3">
+        <v>7.4474062999999993E-2</v>
+      </c>
+      <c r="R79" s="3">
+        <v>7.1542890000000003E-3</v>
+      </c>
+      <c r="S79" s="3">
+        <v>4.9539229999999998E-3</v>
+      </c>
+      <c r="T79" s="2">
+        <v>0</v>
+      </c>
+      <c r="U79" s="3">
+        <v>3.3335779999999998E-3</v>
+      </c>
+      <c r="V79" s="3">
+        <v>3.3335779999999998E-3</v>
+      </c>
+      <c r="W79" s="2">
+        <v>8.5227272729999992</v>
+      </c>
+      <c r="X79" s="3">
+        <v>3.3335779999999998E-3</v>
+      </c>
+      <c r="Y79" s="3">
+        <v>3.3335779999999998E-3</v>
+      </c>
+      <c r="Z79" s="3">
+        <v>0.29520000000000002</v>
+      </c>
+      <c r="AA79" s="3">
+        <v>1.5960000000000001</v>
+      </c>
+      <c r="AB79" s="2">
+        <v>41.477272730000003</v>
+      </c>
+      <c r="AC79" s="3">
+        <v>4.5625</v>
+      </c>
+      <c r="AD79" s="2">
+        <v>16165.30091</v>
+      </c>
+    </row>
+    <row r="80" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A80" s="21"/>
       <c r="B80" s="21"/>
       <c r="C80" s="21"/>
@@ -8638,11 +9749,11 @@
       <c r="L80" s="21"/>
       <c r="M80" s="21"/>
       <c r="N80" s="21"/>
-      <c r="O80" s="21" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="81" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="O80" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="81" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A81" s="21"/>
       <c r="B81" s="21"/>
       <c r="C81" s="21"/>
@@ -8657,8 +9768,103 @@
       <c r="L81" s="21"/>
       <c r="M81" s="21"/>
       <c r="N81" s="21"/>
-      <c r="O81" s="21" t="s">
-        <v>38</v>
+      <c r="O81" t="s">
+        <v>36</v>
+      </c>
+      <c r="P81" s="3">
+        <v>2.5382371000000001E-2</v>
+      </c>
+      <c r="Q81" s="3">
+        <v>7.4474062999999993E-2</v>
+      </c>
+      <c r="R81" s="3">
+        <v>7.1542890000000003E-3</v>
+      </c>
+      <c r="S81" s="3">
+        <v>4.9539229999999998E-3</v>
+      </c>
+      <c r="T81" s="2">
+        <v>0</v>
+      </c>
+      <c r="U81" s="3">
+        <v>3.3335779999999998E-3</v>
+      </c>
+      <c r="V81" s="3">
+        <v>3.3335779999999998E-3</v>
+      </c>
+      <c r="W81" s="2">
+        <v>8.5227272729999992</v>
+      </c>
+      <c r="X81" s="3">
+        <v>3.3335779999999998E-3</v>
+      </c>
+      <c r="Y81" s="3">
+        <v>3.3335779999999998E-3</v>
+      </c>
+      <c r="Z81" s="3">
+        <v>0.29520000000000002</v>
+      </c>
+      <c r="AA81" s="3">
+        <v>1.5960000000000001</v>
+      </c>
+      <c r="AB81" s="2">
+        <v>41.477272730000003</v>
+      </c>
+      <c r="AC81" s="3">
+        <v>4.5625</v>
+      </c>
+      <c r="AD81" s="2">
+        <v>16165.30091</v>
+      </c>
+    </row>
+    <row r="82" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="O82" t="s">
+        <v>37</v>
+      </c>
+      <c r="P82" s="3">
+        <v>2.5382371000000001E-2</v>
+      </c>
+      <c r="Q82" s="3">
+        <v>7.4474062999999993E-2</v>
+      </c>
+      <c r="R82" s="3">
+        <v>7.1542890000000003E-3</v>
+      </c>
+      <c r="S82" s="3">
+        <v>4.9539229999999998E-3</v>
+      </c>
+      <c r="T82" s="2">
+        <v>0</v>
+      </c>
+      <c r="U82" s="3">
+        <v>3.3335779999999998E-3</v>
+      </c>
+      <c r="V82" s="3">
+        <v>3.3335779999999998E-3</v>
+      </c>
+      <c r="W82" s="2">
+        <v>8.5227272729999992</v>
+      </c>
+      <c r="X82" s="3">
+        <v>3.3335779999999998E-3</v>
+      </c>
+      <c r="Y82" s="3">
+        <v>3.3335779999999998E-3</v>
+      </c>
+      <c r="Z82" s="3">
+        <v>0.29520000000000002</v>
+      </c>
+      <c r="AA82" s="3">
+        <v>1.5960000000000001</v>
+      </c>
+      <c r="AB82" s="2">
+        <v>41.477272730000003</v>
+      </c>
+      <c r="AC82" s="3">
+        <v>4.5625</v>
+      </c>
+      <c r="AD82" s="2">
+        <v>16165.30091</v>
       </c>
     </row>
   </sheetData>
@@ -8686,15 +9892,23 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB1CCC97-D0A7-4837-9497-07689BD5D6D2}">
-  <dimension ref="A1:AD82"/>
+  <dimension ref="A1:AD83"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.77734375" customWidth="1"/>
+    <col min="16" max="19" width="8.88671875" style="42"/>
+    <col min="20" max="20" width="8.88671875" style="39"/>
+    <col min="21" max="22" width="8.88671875" style="42"/>
+    <col min="23" max="23" width="8.88671875" style="39"/>
+    <col min="24" max="27" width="8.88671875" style="42"/>
+    <col min="28" max="28" width="8.88671875" style="39"/>
+    <col min="29" max="29" width="8.88671875" style="41"/>
+    <col min="30" max="30" width="11.33203125" style="39" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:30" x14ac:dyDescent="0.3">
@@ -8702,22 +9916,22 @@
         <v>0</v>
       </c>
       <c r="B2" s="31" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C2" s="32"/>
       <c r="D2" s="33"/>
       <c r="E2" s="32" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F2" s="32"/>
       <c r="G2" s="33"/>
       <c r="H2" s="32" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I2" s="32"/>
       <c r="J2" s="32"/>
       <c r="K2" s="31" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L2" s="32"/>
       <c r="M2" s="32"/>
@@ -9018,7 +10232,7 @@
       <c r="T11" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="U11" s="4" t="s">
+      <c r="U11" s="3" t="s">
         <v>23</v>
       </c>
       <c r="V11" s="3" t="s">
@@ -9042,7 +10256,7 @@
       <c r="AB11" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="AC11" s="3" t="s">
+      <c r="AC11" s="40" t="s">
         <v>31</v>
       </c>
       <c r="AD11" s="2" t="s">
@@ -9056,70 +10270,345 @@
     </row>
     <row r="13" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O13" t="s">
-        <v>34</v>
+        <v>49</v>
+      </c>
+      <c r="P13" s="42">
+        <v>2.0422105999999999E-2</v>
+      </c>
+      <c r="Q13" s="42">
+        <v>6.6577413000000002E-2</v>
+      </c>
+      <c r="R13" s="42">
+        <v>4.2976079999999996E-3</v>
+      </c>
+      <c r="S13" s="42">
+        <v>3.4186780000000001E-3</v>
+      </c>
+      <c r="T13" s="39">
+        <v>0</v>
+      </c>
+      <c r="U13" s="42">
+        <v>0</v>
+      </c>
+      <c r="V13" s="42">
+        <v>0</v>
+      </c>
+      <c r="W13" s="39">
+        <v>0</v>
+      </c>
+      <c r="X13" s="42">
+        <v>1.4738187E-2</v>
+      </c>
+      <c r="Y13" s="42">
+        <v>1.4738187E-2</v>
+      </c>
+      <c r="Z13" s="42">
+        <v>0</v>
+      </c>
+      <c r="AA13" s="42">
+        <v>3.8163360000000002</v>
+      </c>
+      <c r="AB13" s="39">
+        <v>99.962121210000006</v>
+      </c>
+      <c r="AC13" s="41">
+        <v>10.99583333</v>
+      </c>
+      <c r="AD13" s="39">
+        <v>16783.498909999998</v>
       </c>
     </row>
     <row r="14" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O14" t="s">
-        <v>33</v>
+        <v>50</v>
+      </c>
+      <c r="P14" s="42">
+        <v>2.0422105999999999E-2</v>
+      </c>
+      <c r="Q14" s="42">
+        <v>6.6577413000000002E-2</v>
+      </c>
+      <c r="R14" s="42">
+        <v>4.2976079999999996E-3</v>
+      </c>
+      <c r="S14" s="42">
+        <v>3.4186780000000001E-3</v>
+      </c>
+      <c r="T14" s="39">
+        <v>0</v>
+      </c>
+      <c r="U14" s="42">
+        <v>0</v>
+      </c>
+      <c r="V14" s="42">
+        <v>0</v>
+      </c>
+      <c r="W14" s="39">
+        <v>0</v>
+      </c>
+      <c r="X14" s="42">
+        <v>1.4738187E-2</v>
+      </c>
+      <c r="Y14" s="42">
+        <v>1.4738187E-2</v>
+      </c>
+      <c r="Z14" s="42">
+        <v>0</v>
+      </c>
+      <c r="AA14" s="42">
+        <v>3.8163360000000002</v>
+      </c>
+      <c r="AB14" s="39">
+        <v>99.962121210000006</v>
+      </c>
+      <c r="AC14" s="41">
+        <v>10.99583333</v>
+      </c>
+      <c r="AD14" s="39">
+        <v>16783.498909999998</v>
       </c>
     </row>
     <row r="15" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O15" t="s">
-        <v>32</v>
+        <v>33</v>
+      </c>
+      <c r="P15" s="42">
+        <v>2.2174191999999999E-2</v>
+      </c>
+      <c r="Q15" s="42">
+        <v>6.8021499999999999E-2</v>
+      </c>
+      <c r="R15" s="42">
+        <v>5.6011979999999999E-3</v>
+      </c>
+      <c r="S15" s="42">
+        <v>3.7126630000000002E-3</v>
+      </c>
+      <c r="T15" s="39">
+        <v>0</v>
+      </c>
+      <c r="U15" s="42">
+        <v>1.5541200000000001E-4</v>
+      </c>
+      <c r="V15" s="42">
+        <v>1.5541200000000001E-4</v>
+      </c>
+      <c r="W15" s="39">
+        <v>0</v>
+      </c>
+      <c r="X15" s="42">
+        <v>1.4027168E-2</v>
+      </c>
+      <c r="Y15" s="42">
+        <v>1.4027168E-2</v>
+      </c>
+      <c r="Z15" s="42">
+        <v>5.1679999999999997E-2</v>
+      </c>
+      <c r="AA15" s="42">
+        <v>3.3281999999999998</v>
+      </c>
+      <c r="AB15" s="39">
+        <v>0.15151515199999999</v>
+      </c>
+      <c r="AC15" s="41">
+        <v>1.6666667E-2</v>
+      </c>
+      <c r="AD15" s="39">
+        <v>16726.551950000001</v>
       </c>
     </row>
     <row r="16" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O16" t="s">
+        <v>32</v>
+      </c>
+      <c r="P16" s="42">
+        <v>0.47406991900000001</v>
+      </c>
+      <c r="Q16" s="42">
+        <v>7.1940545999999994E-2</v>
+      </c>
+      <c r="R16" s="42">
+        <v>0.47826287499999998</v>
+      </c>
+      <c r="S16" s="42">
+        <v>7.3811294999999999E-2</v>
+      </c>
+      <c r="T16" s="39">
+        <v>0</v>
+      </c>
+      <c r="U16" s="42">
+        <v>2.148166E-3</v>
+      </c>
+      <c r="V16" s="42">
+        <v>2.148166E-3</v>
+      </c>
+      <c r="W16" s="39">
+        <v>100</v>
+      </c>
+      <c r="X16" s="42">
+        <v>2.9114729999999999E-3</v>
+      </c>
+      <c r="Y16" s="42">
+        <v>2.9114729999999999E-3</v>
+      </c>
+      <c r="Z16" s="42">
+        <v>0.16416</v>
+      </c>
+      <c r="AA16" s="42">
+        <v>0.27753</v>
+      </c>
+      <c r="AB16" s="39">
+        <v>100</v>
+      </c>
+      <c r="AC16" s="41">
+        <v>11</v>
+      </c>
+      <c r="AD16" s="39">
+        <v>14903.962009999999</v>
+      </c>
+    </row>
+    <row r="17" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="O17" t="s">
+        <v>34</v>
+      </c>
+      <c r="P17" s="42">
+        <v>0.38654200399999999</v>
+      </c>
+      <c r="Q17" s="42">
+        <v>7.5658416000000006E-2</v>
+      </c>
+      <c r="R17" s="42">
+        <v>0.38150645599999999</v>
+      </c>
+      <c r="S17" s="42">
+        <v>7.7287566000000002E-2</v>
+      </c>
+      <c r="T17" s="39">
+        <v>0</v>
+      </c>
+      <c r="U17" s="42">
+        <v>2.148166E-3</v>
+      </c>
+      <c r="V17" s="42">
+        <v>2.148166E-3</v>
+      </c>
+      <c r="W17" s="39">
+        <v>100</v>
+      </c>
+      <c r="X17" s="42">
+        <v>2.9719070000000002E-3</v>
+      </c>
+      <c r="Y17" s="42">
+        <v>2.9719070000000002E-3</v>
+      </c>
+      <c r="Z17" s="42">
+        <v>0.16416</v>
+      </c>
+      <c r="AA17" s="42">
+        <v>0.441</v>
+      </c>
+      <c r="AB17" s="39">
+        <v>100</v>
+      </c>
+      <c r="AC17" s="41">
+        <v>11</v>
+      </c>
+      <c r="AD17" s="39">
+        <v>12736.34367</v>
+      </c>
+    </row>
+    <row r="18" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="O18" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="O17" t="s">
+    <row r="19" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="O19" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="O18" t="s">
+      <c r="P19" s="42">
+        <v>0.47509609200000003</v>
+      </c>
+      <c r="Q19" s="42">
+        <v>7.3223063000000005E-2</v>
+      </c>
+      <c r="R19" s="42">
+        <v>0.47984376499999998</v>
+      </c>
+      <c r="S19" s="42">
+        <v>7.4750901999999994E-2</v>
+      </c>
+      <c r="T19" s="39">
+        <v>0</v>
+      </c>
+      <c r="U19" s="42">
+        <v>2.148166E-3</v>
+      </c>
+      <c r="V19" s="42">
+        <v>2.148166E-3</v>
+      </c>
+      <c r="W19" s="39">
+        <v>100</v>
+      </c>
+      <c r="X19" s="42">
+        <v>3.1957259999999999E-3</v>
+      </c>
+      <c r="Y19" s="42">
+        <v>3.1957259999999999E-3</v>
+      </c>
+      <c r="Z19" s="42">
+        <v>0.16416</v>
+      </c>
+      <c r="AA19" s="42">
+        <v>0.34223999999999999</v>
+      </c>
+      <c r="AB19" s="39">
+        <v>100</v>
+      </c>
+      <c r="AC19" s="41">
+        <v>11</v>
+      </c>
+      <c r="AD19" s="39">
+        <v>16872.860240000002</v>
+      </c>
+    </row>
+    <row r="20" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="O20" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="O19" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.3">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="23" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A23" s="5" t="s">
         <v>0</v>
       </c>
       <c r="B23" s="31" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C23" s="32"/>
       <c r="D23" s="33"/>
       <c r="E23" s="32" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F23" s="32"/>
       <c r="G23" s="33"/>
       <c r="H23" s="32" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I23" s="32"/>
       <c r="J23" s="32"/>
       <c r="K23" s="31" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L23" s="32"/>
       <c r="M23" s="32"/>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A24" s="14" t="s">
         <v>1</v>
       </c>
@@ -9160,7 +10649,7 @@
         <v>0.89999997615814198</v>
       </c>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A25" s="12" t="s">
         <v>2</v>
       </c>
@@ -9201,7 +10690,7 @@
         <v>1.83500003814697</v>
       </c>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A26" s="5" t="s">
         <v>3</v>
       </c>
@@ -9242,7 +10731,7 @@
         <v>1.0740000009536701</v>
       </c>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A27" s="14" t="s">
         <v>4</v>
       </c>
@@ -9283,7 +10772,7 @@
         <v>0.60000002384185702</v>
       </c>
     </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A28" s="5" t="s">
         <v>7</v>
       </c>
@@ -9324,7 +10813,7 @@
         <v>0.44900000095367398</v>
       </c>
     </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A29" s="12" t="s">
         <v>5</v>
       </c>
@@ -9341,7 +10830,7 @@
       <c r="L29" s="2"/>
       <c r="M29" s="2"/>
     </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A30" s="12" t="s">
         <v>17</v>
       </c>
@@ -9382,7 +10871,7 @@
         <v>0.60000002384185702</v>
       </c>
     </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A31" s="13" t="s">
         <v>6</v>
       </c>
@@ -9399,77 +10888,352 @@
       <c r="L31" s="10"/>
       <c r="M31" s="10"/>
     </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O33" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O34" t="s">
+        <v>49</v>
+      </c>
+      <c r="P34" s="42">
+        <v>0.49276842999999998</v>
+      </c>
+      <c r="Q34" s="42">
+        <v>7.2156964000000004E-2</v>
+      </c>
+      <c r="R34" s="42">
+        <v>0.49537018199999999</v>
+      </c>
+      <c r="S34" s="42">
+        <v>7.5086813000000002E-2</v>
+      </c>
+      <c r="T34" s="39">
+        <v>100</v>
+      </c>
+      <c r="U34" s="42">
+        <v>0</v>
+      </c>
+      <c r="V34" s="42">
+        <v>0</v>
+      </c>
+      <c r="W34" s="39">
+        <v>100</v>
+      </c>
+      <c r="X34" s="42">
+        <v>2.644927E-3</v>
+      </c>
+      <c r="Y34" s="42">
+        <v>2.644927E-3</v>
+      </c>
+      <c r="Z34" s="42">
+        <v>2.8800000000000002E-3</v>
+      </c>
+      <c r="AA34" s="42">
+        <v>0.192</v>
+      </c>
+      <c r="AB34" s="39">
+        <v>100</v>
+      </c>
+      <c r="AC34" s="41">
+        <v>11</v>
+      </c>
+      <c r="AD34" s="39">
+        <v>10854.593210000001</v>
+      </c>
+    </row>
+    <row r="35" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="O35" t="s">
+        <v>50</v>
+      </c>
+      <c r="P35" s="42">
+        <v>0.27102898600000003</v>
+      </c>
+      <c r="Q35" s="42">
+        <v>4.4745095999999998E-2</v>
+      </c>
+      <c r="R35" s="42">
+        <v>0.27289521300000003</v>
+      </c>
+      <c r="S35" s="42">
+        <v>3.7710198E-2</v>
+      </c>
+      <c r="T35" s="39">
+        <v>89.886363639999999</v>
+      </c>
+      <c r="U35" s="42">
+        <v>0</v>
+      </c>
+      <c r="V35" s="42">
+        <v>0</v>
+      </c>
+      <c r="W35" s="39">
+        <v>100</v>
+      </c>
+      <c r="X35" s="42">
+        <v>0</v>
+      </c>
+      <c r="Y35" s="42">
+        <v>0</v>
+      </c>
+      <c r="Z35" s="42">
+        <v>0</v>
+      </c>
+      <c r="AA35" s="42">
+        <v>0.93202499999999999</v>
+      </c>
+      <c r="AB35" s="39">
+        <v>100</v>
+      </c>
+      <c r="AC35" s="41">
+        <v>11</v>
+      </c>
+      <c r="AD35" s="39">
+        <v>24341.61377</v>
+      </c>
+    </row>
+    <row r="36" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="O36" t="s">
+        <v>33</v>
+      </c>
+      <c r="P36" s="42">
+        <v>0.16763552700000001</v>
+      </c>
+      <c r="Q36" s="42">
+        <v>7.8511710999999998E-2</v>
+      </c>
+      <c r="R36" s="42">
+        <v>0.16305029500000001</v>
+      </c>
+      <c r="S36" s="42">
+        <v>7.1120540999999995E-2</v>
+      </c>
+      <c r="T36" s="39">
+        <v>96.590909089999997</v>
+      </c>
+      <c r="U36" s="42">
+        <v>0</v>
+      </c>
+      <c r="V36" s="42">
+        <v>0</v>
+      </c>
+      <c r="W36" s="39">
+        <v>0</v>
+      </c>
+      <c r="X36" s="42">
+        <v>1.4738187E-2</v>
+      </c>
+      <c r="Y36" s="42">
+        <v>1.4738187E-2</v>
+      </c>
+      <c r="Z36" s="42">
+        <v>3.6259999999999999E-3</v>
+      </c>
+      <c r="AA36" s="42">
+        <v>3.8163360000000002</v>
+      </c>
+      <c r="AB36" s="39">
+        <v>92.613636360000001</v>
+      </c>
+      <c r="AC36" s="41">
+        <v>10.1875</v>
+      </c>
+      <c r="AD36" s="39">
+        <v>5104.3859670000002</v>
+      </c>
+    </row>
+    <row r="37" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="O37" t="s">
+        <v>32</v>
+      </c>
+      <c r="P37" s="42">
+        <v>6.9194680999999994E-2</v>
+      </c>
+      <c r="Q37" s="42">
+        <v>6.8214596000000002E-2</v>
+      </c>
+      <c r="R37" s="42">
+        <v>5.8914656000000003E-2</v>
+      </c>
+      <c r="S37" s="42">
+        <v>3.5449247000000003E-2</v>
+      </c>
+      <c r="T37" s="39">
+        <v>0</v>
+      </c>
+      <c r="U37" s="42">
+        <v>0</v>
+      </c>
+      <c r="V37" s="42">
+        <v>0</v>
+      </c>
+      <c r="W37" s="39">
+        <v>100</v>
+      </c>
+      <c r="X37" s="42">
+        <v>2.644927E-3</v>
+      </c>
+      <c r="Y37" s="42">
+        <v>2.644927E-3</v>
+      </c>
+      <c r="Z37" s="42">
+        <v>1.1039999999999999E-2</v>
+      </c>
+      <c r="AA37" s="42">
+        <v>0.378</v>
+      </c>
+      <c r="AB37" s="39">
+        <v>100</v>
+      </c>
+      <c r="AC37" s="41">
+        <v>11</v>
+      </c>
+      <c r="AD37" s="39">
+        <v>24308.732680000001</v>
+      </c>
+    </row>
+    <row r="38" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="O38" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="O35" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="O36" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="O37" t="s">
+      <c r="P38" s="42">
+        <v>0.55872443800000005</v>
+      </c>
+      <c r="Q38" s="42">
+        <v>7.0912995000000006E-2</v>
+      </c>
+      <c r="R38" s="42">
+        <v>0.56479812600000001</v>
+      </c>
+      <c r="S38" s="42">
+        <v>7.1431786999999997E-2</v>
+      </c>
+      <c r="T38" s="39">
+        <v>0</v>
+      </c>
+      <c r="U38" s="42">
+        <v>0</v>
+      </c>
+      <c r="V38" s="42">
+        <v>0</v>
+      </c>
+      <c r="W38" s="39">
+        <v>100</v>
+      </c>
+      <c r="X38" s="42">
+        <v>1.2383979999999999E-3</v>
+      </c>
+      <c r="Y38" s="42">
+        <v>1.2383979999999999E-3</v>
+      </c>
+      <c r="Z38" s="42">
+        <v>1.1039999999999999E-2</v>
+      </c>
+      <c r="AA38" s="42">
+        <v>0.13202</v>
+      </c>
+      <c r="AB38" s="39">
+        <v>100</v>
+      </c>
+      <c r="AC38" s="41">
+        <v>11</v>
+      </c>
+      <c r="AD38" s="39">
+        <v>8681.5015750000002</v>
+      </c>
+    </row>
+    <row r="39" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="O39" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="O38" t="s">
+    <row r="40" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="O40" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="O39" t="s">
+      <c r="P40" s="42">
+        <v>6.9194711000000006E-2</v>
+      </c>
+      <c r="Q40" s="42">
+        <v>6.8214580999999996E-2</v>
+      </c>
+      <c r="R40" s="42">
+        <v>5.8914682000000003E-2</v>
+      </c>
+      <c r="S40" s="42">
+        <v>3.5449245999999997E-2</v>
+      </c>
+      <c r="T40" s="39">
+        <v>0</v>
+      </c>
+      <c r="U40" s="42">
+        <v>0</v>
+      </c>
+      <c r="V40" s="42">
+        <v>0</v>
+      </c>
+      <c r="W40" s="39">
+        <v>100</v>
+      </c>
+      <c r="X40" s="42">
+        <v>2.644927E-3</v>
+      </c>
+      <c r="Y40" s="42">
+        <v>2.644927E-3</v>
+      </c>
+      <c r="Z40" s="42">
+        <v>1.1039999999999999E-2</v>
+      </c>
+      <c r="AA40" s="42">
+        <v>0.35099999999999998</v>
+      </c>
+      <c r="AB40" s="39">
+        <v>100</v>
+      </c>
+      <c r="AC40" s="41">
+        <v>11</v>
+      </c>
+      <c r="AD40" s="39">
+        <v>24308.737099999998</v>
+      </c>
+    </row>
+    <row r="41" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="O41" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="O40" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.3">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="44" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A44" s="5" t="s">
         <v>0</v>
       </c>
       <c r="B44" s="31" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C44" s="32"/>
       <c r="D44" s="33"/>
       <c r="E44" s="32" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F44" s="32"/>
       <c r="G44" s="33"/>
       <c r="H44" s="32" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I44" s="32"/>
       <c r="J44" s="32"/>
       <c r="K44" s="31" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L44" s="32"/>
       <c r="M44" s="32"/>
     </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A45" s="14" t="s">
         <v>1</v>
       </c>
@@ -9510,7 +11274,7 @@
         <v>0.57999998331069902</v>
       </c>
     </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A46" s="12" t="s">
         <v>2</v>
       </c>
@@ -9551,7 +11315,7 @@
         <v>0.46000000834464999</v>
       </c>
     </row>
-    <row r="47" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A47" s="5" t="s">
         <v>3</v>
       </c>
@@ -9592,7 +11356,7 @@
         <v>0.44999998807907099</v>
       </c>
     </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A48" s="14" t="s">
         <v>4</v>
       </c>
@@ -9633,7 +11397,7 @@
         <v>0.46000000834464999</v>
       </c>
     </row>
-    <row r="49" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A49" s="5" t="s">
         <v>7</v>
       </c>
@@ -9674,7 +11438,7 @@
         <v>1.1900000572204501</v>
       </c>
     </row>
-    <row r="50" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A50" s="12" t="s">
         <v>5</v>
       </c>
@@ -9691,7 +11455,7 @@
       <c r="L50" s="2"/>
       <c r="M50" s="2"/>
     </row>
-    <row r="51" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A51" s="12" t="s">
         <v>17</v>
       </c>
@@ -9708,7 +11472,7 @@
       <c r="L51" s="2"/>
       <c r="M51" s="2"/>
     </row>
-    <row r="52" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A52" s="13" t="s">
         <v>6</v>
       </c>
@@ -9725,79 +11489,309 @@
       <c r="L52" s="10"/>
       <c r="M52" s="10"/>
     </row>
-    <row r="54" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O54" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="55" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:30" x14ac:dyDescent="0.3">
       <c r="O55" t="s">
+        <v>49</v>
+      </c>
+      <c r="P55" s="42">
+        <v>0.62736285400000003</v>
+      </c>
+      <c r="Q55" s="42">
+        <v>7.1781017000000003E-2</v>
+      </c>
+      <c r="R55" s="42">
+        <v>0.63531370399999998</v>
+      </c>
+      <c r="S55" s="42">
+        <v>6.9879844999999996E-2</v>
+      </c>
+      <c r="T55" s="39">
+        <v>92.840909089999997</v>
+      </c>
+      <c r="U55" s="42">
+        <v>0</v>
+      </c>
+      <c r="V55" s="42">
+        <v>0</v>
+      </c>
+      <c r="W55" s="39">
+        <v>100</v>
+      </c>
+      <c r="X55" s="42">
+        <v>6.7561699999999999E-4</v>
+      </c>
+      <c r="Y55" s="42">
+        <v>6.7561699999999999E-4</v>
+      </c>
+      <c r="Z55" s="42">
+        <v>4.1599999999999996E-3</v>
+      </c>
+      <c r="AA55" s="42">
+        <v>1.584E-2</v>
+      </c>
+      <c r="AB55" s="39">
+        <v>100</v>
+      </c>
+      <c r="AC55" s="41">
+        <v>11</v>
+      </c>
+      <c r="AD55" s="39">
+        <v>3229.7740749999998</v>
+      </c>
+    </row>
+    <row r="56" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="O56" t="s">
+        <v>50</v>
+      </c>
+      <c r="P56" s="42">
+        <v>0.61607394599999998</v>
+      </c>
+      <c r="Q56" s="42">
+        <v>7.4070856000000004E-2</v>
+      </c>
+      <c r="R56" s="42">
+        <v>0.62477324099999998</v>
+      </c>
+      <c r="S56" s="42">
+        <v>7.1897643999999997E-2</v>
+      </c>
+      <c r="T56" s="39">
+        <v>100</v>
+      </c>
+      <c r="U56" s="42">
+        <v>0</v>
+      </c>
+      <c r="V56" s="42">
+        <v>0</v>
+      </c>
+      <c r="W56" s="39">
+        <v>100</v>
+      </c>
+      <c r="X56" s="42">
+        <v>7.4172400000000003E-4</v>
+      </c>
+      <c r="Y56" s="42">
+        <v>7.4172400000000003E-4</v>
+      </c>
+      <c r="Z56" s="42">
+        <v>2.7999999999999998E-4</v>
+      </c>
+      <c r="AA56" s="42">
+        <v>1.584E-2</v>
+      </c>
+      <c r="AB56" s="39">
+        <v>100</v>
+      </c>
+      <c r="AC56" s="41">
+        <v>11</v>
+      </c>
+      <c r="AD56" s="39">
+        <v>3836.9429270000001</v>
+      </c>
+    </row>
+    <row r="57" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="O57" t="s">
+        <v>33</v>
+      </c>
+      <c r="P57" s="42">
+        <v>0.40469522800000002</v>
+      </c>
+      <c r="Q57" s="42">
+        <v>6.9731839000000004E-2</v>
+      </c>
+      <c r="R57" s="42">
+        <v>0.40629886599999998</v>
+      </c>
+      <c r="S57" s="42">
+        <v>7.0271370999999999E-2</v>
+      </c>
+      <c r="T57" s="39">
+        <v>0</v>
+      </c>
+      <c r="U57" s="42">
+        <v>0</v>
+      </c>
+      <c r="V57" s="42">
+        <v>0</v>
+      </c>
+      <c r="W57" s="39">
+        <v>76.212121210000006</v>
+      </c>
+      <c r="X57" s="42">
+        <v>4.4247619999999996E-3</v>
+      </c>
+      <c r="Y57" s="42">
+        <v>4.4247619999999996E-3</v>
+      </c>
+      <c r="Z57" s="42">
+        <v>1.0880000000000001E-2</v>
+      </c>
+      <c r="AA57" s="42">
+        <v>0.83638100000000004</v>
+      </c>
+      <c r="AB57" s="39">
+        <v>100</v>
+      </c>
+      <c r="AC57" s="41">
+        <v>11</v>
+      </c>
+      <c r="AD57" s="39">
+        <v>3455.1726140000001</v>
+      </c>
+    </row>
+    <row r="58" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="O58" t="s">
+        <v>32</v>
+      </c>
+      <c r="P58" s="42">
+        <v>0.58641906600000004</v>
+      </c>
+      <c r="Q58" s="42">
+        <v>7.4058140999999994E-2</v>
+      </c>
+      <c r="R58" s="42">
+        <v>0.59317042200000003</v>
+      </c>
+      <c r="S58" s="42">
+        <v>7.4066038000000001E-2</v>
+      </c>
+      <c r="T58" s="39">
+        <v>0</v>
+      </c>
+      <c r="U58" s="42">
+        <v>0</v>
+      </c>
+      <c r="V58" s="42">
+        <v>0</v>
+      </c>
+      <c r="W58" s="39">
+        <v>100</v>
+      </c>
+      <c r="X58" s="42">
+        <v>1.382154E-3</v>
+      </c>
+      <c r="Y58" s="42">
+        <v>1.382154E-3</v>
+      </c>
+      <c r="Z58" s="42">
+        <v>1.1039999999999999E-2</v>
+      </c>
+      <c r="AA58" s="42">
+        <v>0.150672</v>
+      </c>
+      <c r="AB58" s="39">
+        <v>100</v>
+      </c>
+      <c r="AC58" s="41">
+        <v>11</v>
+      </c>
+      <c r="AD58" s="39">
+        <v>9353.5133420000002</v>
+      </c>
+    </row>
+    <row r="59" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="O59" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="56" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="O56" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="57" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="O57" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="58" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="O58" t="s">
+      <c r="P59" s="42">
+        <v>2.2153664E-2</v>
+      </c>
+      <c r="Q59" s="42">
+        <v>6.8025735000000004E-2</v>
+      </c>
+      <c r="R59" s="42">
+        <v>5.5786159999999998E-3</v>
+      </c>
+      <c r="S59" s="42">
+        <v>3.6971740000000001E-3</v>
+      </c>
+      <c r="T59" s="39">
+        <v>0</v>
+      </c>
+      <c r="U59" s="42">
+        <v>0</v>
+      </c>
+      <c r="V59" s="42">
+        <v>0</v>
+      </c>
+      <c r="W59" s="39">
+        <v>0</v>
+      </c>
+      <c r="X59" s="42">
+        <v>1.4738187E-2</v>
+      </c>
+      <c r="Y59" s="42">
+        <v>1.4738187E-2</v>
+      </c>
+      <c r="Z59" s="42">
+        <v>1.1039999999999999E-2</v>
+      </c>
+      <c r="AA59" s="42">
+        <v>3.8163360000000002</v>
+      </c>
+      <c r="AB59" s="39">
+        <v>7.348484848</v>
+      </c>
+      <c r="AC59" s="41">
+        <v>0.80833333299999999</v>
+      </c>
+      <c r="AD59" s="39">
+        <v>16727.630369999999</v>
+      </c>
+    </row>
+    <row r="60" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="O60" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="59" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="O59" t="s">
+    <row r="61" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="O61" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="60" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="O60" t="s">
+    <row r="62" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="O62" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="61" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="O61" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="64" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="65" spans="1:15" x14ac:dyDescent="0.3">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="65" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A65" s="19" t="s">
         <v>0</v>
       </c>
       <c r="B65" s="34" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C65" s="35"/>
       <c r="D65" s="36"/>
       <c r="E65" s="37" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F65" s="35"/>
       <c r="G65" s="36"/>
       <c r="H65" s="37" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I65" s="35"/>
       <c r="J65" s="38"/>
       <c r="K65" s="34" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L65" s="35"/>
       <c r="M65" s="35"/>
       <c r="N65" s="21"/>
       <c r="O65" s="21"/>
     </row>
-    <row r="66" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A66" s="22" t="s">
         <v>1</v>
       </c>
@@ -9840,7 +11834,7 @@
       <c r="N66" s="21"/>
       <c r="O66" s="21"/>
     </row>
-    <row r="67" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A67" s="22" t="s">
         <v>2</v>
       </c>
@@ -9883,7 +11877,7 @@
       <c r="N67" s="21"/>
       <c r="O67" s="21"/>
     </row>
-    <row r="68" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A68" s="19" t="s">
         <v>3</v>
       </c>
@@ -9926,7 +11920,7 @@
       <c r="N68" s="21"/>
       <c r="O68" s="21"/>
     </row>
-    <row r="69" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A69" s="22" t="s">
         <v>4</v>
       </c>
@@ -9969,7 +11963,7 @@
       <c r="N69" s="21"/>
       <c r="O69" s="21"/>
     </row>
-    <row r="70" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A70" s="19" t="s">
         <v>7</v>
       </c>
@@ -10012,7 +12006,7 @@
       <c r="N70" s="21"/>
       <c r="O70" s="21"/>
     </row>
-    <row r="71" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A71" s="22" t="s">
         <v>5</v>
       </c>
@@ -10031,7 +12025,7 @@
       <c r="N71" s="21"/>
       <c r="O71" s="21"/>
     </row>
-    <row r="72" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A72" s="22" t="s">
         <v>17</v>
       </c>
@@ -10074,7 +12068,7 @@
       <c r="N72" s="21"/>
       <c r="O72" s="21"/>
     </row>
-    <row r="73" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A73" s="20" t="s">
         <v>6</v>
       </c>
@@ -10117,7 +12111,7 @@
       <c r="N73" s="21"/>
       <c r="O73" s="21"/>
     </row>
-    <row r="74" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A74" s="21"/>
       <c r="B74" s="21"/>
       <c r="C74" s="21"/>
@@ -10134,7 +12128,7 @@
       <c r="N74" s="21"/>
       <c r="O74" s="21"/>
     </row>
-    <row r="75" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A75" s="21"/>
       <c r="B75" s="21"/>
       <c r="C75" s="21"/>
@@ -10149,11 +12143,11 @@
       <c r="L75" s="21"/>
       <c r="M75" s="21"/>
       <c r="N75" s="21"/>
-      <c r="O75" s="21" t="s">
+      <c r="O75" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="76" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A76" s="21"/>
       <c r="B76" s="21"/>
       <c r="C76" s="21"/>
@@ -10168,11 +12162,56 @@
       <c r="L76" s="21"/>
       <c r="M76" s="21"/>
       <c r="N76" s="21"/>
-      <c r="O76" s="21" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="77" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="O76" t="s">
+        <v>49</v>
+      </c>
+      <c r="P76" s="42">
+        <v>0.60743649200000005</v>
+      </c>
+      <c r="Q76" s="42">
+        <v>0.33138423</v>
+      </c>
+      <c r="R76" s="42">
+        <v>0.63648149200000004</v>
+      </c>
+      <c r="S76" s="42">
+        <v>0.33051121100000003</v>
+      </c>
+      <c r="T76" s="39">
+        <v>70.60606061</v>
+      </c>
+      <c r="U76" s="42">
+        <v>3.6358300000000001E-3</v>
+      </c>
+      <c r="V76" s="42">
+        <v>3.6358300000000001E-3</v>
+      </c>
+      <c r="W76" s="39">
+        <v>100</v>
+      </c>
+      <c r="X76" s="42">
+        <v>1.03353E-2</v>
+      </c>
+      <c r="Y76" s="42">
+        <v>1.03353E-2</v>
+      </c>
+      <c r="Z76" s="42">
+        <v>8.7999999999999995E-2</v>
+      </c>
+      <c r="AA76" s="42">
+        <v>0.28320000000000001</v>
+      </c>
+      <c r="AB76" s="39">
+        <v>100</v>
+      </c>
+      <c r="AC76" s="41">
+        <v>11</v>
+      </c>
+      <c r="AD76" s="39">
+        <v>24321.607189999999</v>
+      </c>
+    </row>
+    <row r="77" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A77" s="21"/>
       <c r="B77" s="21"/>
       <c r="C77" s="21"/>
@@ -10187,11 +12226,56 @@
       <c r="L77" s="21"/>
       <c r="M77" s="21"/>
       <c r="N77" s="21"/>
-      <c r="O77" s="21" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="78" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="O77" t="s">
+        <v>50</v>
+      </c>
+      <c r="P77" s="42">
+        <v>0.60830025099999996</v>
+      </c>
+      <c r="Q77" s="42">
+        <v>0.33140337600000003</v>
+      </c>
+      <c r="R77" s="42">
+        <v>0.63934216300000002</v>
+      </c>
+      <c r="S77" s="42">
+        <v>0.328036889</v>
+      </c>
+      <c r="T77" s="39">
+        <v>70.60606061</v>
+      </c>
+      <c r="U77" s="42">
+        <v>2.9528549999999999E-3</v>
+      </c>
+      <c r="V77" s="42">
+        <v>2.9528549999999999E-3</v>
+      </c>
+      <c r="W77" s="39">
+        <v>100</v>
+      </c>
+      <c r="X77" s="42">
+        <v>1.0672749E-2</v>
+      </c>
+      <c r="Y77" s="42">
+        <v>1.0672749E-2</v>
+      </c>
+      <c r="Z77" s="42">
+        <v>0.08</v>
+      </c>
+      <c r="AA77" s="42">
+        <v>0.30359999999999998</v>
+      </c>
+      <c r="AB77" s="39">
+        <v>100</v>
+      </c>
+      <c r="AC77" s="41">
+        <v>11</v>
+      </c>
+      <c r="AD77" s="39">
+        <v>25447.67641</v>
+      </c>
+    </row>
+    <row r="78" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A78" s="21"/>
       <c r="B78" s="21"/>
       <c r="C78" s="21"/>
@@ -10206,11 +12290,56 @@
       <c r="L78" s="21"/>
       <c r="M78" s="21"/>
       <c r="N78" s="21"/>
-      <c r="O78" s="21" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="79" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="O78" t="s">
+        <v>33</v>
+      </c>
+      <c r="P78" s="42">
+        <v>7.9489345000000003E-2</v>
+      </c>
+      <c r="Q78" s="42">
+        <v>0.108876977</v>
+      </c>
+      <c r="R78" s="42">
+        <v>5.7906882E-2</v>
+      </c>
+      <c r="S78" s="42">
+        <v>7.2164350000000002E-2</v>
+      </c>
+      <c r="T78" s="39">
+        <v>0</v>
+      </c>
+      <c r="U78" s="42">
+        <v>7.5502099999999999E-3</v>
+      </c>
+      <c r="V78" s="42">
+        <v>7.5502099999999999E-3</v>
+      </c>
+      <c r="W78" s="39">
+        <v>15.3030303</v>
+      </c>
+      <c r="X78" s="42">
+        <v>1.2874299000000001E-2</v>
+      </c>
+      <c r="Y78" s="42">
+        <v>1.2874299000000001E-2</v>
+      </c>
+      <c r="Z78" s="42">
+        <v>0.29520000000000002</v>
+      </c>
+      <c r="AA78" s="42">
+        <v>0.84</v>
+      </c>
+      <c r="AB78" s="39">
+        <v>41.363636360000001</v>
+      </c>
+      <c r="AC78" s="41">
+        <v>4.55</v>
+      </c>
+      <c r="AD78" s="39">
+        <v>17572.518039999999</v>
+      </c>
+    </row>
+    <row r="79" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A79" s="21"/>
       <c r="B79" s="21"/>
       <c r="C79" s="21"/>
@@ -10225,11 +12354,56 @@
       <c r="L79" s="21"/>
       <c r="M79" s="21"/>
       <c r="N79" s="21"/>
-      <c r="O79" s="21" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="80" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="O79" t="s">
+        <v>32</v>
+      </c>
+      <c r="P79" s="42">
+        <v>7.9618703999999998E-2</v>
+      </c>
+      <c r="Q79" s="42">
+        <v>0.103620223</v>
+      </c>
+      <c r="R79" s="42">
+        <v>5.8641828E-2</v>
+      </c>
+      <c r="S79" s="42">
+        <v>7.1932098E-2</v>
+      </c>
+      <c r="T79" s="39">
+        <v>0</v>
+      </c>
+      <c r="U79" s="42">
+        <v>7.5502099999999999E-3</v>
+      </c>
+      <c r="V79" s="42">
+        <v>7.5502099999999999E-3</v>
+      </c>
+      <c r="W79" s="39">
+        <v>14.621212119999999</v>
+      </c>
+      <c r="X79" s="42">
+        <v>1.2874299000000001E-2</v>
+      </c>
+      <c r="Y79" s="42">
+        <v>1.2874299000000001E-2</v>
+      </c>
+      <c r="Z79" s="42">
+        <v>0.29520000000000002</v>
+      </c>
+      <c r="AA79" s="42">
+        <v>1.1305000000000001</v>
+      </c>
+      <c r="AB79" s="39">
+        <v>42.765151520000003</v>
+      </c>
+      <c r="AC79" s="41">
+        <v>4.704166667</v>
+      </c>
+      <c r="AD79" s="39">
+        <v>17021.89831</v>
+      </c>
+    </row>
+    <row r="80" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A80" s="21"/>
       <c r="B80" s="21"/>
       <c r="C80" s="21"/>
@@ -10244,11 +12418,56 @@
       <c r="L80" s="21"/>
       <c r="M80" s="21"/>
       <c r="N80" s="21"/>
-      <c r="O80" s="21" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="81" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="O80" t="s">
+        <v>34</v>
+      </c>
+      <c r="P80" s="42">
+        <v>2.4642293999999999E-2</v>
+      </c>
+      <c r="Q80" s="42">
+        <v>7.4684096000000005E-2</v>
+      </c>
+      <c r="R80" s="42">
+        <v>6.3402049999999998E-3</v>
+      </c>
+      <c r="S80" s="42">
+        <v>5.4095860000000001E-3</v>
+      </c>
+      <c r="T80" s="39">
+        <v>0</v>
+      </c>
+      <c r="U80" s="42">
+        <v>7.5502099999999999E-3</v>
+      </c>
+      <c r="V80" s="42">
+        <v>7.5502099999999999E-3</v>
+      </c>
+      <c r="W80" s="39">
+        <v>8.5606060609999997</v>
+      </c>
+      <c r="X80" s="42">
+        <v>1.4027168E-2</v>
+      </c>
+      <c r="Y80" s="42">
+        <v>1.4027168E-2</v>
+      </c>
+      <c r="Z80" s="42">
+        <v>0.29520000000000002</v>
+      </c>
+      <c r="AA80" s="42">
+        <v>1.5960000000000001</v>
+      </c>
+      <c r="AB80" s="39">
+        <v>20.795454549999999</v>
+      </c>
+      <c r="AC80" s="41">
+        <v>2.2875000000000001</v>
+      </c>
+      <c r="AD80" s="39">
+        <v>16124.11807</v>
+      </c>
+    </row>
+    <row r="81" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A81" s="21"/>
       <c r="B81" s="21"/>
       <c r="C81" s="21"/>
@@ -10263,11 +12482,11 @@
       <c r="L81" s="21"/>
       <c r="M81" s="21"/>
       <c r="N81" s="21"/>
-      <c r="O81" s="21" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="82" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="O81" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="82" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A82" s="21"/>
       <c r="B82" s="21"/>
       <c r="C82" s="21"/>
@@ -10282,8 +12501,103 @@
       <c r="L82" s="21"/>
       <c r="M82" s="21"/>
       <c r="N82" s="21"/>
-      <c r="O82" s="21" t="s">
-        <v>38</v>
+      <c r="O82" t="s">
+        <v>36</v>
+      </c>
+      <c r="P82" s="42">
+        <v>2.4642293999999999E-2</v>
+      </c>
+      <c r="Q82" s="42">
+        <v>7.4684096000000005E-2</v>
+      </c>
+      <c r="R82" s="42">
+        <v>6.3402049999999998E-3</v>
+      </c>
+      <c r="S82" s="42">
+        <v>5.4095860000000001E-3</v>
+      </c>
+      <c r="T82" s="39">
+        <v>0</v>
+      </c>
+      <c r="U82" s="42">
+        <v>7.5502099999999999E-3</v>
+      </c>
+      <c r="V82" s="42">
+        <v>7.5502099999999999E-3</v>
+      </c>
+      <c r="W82" s="39">
+        <v>8.5606060609999997</v>
+      </c>
+      <c r="X82" s="42">
+        <v>1.4027168E-2</v>
+      </c>
+      <c r="Y82" s="42">
+        <v>1.4027168E-2</v>
+      </c>
+      <c r="Z82" s="42">
+        <v>0.29520000000000002</v>
+      </c>
+      <c r="AA82" s="42">
+        <v>1.5960000000000001</v>
+      </c>
+      <c r="AB82" s="39">
+        <v>20.795454549999999</v>
+      </c>
+      <c r="AC82" s="41">
+        <v>2.2875000000000001</v>
+      </c>
+      <c r="AD82" s="39">
+        <v>16124.11807</v>
+      </c>
+    </row>
+    <row r="83" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="O83" t="s">
+        <v>37</v>
+      </c>
+      <c r="P83" s="42">
+        <v>2.4642313999999998E-2</v>
+      </c>
+      <c r="Q83" s="42">
+        <v>7.4684087999999996E-2</v>
+      </c>
+      <c r="R83" s="42">
+        <v>6.340226E-3</v>
+      </c>
+      <c r="S83" s="42">
+        <v>5.4095510000000003E-3</v>
+      </c>
+      <c r="T83" s="39">
+        <v>0</v>
+      </c>
+      <c r="U83" s="42">
+        <v>7.5502099999999999E-3</v>
+      </c>
+      <c r="V83" s="42">
+        <v>7.5502099999999999E-3</v>
+      </c>
+      <c r="W83" s="39">
+        <v>8.5606060609999997</v>
+      </c>
+      <c r="X83" s="42">
+        <v>1.4027168E-2</v>
+      </c>
+      <c r="Y83" s="42">
+        <v>1.4027168E-2</v>
+      </c>
+      <c r="Z83" s="42">
+        <v>0.29520000000000002</v>
+      </c>
+      <c r="AA83" s="42">
+        <v>1.444</v>
+      </c>
+      <c r="AB83" s="39">
+        <v>20.9469697</v>
+      </c>
+      <c r="AC83" s="41">
+        <v>2.3041666670000001</v>
+      </c>
+      <c r="AD83" s="39">
+        <v>16124.12119</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added mte plotting file and plots
</commit_message>
<xml_diff>
--- a/results/compiled results.xlsx
+++ b/results/compiled results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\elish\Desktop\Aims Project\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1909A0AB-C71F-4994-83C5-EDF42BF29570}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4C467A0-DE6D-4F87-B6A9-6F98196802D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{DA4D96B0-492C-4945-A9C4-EFCA6D6BC722}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{DA4D96B0-492C-4945-A9C4-EFCA6D6BC722}"/>
   </bookViews>
   <sheets>
     <sheet name="Dynamic results" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="443" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="459" uniqueCount="52">
   <si>
     <t xml:space="preserve">Model </t>
   </si>
@@ -195,6 +195,9 @@
   </si>
   <si>
     <t>l8b</t>
+  </si>
+  <si>
+    <t>--</t>
   </si>
 </sst>
 </file>
@@ -356,7 +359,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -446,6 +449,12 @@
     <xf numFmtId="2" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -470,12 +479,9 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -843,26 +849,26 @@
       <c r="A2" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="31" t="s">
+      <c r="B2" s="35" t="s">
         <v>39</v>
       </c>
-      <c r="C2" s="32"/>
-      <c r="D2" s="33"/>
-      <c r="E2" s="32" t="s">
+      <c r="C2" s="36"/>
+      <c r="D2" s="37"/>
+      <c r="E2" s="36" t="s">
         <v>40</v>
       </c>
-      <c r="F2" s="32"/>
-      <c r="G2" s="33"/>
-      <c r="H2" s="32" t="s">
+      <c r="F2" s="36"/>
+      <c r="G2" s="37"/>
+      <c r="H2" s="36" t="s">
         <v>41</v>
       </c>
-      <c r="I2" s="32"/>
-      <c r="J2" s="32"/>
-      <c r="K2" s="31" t="s">
+      <c r="I2" s="36"/>
+      <c r="J2" s="36"/>
+      <c r="K2" s="35" t="s">
         <v>42</v>
       </c>
-      <c r="L2" s="32"/>
-      <c r="M2" s="32"/>
+      <c r="L2" s="36"/>
+      <c r="M2" s="36"/>
     </row>
     <row r="3" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
@@ -1337,6 +1343,51 @@
       <c r="N17" t="s">
         <v>50</v>
       </c>
+      <c r="O17" s="43" t="s">
+        <v>51</v>
+      </c>
+      <c r="P17" s="43" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q17" s="43" t="s">
+        <v>51</v>
+      </c>
+      <c r="R17" s="43" t="s">
+        <v>51</v>
+      </c>
+      <c r="S17" s="43" t="s">
+        <v>51</v>
+      </c>
+      <c r="T17" s="43" t="s">
+        <v>51</v>
+      </c>
+      <c r="U17" s="43" t="s">
+        <v>51</v>
+      </c>
+      <c r="V17" s="43" t="s">
+        <v>51</v>
+      </c>
+      <c r="W17" s="43" t="s">
+        <v>51</v>
+      </c>
+      <c r="X17" s="43" t="s">
+        <v>51</v>
+      </c>
+      <c r="Y17" s="43" t="s">
+        <v>51</v>
+      </c>
+      <c r="Z17" s="43" t="s">
+        <v>51</v>
+      </c>
+      <c r="AA17" s="43" t="s">
+        <v>51</v>
+      </c>
+      <c r="AB17" s="43" t="s">
+        <v>51</v>
+      </c>
+      <c r="AC17" s="43" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="18" spans="1:29" x14ac:dyDescent="0.3">
       <c r="N18" t="s">
@@ -1611,26 +1662,29 @@
       <c r="A27" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B27" s="31" t="s">
+      <c r="B27" s="35" t="s">
         <v>39</v>
       </c>
-      <c r="C27" s="32"/>
-      <c r="D27" s="33"/>
-      <c r="E27" s="32" t="s">
+      <c r="C27" s="36"/>
+      <c r="D27" s="37"/>
+      <c r="E27" s="36" t="s">
         <v>40</v>
       </c>
-      <c r="F27" s="32"/>
-      <c r="G27" s="33"/>
-      <c r="H27" s="32" t="s">
+      <c r="F27" s="36"/>
+      <c r="G27" s="37"/>
+      <c r="H27" s="36" t="s">
         <v>41</v>
       </c>
-      <c r="I27" s="32"/>
-      <c r="J27" s="32"/>
-      <c r="K27" s="31" t="s">
+      <c r="I27" s="36"/>
+      <c r="J27" s="36"/>
+      <c r="K27" s="35" t="s">
         <v>42</v>
       </c>
-      <c r="L27" s="32"/>
-      <c r="M27" s="32"/>
+      <c r="L27" s="36"/>
+      <c r="M27" s="36"/>
+      <c r="O27" s="43" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="28" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A28" s="14" t="s">
@@ -2328,26 +2382,26 @@
       <c r="A47" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B47" s="31" t="s">
+      <c r="B47" s="35" t="s">
         <v>39</v>
       </c>
-      <c r="C47" s="32"/>
-      <c r="D47" s="33"/>
-      <c r="E47" s="32" t="s">
+      <c r="C47" s="36"/>
+      <c r="D47" s="37"/>
+      <c r="E47" s="36" t="s">
         <v>40</v>
       </c>
-      <c r="F47" s="32"/>
-      <c r="G47" s="33"/>
-      <c r="H47" s="32" t="s">
+      <c r="F47" s="36"/>
+      <c r="G47" s="37"/>
+      <c r="H47" s="36" t="s">
         <v>41</v>
       </c>
-      <c r="I47" s="32"/>
-      <c r="J47" s="32"/>
-      <c r="K47" s="31" t="s">
+      <c r="I47" s="36"/>
+      <c r="J47" s="36"/>
+      <c r="K47" s="35" t="s">
         <v>42</v>
       </c>
-      <c r="L47" s="32"/>
-      <c r="M47" s="32"/>
+      <c r="L47" s="36"/>
+      <c r="M47" s="36"/>
     </row>
     <row r="48" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A48" s="12" t="s">
@@ -3043,26 +3097,26 @@
       <c r="A70" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B70" s="31" t="s">
+      <c r="B70" s="35" t="s">
         <v>39</v>
       </c>
-      <c r="C70" s="32"/>
-      <c r="D70" s="33"/>
-      <c r="E70" s="32" t="s">
+      <c r="C70" s="36"/>
+      <c r="D70" s="37"/>
+      <c r="E70" s="36" t="s">
         <v>40</v>
       </c>
-      <c r="F70" s="32"/>
-      <c r="G70" s="33"/>
-      <c r="H70" s="32" t="s">
+      <c r="F70" s="36"/>
+      <c r="G70" s="37"/>
+      <c r="H70" s="36" t="s">
         <v>41</v>
       </c>
-      <c r="I70" s="32"/>
-      <c r="J70" s="32"/>
-      <c r="K70" s="31" t="s">
+      <c r="I70" s="36"/>
+      <c r="J70" s="36"/>
+      <c r="K70" s="35" t="s">
         <v>42</v>
       </c>
-      <c r="L70" s="32"/>
-      <c r="M70" s="32"/>
+      <c r="L70" s="36"/>
+      <c r="M70" s="36"/>
     </row>
     <row r="71" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A71" s="14" t="s">
@@ -3798,6 +3852,14 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="B70:D70"/>
+    <mergeCell ref="E70:G70"/>
+    <mergeCell ref="H70:J70"/>
+    <mergeCell ref="K70:M70"/>
+    <mergeCell ref="B47:D47"/>
+    <mergeCell ref="E47:G47"/>
+    <mergeCell ref="H47:J47"/>
+    <mergeCell ref="K47:M47"/>
     <mergeCell ref="B2:D2"/>
     <mergeCell ref="E2:G2"/>
     <mergeCell ref="H2:J2"/>
@@ -3806,14 +3868,6 @@
     <mergeCell ref="E27:G27"/>
     <mergeCell ref="H27:J27"/>
     <mergeCell ref="K27:M27"/>
-    <mergeCell ref="B70:D70"/>
-    <mergeCell ref="E70:G70"/>
-    <mergeCell ref="H70:J70"/>
-    <mergeCell ref="K70:M70"/>
-    <mergeCell ref="B47:D47"/>
-    <mergeCell ref="E47:G47"/>
-    <mergeCell ref="H47:J47"/>
-    <mergeCell ref="K47:M47"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3845,26 +3899,26 @@
       <c r="A2" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="31" t="s">
+      <c r="B2" s="35" t="s">
         <v>39</v>
       </c>
-      <c r="C2" s="32"/>
-      <c r="D2" s="33"/>
-      <c r="E2" s="32" t="s">
+      <c r="C2" s="36"/>
+      <c r="D2" s="37"/>
+      <c r="E2" s="36" t="s">
         <v>40</v>
       </c>
-      <c r="F2" s="32"/>
-      <c r="G2" s="33"/>
-      <c r="H2" s="32" t="s">
+      <c r="F2" s="36"/>
+      <c r="G2" s="37"/>
+      <c r="H2" s="36" t="s">
         <v>41</v>
       </c>
-      <c r="I2" s="32"/>
-      <c r="J2" s="32"/>
-      <c r="K2" s="31" t="s">
+      <c r="I2" s="36"/>
+      <c r="J2" s="36"/>
+      <c r="K2" s="35" t="s">
         <v>42</v>
       </c>
-      <c r="L2" s="32"/>
-      <c r="M2" s="32"/>
+      <c r="L2" s="36"/>
+      <c r="M2" s="36"/>
     </row>
     <row r="3" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
@@ -4631,26 +4685,26 @@
       <c r="A24" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B24" s="31" t="s">
+      <c r="B24" s="35" t="s">
         <v>39</v>
       </c>
-      <c r="C24" s="32"/>
-      <c r="D24" s="33"/>
-      <c r="E24" s="32" t="s">
+      <c r="C24" s="36"/>
+      <c r="D24" s="37"/>
+      <c r="E24" s="36" t="s">
         <v>40</v>
       </c>
-      <c r="F24" s="32"/>
-      <c r="G24" s="33"/>
-      <c r="H24" s="32" t="s">
+      <c r="F24" s="36"/>
+      <c r="G24" s="37"/>
+      <c r="H24" s="36" t="s">
         <v>41</v>
       </c>
-      <c r="I24" s="32"/>
-      <c r="J24" s="32"/>
-      <c r="K24" s="31" t="s">
+      <c r="I24" s="36"/>
+      <c r="J24" s="36"/>
+      <c r="K24" s="35" t="s">
         <v>42</v>
       </c>
-      <c r="L24" s="32"/>
-      <c r="M24" s="32"/>
+      <c r="L24" s="36"/>
+      <c r="M24" s="36"/>
     </row>
     <row r="25" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A25" s="14" t="s">
@@ -5394,26 +5448,26 @@
       <c r="A44" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B44" s="31" t="s">
+      <c r="B44" s="35" t="s">
         <v>39</v>
       </c>
-      <c r="C44" s="32"/>
-      <c r="D44" s="33"/>
-      <c r="E44" s="32" t="s">
+      <c r="C44" s="36"/>
+      <c r="D44" s="37"/>
+      <c r="E44" s="36" t="s">
         <v>40</v>
       </c>
-      <c r="F44" s="32"/>
-      <c r="G44" s="33"/>
-      <c r="H44" s="32" t="s">
+      <c r="F44" s="36"/>
+      <c r="G44" s="37"/>
+      <c r="H44" s="36" t="s">
         <v>41</v>
       </c>
-      <c r="I44" s="32"/>
-      <c r="J44" s="32"/>
-      <c r="K44" s="31" t="s">
+      <c r="I44" s="36"/>
+      <c r="J44" s="36"/>
+      <c r="K44" s="35" t="s">
         <v>42</v>
       </c>
-      <c r="L44" s="32"/>
-      <c r="M44" s="32"/>
+      <c r="L44" s="36"/>
+      <c r="M44" s="36"/>
     </row>
     <row r="45" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A45" s="14" t="s">
@@ -6157,26 +6211,26 @@
       <c r="A65" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="B65" s="34" t="s">
+      <c r="B65" s="38" t="s">
         <v>39</v>
       </c>
-      <c r="C65" s="35"/>
-      <c r="D65" s="36"/>
-      <c r="E65" s="37" t="s">
+      <c r="C65" s="39"/>
+      <c r="D65" s="40"/>
+      <c r="E65" s="41" t="s">
         <v>40</v>
       </c>
-      <c r="F65" s="35"/>
-      <c r="G65" s="36"/>
-      <c r="H65" s="37" t="s">
+      <c r="F65" s="39"/>
+      <c r="G65" s="40"/>
+      <c r="H65" s="41" t="s">
         <v>41</v>
       </c>
-      <c r="I65" s="35"/>
-      <c r="J65" s="38"/>
-      <c r="K65" s="34" t="s">
+      <c r="I65" s="39"/>
+      <c r="J65" s="42"/>
+      <c r="K65" s="38" t="s">
         <v>42</v>
       </c>
-      <c r="L65" s="35"/>
-      <c r="M65" s="35"/>
+      <c r="L65" s="39"/>
+      <c r="M65" s="39"/>
       <c r="N65" s="21"/>
       <c r="O65" s="21"/>
     </row>
@@ -6991,6 +7045,14 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="B65:D65"/>
+    <mergeCell ref="E65:G65"/>
+    <mergeCell ref="H65:J65"/>
+    <mergeCell ref="K65:M65"/>
+    <mergeCell ref="B44:D44"/>
+    <mergeCell ref="E44:G44"/>
+    <mergeCell ref="H44:J44"/>
+    <mergeCell ref="K44:M44"/>
     <mergeCell ref="B2:D2"/>
     <mergeCell ref="E2:G2"/>
     <mergeCell ref="H2:J2"/>
@@ -6999,14 +7061,6 @@
     <mergeCell ref="E24:G24"/>
     <mergeCell ref="H24:J24"/>
     <mergeCell ref="K24:M24"/>
-    <mergeCell ref="B65:D65"/>
-    <mergeCell ref="E65:G65"/>
-    <mergeCell ref="H65:J65"/>
-    <mergeCell ref="K65:M65"/>
-    <mergeCell ref="B44:D44"/>
-    <mergeCell ref="E44:G44"/>
-    <mergeCell ref="H44:J44"/>
-    <mergeCell ref="K44:M44"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -7041,26 +7095,26 @@
       <c r="A2" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="31" t="s">
+      <c r="B2" s="35" t="s">
         <v>39</v>
       </c>
-      <c r="C2" s="32"/>
-      <c r="D2" s="33"/>
-      <c r="E2" s="32" t="s">
+      <c r="C2" s="36"/>
+      <c r="D2" s="37"/>
+      <c r="E2" s="36" t="s">
         <v>40</v>
       </c>
-      <c r="F2" s="32"/>
-      <c r="G2" s="33"/>
-      <c r="H2" s="32" t="s">
+      <c r="F2" s="36"/>
+      <c r="G2" s="37"/>
+      <c r="H2" s="36" t="s">
         <v>41</v>
       </c>
-      <c r="I2" s="32"/>
-      <c r="J2" s="32"/>
-      <c r="K2" s="31" t="s">
+      <c r="I2" s="36"/>
+      <c r="J2" s="36"/>
+      <c r="K2" s="35" t="s">
         <v>42</v>
       </c>
-      <c r="L2" s="32"/>
-      <c r="M2" s="32"/>
+      <c r="L2" s="36"/>
+      <c r="M2" s="36"/>
     </row>
     <row r="3" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
@@ -7737,26 +7791,26 @@
       <c r="A23" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B23" s="31" t="s">
+      <c r="B23" s="35" t="s">
         <v>39</v>
       </c>
-      <c r="C23" s="32"/>
-      <c r="D23" s="33"/>
-      <c r="E23" s="32" t="s">
+      <c r="C23" s="36"/>
+      <c r="D23" s="37"/>
+      <c r="E23" s="36" t="s">
         <v>40</v>
       </c>
-      <c r="F23" s="32"/>
-      <c r="G23" s="33"/>
-      <c r="H23" s="32" t="s">
+      <c r="F23" s="36"/>
+      <c r="G23" s="37"/>
+      <c r="H23" s="36" t="s">
         <v>41</v>
       </c>
-      <c r="I23" s="32"/>
-      <c r="J23" s="32"/>
-      <c r="K23" s="31" t="s">
+      <c r="I23" s="36"/>
+      <c r="J23" s="36"/>
+      <c r="K23" s="35" t="s">
         <v>42</v>
       </c>
-      <c r="L23" s="32"/>
-      <c r="M23" s="32"/>
+      <c r="L23" s="36"/>
+      <c r="M23" s="36"/>
     </row>
     <row r="24" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A24" s="14" t="s">
@@ -8386,26 +8440,26 @@
       <c r="A44" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B44" s="31" t="s">
+      <c r="B44" s="35" t="s">
         <v>39</v>
       </c>
-      <c r="C44" s="32"/>
-      <c r="D44" s="33"/>
-      <c r="E44" s="32" t="s">
+      <c r="C44" s="36"/>
+      <c r="D44" s="37"/>
+      <c r="E44" s="36" t="s">
         <v>40</v>
       </c>
-      <c r="F44" s="32"/>
-      <c r="G44" s="33"/>
-      <c r="H44" s="32" t="s">
+      <c r="F44" s="36"/>
+      <c r="G44" s="37"/>
+      <c r="H44" s="36" t="s">
         <v>41</v>
       </c>
-      <c r="I44" s="32"/>
-      <c r="J44" s="32"/>
-      <c r="K44" s="31" t="s">
+      <c r="I44" s="36"/>
+      <c r="J44" s="36"/>
+      <c r="K44" s="35" t="s">
         <v>42</v>
       </c>
-      <c r="L44" s="32"/>
-      <c r="M44" s="32"/>
+      <c r="L44" s="36"/>
+      <c r="M44" s="36"/>
     </row>
     <row r="45" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A45" s="14" t="s">
@@ -9035,26 +9089,26 @@
       <c r="A64" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="B64" s="34" t="s">
+      <c r="B64" s="38" t="s">
         <v>39</v>
       </c>
-      <c r="C64" s="35"/>
-      <c r="D64" s="36"/>
-      <c r="E64" s="37" t="s">
+      <c r="C64" s="39"/>
+      <c r="D64" s="40"/>
+      <c r="E64" s="41" t="s">
         <v>40</v>
       </c>
-      <c r="F64" s="35"/>
-      <c r="G64" s="36"/>
-      <c r="H64" s="37" t="s">
+      <c r="F64" s="39"/>
+      <c r="G64" s="40"/>
+      <c r="H64" s="41" t="s">
         <v>41</v>
       </c>
-      <c r="I64" s="35"/>
-      <c r="J64" s="38"/>
-      <c r="K64" s="34" t="s">
+      <c r="I64" s="39"/>
+      <c r="J64" s="42"/>
+      <c r="K64" s="38" t="s">
         <v>42</v>
       </c>
-      <c r="L64" s="35"/>
-      <c r="M64" s="35"/>
+      <c r="L64" s="39"/>
+      <c r="M64" s="39"/>
       <c r="N64" s="21"/>
       <c r="O64" s="21"/>
     </row>
@@ -9869,6 +9923,14 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="B44:D44"/>
+    <mergeCell ref="E44:G44"/>
+    <mergeCell ref="H44:J44"/>
+    <mergeCell ref="K44:M44"/>
+    <mergeCell ref="B64:D64"/>
+    <mergeCell ref="E64:G64"/>
+    <mergeCell ref="H64:J64"/>
+    <mergeCell ref="K64:M64"/>
     <mergeCell ref="B2:D2"/>
     <mergeCell ref="E2:G2"/>
     <mergeCell ref="H2:J2"/>
@@ -9877,14 +9939,6 @@
     <mergeCell ref="E23:G23"/>
     <mergeCell ref="H23:J23"/>
     <mergeCell ref="K23:M23"/>
-    <mergeCell ref="B44:D44"/>
-    <mergeCell ref="E44:G44"/>
-    <mergeCell ref="H44:J44"/>
-    <mergeCell ref="K44:M44"/>
-    <mergeCell ref="B64:D64"/>
-    <mergeCell ref="E64:G64"/>
-    <mergeCell ref="H64:J64"/>
-    <mergeCell ref="K64:M64"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -9896,14 +9950,14 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.77734375" customWidth="1"/>
-    <col min="16" max="19" width="8.88671875" style="42"/>
-    <col min="20" max="20" width="8.88671875" style="39"/>
-    <col min="21" max="22" width="8.88671875" style="42"/>
-    <col min="23" max="23" width="8.88671875" style="39"/>
-    <col min="24" max="27" width="8.88671875" style="42"/>
-    <col min="28" max="28" width="8.88671875" style="39"/>
-    <col min="29" max="29" width="8.88671875" style="41"/>
-    <col min="30" max="30" width="11.33203125" style="39" customWidth="1"/>
+    <col min="16" max="19" width="8.88671875" style="34"/>
+    <col min="20" max="20" width="8.88671875" style="31"/>
+    <col min="21" max="22" width="8.88671875" style="34"/>
+    <col min="23" max="23" width="8.88671875" style="31"/>
+    <col min="24" max="27" width="8.88671875" style="34"/>
+    <col min="28" max="28" width="8.88671875" style="31"/>
+    <col min="29" max="29" width="8.88671875" style="33"/>
+    <col min="30" max="30" width="11.33203125" style="31" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:30" x14ac:dyDescent="0.3">
@@ -9915,26 +9969,26 @@
       <c r="A2" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="31" t="s">
+      <c r="B2" s="35" t="s">
         <v>39</v>
       </c>
-      <c r="C2" s="32"/>
-      <c r="D2" s="33"/>
-      <c r="E2" s="32" t="s">
+      <c r="C2" s="36"/>
+      <c r="D2" s="37"/>
+      <c r="E2" s="36" t="s">
         <v>40</v>
       </c>
-      <c r="F2" s="32"/>
-      <c r="G2" s="33"/>
-      <c r="H2" s="32" t="s">
+      <c r="F2" s="36"/>
+      <c r="G2" s="37"/>
+      <c r="H2" s="36" t="s">
         <v>41</v>
       </c>
-      <c r="I2" s="32"/>
-      <c r="J2" s="32"/>
-      <c r="K2" s="31" t="s">
+      <c r="I2" s="36"/>
+      <c r="J2" s="36"/>
+      <c r="K2" s="35" t="s">
         <v>42</v>
       </c>
-      <c r="L2" s="32"/>
-      <c r="M2" s="32"/>
+      <c r="L2" s="36"/>
+      <c r="M2" s="36"/>
     </row>
     <row r="3" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
@@ -10256,7 +10310,7 @@
       <c r="AB11" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="AC11" s="40" t="s">
+      <c r="AC11" s="32" t="s">
         <v>31</v>
       </c>
       <c r="AD11" s="2" t="s">
@@ -10272,49 +10326,49 @@
       <c r="O13" t="s">
         <v>49</v>
       </c>
-      <c r="P13" s="42">
+      <c r="P13" s="34">
         <v>2.0422105999999999E-2</v>
       </c>
-      <c r="Q13" s="42">
+      <c r="Q13" s="34">
         <v>6.6577413000000002E-2</v>
       </c>
-      <c r="R13" s="42">
+      <c r="R13" s="34">
         <v>4.2976079999999996E-3</v>
       </c>
-      <c r="S13" s="42">
+      <c r="S13" s="34">
         <v>3.4186780000000001E-3</v>
       </c>
-      <c r="T13" s="39">
-        <v>0</v>
-      </c>
-      <c r="U13" s="42">
-        <v>0</v>
-      </c>
-      <c r="V13" s="42">
-        <v>0</v>
-      </c>
-      <c r="W13" s="39">
-        <v>0</v>
-      </c>
-      <c r="X13" s="42">
+      <c r="T13" s="31">
+        <v>0</v>
+      </c>
+      <c r="U13" s="34">
+        <v>0</v>
+      </c>
+      <c r="V13" s="34">
+        <v>0</v>
+      </c>
+      <c r="W13" s="31">
+        <v>0</v>
+      </c>
+      <c r="X13" s="34">
         <v>1.4738187E-2</v>
       </c>
-      <c r="Y13" s="42">
+      <c r="Y13" s="34">
         <v>1.4738187E-2</v>
       </c>
-      <c r="Z13" s="42">
-        <v>0</v>
-      </c>
-      <c r="AA13" s="42">
+      <c r="Z13" s="34">
+        <v>0</v>
+      </c>
+      <c r="AA13" s="34">
         <v>3.8163360000000002</v>
       </c>
-      <c r="AB13" s="39">
+      <c r="AB13" s="31">
         <v>99.962121210000006</v>
       </c>
-      <c r="AC13" s="41">
+      <c r="AC13" s="33">
         <v>10.99583333</v>
       </c>
-      <c r="AD13" s="39">
+      <c r="AD13" s="31">
         <v>16783.498909999998</v>
       </c>
     </row>
@@ -10322,49 +10376,49 @@
       <c r="O14" t="s">
         <v>50</v>
       </c>
-      <c r="P14" s="42">
+      <c r="P14" s="34">
         <v>2.0422105999999999E-2</v>
       </c>
-      <c r="Q14" s="42">
+      <c r="Q14" s="34">
         <v>6.6577413000000002E-2</v>
       </c>
-      <c r="R14" s="42">
+      <c r="R14" s="34">
         <v>4.2976079999999996E-3</v>
       </c>
-      <c r="S14" s="42">
+      <c r="S14" s="34">
         <v>3.4186780000000001E-3</v>
       </c>
-      <c r="T14" s="39">
-        <v>0</v>
-      </c>
-      <c r="U14" s="42">
-        <v>0</v>
-      </c>
-      <c r="V14" s="42">
-        <v>0</v>
-      </c>
-      <c r="W14" s="39">
-        <v>0</v>
-      </c>
-      <c r="X14" s="42">
+      <c r="T14" s="31">
+        <v>0</v>
+      </c>
+      <c r="U14" s="34">
+        <v>0</v>
+      </c>
+      <c r="V14" s="34">
+        <v>0</v>
+      </c>
+      <c r="W14" s="31">
+        <v>0</v>
+      </c>
+      <c r="X14" s="34">
         <v>1.4738187E-2</v>
       </c>
-      <c r="Y14" s="42">
+      <c r="Y14" s="34">
         <v>1.4738187E-2</v>
       </c>
-      <c r="Z14" s="42">
-        <v>0</v>
-      </c>
-      <c r="AA14" s="42">
+      <c r="Z14" s="34">
+        <v>0</v>
+      </c>
+      <c r="AA14" s="34">
         <v>3.8163360000000002</v>
       </c>
-      <c r="AB14" s="39">
+      <c r="AB14" s="31">
         <v>99.962121210000006</v>
       </c>
-      <c r="AC14" s="41">
+      <c r="AC14" s="33">
         <v>10.99583333</v>
       </c>
-      <c r="AD14" s="39">
+      <c r="AD14" s="31">
         <v>16783.498909999998</v>
       </c>
     </row>
@@ -10372,49 +10426,49 @@
       <c r="O15" t="s">
         <v>33</v>
       </c>
-      <c r="P15" s="42">
+      <c r="P15" s="34">
         <v>2.2174191999999999E-2</v>
       </c>
-      <c r="Q15" s="42">
+      <c r="Q15" s="34">
         <v>6.8021499999999999E-2</v>
       </c>
-      <c r="R15" s="42">
+      <c r="R15" s="34">
         <v>5.6011979999999999E-3</v>
       </c>
-      <c r="S15" s="42">
+      <c r="S15" s="34">
         <v>3.7126630000000002E-3</v>
       </c>
-      <c r="T15" s="39">
-        <v>0</v>
-      </c>
-      <c r="U15" s="42">
+      <c r="T15" s="31">
+        <v>0</v>
+      </c>
+      <c r="U15" s="34">
         <v>1.5541200000000001E-4</v>
       </c>
-      <c r="V15" s="42">
+      <c r="V15" s="34">
         <v>1.5541200000000001E-4</v>
       </c>
-      <c r="W15" s="39">
-        <v>0</v>
-      </c>
-      <c r="X15" s="42">
+      <c r="W15" s="31">
+        <v>0</v>
+      </c>
+      <c r="X15" s="34">
         <v>1.4027168E-2</v>
       </c>
-      <c r="Y15" s="42">
+      <c r="Y15" s="34">
         <v>1.4027168E-2</v>
       </c>
-      <c r="Z15" s="42">
+      <c r="Z15" s="34">
         <v>5.1679999999999997E-2</v>
       </c>
-      <c r="AA15" s="42">
+      <c r="AA15" s="34">
         <v>3.3281999999999998</v>
       </c>
-      <c r="AB15" s="39">
+      <c r="AB15" s="31">
         <v>0.15151515199999999</v>
       </c>
-      <c r="AC15" s="41">
+      <c r="AC15" s="33">
         <v>1.6666667E-2</v>
       </c>
-      <c r="AD15" s="39">
+      <c r="AD15" s="31">
         <v>16726.551950000001</v>
       </c>
     </row>
@@ -10422,49 +10476,49 @@
       <c r="O16" t="s">
         <v>32</v>
       </c>
-      <c r="P16" s="42">
+      <c r="P16" s="34">
         <v>0.47406991900000001</v>
       </c>
-      <c r="Q16" s="42">
+      <c r="Q16" s="34">
         <v>7.1940545999999994E-2</v>
       </c>
-      <c r="R16" s="42">
+      <c r="R16" s="34">
         <v>0.47826287499999998</v>
       </c>
-      <c r="S16" s="42">
+      <c r="S16" s="34">
         <v>7.3811294999999999E-2</v>
       </c>
-      <c r="T16" s="39">
-        <v>0</v>
-      </c>
-      <c r="U16" s="42">
+      <c r="T16" s="31">
+        <v>0</v>
+      </c>
+      <c r="U16" s="34">
         <v>2.148166E-3</v>
       </c>
-      <c r="V16" s="42">
+      <c r="V16" s="34">
         <v>2.148166E-3</v>
       </c>
-      <c r="W16" s="39">
+      <c r="W16" s="31">
         <v>100</v>
       </c>
-      <c r="X16" s="42">
+      <c r="X16" s="34">
         <v>2.9114729999999999E-3</v>
       </c>
-      <c r="Y16" s="42">
+      <c r="Y16" s="34">
         <v>2.9114729999999999E-3</v>
       </c>
-      <c r="Z16" s="42">
+      <c r="Z16" s="34">
         <v>0.16416</v>
       </c>
-      <c r="AA16" s="42">
+      <c r="AA16" s="34">
         <v>0.27753</v>
       </c>
-      <c r="AB16" s="39">
+      <c r="AB16" s="31">
         <v>100</v>
       </c>
-      <c r="AC16" s="41">
+      <c r="AC16" s="33">
         <v>11</v>
       </c>
-      <c r="AD16" s="39">
+      <c r="AD16" s="31">
         <v>14903.962009999999</v>
       </c>
     </row>
@@ -10472,49 +10526,49 @@
       <c r="O17" t="s">
         <v>34</v>
       </c>
-      <c r="P17" s="42">
+      <c r="P17" s="34">
         <v>0.38654200399999999</v>
       </c>
-      <c r="Q17" s="42">
+      <c r="Q17" s="34">
         <v>7.5658416000000006E-2</v>
       </c>
-      <c r="R17" s="42">
+      <c r="R17" s="34">
         <v>0.38150645599999999</v>
       </c>
-      <c r="S17" s="42">
+      <c r="S17" s="34">
         <v>7.7287566000000002E-2</v>
       </c>
-      <c r="T17" s="39">
-        <v>0</v>
-      </c>
-      <c r="U17" s="42">
+      <c r="T17" s="31">
+        <v>0</v>
+      </c>
+      <c r="U17" s="34">
         <v>2.148166E-3</v>
       </c>
-      <c r="V17" s="42">
+      <c r="V17" s="34">
         <v>2.148166E-3</v>
       </c>
-      <c r="W17" s="39">
+      <c r="W17" s="31">
         <v>100</v>
       </c>
-      <c r="X17" s="42">
+      <c r="X17" s="34">
         <v>2.9719070000000002E-3</v>
       </c>
-      <c r="Y17" s="42">
+      <c r="Y17" s="34">
         <v>2.9719070000000002E-3</v>
       </c>
-      <c r="Z17" s="42">
+      <c r="Z17" s="34">
         <v>0.16416</v>
       </c>
-      <c r="AA17" s="42">
+      <c r="AA17" s="34">
         <v>0.441</v>
       </c>
-      <c r="AB17" s="39">
+      <c r="AB17" s="31">
         <v>100</v>
       </c>
-      <c r="AC17" s="41">
+      <c r="AC17" s="33">
         <v>11</v>
       </c>
-      <c r="AD17" s="39">
+      <c r="AD17" s="31">
         <v>12736.34367</v>
       </c>
     </row>
@@ -10527,49 +10581,49 @@
       <c r="O19" t="s">
         <v>36</v>
       </c>
-      <c r="P19" s="42">
+      <c r="P19" s="34">
         <v>0.47509609200000003</v>
       </c>
-      <c r="Q19" s="42">
+      <c r="Q19" s="34">
         <v>7.3223063000000005E-2</v>
       </c>
-      <c r="R19" s="42">
+      <c r="R19" s="34">
         <v>0.47984376499999998</v>
       </c>
-      <c r="S19" s="42">
+      <c r="S19" s="34">
         <v>7.4750901999999994E-2</v>
       </c>
-      <c r="T19" s="39">
-        <v>0</v>
-      </c>
-      <c r="U19" s="42">
+      <c r="T19" s="31">
+        <v>0</v>
+      </c>
+      <c r="U19" s="34">
         <v>2.148166E-3</v>
       </c>
-      <c r="V19" s="42">
+      <c r="V19" s="34">
         <v>2.148166E-3</v>
       </c>
-      <c r="W19" s="39">
+      <c r="W19" s="31">
         <v>100</v>
       </c>
-      <c r="X19" s="42">
+      <c r="X19" s="34">
         <v>3.1957259999999999E-3</v>
       </c>
-      <c r="Y19" s="42">
+      <c r="Y19" s="34">
         <v>3.1957259999999999E-3</v>
       </c>
-      <c r="Z19" s="42">
+      <c r="Z19" s="34">
         <v>0.16416</v>
       </c>
-      <c r="AA19" s="42">
+      <c r="AA19" s="34">
         <v>0.34223999999999999</v>
       </c>
-      <c r="AB19" s="39">
+      <c r="AB19" s="31">
         <v>100</v>
       </c>
-      <c r="AC19" s="41">
+      <c r="AC19" s="33">
         <v>11</v>
       </c>
-      <c r="AD19" s="39">
+      <c r="AD19" s="31">
         <v>16872.860240000002</v>
       </c>
     </row>
@@ -10587,26 +10641,26 @@
       <c r="A23" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B23" s="31" t="s">
+      <c r="B23" s="35" t="s">
         <v>39</v>
       </c>
-      <c r="C23" s="32"/>
-      <c r="D23" s="33"/>
-      <c r="E23" s="32" t="s">
+      <c r="C23" s="36"/>
+      <c r="D23" s="37"/>
+      <c r="E23" s="36" t="s">
         <v>40</v>
       </c>
-      <c r="F23" s="32"/>
-      <c r="G23" s="33"/>
-      <c r="H23" s="32" t="s">
+      <c r="F23" s="36"/>
+      <c r="G23" s="37"/>
+      <c r="H23" s="36" t="s">
         <v>41</v>
       </c>
-      <c r="I23" s="32"/>
-      <c r="J23" s="32"/>
-      <c r="K23" s="31" t="s">
+      <c r="I23" s="36"/>
+      <c r="J23" s="36"/>
+      <c r="K23" s="35" t="s">
         <v>42</v>
       </c>
-      <c r="L23" s="32"/>
-      <c r="M23" s="32"/>
+      <c r="L23" s="36"/>
+      <c r="M23" s="36"/>
     </row>
     <row r="24" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A24" s="14" t="s">
@@ -10897,49 +10951,49 @@
       <c r="O34" t="s">
         <v>49</v>
       </c>
-      <c r="P34" s="42">
+      <c r="P34" s="34">
         <v>0.49276842999999998</v>
       </c>
-      <c r="Q34" s="42">
+      <c r="Q34" s="34">
         <v>7.2156964000000004E-2</v>
       </c>
-      <c r="R34" s="42">
+      <c r="R34" s="34">
         <v>0.49537018199999999</v>
       </c>
-      <c r="S34" s="42">
+      <c r="S34" s="34">
         <v>7.5086813000000002E-2</v>
       </c>
-      <c r="T34" s="39">
+      <c r="T34" s="31">
         <v>100</v>
       </c>
-      <c r="U34" s="42">
-        <v>0</v>
-      </c>
-      <c r="V34" s="42">
-        <v>0</v>
-      </c>
-      <c r="W34" s="39">
+      <c r="U34" s="34">
+        <v>0</v>
+      </c>
+      <c r="V34" s="34">
+        <v>0</v>
+      </c>
+      <c r="W34" s="31">
         <v>100</v>
       </c>
-      <c r="X34" s="42">
+      <c r="X34" s="34">
         <v>2.644927E-3</v>
       </c>
-      <c r="Y34" s="42">
+      <c r="Y34" s="34">
         <v>2.644927E-3</v>
       </c>
-      <c r="Z34" s="42">
+      <c r="Z34" s="34">
         <v>2.8800000000000002E-3</v>
       </c>
-      <c r="AA34" s="42">
+      <c r="AA34" s="34">
         <v>0.192</v>
       </c>
-      <c r="AB34" s="39">
+      <c r="AB34" s="31">
         <v>100</v>
       </c>
-      <c r="AC34" s="41">
+      <c r="AC34" s="33">
         <v>11</v>
       </c>
-      <c r="AD34" s="39">
+      <c r="AD34" s="31">
         <v>10854.593210000001</v>
       </c>
     </row>
@@ -10947,49 +11001,49 @@
       <c r="O35" t="s">
         <v>50</v>
       </c>
-      <c r="P35" s="42">
+      <c r="P35" s="34">
         <v>0.27102898600000003</v>
       </c>
-      <c r="Q35" s="42">
+      <c r="Q35" s="34">
         <v>4.4745095999999998E-2</v>
       </c>
-      <c r="R35" s="42">
+      <c r="R35" s="34">
         <v>0.27289521300000003</v>
       </c>
-      <c r="S35" s="42">
+      <c r="S35" s="34">
         <v>3.7710198E-2</v>
       </c>
-      <c r="T35" s="39">
+      <c r="T35" s="31">
         <v>89.886363639999999</v>
       </c>
-      <c r="U35" s="42">
-        <v>0</v>
-      </c>
-      <c r="V35" s="42">
-        <v>0</v>
-      </c>
-      <c r="W35" s="39">
+      <c r="U35" s="34">
+        <v>0</v>
+      </c>
+      <c r="V35" s="34">
+        <v>0</v>
+      </c>
+      <c r="W35" s="31">
         <v>100</v>
       </c>
-      <c r="X35" s="42">
-        <v>0</v>
-      </c>
-      <c r="Y35" s="42">
-        <v>0</v>
-      </c>
-      <c r="Z35" s="42">
-        <v>0</v>
-      </c>
-      <c r="AA35" s="42">
+      <c r="X35" s="34">
+        <v>0</v>
+      </c>
+      <c r="Y35" s="34">
+        <v>0</v>
+      </c>
+      <c r="Z35" s="34">
+        <v>0</v>
+      </c>
+      <c r="AA35" s="34">
         <v>0.93202499999999999</v>
       </c>
-      <c r="AB35" s="39">
+      <c r="AB35" s="31">
         <v>100</v>
       </c>
-      <c r="AC35" s="41">
+      <c r="AC35" s="33">
         <v>11</v>
       </c>
-      <c r="AD35" s="39">
+      <c r="AD35" s="31">
         <v>24341.61377</v>
       </c>
     </row>
@@ -10997,49 +11051,49 @@
       <c r="O36" t="s">
         <v>33</v>
       </c>
-      <c r="P36" s="42">
+      <c r="P36" s="34">
         <v>0.16763552700000001</v>
       </c>
-      <c r="Q36" s="42">
+      <c r="Q36" s="34">
         <v>7.8511710999999998E-2</v>
       </c>
-      <c r="R36" s="42">
+      <c r="R36" s="34">
         <v>0.16305029500000001</v>
       </c>
-      <c r="S36" s="42">
+      <c r="S36" s="34">
         <v>7.1120540999999995E-2</v>
       </c>
-      <c r="T36" s="39">
+      <c r="T36" s="31">
         <v>96.590909089999997</v>
       </c>
-      <c r="U36" s="42">
-        <v>0</v>
-      </c>
-      <c r="V36" s="42">
-        <v>0</v>
-      </c>
-      <c r="W36" s="39">
-        <v>0</v>
-      </c>
-      <c r="X36" s="42">
+      <c r="U36" s="34">
+        <v>0</v>
+      </c>
+      <c r="V36" s="34">
+        <v>0</v>
+      </c>
+      <c r="W36" s="31">
+        <v>0</v>
+      </c>
+      <c r="X36" s="34">
         <v>1.4738187E-2</v>
       </c>
-      <c r="Y36" s="42">
+      <c r="Y36" s="34">
         <v>1.4738187E-2</v>
       </c>
-      <c r="Z36" s="42">
+      <c r="Z36" s="34">
         <v>3.6259999999999999E-3</v>
       </c>
-      <c r="AA36" s="42">
+      <c r="AA36" s="34">
         <v>3.8163360000000002</v>
       </c>
-      <c r="AB36" s="39">
+      <c r="AB36" s="31">
         <v>92.613636360000001</v>
       </c>
-      <c r="AC36" s="41">
+      <c r="AC36" s="33">
         <v>10.1875</v>
       </c>
-      <c r="AD36" s="39">
+      <c r="AD36" s="31">
         <v>5104.3859670000002</v>
       </c>
     </row>
@@ -11047,49 +11101,49 @@
       <c r="O37" t="s">
         <v>32</v>
       </c>
-      <c r="P37" s="42">
+      <c r="P37" s="34">
         <v>6.9194680999999994E-2</v>
       </c>
-      <c r="Q37" s="42">
+      <c r="Q37" s="34">
         <v>6.8214596000000002E-2</v>
       </c>
-      <c r="R37" s="42">
+      <c r="R37" s="34">
         <v>5.8914656000000003E-2</v>
       </c>
-      <c r="S37" s="42">
+      <c r="S37" s="34">
         <v>3.5449247000000003E-2</v>
       </c>
-      <c r="T37" s="39">
-        <v>0</v>
-      </c>
-      <c r="U37" s="42">
-        <v>0</v>
-      </c>
-      <c r="V37" s="42">
-        <v>0</v>
-      </c>
-      <c r="W37" s="39">
+      <c r="T37" s="31">
+        <v>0</v>
+      </c>
+      <c r="U37" s="34">
+        <v>0</v>
+      </c>
+      <c r="V37" s="34">
+        <v>0</v>
+      </c>
+      <c r="W37" s="31">
         <v>100</v>
       </c>
-      <c r="X37" s="42">
+      <c r="X37" s="34">
         <v>2.644927E-3</v>
       </c>
-      <c r="Y37" s="42">
+      <c r="Y37" s="34">
         <v>2.644927E-3</v>
       </c>
-      <c r="Z37" s="42">
+      <c r="Z37" s="34">
         <v>1.1039999999999999E-2</v>
       </c>
-      <c r="AA37" s="42">
+      <c r="AA37" s="34">
         <v>0.378</v>
       </c>
-      <c r="AB37" s="39">
+      <c r="AB37" s="31">
         <v>100</v>
       </c>
-      <c r="AC37" s="41">
+      <c r="AC37" s="33">
         <v>11</v>
       </c>
-      <c r="AD37" s="39">
+      <c r="AD37" s="31">
         <v>24308.732680000001</v>
       </c>
     </row>
@@ -11097,49 +11151,49 @@
       <c r="O38" t="s">
         <v>34</v>
       </c>
-      <c r="P38" s="42">
+      <c r="P38" s="34">
         <v>0.55872443800000005</v>
       </c>
-      <c r="Q38" s="42">
+      <c r="Q38" s="34">
         <v>7.0912995000000006E-2</v>
       </c>
-      <c r="R38" s="42">
+      <c r="R38" s="34">
         <v>0.56479812600000001</v>
       </c>
-      <c r="S38" s="42">
+      <c r="S38" s="34">
         <v>7.1431786999999997E-2</v>
       </c>
-      <c r="T38" s="39">
-        <v>0</v>
-      </c>
-      <c r="U38" s="42">
-        <v>0</v>
-      </c>
-      <c r="V38" s="42">
-        <v>0</v>
-      </c>
-      <c r="W38" s="39">
+      <c r="T38" s="31">
+        <v>0</v>
+      </c>
+      <c r="U38" s="34">
+        <v>0</v>
+      </c>
+      <c r="V38" s="34">
+        <v>0</v>
+      </c>
+      <c r="W38" s="31">
         <v>100</v>
       </c>
-      <c r="X38" s="42">
+      <c r="X38" s="34">
         <v>1.2383979999999999E-3</v>
       </c>
-      <c r="Y38" s="42">
+      <c r="Y38" s="34">
         <v>1.2383979999999999E-3</v>
       </c>
-      <c r="Z38" s="42">
+      <c r="Z38" s="34">
         <v>1.1039999999999999E-2</v>
       </c>
-      <c r="AA38" s="42">
+      <c r="AA38" s="34">
         <v>0.13202</v>
       </c>
-      <c r="AB38" s="39">
+      <c r="AB38" s="31">
         <v>100</v>
       </c>
-      <c r="AC38" s="41">
+      <c r="AC38" s="33">
         <v>11</v>
       </c>
-      <c r="AD38" s="39">
+      <c r="AD38" s="31">
         <v>8681.5015750000002</v>
       </c>
     </row>
@@ -11152,49 +11206,49 @@
       <c r="O40" t="s">
         <v>36</v>
       </c>
-      <c r="P40" s="42">
+      <c r="P40" s="34">
         <v>6.9194711000000006E-2</v>
       </c>
-      <c r="Q40" s="42">
+      <c r="Q40" s="34">
         <v>6.8214580999999996E-2</v>
       </c>
-      <c r="R40" s="42">
+      <c r="R40" s="34">
         <v>5.8914682000000003E-2</v>
       </c>
-      <c r="S40" s="42">
+      <c r="S40" s="34">
         <v>3.5449245999999997E-2</v>
       </c>
-      <c r="T40" s="39">
-        <v>0</v>
-      </c>
-      <c r="U40" s="42">
-        <v>0</v>
-      </c>
-      <c r="V40" s="42">
-        <v>0</v>
-      </c>
-      <c r="W40" s="39">
+      <c r="T40" s="31">
+        <v>0</v>
+      </c>
+      <c r="U40" s="34">
+        <v>0</v>
+      </c>
+      <c r="V40" s="34">
+        <v>0</v>
+      </c>
+      <c r="W40" s="31">
         <v>100</v>
       </c>
-      <c r="X40" s="42">
+      <c r="X40" s="34">
         <v>2.644927E-3</v>
       </c>
-      <c r="Y40" s="42">
+      <c r="Y40" s="34">
         <v>2.644927E-3</v>
       </c>
-      <c r="Z40" s="42">
+      <c r="Z40" s="34">
         <v>1.1039999999999999E-2</v>
       </c>
-      <c r="AA40" s="42">
+      <c r="AA40" s="34">
         <v>0.35099999999999998</v>
       </c>
-      <c r="AB40" s="39">
+      <c r="AB40" s="31">
         <v>100</v>
       </c>
-      <c r="AC40" s="41">
+      <c r="AC40" s="33">
         <v>11</v>
       </c>
-      <c r="AD40" s="39">
+      <c r="AD40" s="31">
         <v>24308.737099999998</v>
       </c>
     </row>
@@ -11212,26 +11266,26 @@
       <c r="A44" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B44" s="31" t="s">
+      <c r="B44" s="35" t="s">
         <v>39</v>
       </c>
-      <c r="C44" s="32"/>
-      <c r="D44" s="33"/>
-      <c r="E44" s="32" t="s">
+      <c r="C44" s="36"/>
+      <c r="D44" s="37"/>
+      <c r="E44" s="36" t="s">
         <v>40</v>
       </c>
-      <c r="F44" s="32"/>
-      <c r="G44" s="33"/>
-      <c r="H44" s="32" t="s">
+      <c r="F44" s="36"/>
+      <c r="G44" s="37"/>
+      <c r="H44" s="36" t="s">
         <v>41</v>
       </c>
-      <c r="I44" s="32"/>
-      <c r="J44" s="32"/>
-      <c r="K44" s="31" t="s">
+      <c r="I44" s="36"/>
+      <c r="J44" s="36"/>
+      <c r="K44" s="35" t="s">
         <v>42</v>
       </c>
-      <c r="L44" s="32"/>
-      <c r="M44" s="32"/>
+      <c r="L44" s="36"/>
+      <c r="M44" s="36"/>
     </row>
     <row r="45" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A45" s="14" t="s">
@@ -11498,49 +11552,49 @@
       <c r="O55" t="s">
         <v>49</v>
       </c>
-      <c r="P55" s="42">
+      <c r="P55" s="34">
         <v>0.62736285400000003</v>
       </c>
-      <c r="Q55" s="42">
+      <c r="Q55" s="34">
         <v>7.1781017000000003E-2</v>
       </c>
-      <c r="R55" s="42">
+      <c r="R55" s="34">
         <v>0.63531370399999998</v>
       </c>
-      <c r="S55" s="42">
+      <c r="S55" s="34">
         <v>6.9879844999999996E-2</v>
       </c>
-      <c r="T55" s="39">
+      <c r="T55" s="31">
         <v>92.840909089999997</v>
       </c>
-      <c r="U55" s="42">
-        <v>0</v>
-      </c>
-      <c r="V55" s="42">
-        <v>0</v>
-      </c>
-      <c r="W55" s="39">
+      <c r="U55" s="34">
+        <v>0</v>
+      </c>
+      <c r="V55" s="34">
+        <v>0</v>
+      </c>
+      <c r="W55" s="31">
         <v>100</v>
       </c>
-      <c r="X55" s="42">
+      <c r="X55" s="34">
         <v>6.7561699999999999E-4</v>
       </c>
-      <c r="Y55" s="42">
+      <c r="Y55" s="34">
         <v>6.7561699999999999E-4</v>
       </c>
-      <c r="Z55" s="42">
+      <c r="Z55" s="34">
         <v>4.1599999999999996E-3</v>
       </c>
-      <c r="AA55" s="42">
+      <c r="AA55" s="34">
         <v>1.584E-2</v>
       </c>
-      <c r="AB55" s="39">
+      <c r="AB55" s="31">
         <v>100</v>
       </c>
-      <c r="AC55" s="41">
+      <c r="AC55" s="33">
         <v>11</v>
       </c>
-      <c r="AD55" s="39">
+      <c r="AD55" s="31">
         <v>3229.7740749999998</v>
       </c>
     </row>
@@ -11548,49 +11602,49 @@
       <c r="O56" t="s">
         <v>50</v>
       </c>
-      <c r="P56" s="42">
+      <c r="P56" s="34">
         <v>0.61607394599999998</v>
       </c>
-      <c r="Q56" s="42">
+      <c r="Q56" s="34">
         <v>7.4070856000000004E-2</v>
       </c>
-      <c r="R56" s="42">
+      <c r="R56" s="34">
         <v>0.62477324099999998</v>
       </c>
-      <c r="S56" s="42">
+      <c r="S56" s="34">
         <v>7.1897643999999997E-2</v>
       </c>
-      <c r="T56" s="39">
+      <c r="T56" s="31">
         <v>100</v>
       </c>
-      <c r="U56" s="42">
-        <v>0</v>
-      </c>
-      <c r="V56" s="42">
-        <v>0</v>
-      </c>
-      <c r="W56" s="39">
+      <c r="U56" s="34">
+        <v>0</v>
+      </c>
+      <c r="V56" s="34">
+        <v>0</v>
+      </c>
+      <c r="W56" s="31">
         <v>100</v>
       </c>
-      <c r="X56" s="42">
+      <c r="X56" s="34">
         <v>7.4172400000000003E-4</v>
       </c>
-      <c r="Y56" s="42">
+      <c r="Y56" s="34">
         <v>7.4172400000000003E-4</v>
       </c>
-      <c r="Z56" s="42">
+      <c r="Z56" s="34">
         <v>2.7999999999999998E-4</v>
       </c>
-      <c r="AA56" s="42">
+      <c r="AA56" s="34">
         <v>1.584E-2</v>
       </c>
-      <c r="AB56" s="39">
+      <c r="AB56" s="31">
         <v>100</v>
       </c>
-      <c r="AC56" s="41">
+      <c r="AC56" s="33">
         <v>11</v>
       </c>
-      <c r="AD56" s="39">
+      <c r="AD56" s="31">
         <v>3836.9429270000001</v>
       </c>
     </row>
@@ -11598,49 +11652,49 @@
       <c r="O57" t="s">
         <v>33</v>
       </c>
-      <c r="P57" s="42">
+      <c r="P57" s="34">
         <v>0.40469522800000002</v>
       </c>
-      <c r="Q57" s="42">
+      <c r="Q57" s="34">
         <v>6.9731839000000004E-2</v>
       </c>
-      <c r="R57" s="42">
+      <c r="R57" s="34">
         <v>0.40629886599999998</v>
       </c>
-      <c r="S57" s="42">
+      <c r="S57" s="34">
         <v>7.0271370999999999E-2</v>
       </c>
-      <c r="T57" s="39">
-        <v>0</v>
-      </c>
-      <c r="U57" s="42">
-        <v>0</v>
-      </c>
-      <c r="V57" s="42">
-        <v>0</v>
-      </c>
-      <c r="W57" s="39">
+      <c r="T57" s="31">
+        <v>0</v>
+      </c>
+      <c r="U57" s="34">
+        <v>0</v>
+      </c>
+      <c r="V57" s="34">
+        <v>0</v>
+      </c>
+      <c r="W57" s="31">
         <v>76.212121210000006</v>
       </c>
-      <c r="X57" s="42">
+      <c r="X57" s="34">
         <v>4.4247619999999996E-3</v>
       </c>
-      <c r="Y57" s="42">
+      <c r="Y57" s="34">
         <v>4.4247619999999996E-3</v>
       </c>
-      <c r="Z57" s="42">
+      <c r="Z57" s="34">
         <v>1.0880000000000001E-2</v>
       </c>
-      <c r="AA57" s="42">
+      <c r="AA57" s="34">
         <v>0.83638100000000004</v>
       </c>
-      <c r="AB57" s="39">
+      <c r="AB57" s="31">
         <v>100</v>
       </c>
-      <c r="AC57" s="41">
+      <c r="AC57" s="33">
         <v>11</v>
       </c>
-      <c r="AD57" s="39">
+      <c r="AD57" s="31">
         <v>3455.1726140000001</v>
       </c>
     </row>
@@ -11648,49 +11702,49 @@
       <c r="O58" t="s">
         <v>32</v>
       </c>
-      <c r="P58" s="42">
+      <c r="P58" s="34">
         <v>0.58641906600000004</v>
       </c>
-      <c r="Q58" s="42">
+      <c r="Q58" s="34">
         <v>7.4058140999999994E-2</v>
       </c>
-      <c r="R58" s="42">
+      <c r="R58" s="34">
         <v>0.59317042200000003</v>
       </c>
-      <c r="S58" s="42">
+      <c r="S58" s="34">
         <v>7.4066038000000001E-2</v>
       </c>
-      <c r="T58" s="39">
-        <v>0</v>
-      </c>
-      <c r="U58" s="42">
-        <v>0</v>
-      </c>
-      <c r="V58" s="42">
-        <v>0</v>
-      </c>
-      <c r="W58" s="39">
+      <c r="T58" s="31">
+        <v>0</v>
+      </c>
+      <c r="U58" s="34">
+        <v>0</v>
+      </c>
+      <c r="V58" s="34">
+        <v>0</v>
+      </c>
+      <c r="W58" s="31">
         <v>100</v>
       </c>
-      <c r="X58" s="42">
+      <c r="X58" s="34">
         <v>1.382154E-3</v>
       </c>
-      <c r="Y58" s="42">
+      <c r="Y58" s="34">
         <v>1.382154E-3</v>
       </c>
-      <c r="Z58" s="42">
+      <c r="Z58" s="34">
         <v>1.1039999999999999E-2</v>
       </c>
-      <c r="AA58" s="42">
+      <c r="AA58" s="34">
         <v>0.150672</v>
       </c>
-      <c r="AB58" s="39">
+      <c r="AB58" s="31">
         <v>100</v>
       </c>
-      <c r="AC58" s="41">
+      <c r="AC58" s="33">
         <v>11</v>
       </c>
-      <c r="AD58" s="39">
+      <c r="AD58" s="31">
         <v>9353.5133420000002</v>
       </c>
     </row>
@@ -11698,49 +11752,49 @@
       <c r="O59" t="s">
         <v>34</v>
       </c>
-      <c r="P59" s="42">
+      <c r="P59" s="34">
         <v>2.2153664E-2</v>
       </c>
-      <c r="Q59" s="42">
+      <c r="Q59" s="34">
         <v>6.8025735000000004E-2</v>
       </c>
-      <c r="R59" s="42">
+      <c r="R59" s="34">
         <v>5.5786159999999998E-3</v>
       </c>
-      <c r="S59" s="42">
+      <c r="S59" s="34">
         <v>3.6971740000000001E-3</v>
       </c>
-      <c r="T59" s="39">
-        <v>0</v>
-      </c>
-      <c r="U59" s="42">
-        <v>0</v>
-      </c>
-      <c r="V59" s="42">
-        <v>0</v>
-      </c>
-      <c r="W59" s="39">
-        <v>0</v>
-      </c>
-      <c r="X59" s="42">
+      <c r="T59" s="31">
+        <v>0</v>
+      </c>
+      <c r="U59" s="34">
+        <v>0</v>
+      </c>
+      <c r="V59" s="34">
+        <v>0</v>
+      </c>
+      <c r="W59" s="31">
+        <v>0</v>
+      </c>
+      <c r="X59" s="34">
         <v>1.4738187E-2</v>
       </c>
-      <c r="Y59" s="42">
+      <c r="Y59" s="34">
         <v>1.4738187E-2</v>
       </c>
-      <c r="Z59" s="42">
+      <c r="Z59" s="34">
         <v>1.1039999999999999E-2</v>
       </c>
-      <c r="AA59" s="42">
+      <c r="AA59" s="34">
         <v>3.8163360000000002</v>
       </c>
-      <c r="AB59" s="39">
+      <c r="AB59" s="31">
         <v>7.348484848</v>
       </c>
-      <c r="AC59" s="41">
+      <c r="AC59" s="33">
         <v>0.80833333299999999</v>
       </c>
-      <c r="AD59" s="39">
+      <c r="AD59" s="31">
         <v>16727.630369999999</v>
       </c>
     </row>
@@ -11768,26 +11822,26 @@
       <c r="A65" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="B65" s="34" t="s">
+      <c r="B65" s="38" t="s">
         <v>39</v>
       </c>
-      <c r="C65" s="35"/>
-      <c r="D65" s="36"/>
-      <c r="E65" s="37" t="s">
+      <c r="C65" s="39"/>
+      <c r="D65" s="40"/>
+      <c r="E65" s="41" t="s">
         <v>40</v>
       </c>
-      <c r="F65" s="35"/>
-      <c r="G65" s="36"/>
-      <c r="H65" s="37" t="s">
+      <c r="F65" s="39"/>
+      <c r="G65" s="40"/>
+      <c r="H65" s="41" t="s">
         <v>41</v>
       </c>
-      <c r="I65" s="35"/>
-      <c r="J65" s="38"/>
-      <c r="K65" s="34" t="s">
+      <c r="I65" s="39"/>
+      <c r="J65" s="42"/>
+      <c r="K65" s="38" t="s">
         <v>42</v>
       </c>
-      <c r="L65" s="35"/>
-      <c r="M65" s="35"/>
+      <c r="L65" s="39"/>
+      <c r="M65" s="39"/>
       <c r="N65" s="21"/>
       <c r="O65" s="21"/>
     </row>
@@ -12165,49 +12219,49 @@
       <c r="O76" t="s">
         <v>49</v>
       </c>
-      <c r="P76" s="42">
+      <c r="P76" s="34">
         <v>0.60743649200000005</v>
       </c>
-      <c r="Q76" s="42">
+      <c r="Q76" s="34">
         <v>0.33138423</v>
       </c>
-      <c r="R76" s="42">
+      <c r="R76" s="34">
         <v>0.63648149200000004</v>
       </c>
-      <c r="S76" s="42">
+      <c r="S76" s="34">
         <v>0.33051121100000003</v>
       </c>
-      <c r="T76" s="39">
+      <c r="T76" s="31">
         <v>70.60606061</v>
       </c>
-      <c r="U76" s="42">
+      <c r="U76" s="34">
         <v>3.6358300000000001E-3</v>
       </c>
-      <c r="V76" s="42">
+      <c r="V76" s="34">
         <v>3.6358300000000001E-3</v>
       </c>
-      <c r="W76" s="39">
+      <c r="W76" s="31">
         <v>100</v>
       </c>
-      <c r="X76" s="42">
+      <c r="X76" s="34">
         <v>1.03353E-2</v>
       </c>
-      <c r="Y76" s="42">
+      <c r="Y76" s="34">
         <v>1.03353E-2</v>
       </c>
-      <c r="Z76" s="42">
+      <c r="Z76" s="34">
         <v>8.7999999999999995E-2</v>
       </c>
-      <c r="AA76" s="42">
+      <c r="AA76" s="34">
         <v>0.28320000000000001</v>
       </c>
-      <c r="AB76" s="39">
+      <c r="AB76" s="31">
         <v>100</v>
       </c>
-      <c r="AC76" s="41">
+      <c r="AC76" s="33">
         <v>11</v>
       </c>
-      <c r="AD76" s="39">
+      <c r="AD76" s="31">
         <v>24321.607189999999</v>
       </c>
     </row>
@@ -12229,49 +12283,49 @@
       <c r="O77" t="s">
         <v>50</v>
       </c>
-      <c r="P77" s="42">
+      <c r="P77" s="34">
         <v>0.60830025099999996</v>
       </c>
-      <c r="Q77" s="42">
+      <c r="Q77" s="34">
         <v>0.33140337600000003</v>
       </c>
-      <c r="R77" s="42">
+      <c r="R77" s="34">
         <v>0.63934216300000002</v>
       </c>
-      <c r="S77" s="42">
+      <c r="S77" s="34">
         <v>0.328036889</v>
       </c>
-      <c r="T77" s="39">
+      <c r="T77" s="31">
         <v>70.60606061</v>
       </c>
-      <c r="U77" s="42">
+      <c r="U77" s="34">
         <v>2.9528549999999999E-3</v>
       </c>
-      <c r="V77" s="42">
+      <c r="V77" s="34">
         <v>2.9528549999999999E-3</v>
       </c>
-      <c r="W77" s="39">
+      <c r="W77" s="31">
         <v>100</v>
       </c>
-      <c r="X77" s="42">
+      <c r="X77" s="34">
         <v>1.0672749E-2</v>
       </c>
-      <c r="Y77" s="42">
+      <c r="Y77" s="34">
         <v>1.0672749E-2</v>
       </c>
-      <c r="Z77" s="42">
+      <c r="Z77" s="34">
         <v>0.08</v>
       </c>
-      <c r="AA77" s="42">
+      <c r="AA77" s="34">
         <v>0.30359999999999998</v>
       </c>
-      <c r="AB77" s="39">
+      <c r="AB77" s="31">
         <v>100</v>
       </c>
-      <c r="AC77" s="41">
+      <c r="AC77" s="33">
         <v>11</v>
       </c>
-      <c r="AD77" s="39">
+      <c r="AD77" s="31">
         <v>25447.67641</v>
       </c>
     </row>
@@ -12293,49 +12347,49 @@
       <c r="O78" t="s">
         <v>33</v>
       </c>
-      <c r="P78" s="42">
+      <c r="P78" s="34">
         <v>7.9489345000000003E-2</v>
       </c>
-      <c r="Q78" s="42">
+      <c r="Q78" s="34">
         <v>0.108876977</v>
       </c>
-      <c r="R78" s="42">
+      <c r="R78" s="34">
         <v>5.7906882E-2</v>
       </c>
-      <c r="S78" s="42">
+      <c r="S78" s="34">
         <v>7.2164350000000002E-2</v>
       </c>
-      <c r="T78" s="39">
-        <v>0</v>
-      </c>
-      <c r="U78" s="42">
+      <c r="T78" s="31">
+        <v>0</v>
+      </c>
+      <c r="U78" s="34">
         <v>7.5502099999999999E-3</v>
       </c>
-      <c r="V78" s="42">
+      <c r="V78" s="34">
         <v>7.5502099999999999E-3</v>
       </c>
-      <c r="W78" s="39">
+      <c r="W78" s="31">
         <v>15.3030303</v>
       </c>
-      <c r="X78" s="42">
+      <c r="X78" s="34">
         <v>1.2874299000000001E-2</v>
       </c>
-      <c r="Y78" s="42">
+      <c r="Y78" s="34">
         <v>1.2874299000000001E-2</v>
       </c>
-      <c r="Z78" s="42">
+      <c r="Z78" s="34">
         <v>0.29520000000000002</v>
       </c>
-      <c r="AA78" s="42">
+      <c r="AA78" s="34">
         <v>0.84</v>
       </c>
-      <c r="AB78" s="39">
+      <c r="AB78" s="31">
         <v>41.363636360000001</v>
       </c>
-      <c r="AC78" s="41">
+      <c r="AC78" s="33">
         <v>4.55</v>
       </c>
-      <c r="AD78" s="39">
+      <c r="AD78" s="31">
         <v>17572.518039999999</v>
       </c>
     </row>
@@ -12357,49 +12411,49 @@
       <c r="O79" t="s">
         <v>32</v>
       </c>
-      <c r="P79" s="42">
+      <c r="P79" s="34">
         <v>7.9618703999999998E-2</v>
       </c>
-      <c r="Q79" s="42">
+      <c r="Q79" s="34">
         <v>0.103620223</v>
       </c>
-      <c r="R79" s="42">
+      <c r="R79" s="34">
         <v>5.8641828E-2</v>
       </c>
-      <c r="S79" s="42">
+      <c r="S79" s="34">
         <v>7.1932098E-2</v>
       </c>
-      <c r="T79" s="39">
-        <v>0</v>
-      </c>
-      <c r="U79" s="42">
+      <c r="T79" s="31">
+        <v>0</v>
+      </c>
+      <c r="U79" s="34">
         <v>7.5502099999999999E-3</v>
       </c>
-      <c r="V79" s="42">
+      <c r="V79" s="34">
         <v>7.5502099999999999E-3</v>
       </c>
-      <c r="W79" s="39">
+      <c r="W79" s="31">
         <v>14.621212119999999</v>
       </c>
-      <c r="X79" s="42">
+      <c r="X79" s="34">
         <v>1.2874299000000001E-2</v>
       </c>
-      <c r="Y79" s="42">
+      <c r="Y79" s="34">
         <v>1.2874299000000001E-2</v>
       </c>
-      <c r="Z79" s="42">
+      <c r="Z79" s="34">
         <v>0.29520000000000002</v>
       </c>
-      <c r="AA79" s="42">
+      <c r="AA79" s="34">
         <v>1.1305000000000001</v>
       </c>
-      <c r="AB79" s="39">
+      <c r="AB79" s="31">
         <v>42.765151520000003</v>
       </c>
-      <c r="AC79" s="41">
+      <c r="AC79" s="33">
         <v>4.704166667</v>
       </c>
-      <c r="AD79" s="39">
+      <c r="AD79" s="31">
         <v>17021.89831</v>
       </c>
     </row>
@@ -12421,49 +12475,49 @@
       <c r="O80" t="s">
         <v>34</v>
       </c>
-      <c r="P80" s="42">
+      <c r="P80" s="34">
         <v>2.4642293999999999E-2</v>
       </c>
-      <c r="Q80" s="42">
+      <c r="Q80" s="34">
         <v>7.4684096000000005E-2</v>
       </c>
-      <c r="R80" s="42">
+      <c r="R80" s="34">
         <v>6.3402049999999998E-3</v>
       </c>
-      <c r="S80" s="42">
+      <c r="S80" s="34">
         <v>5.4095860000000001E-3</v>
       </c>
-      <c r="T80" s="39">
-        <v>0</v>
-      </c>
-      <c r="U80" s="42">
+      <c r="T80" s="31">
+        <v>0</v>
+      </c>
+      <c r="U80" s="34">
         <v>7.5502099999999999E-3</v>
       </c>
-      <c r="V80" s="42">
+      <c r="V80" s="34">
         <v>7.5502099999999999E-3</v>
       </c>
-      <c r="W80" s="39">
+      <c r="W80" s="31">
         <v>8.5606060609999997</v>
       </c>
-      <c r="X80" s="42">
+      <c r="X80" s="34">
         <v>1.4027168E-2</v>
       </c>
-      <c r="Y80" s="42">
+      <c r="Y80" s="34">
         <v>1.4027168E-2</v>
       </c>
-      <c r="Z80" s="42">
+      <c r="Z80" s="34">
         <v>0.29520000000000002</v>
       </c>
-      <c r="AA80" s="42">
+      <c r="AA80" s="34">
         <v>1.5960000000000001</v>
       </c>
-      <c r="AB80" s="39">
+      <c r="AB80" s="31">
         <v>20.795454549999999</v>
       </c>
-      <c r="AC80" s="41">
+      <c r="AC80" s="33">
         <v>2.2875000000000001</v>
       </c>
-      <c r="AD80" s="39">
+      <c r="AD80" s="31">
         <v>16124.11807</v>
       </c>
     </row>
@@ -12504,49 +12558,49 @@
       <c r="O82" t="s">
         <v>36</v>
       </c>
-      <c r="P82" s="42">
+      <c r="P82" s="34">
         <v>2.4642293999999999E-2</v>
       </c>
-      <c r="Q82" s="42">
+      <c r="Q82" s="34">
         <v>7.4684096000000005E-2</v>
       </c>
-      <c r="R82" s="42">
+      <c r="R82" s="34">
         <v>6.3402049999999998E-3</v>
       </c>
-      <c r="S82" s="42">
+      <c r="S82" s="34">
         <v>5.4095860000000001E-3</v>
       </c>
-      <c r="T82" s="39">
-        <v>0</v>
-      </c>
-      <c r="U82" s="42">
+      <c r="T82" s="31">
+        <v>0</v>
+      </c>
+      <c r="U82" s="34">
         <v>7.5502099999999999E-3</v>
       </c>
-      <c r="V82" s="42">
+      <c r="V82" s="34">
         <v>7.5502099999999999E-3</v>
       </c>
-      <c r="W82" s="39">
+      <c r="W82" s="31">
         <v>8.5606060609999997</v>
       </c>
-      <c r="X82" s="42">
+      <c r="X82" s="34">
         <v>1.4027168E-2</v>
       </c>
-      <c r="Y82" s="42">
+      <c r="Y82" s="34">
         <v>1.4027168E-2</v>
       </c>
-      <c r="Z82" s="42">
+      <c r="Z82" s="34">
         <v>0.29520000000000002</v>
       </c>
-      <c r="AA82" s="42">
+      <c r="AA82" s="34">
         <v>1.5960000000000001</v>
       </c>
-      <c r="AB82" s="39">
+      <c r="AB82" s="31">
         <v>20.795454549999999</v>
       </c>
-      <c r="AC82" s="41">
+      <c r="AC82" s="33">
         <v>2.2875000000000001</v>
       </c>
-      <c r="AD82" s="39">
+      <c r="AD82" s="31">
         <v>16124.11807</v>
       </c>
     </row>
@@ -12554,54 +12608,62 @@
       <c r="O83" t="s">
         <v>37</v>
       </c>
-      <c r="P83" s="42">
+      <c r="P83" s="34">
         <v>2.4642313999999998E-2</v>
       </c>
-      <c r="Q83" s="42">
+      <c r="Q83" s="34">
         <v>7.4684087999999996E-2</v>
       </c>
-      <c r="R83" s="42">
+      <c r="R83" s="34">
         <v>6.340226E-3</v>
       </c>
-      <c r="S83" s="42">
+      <c r="S83" s="34">
         <v>5.4095510000000003E-3</v>
       </c>
-      <c r="T83" s="39">
-        <v>0</v>
-      </c>
-      <c r="U83" s="42">
+      <c r="T83" s="31">
+        <v>0</v>
+      </c>
+      <c r="U83" s="34">
         <v>7.5502099999999999E-3</v>
       </c>
-      <c r="V83" s="42">
+      <c r="V83" s="34">
         <v>7.5502099999999999E-3</v>
       </c>
-      <c r="W83" s="39">
+      <c r="W83" s="31">
         <v>8.5606060609999997</v>
       </c>
-      <c r="X83" s="42">
+      <c r="X83" s="34">
         <v>1.4027168E-2</v>
       </c>
-      <c r="Y83" s="42">
+      <c r="Y83" s="34">
         <v>1.4027168E-2</v>
       </c>
-      <c r="Z83" s="42">
+      <c r="Z83" s="34">
         <v>0.29520000000000002</v>
       </c>
-      <c r="AA83" s="42">
+      <c r="AA83" s="34">
         <v>1.444</v>
       </c>
-      <c r="AB83" s="39">
+      <c r="AB83" s="31">
         <v>20.9469697</v>
       </c>
-      <c r="AC83" s="41">
+      <c r="AC83" s="33">
         <v>2.3041666670000001</v>
       </c>
-      <c r="AD83" s="39">
+      <c r="AD83" s="31">
         <v>16124.12119</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="B44:D44"/>
+    <mergeCell ref="E44:G44"/>
+    <mergeCell ref="H44:J44"/>
+    <mergeCell ref="K44:M44"/>
+    <mergeCell ref="B65:D65"/>
+    <mergeCell ref="E65:G65"/>
+    <mergeCell ref="H65:J65"/>
+    <mergeCell ref="K65:M65"/>
     <mergeCell ref="B2:D2"/>
     <mergeCell ref="E2:G2"/>
     <mergeCell ref="H2:J2"/>
@@ -12610,14 +12672,6 @@
     <mergeCell ref="E23:G23"/>
     <mergeCell ref="H23:J23"/>
     <mergeCell ref="K23:M23"/>
-    <mergeCell ref="B44:D44"/>
-    <mergeCell ref="E44:G44"/>
-    <mergeCell ref="H44:J44"/>
-    <mergeCell ref="K44:M44"/>
-    <mergeCell ref="B65:D65"/>
-    <mergeCell ref="E65:G65"/>
-    <mergeCell ref="H65:J65"/>
-    <mergeCell ref="K65:M65"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>

<commit_message>
removed Jax 0.9 forcing and plot names txt for appendix 3
</commit_message>
<xml_diff>
--- a/results/compiled results.xlsx
+++ b/results/compiled results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\elish\Desktop\Aims Project\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C754F34-DD0B-4B78-87CD-30C401DE1700}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{328B73AB-1AC0-4BCD-9E3C-AF7DFC5CD9B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{DA4D96B0-492C-4945-A9C4-EFCA6D6BC722}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{DA4D96B0-492C-4945-A9C4-EFCA6D6BC722}"/>
   </bookViews>
   <sheets>
     <sheet name="Dynamic results" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="733" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="733" uniqueCount="83">
   <si>
     <t xml:space="preserve">Model </t>
   </si>
@@ -290,6 +290,9 @@
   <si>
     <t>Qwen 3.5 35b</t>
   </si>
+  <si>
+    <t xml:space="preserve">$\mathcal{C}vol_{wb}~(m^3)$ </t>
+  </si>
 </sst>
 </file>
 
@@ -515,7 +518,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="92">
+  <cellXfs count="91">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -709,6 +712,30 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="14" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -733,33 +760,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="14" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1130,26 +1130,26 @@
       <c r="A2" s="67" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="69" t="s">
+      <c r="B2" s="83" t="s">
         <v>24</v>
       </c>
-      <c r="C2" s="70"/>
-      <c r="D2" s="71"/>
-      <c r="E2" s="70" t="s">
+      <c r="C2" s="84"/>
+      <c r="D2" s="85"/>
+      <c r="E2" s="84" t="s">
         <v>25</v>
       </c>
-      <c r="F2" s="70"/>
-      <c r="G2" s="71"/>
-      <c r="H2" s="70" t="s">
+      <c r="F2" s="84"/>
+      <c r="G2" s="85"/>
+      <c r="H2" s="84" t="s">
         <v>26</v>
       </c>
-      <c r="I2" s="70"/>
-      <c r="J2" s="70"/>
-      <c r="K2" s="69" t="s">
+      <c r="I2" s="84"/>
+      <c r="J2" s="84"/>
+      <c r="K2" s="83" t="s">
         <v>27</v>
       </c>
-      <c r="L2" s="70"/>
-      <c r="M2" s="70"/>
+      <c r="L2" s="84"/>
+      <c r="M2" s="84"/>
       <c r="N2" s="1" t="s">
         <v>56</v>
       </c>
@@ -1593,7 +1593,7 @@
       <c r="T14" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="U14" s="79" t="s">
+      <c r="U14" s="71" t="s">
         <v>15</v>
       </c>
       <c r="V14" s="3" t="s">
@@ -1643,7 +1643,7 @@
       <c r="T15" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="U15" s="80" t="s">
+      <c r="U15" s="72" t="s">
         <v>71</v>
       </c>
       <c r="V15" s="49" t="s">
@@ -1690,10 +1690,10 @@
       <c r="S16" s="2">
         <v>0</v>
       </c>
-      <c r="T16" s="77">
-        <v>0</v>
-      </c>
-      <c r="U16" s="79">
+      <c r="T16" s="69">
+        <v>0</v>
+      </c>
+      <c r="U16" s="71">
         <v>0</v>
       </c>
       <c r="V16" s="3">
@@ -1737,7 +1737,7 @@
       <c r="T17" s="59" t="s">
         <v>34</v>
       </c>
-      <c r="U17" s="81" t="s">
+      <c r="U17" s="73" t="s">
         <v>34</v>
       </c>
       <c r="V17" s="34" t="s">
@@ -1784,10 +1784,10 @@
       <c r="S18" s="10">
         <v>0</v>
       </c>
-      <c r="T18" s="78">
-        <v>0</v>
-      </c>
-      <c r="U18" s="80">
+      <c r="T18" s="70">
+        <v>0</v>
+      </c>
+      <c r="U18" s="72">
         <v>0</v>
       </c>
       <c r="V18" s="49">
@@ -1828,10 +1828,10 @@
       <c r="S19" s="2">
         <v>0</v>
       </c>
-      <c r="T19" s="77">
+      <c r="T19" s="69">
         <v>100</v>
       </c>
-      <c r="U19" s="79">
+      <c r="U19" s="71">
         <v>0</v>
       </c>
       <c r="V19" s="3">
@@ -1872,10 +1872,10 @@
       <c r="S20" s="10">
         <v>0</v>
       </c>
-      <c r="T20" s="78">
-        <v>0</v>
-      </c>
-      <c r="U20" s="80">
+      <c r="T20" s="70">
+        <v>0</v>
+      </c>
+      <c r="U20" s="72">
         <v>0</v>
       </c>
       <c r="V20" s="49">
@@ -1916,10 +1916,10 @@
       <c r="S21" s="2">
         <v>0</v>
       </c>
-      <c r="T21" s="77">
-        <v>0</v>
-      </c>
-      <c r="U21" s="79">
+      <c r="T21" s="69">
+        <v>0</v>
+      </c>
+      <c r="U21" s="71">
         <v>0</v>
       </c>
       <c r="V21" s="3">
@@ -1960,10 +1960,10 @@
       <c r="S22" s="2">
         <v>0</v>
       </c>
-      <c r="T22" s="77">
+      <c r="T22" s="69">
         <v>100</v>
       </c>
-      <c r="U22" s="79">
+      <c r="U22" s="71">
         <v>0</v>
       </c>
       <c r="V22" s="3">
@@ -2004,10 +2004,10 @@
       <c r="S23" s="10">
         <v>0</v>
       </c>
-      <c r="T23" s="78">
-        <v>0</v>
-      </c>
-      <c r="U23" s="80">
+      <c r="T23" s="70">
+        <v>0</v>
+      </c>
+      <c r="U23" s="72">
         <v>0</v>
       </c>
       <c r="V23" s="49">
@@ -2045,26 +2045,26 @@
       <c r="A27" s="67" t="s">
         <v>0</v>
       </c>
-      <c r="B27" s="69" t="s">
+      <c r="B27" s="83" t="s">
         <v>24</v>
       </c>
-      <c r="C27" s="70"/>
-      <c r="D27" s="71"/>
-      <c r="E27" s="70" t="s">
+      <c r="C27" s="84"/>
+      <c r="D27" s="85"/>
+      <c r="E27" s="84" t="s">
         <v>25</v>
       </c>
-      <c r="F27" s="70"/>
-      <c r="G27" s="71"/>
-      <c r="H27" s="70" t="s">
+      <c r="F27" s="84"/>
+      <c r="G27" s="85"/>
+      <c r="H27" s="84" t="s">
         <v>26</v>
       </c>
-      <c r="I27" s="70"/>
-      <c r="J27" s="70"/>
-      <c r="K27" s="69" t="s">
+      <c r="I27" s="84"/>
+      <c r="J27" s="84"/>
+      <c r="K27" s="83" t="s">
         <v>27</v>
       </c>
-      <c r="L27" s="70"/>
-      <c r="M27" s="70"/>
+      <c r="L27" s="84"/>
+      <c r="M27" s="84"/>
       <c r="O27" s="34" t="s">
         <v>34</v>
       </c>
@@ -2431,7 +2431,7 @@
       <c r="T37" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="U37" s="80" t="s">
+      <c r="U37" s="72" t="s">
         <v>71</v>
       </c>
       <c r="V37" s="49" t="s">
@@ -2469,7 +2469,7 @@
       <c r="S38" s="2">
         <v>65.245454545454507</v>
       </c>
-      <c r="T38" s="77">
+      <c r="T38" s="69">
         <v>100</v>
       </c>
       <c r="U38" s="12">
@@ -2515,7 +2515,7 @@
       <c r="S39" s="2">
         <v>0</v>
       </c>
-      <c r="T39" s="77">
+      <c r="T39" s="69">
         <v>100</v>
       </c>
       <c r="U39" s="63">
@@ -2559,7 +2559,7 @@
       <c r="S40" s="10">
         <v>79.445454545454496</v>
       </c>
-      <c r="T40" s="78">
+      <c r="T40" s="70">
         <v>0</v>
       </c>
       <c r="U40" s="66">
@@ -2603,7 +2603,7 @@
       <c r="S41" s="2">
         <v>0</v>
       </c>
-      <c r="T41" s="77">
+      <c r="T41" s="69">
         <v>100</v>
       </c>
       <c r="U41" s="63">
@@ -2647,7 +2647,7 @@
       <c r="S42" s="10">
         <v>0</v>
       </c>
-      <c r="T42" s="78">
+      <c r="T42" s="70">
         <v>100</v>
       </c>
       <c r="U42" s="66">
@@ -2691,7 +2691,7 @@
       <c r="S43" s="2">
         <v>0</v>
       </c>
-      <c r="T43" s="77">
+      <c r="T43" s="69">
         <v>100</v>
       </c>
       <c r="U43" s="63">
@@ -2735,7 +2735,7 @@
       <c r="S44" s="2">
         <v>0</v>
       </c>
-      <c r="T44" s="77">
+      <c r="T44" s="69">
         <v>100</v>
       </c>
       <c r="U44" s="63">
@@ -2779,7 +2779,7 @@
       <c r="S45" s="10">
         <v>0</v>
       </c>
-      <c r="T45" s="78">
+      <c r="T45" s="70">
         <v>0</v>
       </c>
       <c r="U45" s="66">
@@ -2814,26 +2814,26 @@
       <c r="A47" s="67" t="s">
         <v>0</v>
       </c>
-      <c r="B47" s="69" t="s">
+      <c r="B47" s="83" t="s">
         <v>24</v>
       </c>
-      <c r="C47" s="70"/>
-      <c r="D47" s="71"/>
-      <c r="E47" s="70" t="s">
+      <c r="C47" s="84"/>
+      <c r="D47" s="85"/>
+      <c r="E47" s="84" t="s">
         <v>25</v>
       </c>
-      <c r="F47" s="70"/>
-      <c r="G47" s="71"/>
-      <c r="H47" s="70" t="s">
+      <c r="F47" s="84"/>
+      <c r="G47" s="85"/>
+      <c r="H47" s="84" t="s">
         <v>26</v>
       </c>
-      <c r="I47" s="70"/>
-      <c r="J47" s="70"/>
-      <c r="K47" s="69" t="s">
+      <c r="I47" s="84"/>
+      <c r="J47" s="84"/>
+      <c r="K47" s="83" t="s">
         <v>27</v>
       </c>
-      <c r="L47" s="70"/>
-      <c r="M47" s="70"/>
+      <c r="L47" s="84"/>
+      <c r="M47" s="84"/>
       <c r="T47" s="31"/>
     </row>
     <row r="48" spans="1:29" x14ac:dyDescent="0.3">
@@ -3200,7 +3200,7 @@
       <c r="T58" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="U58" s="80" t="s">
+      <c r="U58" s="72" t="s">
         <v>71</v>
       </c>
       <c r="V58" s="49" t="s">
@@ -3238,7 +3238,7 @@
       <c r="S59" s="2">
         <v>0</v>
       </c>
-      <c r="T59" s="77">
+      <c r="T59" s="69">
         <v>100</v>
       </c>
       <c r="U59" s="63">
@@ -3282,7 +3282,7 @@
       <c r="S60" s="2">
         <v>100</v>
       </c>
-      <c r="T60" s="77">
+      <c r="T60" s="69">
         <v>100</v>
       </c>
       <c r="U60" s="63">
@@ -3326,7 +3326,7 @@
       <c r="S61" s="10">
         <v>0</v>
       </c>
-      <c r="T61" s="78">
+      <c r="T61" s="70">
         <v>100</v>
       </c>
       <c r="U61" s="66">
@@ -3370,7 +3370,7 @@
       <c r="S62" s="2">
         <v>0</v>
       </c>
-      <c r="T62" s="77">
+      <c r="T62" s="69">
         <v>100</v>
       </c>
       <c r="U62" s="63">
@@ -3414,7 +3414,7 @@
       <c r="S63" s="10">
         <v>0</v>
       </c>
-      <c r="T63" s="78">
+      <c r="T63" s="70">
         <v>0</v>
       </c>
       <c r="U63" s="66">
@@ -3458,7 +3458,7 @@
       <c r="S64" s="2">
         <v>0</v>
       </c>
-      <c r="T64" s="77">
+      <c r="T64" s="69">
         <v>0</v>
       </c>
       <c r="U64" s="63">
@@ -3502,7 +3502,7 @@
       <c r="S65" s="2">
         <v>0</v>
       </c>
-      <c r="T65" s="77">
+      <c r="T65" s="69">
         <v>100</v>
       </c>
       <c r="U65" s="63">
@@ -3546,7 +3546,7 @@
       <c r="S66" s="10">
         <v>0</v>
       </c>
-      <c r="T66" s="78">
+      <c r="T66" s="70">
         <v>0</v>
       </c>
       <c r="U66" s="66">
@@ -3587,26 +3587,26 @@
       <c r="A70" s="67" t="s">
         <v>0</v>
       </c>
-      <c r="B70" s="69" t="s">
+      <c r="B70" s="83" t="s">
         <v>24</v>
       </c>
-      <c r="C70" s="70"/>
-      <c r="D70" s="71"/>
-      <c r="E70" s="70" t="s">
+      <c r="C70" s="84"/>
+      <c r="D70" s="85"/>
+      <c r="E70" s="84" t="s">
         <v>25</v>
       </c>
-      <c r="F70" s="70"/>
-      <c r="G70" s="71"/>
-      <c r="H70" s="70" t="s">
+      <c r="F70" s="84"/>
+      <c r="G70" s="85"/>
+      <c r="H70" s="84" t="s">
         <v>26</v>
       </c>
-      <c r="I70" s="70"/>
-      <c r="J70" s="70"/>
-      <c r="K70" s="69" t="s">
+      <c r="I70" s="84"/>
+      <c r="J70" s="84"/>
+      <c r="K70" s="83" t="s">
         <v>27</v>
       </c>
-      <c r="L70" s="70"/>
-      <c r="M70" s="70"/>
+      <c r="L70" s="84"/>
+      <c r="M70" s="84"/>
       <c r="T70" s="31"/>
     </row>
     <row r="71" spans="1:27" x14ac:dyDescent="0.3">
@@ -3970,7 +3970,7 @@
       <c r="T80" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="U80" s="80" t="s">
+      <c r="U80" s="72" t="s">
         <v>71</v>
       </c>
       <c r="V80" s="49" t="s">
@@ -4020,7 +4020,7 @@
       <c r="S81" s="2">
         <v>0</v>
       </c>
-      <c r="T81" s="77">
+      <c r="T81" s="69">
         <v>100</v>
       </c>
       <c r="U81" s="63">
@@ -4076,7 +4076,7 @@
       <c r="S82" s="2">
         <v>0</v>
       </c>
-      <c r="T82" s="77">
+      <c r="T82" s="69">
         <v>44.045454545454497</v>
       </c>
       <c r="U82" s="63">
@@ -4132,7 +4132,7 @@
       <c r="S83" s="10">
         <v>0</v>
       </c>
-      <c r="T83" s="78">
+      <c r="T83" s="70">
         <v>0</v>
       </c>
       <c r="U83" s="66">
@@ -4188,7 +4188,7 @@
       <c r="S84" s="2">
         <v>0</v>
       </c>
-      <c r="T84" s="77">
+      <c r="T84" s="69">
         <v>100</v>
       </c>
       <c r="U84" s="63">
@@ -4244,7 +4244,7 @@
       <c r="S85" s="10">
         <v>0</v>
       </c>
-      <c r="T85" s="78">
+      <c r="T85" s="70">
         <v>19.063636363636299</v>
       </c>
       <c r="U85" s="66">
@@ -4303,7 +4303,7 @@
       <c r="T86" s="59" t="s">
         <v>34</v>
       </c>
-      <c r="U86" s="81" t="s">
+      <c r="U86" s="73" t="s">
         <v>34</v>
       </c>
       <c r="V86" s="34" t="s">
@@ -4353,7 +4353,7 @@
       <c r="S87" s="2">
         <v>0</v>
       </c>
-      <c r="T87" s="77">
+      <c r="T87" s="69">
         <v>19.063636363636299</v>
       </c>
       <c r="U87" s="63">
@@ -4397,7 +4397,7 @@
       <c r="S88" s="10">
         <v>0</v>
       </c>
-      <c r="T88" s="78">
+      <c r="T88" s="70">
         <v>19.063636363636299</v>
       </c>
       <c r="U88" s="66">
@@ -4424,6 +4424,14 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="E2:G2"/>
+    <mergeCell ref="H2:J2"/>
+    <mergeCell ref="K2:M2"/>
+    <mergeCell ref="B27:D27"/>
+    <mergeCell ref="E27:G27"/>
+    <mergeCell ref="H27:J27"/>
+    <mergeCell ref="K27:M27"/>
     <mergeCell ref="B70:D70"/>
     <mergeCell ref="E70:G70"/>
     <mergeCell ref="H70:J70"/>
@@ -4432,14 +4440,6 @@
     <mergeCell ref="E47:G47"/>
     <mergeCell ref="H47:J47"/>
     <mergeCell ref="K47:M47"/>
-    <mergeCell ref="B2:D2"/>
-    <mergeCell ref="E2:G2"/>
-    <mergeCell ref="H2:J2"/>
-    <mergeCell ref="K2:M2"/>
-    <mergeCell ref="B27:D27"/>
-    <mergeCell ref="E27:G27"/>
-    <mergeCell ref="H27:J27"/>
-    <mergeCell ref="K27:M27"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4837,14 +4837,14 @@
     <col min="16" max="18" width="12.44140625" style="3" customWidth="1"/>
     <col min="19" max="19" width="12.44140625" style="58" customWidth="1"/>
     <col min="20" max="20" width="8.88671875" style="31"/>
-    <col min="21" max="21" width="10.77734375" style="77" customWidth="1"/>
+    <col min="21" max="21" width="10.77734375" style="69" customWidth="1"/>
     <col min="22" max="22" width="14.5546875" style="3" customWidth="1"/>
     <col min="23" max="23" width="15.77734375" style="58" customWidth="1"/>
     <col min="24" max="24" width="12.44140625" style="3" customWidth="1"/>
     <col min="25" max="25" width="12.44140625" style="58" customWidth="1"/>
     <col min="26" max="26" width="13.77734375" style="31" customWidth="1"/>
     <col min="27" max="27" width="12.44140625" style="31" customWidth="1"/>
-    <col min="28" max="28" width="14.109375" style="86" customWidth="1"/>
+    <col min="28" max="28" width="14.109375" style="31" customWidth="1"/>
     <col min="30" max="31" width="12.44140625" style="3" customWidth="1"/>
   </cols>
   <sheetData>
@@ -4857,26 +4857,26 @@
       <c r="A2" s="67" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="69" t="s">
+      <c r="B2" s="83" t="s">
         <v>24</v>
       </c>
-      <c r="C2" s="70"/>
-      <c r="D2" s="71"/>
-      <c r="E2" s="70" t="s">
+      <c r="C2" s="84"/>
+      <c r="D2" s="85"/>
+      <c r="E2" s="84" t="s">
         <v>25</v>
       </c>
-      <c r="F2" s="70"/>
-      <c r="G2" s="71"/>
-      <c r="H2" s="70" t="s">
+      <c r="F2" s="84"/>
+      <c r="G2" s="85"/>
+      <c r="H2" s="84" t="s">
         <v>26</v>
       </c>
-      <c r="I2" s="70"/>
-      <c r="J2" s="70"/>
-      <c r="K2" s="69" t="s">
+      <c r="I2" s="84"/>
+      <c r="J2" s="84"/>
+      <c r="K2" s="83" t="s">
         <v>27</v>
       </c>
-      <c r="L2" s="70"/>
-      <c r="M2" s="70"/>
+      <c r="L2" s="84"/>
+      <c r="M2" s="84"/>
     </row>
     <row r="3" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
@@ -5198,7 +5198,7 @@
       <c r="T11" s="31" t="s">
         <v>70</v>
       </c>
-      <c r="U11" s="77" t="s">
+      <c r="U11" s="69" t="s">
         <v>72</v>
       </c>
       <c r="V11" s="3" t="s">
@@ -5219,7 +5219,7 @@
       <c r="AA11" s="31" t="s">
         <v>76</v>
       </c>
-      <c r="AB11" s="86" t="s">
+      <c r="AB11" s="31" t="s">
         <v>42</v>
       </c>
       <c r="AD11" s="35" t="s">
@@ -5245,7 +5245,7 @@
       <c r="T12" s="31" t="s">
         <v>14</v>
       </c>
-      <c r="U12" s="77" t="s">
+      <c r="U12" s="69" t="s">
         <v>17</v>
       </c>
       <c r="V12" s="3" t="s">
@@ -5266,7 +5266,7 @@
       <c r="AA12" s="31" t="s">
         <v>23</v>
       </c>
-      <c r="AB12" s="86" t="s">
+      <c r="AB12" s="31" t="s">
         <v>8</v>
       </c>
       <c r="AD12" s="3" t="s">
@@ -5295,14 +5295,14 @@
       <c r="T13" s="51" t="s">
         <v>70</v>
       </c>
-      <c r="U13" s="78" t="s">
+      <c r="U13" s="70" t="s">
         <v>72</v>
       </c>
       <c r="V13" s="49" t="s">
         <v>71</v>
       </c>
-      <c r="W13" s="61" t="s">
-        <v>72</v>
+      <c r="W13" s="49" t="s">
+        <v>82</v>
       </c>
       <c r="X13" s="49" t="s">
         <v>73</v>
@@ -5339,7 +5339,7 @@
       <c r="T14" s="31">
         <v>100</v>
       </c>
-      <c r="U14" s="77">
+      <c r="U14" s="69">
         <v>0</v>
       </c>
       <c r="V14" s="3">
@@ -5360,7 +5360,7 @@
       <c r="AA14" s="31">
         <v>11</v>
       </c>
-      <c r="AB14" s="86">
+      <c r="AB14" s="31">
         <v>5331.3170570000002</v>
       </c>
       <c r="AD14" s="3">
@@ -5389,7 +5389,7 @@
       <c r="T15" s="31">
         <v>100</v>
       </c>
-      <c r="U15" s="77">
+      <c r="U15" s="69">
         <v>0</v>
       </c>
       <c r="V15" s="3">
@@ -5410,7 +5410,7 @@
       <c r="AA15" s="31">
         <v>11</v>
       </c>
-      <c r="AB15" s="86">
+      <c r="AB15" s="31">
         <v>5331.3170567901097</v>
       </c>
       <c r="AD15" s="3">
@@ -5439,7 +5439,7 @@
       <c r="T16" s="51">
         <v>0</v>
       </c>
-      <c r="U16" s="78">
+      <c r="U16" s="70">
         <v>0</v>
       </c>
       <c r="V16" s="49">
@@ -5489,7 +5489,7 @@
       <c r="T17" s="31">
         <v>0</v>
       </c>
-      <c r="U17" s="77">
+      <c r="U17" s="69">
         <v>0</v>
       </c>
       <c r="V17" s="3">
@@ -5510,7 +5510,7 @@
       <c r="AA17" s="31">
         <v>10.881</v>
       </c>
-      <c r="AB17" s="86">
+      <c r="AB17" s="31">
         <v>7108.14468373205</v>
       </c>
       <c r="AD17" s="3">
@@ -5539,7 +5539,7 @@
       <c r="T18" s="51">
         <v>0</v>
       </c>
-      <c r="U18" s="78">
+      <c r="U18" s="70">
         <v>87.1</v>
       </c>
       <c r="V18" s="49">
@@ -5589,7 +5589,7 @@
       <c r="T19" s="31">
         <v>0</v>
       </c>
-      <c r="U19" s="77">
+      <c r="U19" s="69">
         <v>100</v>
       </c>
       <c r="V19" s="3">
@@ -5610,7 +5610,7 @@
       <c r="AA19" s="31">
         <v>11</v>
       </c>
-      <c r="AB19" s="86">
+      <c r="AB19" s="31">
         <v>9698.3661137017607</v>
       </c>
       <c r="AD19" s="3">
@@ -5639,7 +5639,7 @@
       <c r="T20" s="31">
         <v>0</v>
       </c>
-      <c r="U20" s="77">
+      <c r="U20" s="69">
         <v>100</v>
       </c>
       <c r="V20" s="3">
@@ -5660,7 +5660,7 @@
       <c r="AA20" s="31">
         <v>11</v>
       </c>
-      <c r="AB20" s="86">
+      <c r="AB20" s="31">
         <v>13665.8515410358</v>
       </c>
       <c r="AD20" s="3">
@@ -5689,7 +5689,7 @@
       <c r="T21" s="51">
         <v>0</v>
       </c>
-      <c r="U21" s="78">
+      <c r="U21" s="70">
         <v>100</v>
       </c>
       <c r="V21" s="49">
@@ -5729,26 +5729,26 @@
       <c r="A24" s="67" t="s">
         <v>0</v>
       </c>
-      <c r="B24" s="69" t="s">
+      <c r="B24" s="83" t="s">
         <v>24</v>
       </c>
-      <c r="C24" s="70"/>
-      <c r="D24" s="71"/>
-      <c r="E24" s="70" t="s">
+      <c r="C24" s="84"/>
+      <c r="D24" s="85"/>
+      <c r="E24" s="84" t="s">
         <v>25</v>
       </c>
-      <c r="F24" s="70"/>
-      <c r="G24" s="71"/>
-      <c r="H24" s="70" t="s">
+      <c r="F24" s="84"/>
+      <c r="G24" s="85"/>
+      <c r="H24" s="84" t="s">
         <v>26</v>
       </c>
-      <c r="I24" s="70"/>
-      <c r="J24" s="70"/>
-      <c r="K24" s="69" t="s">
+      <c r="I24" s="84"/>
+      <c r="J24" s="84"/>
+      <c r="K24" s="83" t="s">
         <v>27</v>
       </c>
-      <c r="L24" s="70"/>
-      <c r="M24" s="70"/>
+      <c r="L24" s="84"/>
+      <c r="M24" s="84"/>
     </row>
     <row r="25" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A25" s="14" t="s">
@@ -6097,7 +6097,7 @@
       <c r="T34" s="51" t="s">
         <v>70</v>
       </c>
-      <c r="U34" s="78" t="s">
+      <c r="U34" s="70" t="s">
         <v>72</v>
       </c>
       <c r="V34" s="49" t="s">
@@ -6141,7 +6141,7 @@
       <c r="T35" s="31">
         <v>100</v>
       </c>
-      <c r="U35" s="77">
+      <c r="U35" s="69">
         <v>12.2272727272727</v>
       </c>
       <c r="V35" s="3">
@@ -6162,7 +6162,7 @@
       <c r="AA35" s="31">
         <v>11</v>
       </c>
-      <c r="AB35" s="86">
+      <c r="AB35" s="31">
         <v>4943.45004945858</v>
       </c>
       <c r="AD35" s="3">
@@ -6191,7 +6191,7 @@
       <c r="T36" s="31">
         <v>0</v>
       </c>
-      <c r="U36" s="77">
+      <c r="U36" s="69">
         <v>0</v>
       </c>
       <c r="V36" s="3">
@@ -6212,7 +6212,7 @@
       <c r="AA36" s="31">
         <v>10.295999999999999</v>
       </c>
-      <c r="AB36" s="86">
+      <c r="AB36" s="31">
         <v>8331.0174630000001</v>
       </c>
       <c r="AD36" s="3">
@@ -6241,7 +6241,7 @@
       <c r="T37" s="51">
         <v>25.363636363636299</v>
       </c>
-      <c r="U37" s="78">
+      <c r="U37" s="70">
         <v>100</v>
       </c>
       <c r="V37" s="49">
@@ -6291,7 +6291,7 @@
       <c r="T38" s="31">
         <v>100</v>
       </c>
-      <c r="U38" s="77">
+      <c r="U38" s="69">
         <v>54.754545454545401</v>
       </c>
       <c r="V38" s="3">
@@ -6312,7 +6312,7 @@
       <c r="AA38" s="31">
         <v>11</v>
       </c>
-      <c r="AB38" s="86">
+      <c r="AB38" s="31">
         <v>5202.9112099563299</v>
       </c>
       <c r="AD38" s="3">
@@ -6341,7 +6341,7 @@
       <c r="T39" s="51">
         <v>0</v>
       </c>
-      <c r="U39" s="78">
+      <c r="U39" s="70">
         <v>100</v>
       </c>
       <c r="V39" s="49">
@@ -6391,7 +6391,7 @@
       <c r="T40" s="31">
         <v>0</v>
       </c>
-      <c r="U40" s="77">
+      <c r="U40" s="69">
         <v>100</v>
       </c>
       <c r="V40" s="3">
@@ -6412,7 +6412,7 @@
       <c r="AA40" s="31">
         <v>11</v>
       </c>
-      <c r="AB40" s="86">
+      <c r="AB40" s="31">
         <v>9105.1182521936098</v>
       </c>
       <c r="AD40" s="3">
@@ -6441,7 +6441,7 @@
       <c r="T41" s="31">
         <v>0</v>
       </c>
-      <c r="U41" s="77">
+      <c r="U41" s="69">
         <v>100</v>
       </c>
       <c r="V41" s="3">
@@ -6462,7 +6462,7 @@
       <c r="AA41" s="31">
         <v>11</v>
       </c>
-      <c r="AB41" s="86">
+      <c r="AB41" s="31">
         <v>8998.4913450118693</v>
       </c>
       <c r="AD41" s="3">
@@ -6491,7 +6491,7 @@
       <c r="T42" s="51">
         <v>0</v>
       </c>
-      <c r="U42" s="78">
+      <c r="U42" s="70">
         <v>100</v>
       </c>
       <c r="V42" s="49">
@@ -6531,26 +6531,26 @@
       <c r="A44" s="67" t="s">
         <v>0</v>
       </c>
-      <c r="B44" s="69" t="s">
+      <c r="B44" s="83" t="s">
         <v>24</v>
       </c>
-      <c r="C44" s="70"/>
-      <c r="D44" s="71"/>
-      <c r="E44" s="70" t="s">
+      <c r="C44" s="84"/>
+      <c r="D44" s="85"/>
+      <c r="E44" s="84" t="s">
         <v>25</v>
       </c>
-      <c r="F44" s="70"/>
-      <c r="G44" s="71"/>
-      <c r="H44" s="70" t="s">
+      <c r="F44" s="84"/>
+      <c r="G44" s="85"/>
+      <c r="H44" s="84" t="s">
         <v>26</v>
       </c>
-      <c r="I44" s="70"/>
-      <c r="J44" s="70"/>
-      <c r="K44" s="69" t="s">
+      <c r="I44" s="84"/>
+      <c r="J44" s="84"/>
+      <c r="K44" s="83" t="s">
         <v>27</v>
       </c>
-      <c r="L44" s="70"/>
-      <c r="M44" s="70"/>
+      <c r="L44" s="84"/>
+      <c r="M44" s="84"/>
     </row>
     <row r="45" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A45" s="14" t="s">
@@ -6899,7 +6899,7 @@
       <c r="T54" s="51" t="s">
         <v>70</v>
       </c>
-      <c r="U54" s="78" t="s">
+      <c r="U54" s="70" t="s">
         <v>72</v>
       </c>
       <c r="V54" s="49" t="s">
@@ -6943,7 +6943,7 @@
       <c r="T55" s="31">
         <v>89.745454545454507</v>
       </c>
-      <c r="U55" s="77">
+      <c r="U55" s="69">
         <v>0</v>
       </c>
       <c r="V55" s="3">
@@ -6964,7 +6964,7 @@
       <c r="AA55" s="31">
         <v>11</v>
       </c>
-      <c r="AB55" s="86">
+      <c r="AB55" s="31">
         <v>4988.0428367251698</v>
       </c>
       <c r="AD55" s="3">
@@ -6993,7 +6993,7 @@
       <c r="T56" s="31">
         <v>89.745454545454507</v>
       </c>
-      <c r="U56" s="77">
+      <c r="U56" s="69">
         <v>0</v>
       </c>
       <c r="V56" s="3">
@@ -7014,7 +7014,7 @@
       <c r="AA56" s="31">
         <v>11</v>
       </c>
-      <c r="AB56" s="86">
+      <c r="AB56" s="31">
         <v>4988.5894963933697</v>
       </c>
       <c r="AD56" s="3">
@@ -7043,7 +7043,7 @@
       <c r="T57" s="51">
         <v>100</v>
       </c>
-      <c r="U57" s="78">
+      <c r="U57" s="70">
         <v>100</v>
       </c>
       <c r="V57" s="49">
@@ -7093,7 +7093,7 @@
       <c r="T58" s="31">
         <v>77.609090909090895</v>
       </c>
-      <c r="U58" s="77">
+      <c r="U58" s="69">
         <v>100</v>
       </c>
       <c r="V58" s="3">
@@ -7114,7 +7114,7 @@
       <c r="AA58" s="31">
         <v>11</v>
       </c>
-      <c r="AB58" s="86">
+      <c r="AB58" s="31">
         <v>7096.2458818271198</v>
       </c>
       <c r="AD58" s="3">
@@ -7143,7 +7143,7 @@
       <c r="T59" s="51">
         <v>0</v>
       </c>
-      <c r="U59" s="78">
+      <c r="U59" s="70">
         <v>100</v>
       </c>
       <c r="V59" s="49">
@@ -7193,7 +7193,7 @@
       <c r="T60" s="31">
         <v>100</v>
       </c>
-      <c r="U60" s="77">
+      <c r="U60" s="69">
         <v>0</v>
       </c>
       <c r="V60" s="3">
@@ -7214,7 +7214,7 @@
       <c r="AA60" s="31">
         <v>11</v>
       </c>
-      <c r="AB60" s="86">
+      <c r="AB60" s="31">
         <v>2868.1308666606101</v>
       </c>
       <c r="AD60" s="3">
@@ -7243,7 +7243,7 @@
       <c r="T61" s="31">
         <v>0</v>
       </c>
-      <c r="U61" s="77">
+      <c r="U61" s="69">
         <v>100</v>
       </c>
       <c r="V61" s="3">
@@ -7264,7 +7264,7 @@
       <c r="AA61" s="31">
         <v>11</v>
       </c>
-      <c r="AB61" s="86">
+      <c r="AB61" s="31">
         <v>9726.6027333685197</v>
       </c>
       <c r="AD61" s="3">
@@ -7293,7 +7293,7 @@
       <c r="T62" s="51">
         <v>100</v>
       </c>
-      <c r="U62" s="78">
+      <c r="U62" s="70">
         <v>100</v>
       </c>
       <c r="V62" s="49">
@@ -7333,26 +7333,26 @@
       <c r="A65" s="68" t="s">
         <v>0</v>
       </c>
-      <c r="B65" s="72" t="s">
+      <c r="B65" s="86" t="s">
         <v>24</v>
       </c>
-      <c r="C65" s="73"/>
-      <c r="D65" s="74"/>
-      <c r="E65" s="75" t="s">
+      <c r="C65" s="87"/>
+      <c r="D65" s="88"/>
+      <c r="E65" s="89" t="s">
         <v>25</v>
       </c>
-      <c r="F65" s="73"/>
-      <c r="G65" s="74"/>
-      <c r="H65" s="75" t="s">
+      <c r="F65" s="87"/>
+      <c r="G65" s="88"/>
+      <c r="H65" s="89" t="s">
         <v>26</v>
       </c>
-      <c r="I65" s="73"/>
-      <c r="J65" s="76"/>
-      <c r="K65" s="72" t="s">
+      <c r="I65" s="87"/>
+      <c r="J65" s="90"/>
+      <c r="K65" s="86" t="s">
         <v>27</v>
       </c>
-      <c r="L65" s="73"/>
-      <c r="M65" s="73"/>
+      <c r="L65" s="87"/>
+      <c r="M65" s="87"/>
       <c r="N65" s="21"/>
       <c r="O65" s="21"/>
     </row>
@@ -7726,7 +7726,7 @@
       <c r="T75" s="51" t="s">
         <v>70</v>
       </c>
-      <c r="U75" s="78" t="s">
+      <c r="U75" s="70" t="s">
         <v>72</v>
       </c>
       <c r="V75" s="49" t="s">
@@ -7784,7 +7784,7 @@
       <c r="T76" s="31">
         <v>0</v>
       </c>
-      <c r="U76" s="77">
+      <c r="U76" s="69">
         <v>99.754545449999995</v>
       </c>
       <c r="V76" s="3">
@@ -7805,7 +7805,7 @@
       <c r="AA76" s="31">
         <v>11</v>
       </c>
-      <c r="AB76" s="86">
+      <c r="AB76" s="31">
         <v>1510.5934870000001</v>
       </c>
       <c r="AD76" s="3">
@@ -7848,7 +7848,7 @@
       <c r="T77" s="31">
         <v>0</v>
       </c>
-      <c r="U77" s="77">
+      <c r="U77" s="69">
         <v>99.754545454545394</v>
       </c>
       <c r="V77" s="3">
@@ -7869,7 +7869,7 @@
       <c r="AA77" s="31">
         <v>11</v>
       </c>
-      <c r="AB77" s="86">
+      <c r="AB77" s="31">
         <v>1510.59370258337</v>
       </c>
       <c r="AD77" s="3">
@@ -7912,7 +7912,7 @@
       <c r="T78" s="51">
         <v>0</v>
       </c>
-      <c r="U78" s="78">
+      <c r="U78" s="70">
         <v>0</v>
       </c>
       <c r="V78" s="49">
@@ -7976,7 +7976,7 @@
       <c r="T79" s="31">
         <v>0</v>
       </c>
-      <c r="U79" s="77">
+      <c r="U79" s="69">
         <v>48.754545454545401</v>
       </c>
       <c r="V79" s="3">
@@ -7997,7 +7997,7 @@
       <c r="AA79" s="31">
         <v>11</v>
       </c>
-      <c r="AB79" s="86">
+      <c r="AB79" s="31">
         <v>7664.0583359410903</v>
       </c>
       <c r="AD79" s="3">
@@ -8040,7 +8040,7 @@
       <c r="T80" s="51">
         <v>0</v>
       </c>
-      <c r="U80" s="78">
+      <c r="U80" s="70">
         <v>4.1545454545454499</v>
       </c>
       <c r="V80" s="49">
@@ -8123,7 +8123,7 @@
       <c r="T82" s="31">
         <v>0</v>
       </c>
-      <c r="U82" s="77">
+      <c r="U82" s="69">
         <v>4.1545454545454499</v>
       </c>
       <c r="V82" s="3">
@@ -8144,7 +8144,7 @@
       <c r="AA82" s="31">
         <v>9.9190000000000005</v>
       </c>
-      <c r="AB82" s="86">
+      <c r="AB82" s="31">
         <v>9853.7325300468692</v>
       </c>
       <c r="AD82" s="3">
@@ -8173,7 +8173,7 @@
       <c r="T83" s="51">
         <v>0</v>
       </c>
-      <c r="U83" s="78">
+      <c r="U83" s="70">
         <v>4.1545454545454499</v>
       </c>
       <c r="V83" s="49">
@@ -8206,6 +8206,14 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="E2:G2"/>
+    <mergeCell ref="H2:J2"/>
+    <mergeCell ref="K2:M2"/>
+    <mergeCell ref="B24:D24"/>
+    <mergeCell ref="E24:G24"/>
+    <mergeCell ref="H24:J24"/>
+    <mergeCell ref="K24:M24"/>
     <mergeCell ref="B65:D65"/>
     <mergeCell ref="E65:G65"/>
     <mergeCell ref="H65:J65"/>
@@ -8214,14 +8222,6 @@
     <mergeCell ref="E44:G44"/>
     <mergeCell ref="H44:J44"/>
     <mergeCell ref="K44:M44"/>
-    <mergeCell ref="B2:D2"/>
-    <mergeCell ref="E2:G2"/>
-    <mergeCell ref="H2:J2"/>
-    <mergeCell ref="K2:M2"/>
-    <mergeCell ref="B24:D24"/>
-    <mergeCell ref="E24:G24"/>
-    <mergeCell ref="H24:J24"/>
-    <mergeCell ref="K24:M24"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -8233,11 +8233,11 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.77734375" customWidth="1"/>
-    <col min="15" max="15" width="8.88671875" style="82"/>
+    <col min="15" max="15" width="8.88671875" style="74"/>
     <col min="16" max="18" width="9" style="3" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="9" style="58" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="16" style="31" customWidth="1"/>
-    <col min="21" max="21" width="9" style="77" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="9" style="69" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="10.33203125" style="3" customWidth="1"/>
     <col min="23" max="23" width="9" style="58" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="12" style="3" customWidth="1"/>
@@ -8257,26 +8257,26 @@
       <c r="A2" s="67" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="69" t="s">
+      <c r="B2" s="83" t="s">
         <v>24</v>
       </c>
-      <c r="C2" s="70"/>
-      <c r="D2" s="71"/>
-      <c r="E2" s="70" t="s">
+      <c r="C2" s="84"/>
+      <c r="D2" s="85"/>
+      <c r="E2" s="84" t="s">
         <v>25</v>
       </c>
-      <c r="F2" s="70"/>
-      <c r="G2" s="71"/>
-      <c r="H2" s="70" t="s">
+      <c r="F2" s="84"/>
+      <c r="G2" s="85"/>
+      <c r="H2" s="84" t="s">
         <v>26</v>
       </c>
-      <c r="I2" s="70"/>
-      <c r="J2" s="70"/>
-      <c r="K2" s="69" t="s">
+      <c r="I2" s="84"/>
+      <c r="J2" s="84"/>
+      <c r="K2" s="83" t="s">
         <v>27</v>
       </c>
-      <c r="L2" s="70"/>
-      <c r="M2" s="70"/>
+      <c r="L2" s="84"/>
+      <c r="M2" s="84"/>
     </row>
     <row r="3" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
@@ -8574,7 +8574,7 @@
       <c r="T11" s="31" t="s">
         <v>14</v>
       </c>
-      <c r="U11" s="77" t="s">
+      <c r="U11" s="69" t="s">
         <v>17</v>
       </c>
       <c r="V11" s="3" t="s">
@@ -8624,7 +8624,7 @@
       <c r="T12" s="51" t="s">
         <v>70</v>
       </c>
-      <c r="U12" s="78" t="s">
+      <c r="U12" s="70" t="s">
         <v>72</v>
       </c>
       <c r="V12" s="49" t="s">
@@ -8668,7 +8668,7 @@
       <c r="T13" s="31">
         <v>0</v>
       </c>
-      <c r="U13" s="77">
+      <c r="U13" s="69">
         <v>0</v>
       </c>
       <c r="V13" s="3">
@@ -8718,7 +8718,7 @@
       <c r="T14" s="31">
         <v>0</v>
       </c>
-      <c r="U14" s="77">
+      <c r="U14" s="69">
         <v>0</v>
       </c>
       <c r="V14" s="3">
@@ -8768,7 +8768,7 @@
       <c r="T15" s="51">
         <v>0</v>
       </c>
-      <c r="U15" s="78">
+      <c r="U15" s="70">
         <v>0</v>
       </c>
       <c r="V15" s="49">
@@ -8818,7 +8818,7 @@
       <c r="T16" s="31">
         <v>0</v>
       </c>
-      <c r="U16" s="77">
+      <c r="U16" s="69">
         <v>100</v>
       </c>
       <c r="V16" s="3">
@@ -8868,7 +8868,7 @@
       <c r="T17" s="51">
         <v>0</v>
       </c>
-      <c r="U17" s="78">
+      <c r="U17" s="70">
         <v>100</v>
       </c>
       <c r="V17" s="49">
@@ -8923,7 +8923,7 @@
       <c r="T19" s="31">
         <v>0</v>
       </c>
-      <c r="U19" s="77">
+      <c r="U19" s="69">
         <v>35.265151520000003</v>
       </c>
       <c r="V19" s="3">
@@ -8963,7 +8963,7 @@
       <c r="R20" s="49"/>
       <c r="S20" s="61"/>
       <c r="T20" s="51"/>
-      <c r="U20" s="78"/>
+      <c r="U20" s="70"/>
       <c r="V20" s="49"/>
       <c r="W20" s="61"/>
       <c r="X20" s="49"/>
@@ -8981,26 +8981,26 @@
       <c r="A23" s="67" t="s">
         <v>0</v>
       </c>
-      <c r="B23" s="69" t="s">
+      <c r="B23" s="83" t="s">
         <v>24</v>
       </c>
-      <c r="C23" s="70"/>
-      <c r="D23" s="71"/>
-      <c r="E23" s="70" t="s">
+      <c r="C23" s="84"/>
+      <c r="D23" s="85"/>
+      <c r="E23" s="84" t="s">
         <v>25</v>
       </c>
-      <c r="F23" s="70"/>
-      <c r="G23" s="71"/>
-      <c r="H23" s="70" t="s">
+      <c r="F23" s="84"/>
+      <c r="G23" s="85"/>
+      <c r="H23" s="84" t="s">
         <v>26</v>
       </c>
-      <c r="I23" s="70"/>
-      <c r="J23" s="70"/>
-      <c r="K23" s="69" t="s">
+      <c r="I23" s="84"/>
+      <c r="J23" s="84"/>
+      <c r="K23" s="83" t="s">
         <v>27</v>
       </c>
-      <c r="L23" s="70"/>
-      <c r="M23" s="70"/>
+      <c r="L23" s="84"/>
+      <c r="M23" s="84"/>
     </row>
     <row r="24" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A24" s="14" t="s">
@@ -9301,7 +9301,7 @@
       <c r="T33" s="51" t="s">
         <v>70</v>
       </c>
-      <c r="U33" s="78" t="s">
+      <c r="U33" s="70" t="s">
         <v>72</v>
       </c>
       <c r="V33" s="49" t="s">
@@ -9345,7 +9345,7 @@
       <c r="T34" s="31">
         <v>100</v>
       </c>
-      <c r="U34" s="77">
+      <c r="U34" s="69">
         <v>100</v>
       </c>
       <c r="V34" s="3">
@@ -9395,7 +9395,7 @@
       <c r="T35" s="31">
         <v>100</v>
       </c>
-      <c r="U35" s="77">
+      <c r="U35" s="69">
         <v>100</v>
       </c>
       <c r="V35" s="3">
@@ -9445,7 +9445,7 @@
       <c r="T36" s="51">
         <v>0</v>
       </c>
-      <c r="U36" s="78">
+      <c r="U36" s="70">
         <v>0</v>
       </c>
       <c r="V36" s="49">
@@ -9495,7 +9495,7 @@
       <c r="T37" s="31">
         <v>0</v>
       </c>
-      <c r="U37" s="77">
+      <c r="U37" s="69">
         <v>37.462121209999999</v>
       </c>
       <c r="V37" s="3">
@@ -9545,7 +9545,7 @@
       <c r="T38" s="51">
         <v>0</v>
       </c>
-      <c r="U38" s="78">
+      <c r="U38" s="70">
         <v>100</v>
       </c>
       <c r="V38" s="49">
@@ -9600,7 +9600,7 @@
       <c r="T40" s="31">
         <v>0</v>
       </c>
-      <c r="U40" s="77">
+      <c r="U40" s="69">
         <v>100</v>
       </c>
       <c r="V40" s="3">
@@ -9640,7 +9640,7 @@
       <c r="R41" s="49"/>
       <c r="S41" s="61"/>
       <c r="T41" s="51"/>
-      <c r="U41" s="78"/>
+      <c r="U41" s="70"/>
       <c r="V41" s="49"/>
       <c r="W41" s="61"/>
       <c r="X41" s="49"/>
@@ -9658,26 +9658,26 @@
       <c r="A44" s="67" t="s">
         <v>0</v>
       </c>
-      <c r="B44" s="69" t="s">
+      <c r="B44" s="83" t="s">
         <v>24</v>
       </c>
-      <c r="C44" s="70"/>
-      <c r="D44" s="71"/>
-      <c r="E44" s="70" t="s">
+      <c r="C44" s="84"/>
+      <c r="D44" s="85"/>
+      <c r="E44" s="84" t="s">
         <v>25</v>
       </c>
-      <c r="F44" s="70"/>
-      <c r="G44" s="71"/>
-      <c r="H44" s="70" t="s">
+      <c r="F44" s="84"/>
+      <c r="G44" s="85"/>
+      <c r="H44" s="84" t="s">
         <v>26</v>
       </c>
-      <c r="I44" s="70"/>
-      <c r="J44" s="70"/>
-      <c r="K44" s="69" t="s">
+      <c r="I44" s="84"/>
+      <c r="J44" s="84"/>
+      <c r="K44" s="83" t="s">
         <v>27</v>
       </c>
-      <c r="L44" s="70"/>
-      <c r="M44" s="70"/>
+      <c r="L44" s="84"/>
+      <c r="M44" s="84"/>
     </row>
     <row r="45" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A45" s="14" t="s">
@@ -9978,14 +9978,14 @@
       <c r="T54" s="51" t="s">
         <v>70</v>
       </c>
-      <c r="U54" s="78" t="s">
+      <c r="U54" s="70" t="s">
         <v>72</v>
       </c>
       <c r="V54" s="49" t="s">
         <v>71</v>
       </c>
       <c r="W54" s="61" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="X54" s="49" t="s">
         <v>73</v>
@@ -10022,7 +10022,7 @@
       <c r="T55" s="31">
         <v>78.901515151515099</v>
       </c>
-      <c r="U55" s="77">
+      <c r="U55" s="69">
         <v>100</v>
       </c>
       <c r="V55" s="3">
@@ -10072,7 +10072,7 @@
       <c r="T56" s="31">
         <v>76.931818181818102</v>
       </c>
-      <c r="U56" s="77">
+      <c r="U56" s="69">
         <v>100</v>
       </c>
       <c r="V56" s="3">
@@ -10122,7 +10122,7 @@
       <c r="T57" s="51">
         <v>0</v>
       </c>
-      <c r="U57" s="78">
+      <c r="U57" s="70">
         <v>100</v>
       </c>
       <c r="V57" s="49">
@@ -10172,7 +10172,7 @@
       <c r="T58" s="31">
         <v>0</v>
       </c>
-      <c r="U58" s="77">
+      <c r="U58" s="69">
         <v>100</v>
       </c>
       <c r="V58" s="3">
@@ -10222,7 +10222,7 @@
       <c r="T59" s="51">
         <v>0</v>
       </c>
-      <c r="U59" s="78">
+      <c r="U59" s="70">
         <v>74.659090910000003</v>
       </c>
       <c r="V59" s="49">
@@ -10277,7 +10277,7 @@
       <c r="T61" s="31">
         <v>0</v>
       </c>
-      <c r="U61" s="77">
+      <c r="U61" s="69">
         <v>0</v>
       </c>
       <c r="V61" s="3">
@@ -10317,7 +10317,7 @@
       <c r="R62" s="49"/>
       <c r="S62" s="61"/>
       <c r="T62" s="51"/>
-      <c r="U62" s="78"/>
+      <c r="U62" s="70"/>
       <c r="V62" s="49"/>
       <c r="W62" s="61"/>
       <c r="X62" s="49"/>
@@ -10335,28 +10335,28 @@
       <c r="A64" s="68" t="s">
         <v>0</v>
       </c>
-      <c r="B64" s="72" t="s">
+      <c r="B64" s="86" t="s">
         <v>24</v>
       </c>
-      <c r="C64" s="73"/>
-      <c r="D64" s="74"/>
-      <c r="E64" s="75" t="s">
+      <c r="C64" s="87"/>
+      <c r="D64" s="88"/>
+      <c r="E64" s="89" t="s">
         <v>25</v>
       </c>
-      <c r="F64" s="73"/>
-      <c r="G64" s="74"/>
-      <c r="H64" s="75" t="s">
+      <c r="F64" s="87"/>
+      <c r="G64" s="88"/>
+      <c r="H64" s="89" t="s">
         <v>26</v>
       </c>
-      <c r="I64" s="73"/>
-      <c r="J64" s="76"/>
-      <c r="K64" s="72" t="s">
+      <c r="I64" s="87"/>
+      <c r="J64" s="90"/>
+      <c r="K64" s="86" t="s">
         <v>27</v>
       </c>
-      <c r="L64" s="73"/>
-      <c r="M64" s="73"/>
+      <c r="L64" s="87"/>
+      <c r="M64" s="87"/>
       <c r="N64" s="21"/>
-      <c r="O64" s="83"/>
+      <c r="O64" s="75"/>
     </row>
     <row r="65" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A65" s="22" t="s">
@@ -10399,7 +10399,7 @@
         <v>0.65499997138976995</v>
       </c>
       <c r="N65" s="21"/>
-      <c r="O65" s="83"/>
+      <c r="O65" s="75"/>
     </row>
     <row r="66" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A66" s="22" t="s">
@@ -10442,7 +10442,7 @@
         <v>0.67000001668929998</v>
       </c>
       <c r="N66" s="21"/>
-      <c r="O66" s="83"/>
+      <c r="O66" s="75"/>
     </row>
     <row r="67" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A67" s="19" t="s">
@@ -10485,7 +10485,7 @@
         <v>0.72000002861022905</v>
       </c>
       <c r="N67" s="21"/>
-      <c r="O67" s="83"/>
+      <c r="O67" s="75"/>
     </row>
     <row r="68" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A68" s="22" t="s">
@@ -10528,7 +10528,7 @@
         <v>0.85000002384185702</v>
       </c>
       <c r="N68" s="21"/>
-      <c r="O68" s="83"/>
+      <c r="O68" s="75"/>
     </row>
     <row r="69" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A69" s="19" t="s">
@@ -10571,7 +10571,7 @@
         <v>0.85000002384185702</v>
       </c>
       <c r="N69" s="21"/>
-      <c r="O69" s="83"/>
+      <c r="O69" s="75"/>
     </row>
     <row r="70" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A70" s="22" t="s">
@@ -10590,7 +10590,7 @@
       <c r="L70" s="23"/>
       <c r="M70" s="23"/>
       <c r="N70" s="21"/>
-      <c r="O70" s="83"/>
+      <c r="O70" s="75"/>
     </row>
     <row r="71" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A71" s="22" t="s">
@@ -10633,7 +10633,7 @@
         <v>0.85000002384185702</v>
       </c>
       <c r="N71" s="21"/>
-      <c r="O71" s="83"/>
+      <c r="O71" s="75"/>
     </row>
     <row r="72" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A72" s="20" t="s">
@@ -10676,7 +10676,7 @@
         <v>0.85000002384185702</v>
       </c>
       <c r="N72" s="21"/>
-      <c r="O72" s="83"/>
+      <c r="O72" s="75"/>
     </row>
     <row r="73" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A73" s="21"/>
@@ -10693,7 +10693,7 @@
       <c r="L73" s="21"/>
       <c r="M73" s="21"/>
       <c r="N73" s="21"/>
-      <c r="O73" s="83"/>
+      <c r="O73" s="75"/>
     </row>
     <row r="74" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A74" s="21"/>
@@ -10728,7 +10728,7 @@
       <c r="T74" s="51" t="s">
         <v>70</v>
       </c>
-      <c r="U74" s="78" t="s">
+      <c r="U74" s="70" t="s">
         <v>72</v>
       </c>
       <c r="V74" s="49" t="s">
@@ -10786,7 +10786,7 @@
       <c r="T75" s="31">
         <v>0</v>
       </c>
-      <c r="U75" s="77">
+      <c r="U75" s="69">
         <v>28.06818182</v>
       </c>
       <c r="V75" s="3">
@@ -10850,7 +10850,7 @@
       <c r="T76" s="31">
         <v>0</v>
       </c>
-      <c r="U76" s="77">
+      <c r="U76" s="69">
         <v>54.166666669999998</v>
       </c>
       <c r="V76" s="3">
@@ -10914,7 +10914,7 @@
       <c r="T77" s="51">
         <v>0</v>
       </c>
-      <c r="U77" s="78">
+      <c r="U77" s="70">
         <v>40.151515150000002</v>
       </c>
       <c r="V77" s="49">
@@ -10978,7 +10978,7 @@
       <c r="T78" s="31">
         <v>0</v>
       </c>
-      <c r="U78" s="77">
+      <c r="U78" s="69">
         <v>8.5227272729999992</v>
       </c>
       <c r="V78" s="3">
@@ -11042,7 +11042,7 @@
       <c r="T79" s="51">
         <v>0</v>
       </c>
-      <c r="U79" s="78">
+      <c r="U79" s="70">
         <v>8.5227272729999992</v>
       </c>
       <c r="V79" s="49">
@@ -11125,7 +11125,7 @@
       <c r="T81" s="31">
         <v>0</v>
       </c>
-      <c r="U81" s="77">
+      <c r="U81" s="69">
         <v>8.5227272729999992</v>
       </c>
       <c r="V81" s="3">
@@ -11175,7 +11175,7 @@
       <c r="T82" s="51">
         <v>0</v>
       </c>
-      <c r="U82" s="78">
+      <c r="U82" s="70">
         <v>8.5227272729999992</v>
       </c>
       <c r="V82" s="49">
@@ -11208,6 +11208,14 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="E2:G2"/>
+    <mergeCell ref="H2:J2"/>
+    <mergeCell ref="K2:M2"/>
+    <mergeCell ref="B23:D23"/>
+    <mergeCell ref="E23:G23"/>
+    <mergeCell ref="H23:J23"/>
+    <mergeCell ref="K23:M23"/>
     <mergeCell ref="B44:D44"/>
     <mergeCell ref="E44:G44"/>
     <mergeCell ref="H44:J44"/>
@@ -11216,14 +11224,6 @@
     <mergeCell ref="E64:G64"/>
     <mergeCell ref="H64:J64"/>
     <mergeCell ref="K64:M64"/>
-    <mergeCell ref="B2:D2"/>
-    <mergeCell ref="E2:G2"/>
-    <mergeCell ref="H2:J2"/>
-    <mergeCell ref="K2:M2"/>
-    <mergeCell ref="B23:D23"/>
-    <mergeCell ref="E23:G23"/>
-    <mergeCell ref="H23:J23"/>
-    <mergeCell ref="K23:M23"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -11235,17 +11235,17 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.77734375" customWidth="1"/>
-    <col min="15" max="15" width="8.88671875" style="82"/>
+    <col min="15" max="15" width="8.88671875" style="74"/>
     <col min="16" max="16" width="8.88671875" style="33"/>
     <col min="17" max="17" width="11" style="33" customWidth="1"/>
     <col min="18" max="18" width="8.88671875" style="33"/>
-    <col min="19" max="19" width="8.88671875" style="84"/>
+    <col min="19" max="19" width="8.88671875" style="76"/>
     <col min="20" max="20" width="8.88671875" style="32"/>
-    <col min="21" max="21" width="8.88671875" style="85"/>
+    <col min="21" max="21" width="8.88671875" style="77"/>
     <col min="22" max="22" width="8.88671875" style="33"/>
-    <col min="23" max="23" width="8.88671875" style="84"/>
+    <col min="23" max="23" width="8.88671875" style="76"/>
     <col min="24" max="24" width="8.88671875" style="33"/>
-    <col min="25" max="25" width="8.88671875" style="84"/>
+    <col min="25" max="25" width="8.88671875" style="76"/>
     <col min="26" max="27" width="8.88671875" style="32"/>
     <col min="28" max="28" width="11.33203125" style="32" customWidth="1"/>
     <col min="30" max="31" width="8.88671875" style="33"/>
@@ -11260,26 +11260,26 @@
       <c r="A2" s="67" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="69" t="s">
+      <c r="B2" s="83" t="s">
         <v>24</v>
       </c>
-      <c r="C2" s="70"/>
-      <c r="D2" s="71"/>
-      <c r="E2" s="70" t="s">
+      <c r="C2" s="84"/>
+      <c r="D2" s="85"/>
+      <c r="E2" s="84" t="s">
         <v>25</v>
       </c>
-      <c r="F2" s="70"/>
-      <c r="G2" s="71"/>
-      <c r="H2" s="70" t="s">
+      <c r="F2" s="84"/>
+      <c r="G2" s="85"/>
+      <c r="H2" s="84" t="s">
         <v>26</v>
       </c>
-      <c r="I2" s="70"/>
-      <c r="J2" s="70"/>
-      <c r="K2" s="69" t="s">
+      <c r="I2" s="84"/>
+      <c r="J2" s="84"/>
+      <c r="K2" s="83" t="s">
         <v>27</v>
       </c>
-      <c r="L2" s="70"/>
-      <c r="M2" s="70"/>
+      <c r="L2" s="84"/>
+      <c r="M2" s="84"/>
     </row>
     <row r="3" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
@@ -11577,7 +11577,7 @@
       <c r="T11" s="31" t="s">
         <v>14</v>
       </c>
-      <c r="U11" s="77" t="s">
+      <c r="U11" s="69" t="s">
         <v>17</v>
       </c>
       <c r="V11" s="3" t="s">
@@ -11627,7 +11627,7 @@
       <c r="T12" s="51" t="s">
         <v>70</v>
       </c>
-      <c r="U12" s="78" t="s">
+      <c r="U12" s="70" t="s">
         <v>72</v>
       </c>
       <c r="V12" s="49" t="s">
@@ -11665,25 +11665,25 @@
       <c r="R13" s="33">
         <v>4.2976079999999996E-3</v>
       </c>
-      <c r="S13" s="84">
+      <c r="S13" s="76">
         <v>3.4186780000000001E-3</v>
       </c>
       <c r="T13" s="32">
         <v>0</v>
       </c>
-      <c r="U13" s="85">
+      <c r="U13" s="77">
         <v>0</v>
       </c>
       <c r="V13" s="33">
         <v>0</v>
       </c>
-      <c r="W13" s="84">
+      <c r="W13" s="76">
         <v>1.4738187E-2</v>
       </c>
       <c r="X13" s="33">
         <v>0</v>
       </c>
-      <c r="Y13" s="84">
+      <c r="Y13" s="76">
         <v>3.8163360000000002</v>
       </c>
       <c r="Z13" s="32">
@@ -11715,25 +11715,25 @@
       <c r="R14" s="33">
         <v>4.2976079999999996E-3</v>
       </c>
-      <c r="S14" s="84">
+      <c r="S14" s="76">
         <v>3.4186780000000001E-3</v>
       </c>
       <c r="T14" s="32">
         <v>0</v>
       </c>
-      <c r="U14" s="85">
+      <c r="U14" s="77">
         <v>0</v>
       </c>
       <c r="V14" s="33">
         <v>0</v>
       </c>
-      <c r="W14" s="84">
+      <c r="W14" s="76">
         <v>1.4738187E-2</v>
       </c>
       <c r="X14" s="33">
         <v>0</v>
       </c>
-      <c r="Y14" s="84">
+      <c r="Y14" s="76">
         <v>3.8163360000000002</v>
       </c>
       <c r="Z14" s="32">
@@ -11756,43 +11756,43 @@
       <c r="O15" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="P15" s="87">
+      <c r="P15" s="78">
         <v>2.2174191999999999E-2</v>
       </c>
-      <c r="Q15" s="88">
+      <c r="Q15" s="79">
         <v>6.8021499999999999E-2</v>
       </c>
-      <c r="R15" s="88">
+      <c r="R15" s="79">
         <v>5.6011979999999999E-3</v>
       </c>
-      <c r="S15" s="89">
+      <c r="S15" s="80">
         <v>3.7126630000000002E-3</v>
       </c>
-      <c r="T15" s="90">
-        <v>0</v>
-      </c>
-      <c r="U15" s="91">
-        <v>0</v>
-      </c>
-      <c r="V15" s="88">
+      <c r="T15" s="81">
+        <v>0</v>
+      </c>
+      <c r="U15" s="82">
+        <v>0</v>
+      </c>
+      <c r="V15" s="79">
         <v>1.5541200000000001E-4</v>
       </c>
-      <c r="W15" s="89">
+      <c r="W15" s="80">
         <v>1.4027168E-2</v>
       </c>
-      <c r="X15" s="88">
+      <c r="X15" s="79">
         <v>5.1679999999999997E-2</v>
       </c>
-      <c r="Y15" s="89">
+      <c r="Y15" s="80">
         <v>3.3281999999999998</v>
       </c>
-      <c r="Z15" s="90">
+      <c r="Z15" s="81">
         <v>0.15151515199999999</v>
       </c>
-      <c r="AA15" s="90">
+      <c r="AA15" s="81">
         <v>1.6666667E-2</v>
       </c>
-      <c r="AB15" s="90">
+      <c r="AB15" s="81">
         <v>16726.551950000001</v>
       </c>
       <c r="AD15" s="33">
@@ -11815,25 +11815,25 @@
       <c r="R16" s="33">
         <v>0.47826287499999998</v>
       </c>
-      <c r="S16" s="84">
+      <c r="S16" s="76">
         <v>7.3811294999999999E-2</v>
       </c>
       <c r="T16" s="32">
         <v>0</v>
       </c>
-      <c r="U16" s="85">
+      <c r="U16" s="77">
         <v>100</v>
       </c>
       <c r="V16" s="33">
         <v>2.148166E-3</v>
       </c>
-      <c r="W16" s="84">
+      <c r="W16" s="76">
         <v>2.9114729999999999E-3</v>
       </c>
       <c r="X16" s="33">
         <v>0.16416</v>
       </c>
-      <c r="Y16" s="84">
+      <c r="Y16" s="76">
         <v>0.27753</v>
       </c>
       <c r="Z16" s="32">
@@ -11856,43 +11856,43 @@
       <c r="O17" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="P17" s="87">
+      <c r="P17" s="78">
         <v>0.38654200399999999</v>
       </c>
-      <c r="Q17" s="88">
+      <c r="Q17" s="79">
         <v>7.5658416000000006E-2</v>
       </c>
-      <c r="R17" s="88">
+      <c r="R17" s="79">
         <v>0.38150645599999999</v>
       </c>
-      <c r="S17" s="89">
+      <c r="S17" s="80">
         <v>7.7287566000000002E-2</v>
       </c>
-      <c r="T17" s="90">
-        <v>0</v>
-      </c>
-      <c r="U17" s="91">
+      <c r="T17" s="81">
+        <v>0</v>
+      </c>
+      <c r="U17" s="82">
         <v>100</v>
       </c>
-      <c r="V17" s="88">
+      <c r="V17" s="79">
         <v>2.148166E-3</v>
       </c>
-      <c r="W17" s="89">
+      <c r="W17" s="80">
         <v>2.9719070000000002E-3</v>
       </c>
-      <c r="X17" s="88">
+      <c r="X17" s="79">
         <v>0.16416</v>
       </c>
-      <c r="Y17" s="89">
+      <c r="Y17" s="80">
         <v>0.441</v>
       </c>
-      <c r="Z17" s="90">
+      <c r="Z17" s="81">
         <v>100</v>
       </c>
-      <c r="AA17" s="90">
+      <c r="AA17" s="81">
         <v>11</v>
       </c>
-      <c r="AB17" s="90">
+      <c r="AB17" s="81">
         <v>12736.34367</v>
       </c>
       <c r="AD17" s="33">
@@ -11920,25 +11920,25 @@
       <c r="R19" s="33">
         <v>0.47984376499999998</v>
       </c>
-      <c r="S19" s="84">
+      <c r="S19" s="76">
         <v>7.4750901999999994E-2</v>
       </c>
       <c r="T19" s="32">
         <v>0</v>
       </c>
-      <c r="U19" s="85">
+      <c r="U19" s="77">
         <v>100</v>
       </c>
       <c r="V19" s="33">
         <v>2.148166E-3</v>
       </c>
-      <c r="W19" s="84">
+      <c r="W19" s="76">
         <v>3.1957259999999999E-3</v>
       </c>
       <c r="X19" s="33">
         <v>0.16416</v>
       </c>
-      <c r="Y19" s="84">
+      <c r="Y19" s="76">
         <v>0.34223999999999999</v>
       </c>
       <c r="Z19" s="32">
@@ -11961,19 +11961,19 @@
       <c r="O20" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="P20" s="87"/>
-      <c r="Q20" s="88"/>
-      <c r="R20" s="88"/>
-      <c r="S20" s="89"/>
-      <c r="T20" s="90"/>
-      <c r="U20" s="91"/>
-      <c r="V20" s="88"/>
-      <c r="W20" s="89"/>
-      <c r="X20" s="88"/>
-      <c r="Y20" s="89"/>
-      <c r="Z20" s="90"/>
-      <c r="AA20" s="90"/>
-      <c r="AB20" s="90"/>
+      <c r="P20" s="78"/>
+      <c r="Q20" s="79"/>
+      <c r="R20" s="79"/>
+      <c r="S20" s="80"/>
+      <c r="T20" s="81"/>
+      <c r="U20" s="82"/>
+      <c r="V20" s="79"/>
+      <c r="W20" s="80"/>
+      <c r="X20" s="79"/>
+      <c r="Y20" s="80"/>
+      <c r="Z20" s="81"/>
+      <c r="AA20" s="81"/>
+      <c r="AB20" s="81"/>
     </row>
     <row r="22" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
@@ -11984,26 +11984,26 @@
       <c r="A23" s="67" t="s">
         <v>0</v>
       </c>
-      <c r="B23" s="69" t="s">
+      <c r="B23" s="83" t="s">
         <v>24</v>
       </c>
-      <c r="C23" s="70"/>
-      <c r="D23" s="71"/>
-      <c r="E23" s="70" t="s">
+      <c r="C23" s="84"/>
+      <c r="D23" s="85"/>
+      <c r="E23" s="84" t="s">
         <v>25</v>
       </c>
-      <c r="F23" s="70"/>
-      <c r="G23" s="71"/>
-      <c r="H23" s="70" t="s">
+      <c r="F23" s="84"/>
+      <c r="G23" s="85"/>
+      <c r="H23" s="84" t="s">
         <v>26</v>
       </c>
-      <c r="I23" s="70"/>
-      <c r="J23" s="70"/>
-      <c r="K23" s="69" t="s">
+      <c r="I23" s="84"/>
+      <c r="J23" s="84"/>
+      <c r="K23" s="83" t="s">
         <v>27</v>
       </c>
-      <c r="L23" s="70"/>
-      <c r="M23" s="70"/>
+      <c r="L23" s="84"/>
+      <c r="M23" s="84"/>
     </row>
     <row r="24" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A24" s="14" t="s">
@@ -12304,7 +12304,7 @@
       <c r="T33" s="51" t="s">
         <v>70</v>
       </c>
-      <c r="U33" s="78" t="s">
+      <c r="U33" s="70" t="s">
         <v>72</v>
       </c>
       <c r="V33" s="49" t="s">
@@ -12342,25 +12342,25 @@
       <c r="R34" s="33">
         <v>0.49537018199999999</v>
       </c>
-      <c r="S34" s="84">
+      <c r="S34" s="76">
         <v>7.5086813000000002E-2</v>
       </c>
       <c r="T34" s="32">
         <v>100</v>
       </c>
-      <c r="U34" s="85">
+      <c r="U34" s="77">
         <v>100</v>
       </c>
       <c r="V34" s="33">
         <v>0</v>
       </c>
-      <c r="W34" s="84">
+      <c r="W34" s="76">
         <v>2.644927E-3</v>
       </c>
       <c r="X34" s="33">
         <v>2.8800000000000002E-3</v>
       </c>
-      <c r="Y34" s="84">
+      <c r="Y34" s="76">
         <v>0.192</v>
       </c>
       <c r="Z34" s="32">
@@ -12392,25 +12392,25 @@
       <c r="R35" s="33">
         <v>0.27289521300000003</v>
       </c>
-      <c r="S35" s="84">
+      <c r="S35" s="76">
         <v>3.7710198E-2</v>
       </c>
       <c r="T35" s="32">
         <v>89.886363639999999</v>
       </c>
-      <c r="U35" s="85">
+      <c r="U35" s="77">
         <v>100</v>
       </c>
       <c r="V35" s="33">
         <v>0</v>
       </c>
-      <c r="W35" s="84">
+      <c r="W35" s="76">
         <v>0</v>
       </c>
       <c r="X35" s="33">
         <v>0</v>
       </c>
-      <c r="Y35" s="84">
+      <c r="Y35" s="76">
         <v>0.93202499999999999</v>
       </c>
       <c r="Z35" s="32">
@@ -12433,43 +12433,43 @@
       <c r="O36" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="P36" s="87">
+      <c r="P36" s="78">
         <v>0.16763552700000001</v>
       </c>
-      <c r="Q36" s="88">
+      <c r="Q36" s="79">
         <v>7.8511710999999998E-2</v>
       </c>
-      <c r="R36" s="88">
+      <c r="R36" s="79">
         <v>0.16305029500000001</v>
       </c>
-      <c r="S36" s="89">
+      <c r="S36" s="80">
         <v>7.1120540999999995E-2</v>
       </c>
-      <c r="T36" s="90">
+      <c r="T36" s="81">
         <v>96.590909089999997</v>
       </c>
-      <c r="U36" s="91">
-        <v>0</v>
-      </c>
-      <c r="V36" s="88">
-        <v>0</v>
-      </c>
-      <c r="W36" s="89">
+      <c r="U36" s="82">
+        <v>0</v>
+      </c>
+      <c r="V36" s="79">
+        <v>0</v>
+      </c>
+      <c r="W36" s="80">
         <v>1.4738187E-2</v>
       </c>
-      <c r="X36" s="88">
+      <c r="X36" s="79">
         <v>3.6259999999999999E-3</v>
       </c>
-      <c r="Y36" s="89">
+      <c r="Y36" s="80">
         <v>3.8163360000000002</v>
       </c>
-      <c r="Z36" s="90">
+      <c r="Z36" s="81">
         <v>92.613636360000001</v>
       </c>
-      <c r="AA36" s="90">
+      <c r="AA36" s="81">
         <v>10.1875</v>
       </c>
-      <c r="AB36" s="90">
+      <c r="AB36" s="81">
         <v>5104.3859670000002</v>
       </c>
       <c r="AD36" s="33">
@@ -12492,25 +12492,25 @@
       <c r="R37" s="33">
         <v>5.8914656000000003E-2</v>
       </c>
-      <c r="S37" s="84">
+      <c r="S37" s="76">
         <v>3.5449247000000003E-2</v>
       </c>
       <c r="T37" s="32">
         <v>0</v>
       </c>
-      <c r="U37" s="85">
+      <c r="U37" s="77">
         <v>100</v>
       </c>
       <c r="V37" s="33">
         <v>0</v>
       </c>
-      <c r="W37" s="84">
+      <c r="W37" s="76">
         <v>2.644927E-3</v>
       </c>
       <c r="X37" s="33">
         <v>1.1039999999999999E-2</v>
       </c>
-      <c r="Y37" s="84">
+      <c r="Y37" s="76">
         <v>0.378</v>
       </c>
       <c r="Z37" s="32">
@@ -12533,43 +12533,43 @@
       <c r="O38" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="P38" s="87">
+      <c r="P38" s="78">
         <v>0.55872443800000005</v>
       </c>
-      <c r="Q38" s="88">
+      <c r="Q38" s="79">
         <v>7.0912995000000006E-2</v>
       </c>
-      <c r="R38" s="88">
+      <c r="R38" s="79">
         <v>0.56479812600000001</v>
       </c>
-      <c r="S38" s="89">
+      <c r="S38" s="80">
         <v>7.1431786999999997E-2</v>
       </c>
-      <c r="T38" s="90">
-        <v>0</v>
-      </c>
-      <c r="U38" s="91">
+      <c r="T38" s="81">
+        <v>0</v>
+      </c>
+      <c r="U38" s="82">
         <v>100</v>
       </c>
-      <c r="V38" s="88">
-        <v>0</v>
-      </c>
-      <c r="W38" s="89">
+      <c r="V38" s="79">
+        <v>0</v>
+      </c>
+      <c r="W38" s="80">
         <v>1.2383979999999999E-3</v>
       </c>
-      <c r="X38" s="88">
+      <c r="X38" s="79">
         <v>1.1039999999999999E-2</v>
       </c>
-      <c r="Y38" s="89">
+      <c r="Y38" s="80">
         <v>0.13202</v>
       </c>
-      <c r="Z38" s="90">
+      <c r="Z38" s="81">
         <v>100</v>
       </c>
-      <c r="AA38" s="90">
+      <c r="AA38" s="81">
         <v>11</v>
       </c>
-      <c r="AB38" s="90">
+      <c r="AB38" s="81">
         <v>8681.5015750000002</v>
       </c>
       <c r="AD38" s="33">
@@ -12597,25 +12597,25 @@
       <c r="R40" s="33">
         <v>5.8914682000000003E-2</v>
       </c>
-      <c r="S40" s="84">
+      <c r="S40" s="76">
         <v>3.5449245999999997E-2</v>
       </c>
       <c r="T40" s="32">
         <v>0</v>
       </c>
-      <c r="U40" s="85">
+      <c r="U40" s="77">
         <v>100</v>
       </c>
       <c r="V40" s="33">
         <v>0</v>
       </c>
-      <c r="W40" s="84">
+      <c r="W40" s="76">
         <v>2.644927E-3</v>
       </c>
       <c r="X40" s="33">
         <v>1.1039999999999999E-2</v>
       </c>
-      <c r="Y40" s="84">
+      <c r="Y40" s="76">
         <v>0.35099999999999998</v>
       </c>
       <c r="Z40" s="32">
@@ -12638,19 +12638,19 @@
       <c r="O41" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="P41" s="87"/>
-      <c r="Q41" s="88"/>
-      <c r="R41" s="88"/>
-      <c r="S41" s="89"/>
-      <c r="T41" s="90"/>
-      <c r="U41" s="91"/>
-      <c r="V41" s="88"/>
-      <c r="W41" s="89"/>
-      <c r="X41" s="88"/>
-      <c r="Y41" s="89"/>
-      <c r="Z41" s="90"/>
-      <c r="AA41" s="90"/>
-      <c r="AB41" s="90"/>
+      <c r="P41" s="78"/>
+      <c r="Q41" s="79"/>
+      <c r="R41" s="79"/>
+      <c r="S41" s="80"/>
+      <c r="T41" s="81"/>
+      <c r="U41" s="82"/>
+      <c r="V41" s="79"/>
+      <c r="W41" s="80"/>
+      <c r="X41" s="79"/>
+      <c r="Y41" s="80"/>
+      <c r="Z41" s="81"/>
+      <c r="AA41" s="81"/>
+      <c r="AB41" s="81"/>
     </row>
     <row r="43" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
@@ -12661,26 +12661,26 @@
       <c r="A44" s="67" t="s">
         <v>0</v>
       </c>
-      <c r="B44" s="69" t="s">
+      <c r="B44" s="83" t="s">
         <v>24</v>
       </c>
-      <c r="C44" s="70"/>
-      <c r="D44" s="71"/>
-      <c r="E44" s="70" t="s">
+      <c r="C44" s="84"/>
+      <c r="D44" s="85"/>
+      <c r="E44" s="84" t="s">
         <v>25</v>
       </c>
-      <c r="F44" s="70"/>
-      <c r="G44" s="71"/>
-      <c r="H44" s="70" t="s">
+      <c r="F44" s="84"/>
+      <c r="G44" s="85"/>
+      <c r="H44" s="84" t="s">
         <v>26</v>
       </c>
-      <c r="I44" s="70"/>
-      <c r="J44" s="70"/>
-      <c r="K44" s="69" t="s">
+      <c r="I44" s="84"/>
+      <c r="J44" s="84"/>
+      <c r="K44" s="83" t="s">
         <v>27</v>
       </c>
-      <c r="L44" s="70"/>
-      <c r="M44" s="70"/>
+      <c r="L44" s="84"/>
+      <c r="M44" s="84"/>
     </row>
     <row r="45" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A45" s="14" t="s">
@@ -12957,7 +12957,7 @@
       <c r="T54" s="51" t="s">
         <v>70</v>
       </c>
-      <c r="U54" s="78" t="s">
+      <c r="U54" s="70" t="s">
         <v>72</v>
       </c>
       <c r="V54" s="49" t="s">
@@ -12995,25 +12995,25 @@
       <c r="R55" s="33">
         <v>0.63531370399999998</v>
       </c>
-      <c r="S55" s="84">
+      <c r="S55" s="76">
         <v>6.9879844999999996E-2</v>
       </c>
       <c r="T55" s="32">
         <v>92.840909089999997</v>
       </c>
-      <c r="U55" s="85">
+      <c r="U55" s="77">
         <v>100</v>
       </c>
       <c r="V55" s="33">
         <v>0</v>
       </c>
-      <c r="W55" s="84">
+      <c r="W55" s="76">
         <v>6.7561699999999999E-4</v>
       </c>
       <c r="X55" s="33">
         <v>4.1599999999999996E-3</v>
       </c>
-      <c r="Y55" s="84">
+      <c r="Y55" s="76">
         <v>1.584E-2</v>
       </c>
       <c r="Z55" s="32">
@@ -13045,25 +13045,25 @@
       <c r="R56" s="33">
         <v>0.62477324099999998</v>
       </c>
-      <c r="S56" s="84">
+      <c r="S56" s="76">
         <v>7.1897643999999997E-2</v>
       </c>
       <c r="T56" s="32">
         <v>100</v>
       </c>
-      <c r="U56" s="85">
+      <c r="U56" s="77">
         <v>100</v>
       </c>
       <c r="V56" s="33">
         <v>0</v>
       </c>
-      <c r="W56" s="84">
+      <c r="W56" s="76">
         <v>7.4172400000000003E-4</v>
       </c>
       <c r="X56" s="33">
         <v>2.7999999999999998E-4</v>
       </c>
-      <c r="Y56" s="84">
+      <c r="Y56" s="76">
         <v>1.584E-2</v>
       </c>
       <c r="Z56" s="32">
@@ -13086,43 +13086,43 @@
       <c r="O57" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="P57" s="87">
+      <c r="P57" s="78">
         <v>0.40469522800000002</v>
       </c>
-      <c r="Q57" s="88">
+      <c r="Q57" s="79">
         <v>6.9731839000000004E-2</v>
       </c>
-      <c r="R57" s="88">
+      <c r="R57" s="79">
         <v>0.40629886599999998</v>
       </c>
-      <c r="S57" s="89">
+      <c r="S57" s="80">
         <v>7.0271370999999999E-2</v>
       </c>
-      <c r="T57" s="90">
-        <v>0</v>
-      </c>
-      <c r="U57" s="91">
+      <c r="T57" s="81">
+        <v>0</v>
+      </c>
+      <c r="U57" s="82">
         <v>76.212121210000006</v>
       </c>
-      <c r="V57" s="88">
-        <v>0</v>
-      </c>
-      <c r="W57" s="89">
+      <c r="V57" s="79">
+        <v>0</v>
+      </c>
+      <c r="W57" s="80">
         <v>4.4247619999999996E-3</v>
       </c>
-      <c r="X57" s="88">
+      <c r="X57" s="79">
         <v>1.0880000000000001E-2</v>
       </c>
-      <c r="Y57" s="89">
+      <c r="Y57" s="80">
         <v>0.83638100000000004</v>
       </c>
-      <c r="Z57" s="90">
+      <c r="Z57" s="81">
         <v>100</v>
       </c>
-      <c r="AA57" s="90">
+      <c r="AA57" s="81">
         <v>11</v>
       </c>
-      <c r="AB57" s="90">
+      <c r="AB57" s="81">
         <v>3455.1726140000001</v>
       </c>
       <c r="AD57" s="33">
@@ -13145,25 +13145,25 @@
       <c r="R58" s="33">
         <v>0.59317042200000003</v>
       </c>
-      <c r="S58" s="84">
+      <c r="S58" s="76">
         <v>7.4066038000000001E-2</v>
       </c>
       <c r="T58" s="32">
         <v>0</v>
       </c>
-      <c r="U58" s="85">
+      <c r="U58" s="77">
         <v>100</v>
       </c>
       <c r="V58" s="33">
         <v>0</v>
       </c>
-      <c r="W58" s="84">
+      <c r="W58" s="76">
         <v>1.382154E-3</v>
       </c>
       <c r="X58" s="33">
         <v>1.1039999999999999E-2</v>
       </c>
-      <c r="Y58" s="84">
+      <c r="Y58" s="76">
         <v>0.150672</v>
       </c>
       <c r="Z58" s="32">
@@ -13186,43 +13186,43 @@
       <c r="O59" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="P59" s="87">
+      <c r="P59" s="78">
         <v>2.2153664E-2</v>
       </c>
-      <c r="Q59" s="88">
+      <c r="Q59" s="79">
         <v>6.8025735000000004E-2</v>
       </c>
-      <c r="R59" s="88">
+      <c r="R59" s="79">
         <v>5.5786159999999998E-3</v>
       </c>
-      <c r="S59" s="89">
+      <c r="S59" s="80">
         <v>3.6971740000000001E-3</v>
       </c>
-      <c r="T59" s="90">
-        <v>0</v>
-      </c>
-      <c r="U59" s="91">
-        <v>0</v>
-      </c>
-      <c r="V59" s="88">
-        <v>0</v>
-      </c>
-      <c r="W59" s="89">
+      <c r="T59" s="81">
+        <v>0</v>
+      </c>
+      <c r="U59" s="82">
+        <v>0</v>
+      </c>
+      <c r="V59" s="79">
+        <v>0</v>
+      </c>
+      <c r="W59" s="80">
         <v>1.4738187E-2</v>
       </c>
-      <c r="X59" s="88">
+      <c r="X59" s="79">
         <v>1.1039999999999999E-2</v>
       </c>
-      <c r="Y59" s="89">
+      <c r="Y59" s="80">
         <v>3.8163360000000002</v>
       </c>
-      <c r="Z59" s="90">
+      <c r="Z59" s="81">
         <v>7.348484848</v>
       </c>
-      <c r="AA59" s="90">
+      <c r="AA59" s="81">
         <v>0.80833333299999999</v>
       </c>
-      <c r="AB59" s="90">
+      <c r="AB59" s="81">
         <v>16727.630369999999</v>
       </c>
       <c r="AD59" s="33">
@@ -13246,19 +13246,19 @@
       <c r="O62" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="P62" s="87"/>
-      <c r="Q62" s="88"/>
-      <c r="R62" s="88"/>
-      <c r="S62" s="89"/>
-      <c r="T62" s="90"/>
-      <c r="U62" s="91"/>
-      <c r="V62" s="88"/>
-      <c r="W62" s="89"/>
-      <c r="X62" s="88"/>
-      <c r="Y62" s="89"/>
-      <c r="Z62" s="90"/>
-      <c r="AA62" s="90"/>
-      <c r="AB62" s="90"/>
+      <c r="P62" s="78"/>
+      <c r="Q62" s="79"/>
+      <c r="R62" s="79"/>
+      <c r="S62" s="80"/>
+      <c r="T62" s="81"/>
+      <c r="U62" s="82"/>
+      <c r="V62" s="79"/>
+      <c r="W62" s="80"/>
+      <c r="X62" s="79"/>
+      <c r="Y62" s="80"/>
+      <c r="Z62" s="81"/>
+      <c r="AA62" s="81"/>
+      <c r="AB62" s="81"/>
     </row>
     <row r="64" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
@@ -13269,28 +13269,28 @@
       <c r="A65" s="68" t="s">
         <v>0</v>
       </c>
-      <c r="B65" s="72" t="s">
+      <c r="B65" s="86" t="s">
         <v>24</v>
       </c>
-      <c r="C65" s="73"/>
-      <c r="D65" s="74"/>
-      <c r="E65" s="75" t="s">
+      <c r="C65" s="87"/>
+      <c r="D65" s="88"/>
+      <c r="E65" s="89" t="s">
         <v>25</v>
       </c>
-      <c r="F65" s="73"/>
-      <c r="G65" s="74"/>
-      <c r="H65" s="75" t="s">
+      <c r="F65" s="87"/>
+      <c r="G65" s="88"/>
+      <c r="H65" s="89" t="s">
         <v>26</v>
       </c>
-      <c r="I65" s="73"/>
-      <c r="J65" s="76"/>
-      <c r="K65" s="72" t="s">
+      <c r="I65" s="87"/>
+      <c r="J65" s="90"/>
+      <c r="K65" s="86" t="s">
         <v>27</v>
       </c>
-      <c r="L65" s="73"/>
-      <c r="M65" s="73"/>
+      <c r="L65" s="87"/>
+      <c r="M65" s="87"/>
       <c r="N65" s="21"/>
-      <c r="O65" s="83"/>
+      <c r="O65" s="75"/>
     </row>
     <row r="66" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A66" s="22" t="s">
@@ -13333,7 +13333,7 @@
         <v>0.625</v>
       </c>
       <c r="N66" s="21"/>
-      <c r="O66" s="83"/>
+      <c r="O66" s="75"/>
     </row>
     <row r="67" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A67" s="22" t="s">
@@ -13376,7 +13376,7 @@
         <v>0.60000002384185702</v>
       </c>
       <c r="N67" s="21"/>
-      <c r="O67" s="83"/>
+      <c r="O67" s="75"/>
     </row>
     <row r="68" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A68" s="19" t="s">
@@ -13419,7 +13419,7 @@
         <v>0.75</v>
       </c>
       <c r="N68" s="21"/>
-      <c r="O68" s="83"/>
+      <c r="O68" s="75"/>
     </row>
     <row r="69" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A69" s="22" t="s">
@@ -13462,7 +13462,7 @@
         <v>0.75</v>
       </c>
       <c r="N69" s="21"/>
-      <c r="O69" s="83"/>
+      <c r="O69" s="75"/>
     </row>
     <row r="70" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A70" s="19" t="s">
@@ -13505,7 +13505,7 @@
         <v>0.85000002384185702</v>
       </c>
       <c r="N70" s="21"/>
-      <c r="O70" s="83"/>
+      <c r="O70" s="75"/>
     </row>
     <row r="71" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A71" s="22" t="s">
@@ -13524,7 +13524,7 @@
       <c r="L71" s="23"/>
       <c r="M71" s="23"/>
       <c r="N71" s="21"/>
-      <c r="O71" s="83"/>
+      <c r="O71" s="75"/>
     </row>
     <row r="72" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A72" s="22" t="s">
@@ -13567,7 +13567,7 @@
         <v>0.85000002384185702</v>
       </c>
       <c r="N72" s="21"/>
-      <c r="O72" s="83"/>
+      <c r="O72" s="75"/>
     </row>
     <row r="73" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A73" s="20" t="s">
@@ -13610,7 +13610,7 @@
         <v>0.85000002384185702</v>
       </c>
       <c r="N73" s="21"/>
-      <c r="O73" s="83"/>
+      <c r="O73" s="75"/>
     </row>
     <row r="74" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A74" s="21"/>
@@ -13627,7 +13627,7 @@
       <c r="L74" s="21"/>
       <c r="M74" s="21"/>
       <c r="N74" s="21"/>
-      <c r="O74" s="83"/>
+      <c r="O74" s="75"/>
     </row>
     <row r="75" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A75" s="21"/>
@@ -13662,7 +13662,7 @@
       <c r="T75" s="51" t="s">
         <v>70</v>
       </c>
-      <c r="U75" s="78" t="s">
+      <c r="U75" s="70" t="s">
         <v>72</v>
       </c>
       <c r="V75" s="49" t="s">
@@ -13714,25 +13714,25 @@
       <c r="R76" s="33">
         <v>0.63648149200000004</v>
       </c>
-      <c r="S76" s="84">
+      <c r="S76" s="76">
         <v>0.33051121100000003</v>
       </c>
       <c r="T76" s="32">
         <v>70.60606061</v>
       </c>
-      <c r="U76" s="85">
+      <c r="U76" s="77">
         <v>100</v>
       </c>
       <c r="V76" s="33">
         <v>3.6358300000000001E-3</v>
       </c>
-      <c r="W76" s="84">
+      <c r="W76" s="76">
         <v>1.03353E-2</v>
       </c>
       <c r="X76" s="33">
         <v>8.7999999999999995E-2</v>
       </c>
-      <c r="Y76" s="84">
+      <c r="Y76" s="76">
         <v>0.28320000000000001</v>
       </c>
       <c r="Z76" s="32">
@@ -13778,25 +13778,25 @@
       <c r="R77" s="33">
         <v>0.63934216300000002</v>
       </c>
-      <c r="S77" s="84">
+      <c r="S77" s="76">
         <v>0.328036889</v>
       </c>
       <c r="T77" s="32">
         <v>70.60606061</v>
       </c>
-      <c r="U77" s="85">
+      <c r="U77" s="77">
         <v>100</v>
       </c>
       <c r="V77" s="33">
         <v>2.9528549999999999E-3</v>
       </c>
-      <c r="W77" s="84">
+      <c r="W77" s="76">
         <v>1.0672749E-2</v>
       </c>
       <c r="X77" s="33">
         <v>0.08</v>
       </c>
-      <c r="Y77" s="84">
+      <c r="Y77" s="76">
         <v>0.30359999999999998</v>
       </c>
       <c r="Z77" s="32">
@@ -13833,43 +13833,43 @@
       <c r="O78" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="P78" s="87">
+      <c r="P78" s="78">
         <v>7.9489345000000003E-2</v>
       </c>
-      <c r="Q78" s="88">
+      <c r="Q78" s="79">
         <v>0.108876977</v>
       </c>
-      <c r="R78" s="88">
+      <c r="R78" s="79">
         <v>5.7906882E-2</v>
       </c>
-      <c r="S78" s="89">
+      <c r="S78" s="80">
         <v>7.2164350000000002E-2</v>
       </c>
-      <c r="T78" s="90">
-        <v>0</v>
-      </c>
-      <c r="U78" s="91">
+      <c r="T78" s="81">
+        <v>0</v>
+      </c>
+      <c r="U78" s="82">
         <v>15.3030303</v>
       </c>
-      <c r="V78" s="88">
+      <c r="V78" s="79">
         <v>7.5502099999999999E-3</v>
       </c>
-      <c r="W78" s="89">
+      <c r="W78" s="80">
         <v>1.2874299000000001E-2</v>
       </c>
-      <c r="X78" s="88">
+      <c r="X78" s="79">
         <v>0.29520000000000002</v>
       </c>
-      <c r="Y78" s="89">
+      <c r="Y78" s="80">
         <v>0.84</v>
       </c>
-      <c r="Z78" s="90">
+      <c r="Z78" s="81">
         <v>41.363636360000001</v>
       </c>
-      <c r="AA78" s="90">
+      <c r="AA78" s="81">
         <v>4.55</v>
       </c>
-      <c r="AB78" s="90">
+      <c r="AB78" s="81">
         <v>17572.518039999999</v>
       </c>
       <c r="AD78" s="33">
@@ -13906,25 +13906,25 @@
       <c r="R79" s="33">
         <v>5.8641828E-2</v>
       </c>
-      <c r="S79" s="84">
+      <c r="S79" s="76">
         <v>7.1932098E-2</v>
       </c>
       <c r="T79" s="32">
         <v>0</v>
       </c>
-      <c r="U79" s="85">
+      <c r="U79" s="77">
         <v>14.621212119999999</v>
       </c>
       <c r="V79" s="33">
         <v>7.5502099999999999E-3</v>
       </c>
-      <c r="W79" s="84">
+      <c r="W79" s="76">
         <v>1.2874299000000001E-2</v>
       </c>
       <c r="X79" s="33">
         <v>0.29520000000000002</v>
       </c>
-      <c r="Y79" s="84">
+      <c r="Y79" s="76">
         <v>1.1305000000000001</v>
       </c>
       <c r="Z79" s="32">
@@ -13961,43 +13961,43 @@
       <c r="O80" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="P80" s="87">
+      <c r="P80" s="78">
         <v>2.4642293999999999E-2</v>
       </c>
-      <c r="Q80" s="88">
+      <c r="Q80" s="79">
         <v>7.4684096000000005E-2</v>
       </c>
-      <c r="R80" s="88">
+      <c r="R80" s="79">
         <v>6.3402049999999998E-3</v>
       </c>
-      <c r="S80" s="89">
+      <c r="S80" s="80">
         <v>5.4095860000000001E-3</v>
       </c>
-      <c r="T80" s="90">
-        <v>0</v>
-      </c>
-      <c r="U80" s="91">
+      <c r="T80" s="81">
+        <v>0</v>
+      </c>
+      <c r="U80" s="82">
         <v>8.5606060609999997</v>
       </c>
-      <c r="V80" s="88">
+      <c r="V80" s="79">
         <v>7.5502099999999999E-3</v>
       </c>
-      <c r="W80" s="89">
+      <c r="W80" s="80">
         <v>1.4027168E-2</v>
       </c>
-      <c r="X80" s="88">
+      <c r="X80" s="79">
         <v>0.29520000000000002</v>
       </c>
-      <c r="Y80" s="89">
+      <c r="Y80" s="80">
         <v>1.5960000000000001</v>
       </c>
-      <c r="Z80" s="90">
+      <c r="Z80" s="81">
         <v>20.795454549999999</v>
       </c>
-      <c r="AA80" s="90">
+      <c r="AA80" s="81">
         <v>2.2875000000000001</v>
       </c>
-      <c r="AB80" s="90">
+      <c r="AB80" s="81">
         <v>16124.11807</v>
       </c>
       <c r="AD80" s="33">
@@ -14053,25 +14053,25 @@
       <c r="R82" s="33">
         <v>6.3402049999999998E-3</v>
       </c>
-      <c r="S82" s="84">
+      <c r="S82" s="76">
         <v>5.4095860000000001E-3</v>
       </c>
       <c r="T82" s="32">
         <v>0</v>
       </c>
-      <c r="U82" s="85">
+      <c r="U82" s="77">
         <v>8.5606060609999997</v>
       </c>
       <c r="V82" s="33">
         <v>7.5502099999999999E-3</v>
       </c>
-      <c r="W82" s="84">
+      <c r="W82" s="76">
         <v>1.4027168E-2</v>
       </c>
       <c r="X82" s="33">
         <v>0.29520000000000002</v>
       </c>
-      <c r="Y82" s="84">
+      <c r="Y82" s="76">
         <v>1.5960000000000001</v>
       </c>
       <c r="Z82" s="32">
@@ -14094,43 +14094,43 @@
       <c r="O83" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="P83" s="87">
+      <c r="P83" s="78">
         <v>2.4642313999999998E-2</v>
       </c>
-      <c r="Q83" s="88">
+      <c r="Q83" s="79">
         <v>7.4684087999999996E-2</v>
       </c>
-      <c r="R83" s="88">
+      <c r="R83" s="79">
         <v>6.340226E-3</v>
       </c>
-      <c r="S83" s="89">
+      <c r="S83" s="80">
         <v>5.4095510000000003E-3</v>
       </c>
-      <c r="T83" s="90">
-        <v>0</v>
-      </c>
-      <c r="U83" s="91">
+      <c r="T83" s="81">
+        <v>0</v>
+      </c>
+      <c r="U83" s="82">
         <v>8.5606060609999997</v>
       </c>
-      <c r="V83" s="88">
+      <c r="V83" s="79">
         <v>7.5502099999999999E-3</v>
       </c>
-      <c r="W83" s="89">
+      <c r="W83" s="80">
         <v>1.4027168E-2</v>
       </c>
-      <c r="X83" s="88">
+      <c r="X83" s="79">
         <v>0.29520000000000002</v>
       </c>
-      <c r="Y83" s="89">
+      <c r="Y83" s="80">
         <v>1.444</v>
       </c>
-      <c r="Z83" s="90">
+      <c r="Z83" s="81">
         <v>20.9469697</v>
       </c>
-      <c r="AA83" s="90">
+      <c r="AA83" s="81">
         <v>2.3041666670000001</v>
       </c>
-      <c r="AB83" s="90">
+      <c r="AB83" s="81">
         <v>16124.12119</v>
       </c>
       <c r="AD83" s="33">
@@ -14142,6 +14142,14 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="E2:G2"/>
+    <mergeCell ref="H2:J2"/>
+    <mergeCell ref="K2:M2"/>
+    <mergeCell ref="B23:D23"/>
+    <mergeCell ref="E23:G23"/>
+    <mergeCell ref="H23:J23"/>
+    <mergeCell ref="K23:M23"/>
     <mergeCell ref="B44:D44"/>
     <mergeCell ref="E44:G44"/>
     <mergeCell ref="H44:J44"/>
@@ -14150,14 +14158,6 @@
     <mergeCell ref="E65:G65"/>
     <mergeCell ref="H65:J65"/>
     <mergeCell ref="K65:M65"/>
-    <mergeCell ref="B2:D2"/>
-    <mergeCell ref="E2:G2"/>
-    <mergeCell ref="H2:J2"/>
-    <mergeCell ref="K2:M2"/>
-    <mergeCell ref="B23:D23"/>
-    <mergeCell ref="E23:G23"/>
-    <mergeCell ref="H23:J23"/>
-    <mergeCell ref="K23:M23"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>

<commit_message>
fixed wrong multiple safety results and updated box plots and figure results
</commit_message>
<xml_diff>
--- a/results/compiled results.xlsx
+++ b/results/compiled results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\elish\Desktop\Aims Project\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{328B73AB-1AC0-4BCD-9E3C-AF7DFC5CD9B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EDC990E-44D4-4F8D-90BF-896C4D82D818}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{DA4D96B0-492C-4945-A9C4-EFCA6D6BC722}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{DA4D96B0-492C-4945-A9C4-EFCA6D6BC722}"/>
   </bookViews>
   <sheets>
     <sheet name="Dynamic results" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="733" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="721" uniqueCount="83">
   <si>
     <t xml:space="preserve">Model </t>
   </si>
@@ -518,7 +518,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="91">
+  <cellXfs count="92">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -736,6 +736,9 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="14" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1130,26 +1133,26 @@
       <c r="A2" s="67" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="83" t="s">
+      <c r="B2" s="84" t="s">
         <v>24</v>
       </c>
-      <c r="C2" s="84"/>
-      <c r="D2" s="85"/>
-      <c r="E2" s="84" t="s">
+      <c r="C2" s="85"/>
+      <c r="D2" s="86"/>
+      <c r="E2" s="85" t="s">
         <v>25</v>
       </c>
-      <c r="F2" s="84"/>
-      <c r="G2" s="85"/>
-      <c r="H2" s="84" t="s">
+      <c r="F2" s="85"/>
+      <c r="G2" s="86"/>
+      <c r="H2" s="85" t="s">
         <v>26</v>
       </c>
-      <c r="I2" s="84"/>
-      <c r="J2" s="84"/>
-      <c r="K2" s="83" t="s">
+      <c r="I2" s="85"/>
+      <c r="J2" s="85"/>
+      <c r="K2" s="84" t="s">
         <v>27</v>
       </c>
-      <c r="L2" s="84"/>
-      <c r="M2" s="84"/>
+      <c r="L2" s="85"/>
+      <c r="M2" s="85"/>
       <c r="N2" s="1" t="s">
         <v>56</v>
       </c>
@@ -1280,17 +1283,47 @@
       <c r="N4" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="O4" s="34"/>
-      <c r="P4" s="34"/>
-      <c r="Q4" s="34"/>
-      <c r="R4" s="34"/>
-      <c r="S4" s="34"/>
-      <c r="T4" s="34"/>
-      <c r="U4" s="34"/>
-      <c r="V4" s="34"/>
+      <c r="O4" s="34">
+        <v>2.0934814E-2</v>
+      </c>
+      <c r="P4" s="34">
+        <v>6.9102947999999997E-2</v>
+      </c>
+      <c r="Q4" s="34">
+        <v>3.471174E-3</v>
+      </c>
+      <c r="R4" s="34">
+        <v>5.1547609999999999E-3</v>
+      </c>
+      <c r="S4" s="34">
+        <v>0</v>
+      </c>
+      <c r="T4" s="34">
+        <v>0</v>
+      </c>
+      <c r="U4" s="34">
+        <v>0</v>
+      </c>
+      <c r="V4" s="34">
+        <v>0</v>
+      </c>
       <c r="W4" s="34"/>
       <c r="X4" s="34"/>
-      <c r="AC4" s="34"/>
+      <c r="Y4" s="2">
+        <v>1.2800000000000001E-2</v>
+      </c>
+      <c r="Z4" s="31">
+        <v>3.7720889999999998</v>
+      </c>
+      <c r="AA4" s="35">
+        <v>10.62727273</v>
+      </c>
+      <c r="AB4" s="35">
+        <v>1.169</v>
+      </c>
+      <c r="AC4" s="34">
+        <v>13031.07163</v>
+      </c>
     </row>
     <row r="5" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
@@ -1719,41 +1752,41 @@
       <c r="N17" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="O17" s="34" t="s">
-        <v>34</v>
-      </c>
-      <c r="P17" s="34" t="s">
-        <v>34</v>
-      </c>
-      <c r="Q17" s="34" t="s">
-        <v>34</v>
-      </c>
-      <c r="R17" s="59" t="s">
-        <v>34</v>
-      </c>
-      <c r="S17" s="34" t="s">
-        <v>34</v>
-      </c>
-      <c r="T17" s="59" t="s">
-        <v>34</v>
-      </c>
-      <c r="U17" s="73" t="s">
-        <v>34</v>
-      </c>
-      <c r="V17" s="34" t="s">
-        <v>34</v>
-      </c>
-      <c r="W17" s="59" t="s">
-        <v>34</v>
-      </c>
-      <c r="X17" s="34" t="s">
-        <v>34</v>
-      </c>
-      <c r="Y17" s="34" t="s">
-        <v>34</v>
-      </c>
-      <c r="Z17" s="34" t="s">
-        <v>34</v>
+      <c r="O17" s="34">
+        <v>2.0934814E-2</v>
+      </c>
+      <c r="P17" s="34">
+        <v>6.9102947999999997E-2</v>
+      </c>
+      <c r="Q17" s="34">
+        <v>3.471174E-3</v>
+      </c>
+      <c r="R17" s="59">
+        <v>5.1547609999999999E-3</v>
+      </c>
+      <c r="S17" s="38">
+        <v>0</v>
+      </c>
+      <c r="T17" s="39">
+        <v>0</v>
+      </c>
+      <c r="U17" s="83">
+        <v>0</v>
+      </c>
+      <c r="V17" s="3">
+        <v>1.2800000000000001E-2</v>
+      </c>
+      <c r="W17" s="3">
+        <v>3.7720889999999998</v>
+      </c>
+      <c r="X17" s="39">
+        <v>10.62727273</v>
+      </c>
+      <c r="Y17" s="38">
+        <v>1.169</v>
+      </c>
+      <c r="Z17" s="39">
+        <v>13031.07163</v>
       </c>
       <c r="AA17" s="36" t="s">
         <v>34</v>
@@ -2045,26 +2078,26 @@
       <c r="A27" s="67" t="s">
         <v>0</v>
       </c>
-      <c r="B27" s="83" t="s">
+      <c r="B27" s="84" t="s">
         <v>24</v>
       </c>
-      <c r="C27" s="84"/>
-      <c r="D27" s="85"/>
-      <c r="E27" s="84" t="s">
+      <c r="C27" s="85"/>
+      <c r="D27" s="86"/>
+      <c r="E27" s="85" t="s">
         <v>25</v>
       </c>
-      <c r="F27" s="84"/>
-      <c r="G27" s="85"/>
-      <c r="H27" s="84" t="s">
+      <c r="F27" s="85"/>
+      <c r="G27" s="86"/>
+      <c r="H27" s="85" t="s">
         <v>26</v>
       </c>
-      <c r="I27" s="84"/>
-      <c r="J27" s="84"/>
-      <c r="K27" s="83" t="s">
+      <c r="I27" s="85"/>
+      <c r="J27" s="85"/>
+      <c r="K27" s="84" t="s">
         <v>27</v>
       </c>
-      <c r="L27" s="84"/>
-      <c r="M27" s="84"/>
+      <c r="L27" s="85"/>
+      <c r="M27" s="85"/>
       <c r="O27" s="34" t="s">
         <v>34</v>
       </c>
@@ -2814,26 +2847,26 @@
       <c r="A47" s="67" t="s">
         <v>0</v>
       </c>
-      <c r="B47" s="83" t="s">
+      <c r="B47" s="84" t="s">
         <v>24</v>
       </c>
-      <c r="C47" s="84"/>
-      <c r="D47" s="85"/>
-      <c r="E47" s="84" t="s">
+      <c r="C47" s="85"/>
+      <c r="D47" s="86"/>
+      <c r="E47" s="85" t="s">
         <v>25</v>
       </c>
-      <c r="F47" s="84"/>
-      <c r="G47" s="85"/>
-      <c r="H47" s="84" t="s">
+      <c r="F47" s="85"/>
+      <c r="G47" s="86"/>
+      <c r="H47" s="85" t="s">
         <v>26</v>
       </c>
-      <c r="I47" s="84"/>
-      <c r="J47" s="84"/>
-      <c r="K47" s="83" t="s">
+      <c r="I47" s="85"/>
+      <c r="J47" s="85"/>
+      <c r="K47" s="84" t="s">
         <v>27</v>
       </c>
-      <c r="L47" s="84"/>
-      <c r="M47" s="84"/>
+      <c r="L47" s="85"/>
+      <c r="M47" s="85"/>
       <c r="T47" s="31"/>
     </row>
     <row r="48" spans="1:29" x14ac:dyDescent="0.3">
@@ -3587,26 +3620,26 @@
       <c r="A70" s="67" t="s">
         <v>0</v>
       </c>
-      <c r="B70" s="83" t="s">
+      <c r="B70" s="84" t="s">
         <v>24</v>
       </c>
-      <c r="C70" s="84"/>
-      <c r="D70" s="85"/>
-      <c r="E70" s="84" t="s">
+      <c r="C70" s="85"/>
+      <c r="D70" s="86"/>
+      <c r="E70" s="85" t="s">
         <v>25</v>
       </c>
-      <c r="F70" s="84"/>
-      <c r="G70" s="85"/>
-      <c r="H70" s="84" t="s">
+      <c r="F70" s="85"/>
+      <c r="G70" s="86"/>
+      <c r="H70" s="85" t="s">
         <v>26</v>
       </c>
-      <c r="I70" s="84"/>
-      <c r="J70" s="84"/>
-      <c r="K70" s="83" t="s">
+      <c r="I70" s="85"/>
+      <c r="J70" s="85"/>
+      <c r="K70" s="84" t="s">
         <v>27</v>
       </c>
-      <c r="L70" s="84"/>
-      <c r="M70" s="84"/>
+      <c r="L70" s="85"/>
+      <c r="M70" s="85"/>
       <c r="T70" s="31"/>
     </row>
     <row r="71" spans="1:27" x14ac:dyDescent="0.3">
@@ -4424,6 +4457,14 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="B70:D70"/>
+    <mergeCell ref="E70:G70"/>
+    <mergeCell ref="H70:J70"/>
+    <mergeCell ref="K70:M70"/>
+    <mergeCell ref="B47:D47"/>
+    <mergeCell ref="E47:G47"/>
+    <mergeCell ref="H47:J47"/>
+    <mergeCell ref="K47:M47"/>
     <mergeCell ref="B2:D2"/>
     <mergeCell ref="E2:G2"/>
     <mergeCell ref="H2:J2"/>
@@ -4432,14 +4473,6 @@
     <mergeCell ref="E27:G27"/>
     <mergeCell ref="H27:J27"/>
     <mergeCell ref="K27:M27"/>
-    <mergeCell ref="B70:D70"/>
-    <mergeCell ref="E70:G70"/>
-    <mergeCell ref="H70:J70"/>
-    <mergeCell ref="K70:M70"/>
-    <mergeCell ref="B47:D47"/>
-    <mergeCell ref="E47:G47"/>
-    <mergeCell ref="H47:J47"/>
-    <mergeCell ref="K47:M47"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4857,48 +4890,48 @@
       <c r="A2" s="67" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="83" t="s">
+      <c r="B2" s="84" t="s">
         <v>24</v>
       </c>
-      <c r="C2" s="84"/>
-      <c r="D2" s="85"/>
-      <c r="E2" s="84" t="s">
+      <c r="C2" s="85"/>
+      <c r="D2" s="86"/>
+      <c r="E2" s="85" t="s">
         <v>25</v>
       </c>
-      <c r="F2" s="84"/>
-      <c r="G2" s="85"/>
-      <c r="H2" s="84" t="s">
+      <c r="F2" s="85"/>
+      <c r="G2" s="86"/>
+      <c r="H2" s="85" t="s">
         <v>26</v>
       </c>
-      <c r="I2" s="84"/>
-      <c r="J2" s="84"/>
-      <c r="K2" s="83" t="s">
+      <c r="I2" s="85"/>
+      <c r="J2" s="85"/>
+      <c r="K2" s="84" t="s">
         <v>27</v>
       </c>
-      <c r="L2" s="84"/>
-      <c r="M2" s="84"/>
+      <c r="L2" s="85"/>
+      <c r="M2" s="85"/>
     </row>
     <row r="3" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
         <v>1</v>
       </c>
       <c r="B3" s="15">
-        <v>0.28999999165534901</v>
+        <v>0.3</v>
       </c>
       <c r="C3" s="16">
-        <v>0.270000010728836</v>
+        <v>-0.25</v>
       </c>
       <c r="D3" s="17">
-        <v>-0.46000000834464999</v>
+        <v>0.25</v>
       </c>
       <c r="E3" s="16">
-        <v>0.490000009536743</v>
+        <v>0.5</v>
       </c>
       <c r="F3" s="16">
-        <v>0.46999999880790699</v>
+        <v>0.25</v>
       </c>
       <c r="G3" s="17">
-        <v>1.12000000476837</v>
+        <v>0.45</v>
       </c>
       <c r="H3" s="16">
         <v>-0.855000019073486</v>
@@ -5325,43 +5358,43 @@
         <v>1</v>
       </c>
       <c r="P14" s="3">
-        <v>0.20880342800000001</v>
+        <v>0.205705302011014</v>
       </c>
       <c r="Q14" s="3">
-        <v>3.2646891999999997E-2</v>
+        <v>0.10480522342236601</v>
       </c>
       <c r="R14" s="3">
-        <v>0.207741801</v>
+        <v>0.20691336023293999</v>
       </c>
       <c r="S14" s="58">
-        <v>3.1069445000000001E-2</v>
+        <v>0.10594480432336199</v>
       </c>
       <c r="T14" s="31">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="U14" s="69">
         <v>0</v>
       </c>
       <c r="V14" s="3">
-        <v>1.81694E-3</v>
+        <v>4.7640653619619E-2</v>
       </c>
       <c r="W14" s="58">
-        <v>5.6548668000000003E-2</v>
+        <v>5.6548667764616201E-2</v>
       </c>
       <c r="X14" s="3">
-        <v>0.02</v>
+        <v>6.3199999999999895E-2</v>
       </c>
       <c r="Y14" s="58">
-        <v>3.8163360000000002</v>
+        <v>3.81633599999999</v>
       </c>
       <c r="Z14" s="31">
-        <v>100</v>
+        <v>93.6</v>
       </c>
       <c r="AA14" s="31">
-        <v>11</v>
+        <v>10.295999999999999</v>
       </c>
       <c r="AB14" s="31">
-        <v>5331.3170570000002</v>
+        <v>8331.0174627980305</v>
       </c>
       <c r="AD14" s="3">
         <v>5.6548668000000003E-2</v>
@@ -5375,43 +5408,43 @@
         <v>2</v>
       </c>
       <c r="P15" s="3">
-        <v>0.208803427881982</v>
+        <v>0.205705302011014</v>
       </c>
       <c r="Q15" s="3">
-        <v>3.2646891997723602E-2</v>
+        <v>0.10480522342236601</v>
       </c>
       <c r="R15" s="3">
-        <v>0.20774180079319299</v>
+        <v>0.20691336023293999</v>
       </c>
       <c r="S15" s="58">
-        <v>3.1069445262637101E-2</v>
+        <v>0.10594480432336199</v>
       </c>
       <c r="T15" s="31">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="U15" s="69">
         <v>0</v>
       </c>
       <c r="V15" s="3">
-        <v>1.81694009620145E-3</v>
+        <v>4.7640653619619E-2</v>
       </c>
       <c r="W15" s="58">
         <v>5.6548667764616201E-2</v>
       </c>
       <c r="X15" s="3">
-        <v>0.02</v>
+        <v>6.3199999999999895E-2</v>
       </c>
       <c r="Y15" s="58">
         <v>3.81633599999999</v>
       </c>
       <c r="Z15" s="31">
-        <v>100</v>
+        <v>93.6</v>
       </c>
       <c r="AA15" s="31">
-        <v>11</v>
+        <v>10.295999999999999</v>
       </c>
       <c r="AB15" s="31">
-        <v>5331.3170567901097</v>
+        <v>8331.0174627980305</v>
       </c>
       <c r="AD15" s="3">
         <v>5.6548667764616201E-2</v>
@@ -5729,26 +5762,26 @@
       <c r="A24" s="67" t="s">
         <v>0</v>
       </c>
-      <c r="B24" s="83" t="s">
+      <c r="B24" s="84" t="s">
         <v>24</v>
       </c>
-      <c r="C24" s="84"/>
-      <c r="D24" s="85"/>
-      <c r="E24" s="84" t="s">
+      <c r="C24" s="85"/>
+      <c r="D24" s="86"/>
+      <c r="E24" s="85" t="s">
         <v>25</v>
       </c>
-      <c r="F24" s="84"/>
-      <c r="G24" s="85"/>
-      <c r="H24" s="84" t="s">
+      <c r="F24" s="85"/>
+      <c r="G24" s="86"/>
+      <c r="H24" s="85" t="s">
         <v>26</v>
       </c>
-      <c r="I24" s="84"/>
-      <c r="J24" s="84"/>
-      <c r="K24" s="83" t="s">
+      <c r="I24" s="85"/>
+      <c r="J24" s="85"/>
+      <c r="K24" s="84" t="s">
         <v>27</v>
       </c>
-      <c r="L24" s="84"/>
-      <c r="M24" s="84"/>
+      <c r="L24" s="85"/>
+      <c r="M24" s="85"/>
     </row>
     <row r="25" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A25" s="14" t="s">
@@ -6531,26 +6564,26 @@
       <c r="A44" s="67" t="s">
         <v>0</v>
       </c>
-      <c r="B44" s="83" t="s">
+      <c r="B44" s="84" t="s">
         <v>24</v>
       </c>
-      <c r="C44" s="84"/>
-      <c r="D44" s="85"/>
-      <c r="E44" s="84" t="s">
+      <c r="C44" s="85"/>
+      <c r="D44" s="86"/>
+      <c r="E44" s="85" t="s">
         <v>25</v>
       </c>
-      <c r="F44" s="84"/>
-      <c r="G44" s="85"/>
-      <c r="H44" s="84" t="s">
+      <c r="F44" s="85"/>
+      <c r="G44" s="86"/>
+      <c r="H44" s="85" t="s">
         <v>26</v>
       </c>
-      <c r="I44" s="84"/>
-      <c r="J44" s="84"/>
-      <c r="K44" s="83" t="s">
+      <c r="I44" s="85"/>
+      <c r="J44" s="85"/>
+      <c r="K44" s="84" t="s">
         <v>27</v>
       </c>
-      <c r="L44" s="84"/>
-      <c r="M44" s="84"/>
+      <c r="L44" s="85"/>
+      <c r="M44" s="85"/>
     </row>
     <row r="45" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A45" s="14" t="s">
@@ -7333,26 +7366,26 @@
       <c r="A65" s="68" t="s">
         <v>0</v>
       </c>
-      <c r="B65" s="86" t="s">
+      <c r="B65" s="87" t="s">
         <v>24</v>
       </c>
-      <c r="C65" s="87"/>
-      <c r="D65" s="88"/>
-      <c r="E65" s="89" t="s">
+      <c r="C65" s="88"/>
+      <c r="D65" s="89"/>
+      <c r="E65" s="90" t="s">
         <v>25</v>
       </c>
-      <c r="F65" s="87"/>
-      <c r="G65" s="88"/>
-      <c r="H65" s="89" t="s">
+      <c r="F65" s="88"/>
+      <c r="G65" s="89"/>
+      <c r="H65" s="90" t="s">
         <v>26</v>
       </c>
-      <c r="I65" s="87"/>
-      <c r="J65" s="90"/>
-      <c r="K65" s="86" t="s">
+      <c r="I65" s="88"/>
+      <c r="J65" s="91"/>
+      <c r="K65" s="87" t="s">
         <v>27</v>
       </c>
-      <c r="L65" s="87"/>
-      <c r="M65" s="87"/>
+      <c r="L65" s="88"/>
+      <c r="M65" s="88"/>
       <c r="N65" s="21"/>
       <c r="O65" s="21"/>
     </row>
@@ -8206,6 +8239,14 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="B65:D65"/>
+    <mergeCell ref="E65:G65"/>
+    <mergeCell ref="H65:J65"/>
+    <mergeCell ref="K65:M65"/>
+    <mergeCell ref="B44:D44"/>
+    <mergeCell ref="E44:G44"/>
+    <mergeCell ref="H44:J44"/>
+    <mergeCell ref="K44:M44"/>
     <mergeCell ref="B2:D2"/>
     <mergeCell ref="E2:G2"/>
     <mergeCell ref="H2:J2"/>
@@ -8214,14 +8255,6 @@
     <mergeCell ref="E24:G24"/>
     <mergeCell ref="H24:J24"/>
     <mergeCell ref="K24:M24"/>
-    <mergeCell ref="B65:D65"/>
-    <mergeCell ref="E65:G65"/>
-    <mergeCell ref="H65:J65"/>
-    <mergeCell ref="K65:M65"/>
-    <mergeCell ref="B44:D44"/>
-    <mergeCell ref="E44:G44"/>
-    <mergeCell ref="H44:J44"/>
-    <mergeCell ref="K44:M44"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -8257,26 +8290,26 @@
       <c r="A2" s="67" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="83" t="s">
+      <c r="B2" s="84" t="s">
         <v>24</v>
       </c>
-      <c r="C2" s="84"/>
-      <c r="D2" s="85"/>
-      <c r="E2" s="84" t="s">
+      <c r="C2" s="85"/>
+      <c r="D2" s="86"/>
+      <c r="E2" s="85" t="s">
         <v>25</v>
       </c>
-      <c r="F2" s="84"/>
-      <c r="G2" s="85"/>
-      <c r="H2" s="84" t="s">
+      <c r="F2" s="85"/>
+      <c r="G2" s="86"/>
+      <c r="H2" s="85" t="s">
         <v>26</v>
       </c>
-      <c r="I2" s="84"/>
-      <c r="J2" s="84"/>
-      <c r="K2" s="83" t="s">
+      <c r="I2" s="85"/>
+      <c r="J2" s="85"/>
+      <c r="K2" s="84" t="s">
         <v>27</v>
       </c>
-      <c r="L2" s="84"/>
-      <c r="M2" s="84"/>
+      <c r="L2" s="85"/>
+      <c r="M2" s="85"/>
     </row>
     <row r="3" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
@@ -8981,26 +9014,26 @@
       <c r="A23" s="67" t="s">
         <v>0</v>
       </c>
-      <c r="B23" s="83" t="s">
+      <c r="B23" s="84" t="s">
         <v>24</v>
       </c>
-      <c r="C23" s="84"/>
-      <c r="D23" s="85"/>
-      <c r="E23" s="84" t="s">
+      <c r="C23" s="85"/>
+      <c r="D23" s="86"/>
+      <c r="E23" s="85" t="s">
         <v>25</v>
       </c>
-      <c r="F23" s="84"/>
-      <c r="G23" s="85"/>
-      <c r="H23" s="84" t="s">
+      <c r="F23" s="85"/>
+      <c r="G23" s="86"/>
+      <c r="H23" s="85" t="s">
         <v>26</v>
       </c>
-      <c r="I23" s="84"/>
-      <c r="J23" s="84"/>
-      <c r="K23" s="83" t="s">
+      <c r="I23" s="85"/>
+      <c r="J23" s="85"/>
+      <c r="K23" s="84" t="s">
         <v>27</v>
       </c>
-      <c r="L23" s="84"/>
-      <c r="M23" s="84"/>
+      <c r="L23" s="85"/>
+      <c r="M23" s="85"/>
     </row>
     <row r="24" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A24" s="14" t="s">
@@ -9658,26 +9691,26 @@
       <c r="A44" s="67" t="s">
         <v>0</v>
       </c>
-      <c r="B44" s="83" t="s">
+      <c r="B44" s="84" t="s">
         <v>24</v>
       </c>
-      <c r="C44" s="84"/>
-      <c r="D44" s="85"/>
-      <c r="E44" s="84" t="s">
+      <c r="C44" s="85"/>
+      <c r="D44" s="86"/>
+      <c r="E44" s="85" t="s">
         <v>25</v>
       </c>
-      <c r="F44" s="84"/>
-      <c r="G44" s="85"/>
-      <c r="H44" s="84" t="s">
+      <c r="F44" s="85"/>
+      <c r="G44" s="86"/>
+      <c r="H44" s="85" t="s">
         <v>26</v>
       </c>
-      <c r="I44" s="84"/>
-      <c r="J44" s="84"/>
-      <c r="K44" s="83" t="s">
+      <c r="I44" s="85"/>
+      <c r="J44" s="85"/>
+      <c r="K44" s="84" t="s">
         <v>27</v>
       </c>
-      <c r="L44" s="84"/>
-      <c r="M44" s="84"/>
+      <c r="L44" s="85"/>
+      <c r="M44" s="85"/>
     </row>
     <row r="45" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A45" s="14" t="s">
@@ -10335,26 +10368,26 @@
       <c r="A64" s="68" t="s">
         <v>0</v>
       </c>
-      <c r="B64" s="86" t="s">
+      <c r="B64" s="87" t="s">
         <v>24</v>
       </c>
-      <c r="C64" s="87"/>
-      <c r="D64" s="88"/>
-      <c r="E64" s="89" t="s">
+      <c r="C64" s="88"/>
+      <c r="D64" s="89"/>
+      <c r="E64" s="90" t="s">
         <v>25</v>
       </c>
-      <c r="F64" s="87"/>
-      <c r="G64" s="88"/>
-      <c r="H64" s="89" t="s">
+      <c r="F64" s="88"/>
+      <c r="G64" s="89"/>
+      <c r="H64" s="90" t="s">
         <v>26</v>
       </c>
-      <c r="I64" s="87"/>
-      <c r="J64" s="90"/>
-      <c r="K64" s="86" t="s">
+      <c r="I64" s="88"/>
+      <c r="J64" s="91"/>
+      <c r="K64" s="87" t="s">
         <v>27</v>
       </c>
-      <c r="L64" s="87"/>
-      <c r="M64" s="87"/>
+      <c r="L64" s="88"/>
+      <c r="M64" s="88"/>
       <c r="N64" s="21"/>
       <c r="O64" s="75"/>
     </row>
@@ -11208,6 +11241,14 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="B44:D44"/>
+    <mergeCell ref="E44:G44"/>
+    <mergeCell ref="H44:J44"/>
+    <mergeCell ref="K44:M44"/>
+    <mergeCell ref="B64:D64"/>
+    <mergeCell ref="E64:G64"/>
+    <mergeCell ref="H64:J64"/>
+    <mergeCell ref="K64:M64"/>
     <mergeCell ref="B2:D2"/>
     <mergeCell ref="E2:G2"/>
     <mergeCell ref="H2:J2"/>
@@ -11216,14 +11257,6 @@
     <mergeCell ref="E23:G23"/>
     <mergeCell ref="H23:J23"/>
     <mergeCell ref="K23:M23"/>
-    <mergeCell ref="B44:D44"/>
-    <mergeCell ref="E44:G44"/>
-    <mergeCell ref="H44:J44"/>
-    <mergeCell ref="K44:M44"/>
-    <mergeCell ref="B64:D64"/>
-    <mergeCell ref="E64:G64"/>
-    <mergeCell ref="H64:J64"/>
-    <mergeCell ref="K64:M64"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -11260,26 +11293,26 @@
       <c r="A2" s="67" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="83" t="s">
+      <c r="B2" s="84" t="s">
         <v>24</v>
       </c>
-      <c r="C2" s="84"/>
-      <c r="D2" s="85"/>
-      <c r="E2" s="84" t="s">
+      <c r="C2" s="85"/>
+      <c r="D2" s="86"/>
+      <c r="E2" s="85" t="s">
         <v>25</v>
       </c>
-      <c r="F2" s="84"/>
-      <c r="G2" s="85"/>
-      <c r="H2" s="84" t="s">
+      <c r="F2" s="85"/>
+      <c r="G2" s="86"/>
+      <c r="H2" s="85" t="s">
         <v>26</v>
       </c>
-      <c r="I2" s="84"/>
-      <c r="J2" s="84"/>
-      <c r="K2" s="83" t="s">
+      <c r="I2" s="85"/>
+      <c r="J2" s="85"/>
+      <c r="K2" s="84" t="s">
         <v>27</v>
       </c>
-      <c r="L2" s="84"/>
-      <c r="M2" s="84"/>
+      <c r="L2" s="85"/>
+      <c r="M2" s="85"/>
     </row>
     <row r="3" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
@@ -11984,26 +12017,26 @@
       <c r="A23" s="67" t="s">
         <v>0</v>
       </c>
-      <c r="B23" s="83" t="s">
+      <c r="B23" s="84" t="s">
         <v>24</v>
       </c>
-      <c r="C23" s="84"/>
-      <c r="D23" s="85"/>
-      <c r="E23" s="84" t="s">
+      <c r="C23" s="85"/>
+      <c r="D23" s="86"/>
+      <c r="E23" s="85" t="s">
         <v>25</v>
       </c>
-      <c r="F23" s="84"/>
-      <c r="G23" s="85"/>
-      <c r="H23" s="84" t="s">
+      <c r="F23" s="85"/>
+      <c r="G23" s="86"/>
+      <c r="H23" s="85" t="s">
         <v>26</v>
       </c>
-      <c r="I23" s="84"/>
-      <c r="J23" s="84"/>
-      <c r="K23" s="83" t="s">
+      <c r="I23" s="85"/>
+      <c r="J23" s="85"/>
+      <c r="K23" s="84" t="s">
         <v>27</v>
       </c>
-      <c r="L23" s="84"/>
-      <c r="M23" s="84"/>
+      <c r="L23" s="85"/>
+      <c r="M23" s="85"/>
     </row>
     <row r="24" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A24" s="14" t="s">
@@ -12661,26 +12694,26 @@
       <c r="A44" s="67" t="s">
         <v>0</v>
       </c>
-      <c r="B44" s="83" t="s">
+      <c r="B44" s="84" t="s">
         <v>24</v>
       </c>
-      <c r="C44" s="84"/>
-      <c r="D44" s="85"/>
-      <c r="E44" s="84" t="s">
+      <c r="C44" s="85"/>
+      <c r="D44" s="86"/>
+      <c r="E44" s="85" t="s">
         <v>25</v>
       </c>
-      <c r="F44" s="84"/>
-      <c r="G44" s="85"/>
-      <c r="H44" s="84" t="s">
+      <c r="F44" s="85"/>
+      <c r="G44" s="86"/>
+      <c r="H44" s="85" t="s">
         <v>26</v>
       </c>
-      <c r="I44" s="84"/>
-      <c r="J44" s="84"/>
-      <c r="K44" s="83" t="s">
+      <c r="I44" s="85"/>
+      <c r="J44" s="85"/>
+      <c r="K44" s="84" t="s">
         <v>27</v>
       </c>
-      <c r="L44" s="84"/>
-      <c r="M44" s="84"/>
+      <c r="L44" s="85"/>
+      <c r="M44" s="85"/>
     </row>
     <row r="45" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A45" s="14" t="s">
@@ -13269,26 +13302,26 @@
       <c r="A65" s="68" t="s">
         <v>0</v>
       </c>
-      <c r="B65" s="86" t="s">
+      <c r="B65" s="87" t="s">
         <v>24</v>
       </c>
-      <c r="C65" s="87"/>
-      <c r="D65" s="88"/>
-      <c r="E65" s="89" t="s">
+      <c r="C65" s="88"/>
+      <c r="D65" s="89"/>
+      <c r="E65" s="90" t="s">
         <v>25</v>
       </c>
-      <c r="F65" s="87"/>
-      <c r="G65" s="88"/>
-      <c r="H65" s="89" t="s">
+      <c r="F65" s="88"/>
+      <c r="G65" s="89"/>
+      <c r="H65" s="90" t="s">
         <v>26</v>
       </c>
-      <c r="I65" s="87"/>
-      <c r="J65" s="90"/>
-      <c r="K65" s="86" t="s">
+      <c r="I65" s="88"/>
+      <c r="J65" s="91"/>
+      <c r="K65" s="87" t="s">
         <v>27</v>
       </c>
-      <c r="L65" s="87"/>
-      <c r="M65" s="87"/>
+      <c r="L65" s="88"/>
+      <c r="M65" s="88"/>
       <c r="N65" s="21"/>
       <c r="O65" s="75"/>
     </row>
@@ -14142,6 +14175,14 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="B44:D44"/>
+    <mergeCell ref="E44:G44"/>
+    <mergeCell ref="H44:J44"/>
+    <mergeCell ref="K44:M44"/>
+    <mergeCell ref="B65:D65"/>
+    <mergeCell ref="E65:G65"/>
+    <mergeCell ref="H65:J65"/>
+    <mergeCell ref="K65:M65"/>
     <mergeCell ref="B2:D2"/>
     <mergeCell ref="E2:G2"/>
     <mergeCell ref="H2:J2"/>
@@ -14150,14 +14191,6 @@
     <mergeCell ref="E23:G23"/>
     <mergeCell ref="H23:J23"/>
     <mergeCell ref="K23:M23"/>
-    <mergeCell ref="B44:D44"/>
-    <mergeCell ref="E44:G44"/>
-    <mergeCell ref="H44:J44"/>
-    <mergeCell ref="K44:M44"/>
-    <mergeCell ref="B65:D65"/>
-    <mergeCell ref="E65:G65"/>
-    <mergeCell ref="H65:J65"/>
-    <mergeCell ref="K65:M65"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>